<commit_message>
feat: add Combined sheet to PDTs.xlsx and ignore per-cell-line workbooks
PDTs.xlsx now has four sheets (MCF7, HL60, NTERA2, Combined).
The Combined sheet contains the union of unique substrates per kinase
across all three cell lines (103 kinases, 28 586 substrate entries).

Also exclude MCF7/HL60/NTERA2_PDTs.xlsx from version control via
.gitignore — the consolidated PDTs.xlsx is the canonical reference.
</commit_message>
<xml_diff>
--- a/PDTs.xlsx
+++ b/PDTs.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCF7" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HL60" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NTERA2" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Combined" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4449,4 +4450,1580 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C104"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>kinase</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>substrates</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AAK1</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>AMBRA1(S1205);CTPS1(Y567);CTU2(S419);DENND4A(S1256);MARK2(S456);MEPCE(T213);PPHLN1(S201);RBL2(S413)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ABL1</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>158</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>AFDN(T1330);AKT1S1(T246);ALDH5A1(S121);ANKRD17(S2401);AP1M1(T154);ARHGAP17(S162);ARHGEF11(S255);ARHGEF5(S606);ARID1A(S772);ASAP2(S822);ASCC3(S2195);ASIC3(S39);ATF7(S434);ATF7IP(S474);ATF7IP(S477);ATXN2L(S32);BICRAL(S675);CAMKV(T435);CAMSAP1(S793);CAMSAP3(S814);CARHSP1(S30);CARHSP1(S32);CDC6(S106);CDK18(S117);CRAMP1(S1268);CRKL(Y207);CRTC1(S172);CRTC1(T149);CSNK1D(S331);DCLRE1C(S518);DDX17(S571);DOCK5(S1834);DUSP27(S965);EEF2K(S72);EEF2K(S74);EEF2K(Y69);EIF2B1(S105);EIF2B1(S107);EIF3A(S1188);EIF4ENIF1(S752);EPX(S670);EPX(S672);ETV6(S203);EVPL(S2025);FAM120A(Y452);FAM189A1(S18);FAM193B(S785);FAM234B(S62);FAM47A(S258);FBXL15(S262);FOXK1(S223);FUBP3(S569);GJA1(S365);GLCCI1(S30);GRAMD1B(S274);GSK3B(S25);GSK3B(S9);GTF2F1(T389);HIPK1(T351);HIPK2(T360);HUWE1(T2889);IKBKB(S672);IRF2BPL(S215);ITSN1(S315);KIAA1522(S327);KIFC1(S26);KIFC1(S349);KIFC1(S351);LARP4(T389);LINC00322(S228);LLGL2(S1000);MAP3K11(S524);MARCKS(S167);MARK2(S486);MCRIP2(S82);MED13(S890);METTL1(S27);MFSD10(S270);MNAT1(S279);MON1B(S59);MON1B(S61);MPHOSPH8(S403);MTA1(S576);MTMR14(S530);MYC(S62);MYCN(S62);MYO18A(S102);NAA30(S39);NECTIN1(T391);NPM1(S70);NSRP1(S33);NSUN2(S456);NSUN2(S473);PAK2(S141);PAK4(T207);PALD1(S406);PALM3(S143);PARD3(S174);PCBP2(S189);PDS5B(S1358);PHACTR1(S505);PKN1(S562);PKP4(S337);PKP4(S406);POLH(S379);PPP1R12A(S903);PPP1R13L(S102);PRAG1(S889);PTPN13(S214);PTPN22(S692);PXN(S258);RAB3IP(S157);RBL2(S639);RBM10(S797);RCSD1(S116);RCSD1(S120);RFX7(S225);RFX7(S424);RHBDF2(S113);RIOK1(S22);RPS6(S235);RREB1(S42);SHC3(S474);SHROOM3(S816);SIRT1(S27);SKIV2L(S133);SLC4A7(S556);SLC9A3R1(S269);SNIP1(S35);SRGAP1(S932);SRRM2(S1404);SRRM2(S2121);SRRM2(S322);SRSF7(S167);STK33(S470);TBKBP1(S365);TEX2(S266);TNS1(S1269);TRAFD1(S470);TRAPPC12(S184);TRIM37(S773);TRIO(S1724);TVP23C(S223);USP1(S67);USP32(S1423);WDR20(S434);XPR1(S668);ZC3H3(S569);ZC3H3(S571);ZNF106(S641);ZNF516(T930);ZNF552(S86);ZNF609(S1055);ZNF75A(S286);ZNF75D(S490);ZNF814(S87);ZNRF2(S21);ZSCAN10(S6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ABL2</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>125</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(S30);AFDN(T1330);ANKRD17(S2401);AP1M1(T154);ARHGAP17(S162);ARHGEF11(S255);ARID1A(S772);ASCC3(S2195);ATF7(S434);ATF7IP(S474);ATF7IP(S477);ATXN2L(S32);BICRAL(S675);CAMKV(T435);CAMSAP1(S793);CAMSAP3(S814);CDC42SE1(S74);CDC6(S106);CDK18(S117);CRAMP1(S1268);CRTC3(S62);CSNK1D(S331);DCLRE1C(S518);EEF2K(S72);EEF2K(S74);EEF2K(Y69);EIF3A(S1188);EIF4ENIF1(S752);EPB41L5(S436);ETV6(S203);EVPL(S2025);FAM120A(Y452);FAM193B(S785);FOXK1(S223);FUBP3(S569);GLCCI1(S30);GRAMD1B(S274);GSK3B(S25);GSK3B(S9);GTF2F1(T389);HIPK1(T351);HIPK1(Y352);HIPK2(T360);HIPK2(Y361);HTT(S1199);HUWE1(T2889);IKBKB(S672);IRF2BPL(S215);IRS1(S374);ITSN1(S315);KIFC1(S26);MAP3K11(S524);MAP4(S928);MAP7D1(S399);MARCKS(S167);MAST2(S1364);MCRIP2(S82);MED13(S890);MNAT1(S279);MON1B(S59);MON1B(S61);MPHOSPH8(S403);MTA1(S576);MYC(S62);MYCN(S62);NAA30(S39);NAV1(S1265);NECTIN1(T391);NSRP1(S33);NSUN2(S456);NSUN2(S473);OTUD4(S416);PAK4(T207);PALD1(S406);PARD3(S174);PDHA1(S232);PDS5B(S1358);PHACTR1(S505);PKN1(S562);PKP2(S329);PKP4(S337);PKP4(S406);PPP1R12A(S903);PPP1R13L(S102);PRAG1(S889);PRAM1(S334);PREX1(S1182);PTPN22(S692);PXN(S258);R3HDM1(S381);RANBP1(S60);RB1(S249);RBM10(S797);RCSD1(S116);RCSD1(S120);RFX7(S225);RFX7(S424);RICTOR(S1284);RIOK1(S22);RREB1(S42);SHC3(S474);SHROOM3(S816);SIRT1(S27);SLC4A7(S556);SNIP1(S35);SRRM1(S429);SRRM2(S1404);SRRM2(S322);STK33(S470);TBKBP1(S365);TEX2(S266);TNS1(S1269);TRA2A(T202);TRAFD1(S470);TRAPPC12(S184);TRIO(S1724);TVP23C(S223);USP1(S67);USP32(S1423);WDR20(S434);ZNF106(S641);ZNF516(T930);ZNF552(S86);ZNF609(S1055);ZNF814(S87)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AKT1.2</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>155</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ABLIM1(S452);ACLY(S455);ADD1(S465);AFF4(S1043);AHNAK(S5731);AKT1S1(T246);ALDH1A3(S95);ALKBH5(S361);ANKRD2(S99);ANLN(S182);ANLN(T194);ARFGAP2(S368);ARHGEF12(S1288);ARHGEF17(S420);ASAP2(S822);ASIC3(S37);ASIC3(S39);BAD(S99);BAIAP2L1(S261);BAIAP2L1(T257);BAZ2A(S1397);BCL9L(S750);BRCA1(S1189);BRCA1(S1191);C2CD5(S260);CAD(S1859);CEP170B(S1179);CEP170B(S421);CLASP1(S1091);CSNK1D(S382);CTDSPL2(S104);DDX17(S571);DENND4C(S989);DENND5B(S1076);DTL(S623);EIF2B1(S105);EIF2B1(S107);EIF4EBP1(S65);EIF4EBP2(T70);EIF4EBP3(S51);EPB41L1(S510);EPX(S670);EPX(S672);FAM117A(S145);FAM189A1(S18);FAM53B(S118);FBXL15(S262);FOXO3(S284);GSK3A(S21);HCLS1(T308);HDGFL2(S454);HNRNPA2B1(S212);IRS1(S312);ITPR3(S1832);JPT1(S28);JPT1(T54);JUN(S63);KANK1(S325);KAZN(S387);KIFC1(S349);KIFC1(S351);KRI1(S171);KRT18(S7);KRT8(S477);LARP1(S766);LARP1(T649);LASP1(S146);LIMD2(S29);LINC00322(S226);LINC00322(S228);LRCH4(S515);LRRTM4(S195);MARCKS(S167);MARCKS(S170);MEPCE(S152);MFSD10(S270);MFSD2B(S491);MKI67(S308);MRGBP(S195);MSH6(S256);MTMR1(S43);MTMR4(S610);MTSS1L(S300);MYC(S62);MYCN(S62);MYO9B(S1405);NBEAL2(S2743);NDRG1(S367);NSD2(T115);PALLD(S893);PATL1(T194);PCBP1(S264);PCM1(S960);PDAP1(S176);PDE3B(S495);PDS5B(S1358);PHACTR4(S590);PHC3(S823);PHIP(S1315);PI4K2A(S462);PKP3(S180);PLEC(S4386);POLH(S379);PPFIA1(S1172);PPHLN1(Y162);PPP1R9A(S840);PRKAG2(S196);PRMT9(S81);RAB3IP(S157);RBM14(S618);RPS6(S235);RPS6(S240);RPS6KB1(S427);RPS6KB1(S441);RRN3(S44);RRN3P2(S44);RRP9(S293);SAFB(S601);SCAMP3(S32);SERBP1(S203);SH3BP1(S612);SH3BP1(S613);SH3PXD2B(S291);SKIV2L(S131);SKIV2L(S133);SRGAP1(S917);SRRM2(S771);SRSF7(S165);SRSF7(S167);STAT5A(S193);STAT5A(S780);TMEM163(S12);TMPO(S67);TRA2B(T201);TRA2B(T212);TRIM33(S1119);TRIM37(S771);TRIM37(S773);TRPV3(S372);UBA1(S816);UBA1(S820);UBE2J1(T267);ULK1(S623);UNK(S385);VIPAS39(S121);VRTN(S432);XPR1(S666);XPR1(S668);YBX1(S209);ZC3H15(S381);ZC3H3(S569);ZC3H3(S571);ZNF185(S64);ZNRF2(S21);ZSCAN10(S6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AKT3</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>13</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ASAP2(S822);CEP170B(S1179);CHEK1(S280);EPB41L1(S510);MEPCE(S152);NUP50(S208);SCAMP3(S32);SERBP1(S203);TMEM163(S12);VIPAS39(S121);YBX1(S209);ZNF185(S64);ZNRF2(S21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ARAF</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1649</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>09/02/18 00:00:00(S218);09/07/18 00:00:00(T228);09/09/18 00:00:00(T142);09/09/18 00:00:00(T49);AAK1(S637);AAK1(T606);AATF(S203);AATF(S321);ABCB11(S694);ABI1(Y213);ABI2(S368);ABLIM1(S216);ABLIM1(S640);ABR(S53);ACIN1(S386);ACIN1(S388);ACIN1(S490);ACIN1(S657);ACSL3(T107);ACSS2(S267);ACTL6A(S233);ADAMTS5(S264);ADD1(S726);ADD2(S600);ADD2(S713);ADD3(S681);ADD3(S693);ADGRA1(S8);ADGRL2(S1334);ADNP(S953);ADNP(S955);ADRM1(T217);AEBP2(S24);AFDN(T1330);AFF4(S1043);AFF4(S487);AGAP1(S422);AGAP1(S521);AGAP1(T836);AGAP2(T809);AGFG1(S181);AGFG1(S293);AHCTF1(S1944);AHNAK(S177);AHNAK(S3412);AHNAK(S3426);AHNAK(S5763);AIFM1(S268);AKAP1(S445);AKAP12(S286);AKAP2(S121);AKAP8(S339);AKIRIN2(S21);AKT1S1(S88);AKT1S1(T246);ALDOA(T9);ALMS1(S3802);ALMS1(T3036);ALX1(S69);AMPD2(S76);ANK1(S15);ANK3(S1459);ANKHD1(S1670);ANKHD1(S1679);ANKMY1(S861);ANKRD17(S1709);ANKRD17(S19);ANKRD17(S1940);ANKRD17(S2067);ANKRD17(S2401);ANKRD2(S99);ANLN(S182);ANLN(S323);ANLN(S362);ANLN(S449);ANLN(S485);ANLN(S927);ANLN(T194);ANXA2(T19);ANXA2P2(T19);AP1M1(T154);AP3B1(S276);APBA2(S11);APRT(S30);ARFGAP2(S368);ARFGEF2(S227);ARFGEF2(S240);ARFGEF2(T244);ARFGEF3(S2061);ARFGEF3(S2097);ARFIP1(S132);ARGLU1(S77);ARHGAP10(S591);ARHGAP17(S162);ARHGAP17(S674);ARHGAP29(S1029);ARHGAP39(S286);ARHGAP39(S366);ARHGEF11(S1413);ARHGEF11(S255);ARHGEF12(T736);ARHGEF16(S107);ARHGEF16(S174);ARHGEF16(S208);ARHGEF17(S420);ARHGEF17(T396);ARHGEF18(S1124);ARHGEF2(S137);ARHGEF26(S80);ARHGEF6(S488);ARHGEF6(S684);ARHGEF7(S518);ARID1A(S382);ARID1A(S696);ARID1A(S772);ARID1A(T1206);ARID1B(S502);ARID3B(S89);ARPC1B(T315);ARPP19(S104);ARPP19(S62);ASAP1(S1027);ASCC3(S2195);ASF1B(T179);ASH1L(S1748);ATAD2(S327);ATF7(S434);ATF7IP(S113);ATF7IP(S474);ATF7IP(S477);ATG13(S361);ATP13A1(S899);ATP13A3(S817);ATP2B1(S1193);ATRX(S1527);ATXN2(S624);ATXN2L(S32);ATXN2L(S559);ATXN2L(S634);AUTS2(S941);AXIN1(S77);B3GNT8(S37);BAG3(S289);BAG3(T285);BAG6(S964);BAIAP2(S366);BAIAP2L1(S261);BAIAP2L1(S414);BAIAP2L1(T257);BARGIN(S183);BAZ1A(S1280);BAZ1B(S349);BBX(S844);BCAM(S600);BCL11A(S205);BCL11A(S630);BCL11A(S718);BCL2L12(S242);BCL7C(S126);BCL9(S1044);BCL9L(S21);BCL9L(S750);BCLAF1(S222);BCLAF1(S397);BCR(S122);BICRA(S1413);BICRAL(S675);BIN1(S298);BIN1(S331);BIRC6(S577);BOD1L1(T2480);BOLA1(S123);BRD1(S128);BRD2(S633);BRIP1(S128);BRSK1(S563);BRSK2(S489);BUD13(S325);C11orf94(S77);C19orf47(S151);C2CD4C(S178);C2CD5(S295);C9orf78(S261);CALD1(T730);CAMKK2(S511);CAMKV(T435);CAMSAP1(S793);CAMSAP3(S1074);CAMSAP3(S1080);CAMSAP3(S368);CAMSAP3(S814);CANX(S583);CARD11(S512);CARHSP1(S30);CASKIN2(S471);CASP8AP2(S567);CBL(S619);CBY1(S9);CC2D1A(S455);CCAR2(S124);CCDC120(S358);CCDC61(T285);CCDC8(S261);CCDC86(S91);CCDC86(T42);CCDC88B(S1379);CCDC88C(S227);CCNE1(S103);CCNK(S340);CCNK(S9);CCNL1(S342);CCNY(S25);CD244(S334);CD2AP(S458);CD3EAP(S27);CDAN1(S160);CDC42BPA(S1651);CDC42EP4(S292);CDC6(S106);CDC6(S54);CDCA2(S98);CDCA3(S29);CDCA3(S87);CDCA5(S75);CDK10(T196);CDK11A(S271);CDK11A(T583);CDK11A(Y582);CDK11B(S283);CDK12(S1083);CDK12(S423);CDK12(T1244);CDK12(T514);CDK12(T893);CDK13(T871);CDK14(S134);CDK14(S78);CDK14(S95);CDK16(S138);CDK17(S137);CDK17(S9);CDK18(S117);CDK18(S74);CDK18(S98);CDK7(T170);CEBPE(S21);CEBPZ(S629);CENPF(S1750);CENPF(S276);CENPF(T144);CENPO(S35);CEP131(S114);CEP192(S1514);CEP57(S55);CEP72(S237);CEP97(S308);CFL1(S3);CHAF1A(S772);CHAF1A(S775);CHAF1B(S538);CHAMP1(S308);CHAMP1(S319);CHAMP1(S376);CHAMP1(S416);CHAMP1(S507);CHAMP1(S603);CHD1(S1677);CHD1(S90);CHD4(T1553);CHD8(S2046);CHD8(T1982);CIR1(S202);CIT(S1940);CIT(S1993);CIZ1(S838);CLASP2(S525);CLASP2(S529);CLASP2(S596);CLASP2(S892);CLIC6(S293);CLK1(S337);CLNS1A(S102);CLSPN(S1289);CLSPN(S516);CNK3/IPCEF1(S873);CNN3(S296);CNNM3(S467);CNNM4(S664);CNOT2(T93);CNTNAP4(S520);COBL(S269);COBL(S347);COG2(T480);COIL(T303);COL19A1(S81);COPA(S173);COPE(S13);CPSF7(T203);CRAMP1(S1268);CRKL(Y198);CRTC3(S329);CRTC3(S62);CSNK1D(S331);CSNK1D(S350);CSNK1E(S363);CSPP1(S966);CSTF3(S691);CTDP1(S416);CTNNB1(S191);CTNND1(Y865);CTPS2(S568);CTTN(S405);CTTN(T411);CTTNBP2NL(S568);CUEDC2(S110);CXADR(S332);CYBRD1(S260);DAXX(S178);DAXX(S495);DBF4(S359);DBF4(T510);DBN1(S381);DCDC2(S270);DCK(S74);DCLK1(S337);DCLRE1C(S518);DCP1A(S525);DCP1B(T392);DCP2(S284);DDX20(S714);DDX20(T552);DDX3X(S594);DDX3Y(S592);DDX5(S480);DENND4A(S1240);DENND4A(S1256);DENND4A(S728);DENND4A(T1019);DENND4C(S1277);DENND4C(S1301);DENR(S73);DFFA(S315);DGCR8(S95);DHX15(T191);DHX29(S200);DIDO1(S1040);DIP2B(S203);DKC1(S494);DLG5(S1209);DLG5(T1279);DLGAP4(S666);DLGAP5(S690);DMAP1(T445);DMWD(S495);DNM1L(S616);DNMT1(S127);DNMT1(T137);DOCK5(S1789);DOCK7(S30);DOCK7(S864);DOCK8(S139);DOT1L(S1001);DPF2(S244);DPF2(T248);DTL(T196);DTL(T429);DYNC1LI1(S398);DYNC1LI1(S465);EAF2(S154);EBAG9(S36);EEF1A1(Y29);EEF1A1P5(Y29);EEF1A2(Y29);EEF1B2(S95);EEF1D(T147);EEF2K(S72);EEF2K(S74);EEF2K(Y69);EHBP1(T378);EHBP1L1(S285);EIF2B1(S107);EIF3A(S1188);EIF3A(S584);EIF3E(S399);EIF4A3(T163);EIF4B(S283);EIF4EBP1(T82);EIF4EBP3(S51);EIF4ENIF1(S5);EIF4ENIF1(S752);EIF4G1(S1092);EIF4G1(S1209);EIF4G2(S395);EIF4G3(S230);EIF4H(S21);EIF5B(S438);ELF2(T374);ELMO1(S344);ELOA(S413);ELP2(S122);EMSY(S1213);ENAH(S531);ENSA(S67);EP300(S1038);EP400(S1547);EPB41L1(S510);EPB41L2(S562);EPB41L2(S715);EPB41L3(S760);EPB41L3(S88);EPB41L3(S962);EPB41L4B(S390);EPB41L5(S550);EPHB4(S502);EPS15(S814);EPS15L1(S108);EPX(S672);ERC1(S21);ERCC6L(S1069);ERF(S327);ERLIN1(S324);ERRFI1(S302);ESCO2(S75);ESS2(S292);ESS2(T110);ESS2(Y102);ETNK2(T322);ETV6(S203);EVPL(S2025);EXOC2(S435);EZH2(T367);FAM110B(S301);FAM117B(S16);FAM117B(S457);FAM120A(Y452);FAM122A(S189);FAM122A(S76);FAM126B(S430);FAM169A(S526);FAM171A1(S422);FAM171A1(S849);FAM193B(S785);FAM208A(S979);FAM53B(S118);FAM53B(S167);FAM53B(S268);FAM53C(S162);FAM53C(S273);FAM83G(S760);FAM83H(S523);FAM83H(S998);FAM98B(S261);FANCI(S407);FARP1(S340);FARP1(S427);FBRSL1(T1010);FBXO28(S344);FCHO2(S387);FERMT3(S497);FGD1(S82);FGFR1OP(T170);FLI1(S241);FNBP1(S497);FNBP1L(S295);FNBP1L(S489);FOCAD(T543);FOXJ3(S223);FOXK1(S213);FOXK1(S223);FOXK1(S257);FOXK2(S398);FOXP1(S83);FRY(T1956);FUBP3(S296);FUBP3(S569);FXR1(S409);FZR1(S163);G3BP2(S141);G3BP2(S149);GAB2(S210);GAB2(S623);GAPVD1(S950);GDI2(S61);GEMIN2(S81);GEMIN5(S770);GFPT1(S261);GJA1(S325);GJA1(Y267);GLCCI1(S223);GLCCI1(S30);GLCCI1(S406);GLCCI1(T110);GMPS(T318);GNL3(S529);GON4L(S346);GORASP1(S220);GPAT3(S68);GPATCH11(S141);GPATCH2(S54);GPATCH4(S128);GPRIN1(S615);GPS1(S468);GRAMD1A(S263);GRAMD1B(S274);GRB10(S104);GREB1(S1193);GRIN3B(S634);GRIP1(S847);GSE1(S710);GSE1(S826);GSE1(S828);GSE1(S857);GSE1(T433);GSK3B(S25);GSK3B(S9);GTF2F1(T389);GTF2I(S210);GTF2I(T558);GTF3C1(S1653);GTF3C2(S893);GTPBP1(S580);GYS1(S649);HAUS6(T584);HBS1L(T231);HCFC1(S1205);HCLS1(S275);HCN4(S1059);HDAC1(S421);HDAC1(S423);HDAC2(S422);HDAC2(S424);HDAC4(S266);HDAC5(S279);HDAC5(S661);HDAC7(S358);HDAC7(S487);HDAC9(S240);HDGF(S133);HDGFL2(S366);HDGFL2(S369);HDGFL2(S370);HDGFL2(S652);HDGFL2(S664);HEATR6(S336);HECW1(S1344);HECW2(S1310);HERC2(S1539);HIPK1(T351);HIPK2(T360);HIPK4(S337);HIRIP3(S530);HIRIP3(S87);HMGN1(S25);HMOX1(S229);HNRNPA1(S338);HNRNPA1(S6);HNRNPA1(S95);HNRNPA1L2(S95);HNRNPA2B1(S212);HNRNPA2B1(S225);HNRNPA2B1(S259);HNRNPK(S216);HNRNPK(S284);HNRNPUL1(S718);HPS5(S534);HR(S6);HRNR(S903);HSP90AA1(S399);HSP90AB1(S255);HSP90AB1(S391);HSP90AB2P(S177);HSP90AB3P(S333);HSPB1(S199);HSPB1(S82);HSPB1(S98);HSPH1(S809);HTT(S1179);HUWE1(S1907);HUWE1(S3127);HUWE1(S3816);HUWE1(T2889);HYLS1(S297);ICE1(S255);IKBKB(S672);ILF3(S62);IMPDH2(S122);IMPDH2(S416);INCENP(S142);INCENP(S312);INTS1(T83);INTS10(S231);INTS3(S994);INTS3(S998);INVS(S617);IPCEF1(S411);IRF2BP2(S175);IRF2BP2(S360);IRF2BP2(S406);IRF2BP2(S71);IRF2BPL(S215);IRF2BPL(S519);IRF3(S175);IRS1(S1078);IRS1(S329);IRS1(T351);IRS2(S1176);IRS2(S915);ISCU(S20);ITSN1(S315);IWS1(S248);IWS1(S250);JMY(S115);JPH1(S216);JPH1(S475);JPH4(S157);JPT1(S131);JPT2(S97);KANSL1(S249);KANSL1(S991);KANSL1(S994);KDM1B(S17);KHSRP(S181);KIAA0754(S25);KIAA0930(S304);KIAA1143(S115);KIAA1217(S1794);KIAA1522(S327);KIAA1522(S971);KIAA1522(S979);KIAA1522(T162);KIAA1551(S1358);KIAA1671(S1488);KIF13B(S1410);KIF13B(S1644);KIF15(S568);KIF21A(S1212);KIF21A(S1239);KIF21A(S383);KIF21B(S1241);KIF21B(T1237);KIFC1(S26);KIFC1(S351);KLC1(S460);KLF3(S250);KMT2A(S2098);KMT2A(S2151);KMT2B(S861);KMT2C(S46);KMT2D(S3130);KRT18(S30);KRT80(S451);KSR1(S334);L3MBTL2(S683);L3MBTL2(S689);L3MBTL3(S608);LAMTOR1(S27);LARP1(T649);LARP4(S583);LARP4(S722);LARP4(T389);LARP6(S409);LAS1L(S617);LASP1(T104);LAT2(S51);LAT2(Y136);LATS1(S464);LEMD3(S144);LEO1(S546);LIG1(S141);LIG1(S51);LIG3(S242);LIMA1(S132);LIMA1(S362);LIMA1(S609);LIMK1(S298);LIMK1(S310);LINC01549(S26);LLGL2(S1000);LMNB1(T20);LRCH4(S457);LRP6(S1490);LRRC41(T327);LRRTM4(S195);LSM14A(S183);LSM14B(S165);LSP1(S189);LSR(S424);LSR(S510);LYSMD2(S24);MAGED2(S191);MAGED2(S247);MAGOH(S106);MAGOHB(S108);MAP1A(S1675);MAP1B(S1378);MAP1B(S1501);MAP1B(S1512);MAP1S(S640);MAP1S(S657);MAP1S(T638);MAP3K1(S1018);MAP3K11(S507);MAP3K11(S524);MAP3K3(T353);MAP3K8(S141);MAP4(S787);MAP4(T521);MAP4(T942);MAP4K3(S616);MAP4K4(S639);MAP4K4(S900);MAP7D1(S311);MAP7D3(S433);MAPRE2(S200);MAPT(S552);MAPT(T548);MARCKS(S167);MARK2(S456);MARK2(S486);MARK2(S619);MARK3(S469);MARK3(S583);MARK3(S585);MARK3(S587);MARK3(S601);MAST2(S1381);MASTL(S619);MATR3(S598);MCM2(S27);MCM3(S704);MCRIP2(S82);MDC1(S495);MDC1(S498);MECP2(S229);MED1(S1207);MED1(S953);MED1(T1215);MED13(S890);MEF2D(S180);MEF2D(S251);MFAP1(S132);MFAP1(S133);MFGE8(S42);MFSD2B(S494);MGA(S2088);MGA(S3020);MGRN1(S524);MICALL1(S295);MICALL1(S486);MICALL1(S578);MICALL1(S621);MICALL2(S153);MICALL2(S249);MID1(S96);MIIP(S303);MIS18BP1(S1042);MIS18BP1(S365);MISP(S394);MISP3(S91);MKI67(S584);MLF2(S238);MLXIPL(S614);MMACHC(S275);MNAT1(S279);MOK(S298);MOK(T291);MON1B(S59);MON1B(S61);MORC2(S696);MPHOSPH8(S403);MPLKIP(S115);MPLKIP(T51);MPLKIP(Y45);MPND(T76);MROH6(S9);MSANTD3(S274);MSH4(S902);MTA1(S576);MTA1(S639);MTBP(S639);MTBP(S755);MTCL1(S43);MTCL1(S549);MTCL1(S87);MTFR1L(S238);MTMR12(S564);MTOR(S2454);MTSS1L(T391);MTX3(S284);MUC16(S12130);MYBBP1A(S1267);MYBPC3(T307);MYC(S62);MYCN(S62);MYO10(S1883);MYO9B(S1267);MYO9B(S1331);MZT2A(S139);MZT2B(S139);NAA25(S691);NAA30(S39);NAA30(S89);NAB1(S183);NAF1(S315);NAP1L4(S125);NASP(S480);NAV1(S1000);NAV1(S1265);NAV1(S1382);NAV1(S648);NAV1(S754);NAV1(S760);NAV2(S1059);NAV2(S1559);NCKAP5L(S473);NCKIPSD(T181);NCL(S145);NCL(S153);NCL(S184);NCL(S206);NCOA2(S565);NCOA3(S1330);NCOA3(S694);NCOA5(T460);NCOR1(S1195);NCOR1(S2120);NCOR1(T2396);NCOR2(S1018);NCOR2(S1025);NCOR2(S1547);NCOR2(S1982);NCOR2(S215);NCOR2(S2424);NCOR2(S956);NDE1(S282);NECTIN1(S422);NECTIN1(T391);NELFA(S233);NEO1(S1214);NES(S325);NES(S475);NES(S476);NES(S548);NEXN(S243);NF1(S1140);NFIA(S287);NFIC(S333);NFIC(S339);NFIC(S473);NFIX(S265);NFIX(S301);NHS(T401);NHSL1(S1386);NIPBL(S2658);NIPBL(S318);NKTR(S379);NKTR(S463);NLN(S485);NME1(T94);NME2(T94);NME2P1(T79);NMT1(S47);NOL4L(S130);NOL6(S283);NOL8(S268);NOL8(S890);NOL8(T888);NOLC1(S456);NOLC1(S508);NOLC1(S698);NOP2(S181);NOP2(S786);NOP2(T185);NOP58(S351);NOP58(S514);NOS1AP(S266);NPFFR2(S54);NPM1(S137);NPM1(S260);NSD2(S421);NSFL1C(S114);NSFL1C(S140);NSRP1(S33);NSUN2(S456);NSUN2(S473);NUCKS1(S113);NUCKS1(S181);NUFIP2(S572);NUMB(S634);NUP160(S1157);NUP210(S1848);NUP214(S1045);NUP214(S940);NUP35(S55);NUP35(T273);NUP98(S1043);NUP98(S839);OBSL1(S1671);OR8J2(S137);ORC1(S199);ORC2(T226);ORC6(T195);OSBPL10(S201);OSBPL11(S181);OSBPL9(S326);OTUD7B(S464);P2RX7(S470);P2RX7(T467);PA2G4(S363);PACS1(S495);PAK1(S115);PAK4(T207);PAK4(T478);PALB2(S781);PALD1(S406);PALLD(S1116);PALLD(S1118);PALLD(S1121);PALM3(S155);PALM3(T151);PAPOLA(T23);PAPOLG(S599);PARD3(S144);PARD3(S174);PARD3(S220);PARG(S137);PARN(S619);PARVA(S10);PARVA(S14);PARVA(S19);PAWR(S259);PAXX(S148);PCBP1(S173);PCBP1(S262);PCBP1(S264);PCBP2(S189);PCBP2(S272);PCDH1(S949);PCDH1(S962);PCDHA13(S356);PCDHA4(S356);PCDHB13(S69);PCDHB8(S69);PCF11(T1530);PCGF6(S115);PCM1(S1958);PCM1(S776);PCM1(S779);PCM1(S960);PCM1_HUMAN_Phospho (ST);PCNP(T139);PCNT(S2355);PCYT1A(S315);PCYT1B(S315);PDCD4(S94);PDHA1(S232);PDLIM5(S111);PDLIM5(S313);PDS5B(S1358);PDZD2(S1270);PDZD4(S564);PER2(S977);PFAS(S569);PGAM1(S118);PGAM4(S118);PGM2(S165);PGM2L1(S175);PHACTR1(S505);PHACTR2(S443);PHACTR2(S445);PHACTR2(S471);PHACTR2(T452);PHACTR2(Y451);PHACTR4(S131);PHACTR4(S443);PHACTR4(S628);PHF3(S1642);PHF6(S154);PHLDA2(S144);PHLDB1(S430);PHLDB1(S461);PHLDB1(S470);PHOX2A(S208);PHRF1(S1124);PHRF1(S1202);PI4KB(S266);PIK3AP1(Y570);PIKFYVE(S299);PIKFYVE(S307);PITPNM1(S621);PJA2(S309);PKN1(S562);PKP2(S293);PKP4(S337);PKP4(S406);PLCH1(S1060);PLCL2(S17);PLEKHA2(S349);PLEKHA5(S140);PLEKHA5(S568);PLEKHA5(S885);PLEKHA5(S933);PLEKHG3(S76);PLEKHO2(S390);PLIN3(S130);PLPPR3(S353);PLPPR3(S508);PML(S527);PNISR(S211);PNN(S100);POGZ(S425);POGZ(S445);POLD3(S307);POLR2A(S1875);POM121(S269);POM121(S435);POM121B(S19);POM121C(S246);POM121C(S412);PPA2(S317);PPAN(S359);PPFIA1(S1172);PPFIA3(S1164);PPFIA4(S684);PPFIBP2(S387);PPHLN1(S163);PPHLN1(S205);PPIG(S356);PPIG(S397);PPIG(T358);PPIP5K1(S964);PPL(S14);PPM1H(S221);PPP1CA(T320);PPP1R12A(S422);PPP1R12A(S903);PPP1R12C(S509);PPP1R13L(S102);PPP1R13L(S358);PPP1R1A(S67);PPP1R35(S87);PPP1R35(T84);PPP1R3D(S74);PPP1R3D(S78);PPP4R2(S159);PPP4R2(S226);PPP4R3A(S741);PPP6R3(S525);PPP6R3(S617);PPP6R3(S853);PQBP1(S247);PRAG1(S889);PRAM1(S298);PRDM2(S1484);PREX1(S1182);PRKAA1(S184);PRKAA2(S173);PRKAR1B(S83);PRKCD(S645);PRKD1(S549);PRKD1(S742);PRKD3(S735);PRKDC(S2612);PRKDC(S3205);PROSER2(S43);PRPF40A(S938);PRPF4B(S277);PRPF4B(S292);PRPF4B(S294);PRPF4B(S852);PRPF4B(Y849);PRPF6(T266);PRPSAP2(S227);PRR15(S49);PRR5(S11);PRRC2A(S1691);PRRC2A(S456);PRRC2A(S761);PRRC2A(T1347);PRRC2B(S1691);PRRC2B(T225);PSD4(S118);PSMD1(T273);PSMD2(S16);PSMF1(S153);PSPC1(S477);PTGES3(S113);PTK2(S29);PTK2(S722);PTPN13(S2032);PTPN13(S240);PTPN13(S890);PTPN2(S304);PTPN21(S660);PTPN22(S692);PTPN23(S1123);PTPRK(S856);PTPRK(Y858);PTPRZ1(S2056);PTS(S19);PTTG1(S165);PTTG2(S165);PWP1(S50);PXN(S258);PXN(Y118);PXN(Y88);PYCR2(S304);QSER1(S1348);QSER1(T1341);R3HDM1(S381);RAB11FIP1(S435);RAB12(S21);RAB3IL1(S168);RAB40C(S268);RABGEF1(S302);RABGEF1(S607);RAD18(S322);RAD51AP1(S120);RAD54B(S14);RALGAPA2(S1629);RALGAPB(T379);RALGPS2(S308);RALGPS2(S329);RALGPS2(S422);RALY(S135);RANBP2(S21);RANBP2(S788);RANBP3(S108);RANBP3(S211);RANBP3(S333);RAPGEF1(S311);RAPGEF1(T216);RAPGEF2(S1080);RAPGEF2(S585);RASAL2(S18);RASGRP2(S391);RASGRP2(S576);RB1(S795);RB1(S807);RB1(T821);RB1(Y790);RB1CC1(T238);RBBP6(S1697);RBBP6(S516);RBBP6(S873);RBBP8(T315);RBL1(S988);RBL2(S639);RBL2(S662);RBM10(S723);RBM10(S797);RBM12B(S638);RBM14(S520);RBM15(S128);RBM15(S741);RBM15B(S552);RBM17(Y214);RBM25(S703);RBMX(S88);RBMX2(S188);RBPMS(T118);RBSN(S429);RCOR1(S460);RCOR2(S63);RCSD1(S116);RCSD1(S120);REXO4(S15);RFC1(S156);RFTN1(S61);RFX7(S225);RFX7(S424);RGL2(T752);RGPD1(S779);RGPD2(S787);RGPD3(S789);RGPD4(S789);RGPD5(S21);RGPD5(S788);RGPD8(S21);RGPD8(S788);RHBDF2(S113);RICTOR(S1284);RIF1(S1707);RIF1(S2161);RIF1(T1047);RIOK1(S22);RIPK2(S363);RIPOR1(S349);RIPOR1(S351);RNF214(S500);RNPS1(S251);ROBO1(S1055);ROBO2(S1156);RPL18A(S71);RPL34(S12);RPP38(S235);RPRD2(S769);RPRD2(S965);RPS6KA3(S369);RPUSD2(S68);RRAS2(S186);RREB1(S1320);RREB1(S161);RREB1(S231);RREB1(S42);RSF1(S1277);RSF1(S1282);RSF1(T1278);RSF1(T1305);RSF1(Y1281);RSL1D1(S396);RSL1D1(T415);RSRC2(S32);RTKN(S543);RTN3(S229);RUFY1(S620);RUNX1(S21);SALL2(S641);SALL3(T935);SALL4(S307);SALL4(S756);SAMD4B(S628);SCAF11(S608);SCAF8(S617);SCNM1(S183);SCRIB(S1306);SCRIB(S504);SCRIB(S853);SEC16A(S136);SEC16A(S391);SEC16A(T19);SEC31A(S527);SEC61A1(S408);SEMA6A(T761);SENP1(S170);SENP6(S350);SENP7(S443);SENP7(S444);SERBP1(S203);SET(S28);SETDB1(S1066);SETX(S1663);SF3B1(T223);SF3B1(T227);SF3B1(T244);SF3B2(S307);SFMBT2(T762);SFN(S45);SFPQ(S33);SGO1(S461);SH2D3C(S440);SH2D5(S231);SH3BP1(S175);SH3BP1(S586);SH3BP1(S598);SH3BP1(S612);SH3BP1(S613);SH3BP1(T626);SH3BP2(S278);SHANK1(S948);SHANK2(S1069);SHANK2(S452);SHARPIN(S131);SHC3(S474);SHROOM2(S1116);SHROOM2(S422);SHROOM3(S242);SHROOM3(S439);SHROOM3(S816);SHROOM3(S913);SIN3A(S1112);SIN3A(T266);SIN3B(S273);SIPA1L1(S1087);SIPA1L1(S1255);SIPA1L1(S1549);SIPA1L1(S1649);SIPA1L1(S1650);SIPA1L3(S1364);SIRT1(S172);SIRT1(S27);SKA3(S119);SLAIN2(S48);SLC12A7(T30);SLC12A7(T980);SLC13A4(S246);SLC16A1(S461);SLC22A17(S515);SLC2A3(S485);SLC38A1(S49);SLC4A1AP(S466);SLC4A1AP(S82);SLC4A7(S556);SLC6A15(S687);SLC7A6OS(S308);SLC9A3R1(S280);SLX4(S1044);SMAP2(S219);SMARCA4(S695);SMARCAD1(S79);SMARCC2(S283);SMARCC2(T548);SMC3(S1083);SMCR8(S498);SMTN(S32);SNAP23(S110);SNAPC4(S599);SNIP1(S35);SNRK(S518);SNTB1(S219);SNTB1(S87);SNTB2(S393);SNTB2(S95);SNX1(S188);SNX17(S336);SNX17(S437);SNX17(S440);SNX2(S277);SNX8(S456);SNX8(T452);SOGA1(S1017);SON(S152);SON(S1782);SORBS2(S278);SORBS3(S530);SOWAHC(S213);SOWAHD(S22);SP110(S380);SPATA19(S148);SPECC1(S847);SPIRE1(T509);SPRY2(S142);SPRY4(S125);SPTBN1(S2341);SQSTM1(S328);SRCAP(S274);SRCAP(S3016);SRF(S224);SRGAP1(S1029);SRGAP1(S932);SRRM1(S260);SRRM1(S391);SRRM1(S402);SRRM1(S431);SRRM1(S549);SRRM1(S551);SRRM1(S696);SRRM1(S715);SRRM1(S738);SRRM1(T406);SRRM2(S1329);SRRM2(S1404);SRRM2(S2071);SRRM2(S2121);SRRM2(S2123);SRRM2(S2272);SRRM2(S2382);SRRM2(S2581);SRRM2(S322);SRRM2(S323);SRRM2(S358);SRRM2(S377);SRRM2(S398);SRRM2(S440);SRRM2(S774);SRRM2(S952);SRRM2(S954);SRRM2(T1003);SRRM2(T1434);SRRM2(T1492);SRRM2(T1531);SRRM2(T2058);SRRM2(T2061);SRRM2(T2069);SRRM2(T315);SRRM2(T400);SRRM2(T983);SRRT(S67);SRSF1(S199);SRSF1(S201);SRSF1(S205);SRSF11(S434);SRSF7(S192);SRSF9(S204);SSBP3(S347);STAMBPL1(S242);STAU2(S486);STIM1(S575);STIM1(S618);STIM2(S523);STK10(S417);STK10(S438);STK11IP(S470);STK33(S470);STRN(S245);STRN(S376);STRN(T143);STRN(Y135);STUB1(S23);SUPT5H(S666);SYAP1(T248);SYN1(S427);SYN1(S551);SYN1(S553);SYNJ1(S1392);SYNJ2(S1124);SYNRG(S473);SZRD1(S74);TAF2(S1185);TAF4B(S595);TAF6(S634);TAF6(S636);TAF9(T144);TALDO1(S237);TANC1(S67);TANC2(S1458);TANC2(S1977);TAOK1(S421);TAOK1(S9);TAOK1(S965);TARDBP(S292);TAX1BP1(S666);TBC1D1(S211);TBC1D10B(S22);TBC1D10B(S658);TBC1D10B(S661);TBC1D10B(S678);TBC1D10B(T152);TBC1D13(S184);TBC1D22A(S167);TBC1D5(S522);TBC1D5(S554);TBC1D5(S730);TBCC(S168);TBKBP1(S365);TC2N(S168);TCF12(S79);TCF20(S559);TCOF1(S1227);TCOF1(S1257);TCOF1(S583);TCOF1(S906);TCOF1(T983);TDRD12(S211);TERF2IP(S154);TET2(S1107);TEX2(S266);TFDP1(S23);TFE3(S548);THOC2(T1443);THOP1_HUMAN_Phospho (ST);TIAM1(S1407);TJAP1(T60);TJP1(S1579);TJP1(S968);TJP3(S591);TLE1(T312);TLE3(S263);TLE4(S292);TLK2(S771);TMC6(S63);TMEM163(S12);TMEM185A(S333);TMEM185B(S333);TMEM201(S443);TMEM201(S466);TMEM41B(T18);TMEM9(S137);TMF1(S328);TMF1(T401);TMPO(S224);TNIK(S548);TNIK(S707);TNK2(Y827);TNKS1BP1(S1620);TNKS1BP1(S1621);TNKS1BP1(S1715);TNRC18(S1925);TNS1(S1269);TNS1(T1173);TNS3(S874);TNS3(T632);TOM1L1(S323);TOR1AIP1(S143);TP53BP1(S1068);TP53BP1(S1320);TP53BP1(S1678);TP53BP1(S294);TP53BP1(S398);TP53BP1(S831);TPD52L2(S21);TPX2(T369);TRA2A(T202);TRAFD1(S470);TRAP1(S401);TRAPPC12(S184);TRIM16(S36);TRIO(S1724);TRIOBP(S1955);TRIT1(S443);TRMT2A(S602);TRPM7(S1477);TRPS1(S1081);TRPS1(S1085);TRPV3(S372);TSC2(S1155);TSC22D4(S62);TSEN2(S81);TSNAX(S33);TSSC4(S132);TTC7A(S182);TTYH3(S496);TVP23C(S223);U2AF2(S79);U2SURP(S67);UBA1(S816);UBA1(S820);UBAP2L(S471);UBAP2L(S609);UBASH3A(S471);UBE2J1(S266);UBE2O(S515);UBR4(S2718);UCKL1(S56);UHRF1(S287);UIMC1(S140);ULK3(S240);UNC80(S3073);UPF1(S1127);USP1(S67);USP11(S648);USP14(S143);USP18(T87);USP28(S1053);USP32(S1423);USP32(S1588);USP33(S439);USP36(S742);USP36(S952);USP41(T87);USP54(S1036);USP6NL(S396);USP6NL(S680);USP7(S18);UTF1(S245);UTF1(S54);UTP18(S121);UTP18(S206);VCL(S346);VCP(S770);VDAC2(S115);VEZT(S696);VGLL4(S149);VIM(S73);VPS13C(T1437);VPS72(S127);VRTN(S432);WAC(S511);WAC(T457);WASF1(S310);WDCP(S690);WDFY3(S2278);WDR20(S434);WDR44(S50);WDR62(S33);WEE1(S139);WIPF2(S235);WIPF3(S149);WIZ(S1017);WIZ(S1151);WNK1(S2121);WNK1(S2370);WNK3(S1095);WWP2(S211);XRCC1(S226);XRCC1(S229);XRCC1(S241);XRCC1(T198);XRCC1(T202);XRCC1(Y211);XRCC4(S237);YEATS2(S447);YTHDC1(S424);YTHDC2(S1279);YTHDF1(S291);YWHAB(S47);YWHAE(S46);YWHAG(S46);YWHAH(S46);YWHAQ(S45);YWHAZ(S45);ZBTB17(S120);ZBTB7A(S549);ZBTB7B(S487);ZC3H11A(T321);ZC3H14(S515);ZC3H18(S67);ZC3H18(S74);ZC3H18(T796);ZC3H3(S571);ZC3H4(S1110);ZDH18_HUMAN_Phospho (ST);ZDHHC18(S19);ZDHHC5(S621);ZDHHC5(T348);ZEB1(S679);ZFP36L1(S54);ZFP36L2(S438);ZFPM1(S786);ZFPM1(S909);ZFR(S1054);ZFYVE19(S463);ZMYM4(S242);ZMYND8(S406);ZMYND8(S444);ZMYND8(S486);ZMYND8(S488);ZNF106(S641);ZNF219(S16);ZNF221(S486);ZNF224(S548);ZNF318(S2035);ZNF326(S270);ZNF326(S56);ZNF462(S455);ZNF507(S545);ZNF516(S852);ZNF516(T930);ZNF552(S86);ZNF592(S573);ZNF609(S1055);ZNF609(S758);ZNF622(S143);ZNF638(S1401);ZNF638(S605);ZNF639(S60);ZNF649(S474);ZNF687(S266);ZNF687(S271);ZNF687(S374);ZNF777(S47);ZNF800(S336);ZNF814(S87);ZNF84(S128);ZNRF2(S135);ZRANB2(S120);ZSCAN29(S153);ZYX(S259);ZZEF1(S1518)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>AURKB</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>74</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ACIN1(S490);ADGRL2(S1430);AHCTF1(S1142);AKIRIN2(S21);APC(S2125);ARHGEF6(S488);ARID1A(S604);ARPP19(S62);ATXN1(S88);BAIAP2(S366);BCL9L(S750);BTF3(S30);CASKIN2(T807);CDC42EP4(S118);CDK2(T160);CDK3(T160);DBF4(S359);DDX3X(S90);DNTTIP2(S141);DSP(S176);DTL(T429);EIF3A(S1188);EIF3A(S882);EIF4B(S207);ENSA(S67);FAM53C(S251);FAM53C(S254);FAM53C(S255);GAPDH(T153);GON4L(S346);GSK3A(S21);HMGCR(S872);HNRNPD(S190);IFIH1(S301);IQSEC1(S180);IRF2BP2(S406);IRS2(S306);KNOP1(T310);KRT80(S45);LRRC40(S71);LUC7L2(S18);MAST2(S148);MPRIP(S993);MTFR1L(S103);MTMR1(S43);MTMR3(S613);NCBP1(S22);PAWR(T163);PFDN4(S125);PGM5(S510);PI4KB(S266);PXN(S258);RB1(S795);RHPN2(T655);RHPN2P1(T552);RIF1(T1047);RPS2(S264);SASH1(S839);SEC31A(S799);SENP7(S443);SENP7(S444);SHROOM3(S890);SIPA1L2(S162);SLC9A3R1(S269);SRRM2(S1124);TIAM1(S311);TJP1(S1579);TPD52(S176);UTP3(S37);VIPAS39(S121);ZC3HC1(S395);ZNF84(S128);ZNRF1(S123);ZZZ3(S113)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BMP2K</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>23</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(T142);CDC25B(S375);CDK12(T893);DENND4A(S1256);HSH2D(S194);MKL2(S921);MPLKIP(S115);MYBBP1A(S11);PALM3(S303);PKP2(S82);PPP4R3B(S840);RB1(T601);RBMX(S208);RBMXL1(S208);SCFD1(S303);SF3B1(T436);SRRM2(S1014);TANC2(S169);TCOF1(S156);TLN1(S425);TNKS1BP1(S1297);TNKS1BP1(S435);WIPI2(S413)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CAMK2A</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>376</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(S30);AAK1(S14);ABI1(S216);ABI1(Y213);ABLIM1(S431);ABR(T74);ADAM17(S791);ADD1(S12);AFDN(S1721);AFF4(S1043);AHCTF1(S528);AHNAK(S115);AHNAK(S216);AHNAK(S3412);AHNAK(S3426);AHNAK(S5739);AJUBA(S263);AKAP11(S1580);AKAP11(S448);AKAP13(S1559);AKAP13(S1929);AKAP13(S2728);AMBRA1(S639);ANKZF1(S675);ARFGAP2(S368);ARFGAP2(S432);ARHGAP17(S625);ARHGEF17(S735);ARHGEF6(S684);ARID1A(S1604);ARL6IP6(S80);ATAD2(S327);ATG2A(S498);ATG2B(S1582);ATG2B(S1583);ATG2B(Y1577);ATN1(S661);ATN1(T653);BAG6(S1081);BAIAP2(S366);BCL11A(S328);BRIP1(S956);BTF3(S30);C1orf198(S175);C2CD5(S281);C6orf132(S449);C7orf50(S175);CARMIL2(S1315);CASC1(S504);CBL(S486);CCDC6(S240);CCDC85C(S246);CCSER1(S448);CD97(S831);CDC25B(S230);CDC25B(S238);CDC25B(S375);CDK12(S383);CDK12(S385);CDK12(T893);CDK16(S138);CDK9(S347);CEP55(S428);CEP57(S55);CHAF1A(S206);CHAMP1(S376);CHAMP1(S507);CHD4(S303);CLASP1(S636);CLINT1(T308);COL4A3BP(S373);CPSF7(S48);CREB1(S111);CREB1(S271);CRTC1(S153);CSPP1(S901);CTU2(S419);DBNL(T291);DIP2B(S259);DLG5(S1000);DLG5(T984);DLGAP4(T975);DLGAP5(S725);DNTTIP2(S434);DVL3(S125);DYNC1LI1(S398);EGLN1(S125);EIF3A(S1188);EIF3A(S1336);EIF3A(S882);EIF3E(S399);EIF4ENIF1(S564);ELAVL1(S202);EML4(S146);EP400(S722);EPN2(S173);ERRFI1(S461);FAM102A(S189);FAM117A(S29);FAM122A(S143);FAM122A(S189);FAM129B(S665);FAM129B(S681);FAM129B(S696);FAM207A(T34);FAM53C(S232);FAM83H(S914);FBRSL1(T1010);FERMT3(S15);FIP1L1(S259);FRMD6(S522);FRMD6(S525);GAB2(S141);GATAD2A(T189);GATAD2B(S334);GATAD2B(S486);GBF1(S1298);GIGYF2(S26);GNL3(S529);GRIP1(S847);GTF2I(S412);GTF3C2(S132);GTF3C2(S167);GTSE1(S575);HCFC1(S666);HIPK1(Y352);HIPK2(Y361);HMGCR(S872);HNRNPA1(S338);HNRNPA2B1(S344);HNRNPA3(S358);IBTK(S1045);INCENP(T292);INPP5D(T963);IRF2BP2(S406);IRF2BPL(S519);ITSN2(S884);ITSN2(S889);JPT2(T76);JUP(S665);KHDRBS1(S20);KHDRBS1(T61);KIAA0319L(S978);KIAA1217(S361);KIAA1522(S858);KIAA1522(S862);KIAA1522(S929);KIF13B(S1410);KIF1A(S1094);KIF1A(S1528);KIF1A(S1532);KLC2(S610);KPNA4(S60);LAD1(S301);LAMTOR1(S27);LARP1(S824);LARP1(T526);LIN54(S310);LINC00337(S30);LMNA(S628);LMNB1(S23);LMNB2(S37);LSM14B(S165);MACF1(S7279);MAP2(S1540);MAP3K4(S1274);MAZ(S361);MCM3AP(S557);MELK(S529);MEPCE(T213);MIA3(S1741);MICAL3(S649);MICALL1(S391);MICALL1(S640);MICALL2(S143);MICALL2(S153);MIS18BP1(S1042);MKI67(S2223);MKI67(T1557);MLC1(S179);MORC2(S696);MPRIP(S993);MTA1(S449);MTA1(S522);MTA2(S435);MTFR1L(S103);MTMR12(S564);MTMR3(S613);MTSS1L(S342);MVB12A(S170);MYC(S62);MYC(T58);NCOA3(Y574);NCOR1(S1980);NCOR1(S1981);NCOR2(S1547);NCOR2(S54);NFATC2(S217);NIFK(T238);NOLC1(S508);NOP58(S351);NUCKS1(T179);NUFIP2(S230);NUMA1(S1862);NUMBL(S263);NUP153(S209);NUP35(S66);OBSL1(S10);PABPN1(S150);PAGR1(S237);PARVA(S19);PBRM1(S13);PBRM1(S14);PCBP1(S190);PCNP(T139);PCYT1A(S315);PCYT1B(S315);PDCD6IP(S730);PGRMC1(S181);PHACTR2(T25);PHAX(S368);PIGT(S235);PKD2(S832);PLEC(S1435);PLEKHA5(T857);PML(S505);POLM(S12);POLR2A(S1878);POLR2A(S1910);PPFIBP1(S601);PPHLN1(S163);PPP1CA(T320);PPP1R13B(S681);PPP1R13L(S358);PPP1R35(S87);PPP1R35(T84);PPP1R9B(S100);PRAG1(S510);PRC1(S4);PRR36(T1082);PRRC2A(S1147);PRRC2A(S1386);PRRC2C(S1544);PSMF1(S153);PTK2(S716);PTPN12(S435);PTPN14(S760);PUM1(S124);PXN(S85);RALGAPA1(T754);RALGAPB(T379);RALY(S135);RANBP3(S211);RASAL3(S51);RB1(S788);RB1(Y790);RBL1(T369);RBM15(S294);RBM15B(S265);RBM15B(S267);RBM17(S169);RBM23(S140);RBM23(S142);RBM39(S97);RBM6(S1025);RBMX(S208);RBMX(S352);RBMXL1(S208);RECQL5(S815);RFX7(S1028);RIPOR1(S351);RLIM(S230);RPA1(T180);RPL28(S115);RPS14(S139);RRBP1(T1046);SAFB(S601);SAMD1(S161);SAMD1(T107);SAP130(S442);SCAF11(S796);SCML2(S267);SCRIB(S1348);SCRIB(S504);SET(S7);SF3B1(T261);SF3B1(T436);SGPP1(S101);SHANK2(S67);SHROOM3(T576);SIK3(T469);SLAIN2(S413);SLTM(S1014);SMAP2(S240);SMARCA2(S588);SMARCD1(S206);SMARCD2(S229);SMARCD3(S181);SMNDC1(S201);SNRK(S518);SNRNP200(S225);SNRNP70(S226);SNRPA1(T180);SNX17(S336);SPTAN1(S1031);SRSF10(S133);SRSF4(S113);SRSF5(S117);SRSF6(S119);SRSF9(S216);SSH3(S37);STAM(S156);STIM2(S523);STK17A(S28);STMN1(S38);STX17(S289);SURF6(S138);SURF6(T229);SYNJ1(S1053);SYTL2(S344);TAF7(S201);TBC1D1(S237);TBX2(S653);THAP4(S128);TJP1(S968);TJP2(S266);TJP2(T462);TJP3(S369);TJP3(S371);TJP3(S591);TK1(S231);TMPO(S306);TMPO(S354);TNIK(S764);TNIK(S766);TNKS1BP1(S1103);TOM1(S464);TP53BP1(S1317);TRA2A(T202);TRA2B(T201);TRA2B(T212);TRAF4(S426);TRAPPC10(S711);TRIM11(S85);TRIP10(S296);TRIP12(S312);TRPM7(S1477);TRPS1(S216);TRPS1(T751);USP10(S211);USP15(S242);USP20(S134);USP32(S1416);USP36(S742);USP54(S1036);USP6(S1214);USP7(S18);UTP20(T1741);VCL(S290);VGLL4(S149);XRCC1(S226);XRCC1(T198);YAP1(S289);YBX3(T67);YTHDC2(S1223);ZC3HAV1(S257);ZC3HAV1(T273);ZCCHC8(T479);ZCCHC8(T485);ZFP64(S547);ZFYVE26(S1764);ZNF136(S405);ZNF318(S1896);ZNF408(T322);ZNF639(S88);ZYX(S308)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CAMK2D</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>122</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(S30);ABI1(S216);ABI1(Y213);ACIN1(T414);ADAM17(S791);AFF4(S1043);AHNAK(S3412);AHNAK(S3426);ANLN(T364);ARAP3(S1444);ARFGAP2(S432);ARHGAP17(S625);BRD4(S1126);BUB1(S655);C2CD5(S662);CDK16(S138);CDK9(S347);CEP170(S881);CEP55(S428);CEP57(S55);CHAMP1(S376);CLINT1(T308);CPSF7(S48);CREB1(S111);CTU2(S419);DBNL(T291);DLGAP5(S725);DOCK7(S898);DYNC1LI1(S398);EIF4B(S207);ELAVL1(S202);EP400(S722);ERRFI1(S461);FAM129B(S696);FAM207A(T34);FGD6(S692);FLYWCH2(S21);GATAD2B(S486);GNL3(S529);GTF3C2(S167);HCFC1(S666);HNRNPA1(S338);HNRNPA2B1(S344);HNRNPC(S253);HNRNPLL(S61);HNRNPM(S528);HUWE1(S1084);JPT2(T76);KHDRBS1(S20);KIAA0319L(S978);LAD1(S301);LMNA(S628);LMNB1(S23);LMNB2(S37);MAST2(S876);MAZ(S361);MEPCE(S217);MEPCE(T213);MTA1(S386);MYC(T58);NADK(S48);NADK(S64);NAV1(S808);NCL(T76);NDRG2(T334);NOLC1(S397);NOLC1(S508);NOLC1(S622);NUFIP2(S230);NUMA1(S1862);NUP35(S66);PABPN1(S150);PCBP1(S190);PCM1(T79);PCM1(T82);PCNP(T139);PDCD6IP(S730);PDLIM2(S129);PHF8(S880);PLEKHG4B(T727);PPP1R13L(S358);PRKDC(T1045);PSMF1(S153);R3HDM2(S349);RALGAPA1(T754);RALY(S135);RBM17(S169);RBM39(Y95);RBMX(S249);RBMXL1(S249);RECQL5(S815);RFX7(S1028);RIF1(S1688);RPA1(T180);RPS27(S78);RPS27L(S78);SAP130(S442);SAPCD2(S157);SCRIB(S1348);SF3B1(T436);SHANK2(S67);SNRPA1(T180);SNRPC(S17);SPEG(S2109);SRSF9(S216);STIM2(S523);STK17A(S28);STMN1(S38);SUPT6H(T1523);TCOF1(S503);TCOF1(T914);THRAP3(S575);TK1(S231);TMPO(S306);TNKS1BP1(S836);TRA2B(T201);TRA2B(T212);UNC13B(S367);VGLL4(S149);ZCCHC8(T479);ZCCHC8(T485);ZYX(S308)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CAMK2G</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>185</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(S30);ABI1(S216);ADAM17(S791);AFF4(S1043);AGAP2(S808);AHNAK(S115);AHNAK(S3412);AHNAK(S3426);AMBRA1(S1205);APPL1(S401);ARAP3(S1444);ARFGAP2(S368);ARFGAP2(S432);ARHGAP17(S625);ARID1A(S1184);BCAM(S600);BRD4(S1126);BUB1(S655);C2CD5(S662);CALU(S35);CALU(S44);CAMSAP1(S563);CDCA7L(S261);CDK16(S138);CDK9(S347);CEP170(S881);CEP55(S428);CEP57(S55);CHAMP1(S376);CLINT1(T308);CPSF7(S48);CREB1(S111);CTU2(S419);DBNL(T291);DENND4C(S1099);DLGAP5(S725);DOCK7(S898);DOCK8(S451);DYNC1LI1(S398);EEPD1(S21);EIF4B(S207);ELAVL1(S202);EP400(S722);ERRFI1(S461);EVL(S331);FAM129B(S696);FAM207A(T34);FGD6(S692);FLYWCH2(S21);GAB2(S141);GAPVD1(S902);GATAD2B(S486);GNL3(S529);GON4L(S206);GPATCH2(S195);GTF3C2(S167);HCFC1(S666);HNRNPA1(S338);HNRNPA2B1(S344);HNRNPLL(S61);HNRNPM(S528);HNRNPM(S618);HUWE1(S1084);IRF2BP2(S318);KHDRBS1(S20);KIAA0319L(S978);LAD1(S301);LIMA1(S617);LMNA(S628);LMNB1(S23);LMNB2(S37);LRCH4(S520);MAP1A(S1675);MARK2(S456);MAST2(S876);MAZ(S361);MEPCE(S217);MEPCE(T213);MICAL3(S649);MICALL1(S486);MTA1(S386);MYC(T58);NADK(S48);NADK(S64);NAV1(S808);NDRG2(T334);NOLC1(S397);NOLC1(S508);NOLC1(S622);NSD1(S2471);NUFIP2(S230);NUMA1(S1862);NUP210(S1881);NUP35(S66);OSBPL8(S68);PABPN1(S150);PCBP1(S190);PCM1(T79);PCM1(T82);PCNP(T139);PDCD6IP(S730);PDLIM2(S129);PDZD8(S521);PFKL(S775);PHAX(S368);PLK1(T214);PLPPR3(S353);PPHLN1(S163);PPP1R13L(S358);PPP1R9B(S100);PRKDC(T1045);PSMF1(S153);PTPN12(S449);R3HDM2(S349);RALGAPA1(T754);RALY(S135);RASAL3(S18);RASAL3(S51);RASAL3(S72);RB1(T356);RBL1(S640);RBL1(S749);RBL1(T369);RBM10(S845);RBM15B(S265);RBM17(S169);RBM39(Y95);RBMX(S249);RBMX(S332);RBMX(S352);RBMXL1(S249);RECQL5(S815);RFX7(S1028);RIF1(S1688);RPA1(T180);RPS27(S78);RPS27L(S78);SAP130(S442);SCRIB(S1348);SF3B1(T436);SFSWAP(S909);SH3BP2(S427);SHANK2(S67);SIK3(S866);SLTM(S551);SNRPA1(T180);SPEG(S2109);SRSF9(S216);STIM2(S523);STK17A(S28);STMN1(S38);SUPT6H(T1523);SVIL(S968);TACC3(S250);TBC1D1(S211);TBC1D9B(S435);TCF20(S574);TCOF1(S1227);TCOF1(S503);TCOF1(T914);THRAP3(S248);THRAP3(S575);TK1(S231);TMEM201(S441);TMX1(S270);TOR1AIP1(S135);TPD52(S176);TPD52L2(S166);TRA2A(T202);TRA2B(T201);TRA2B(T212);UNC13B(S367);UNC93B1(S547);UNC93B1(S550);UNG(T60);UPF3B(T169);USP36(T653);VGLL4(S149);XRCC6(S477);ZCCHC8(S598);ZCCHC8(T479);ZCCHC8(T485);ZFHX4(S2996);ZNF24(S274);ZYX(S308)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CAMKK2</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>750</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(S30);AAK1(S14);ABI1(S216);ABI1(Y213);ABLIM1(S431);ABR(T74);ACIN1(T414);ACTA1(S241);ACTA2(S241);ACTB(S239);ACTBL2(S240);ACTC1(S241);ACTG1(S239);ACTG2(S240);ADAM10(S740);ADAM10(Y741);ADAM17(S791);ADD1(S12);ADD1(S431);ADD1(S726);ADD2(S713);ADD3(S693);AFDN(S1721);AFF4(S1043);AFF4(S1058);AFF4(S32);AGAP2(S808);AHCTF1(S528);AHDC1(S1064);AHDC1(S1507);AHNAK(S115);AHNAK(S216);AHNAK(S3412);AHNAK(S3426);AHNAK(S5731);AKAP11(S1580);AKAP11(S422);AKAP11(S448);AKAP13(S2728);AMBRA1(S1205);AMBRA1(S639);ANAPC1(S355);ANKRD17(S2401);ANKS1A(S382);ANKZF1(S675);ANLN(S518);ANP32B(T244);APPL1(S401);ARAP3(S1444);ARFGAP1(T135);ARFGAP2(S368);ARFGAP2(S432);ARHGAP1(S44);ARHGAP1(S51);ARHGAP17(S625);ARHGAP21(S856);ARHGEF11(S150);ARHGEF11(S35);ARHGEF17(S735);ARHGEF18(S1111);ARHGEF26(S80);ARID1A(S1184);ARID1A(S1604);ARID1A(S730);ARID3B(S381);ARL6IP6(S80);ASF1B(T179);ATAD2(S327);ATG2B(S1582);ATG2B(S1583);ATG2B(Y1577);ATN1(S661);ATN1(T653);ATXN2(S684);ATXN2(T666);BAG3(S289);BAG3(T285);BAP18(S110);BCAM(S600);BCL11A(S328);BCL2L12(S113);BCL2L12(S121);BCL2L12(T117);BCR(S459);BIN2(S259);BPTF(S1300);BRD4(S1126);BRIP1(S956);BRSK2(T459);BRSK2(T463);BUB1(S655);C16orf54(S194);C16orf72(S167);C2CD2L(S662);C2CD5(S281);C2CD5(S662);C6orf132(S449);C7orf50(S175);CABLES1(S291);CALU(S35);CALU(S44);CAMSAP1(S563);CARMIL2(S1315);CAT(S515);CBL(S799);CBX8(S311);CCDC6(S240);CCDC9(S376);CCDC93(S305);CCL13(S44);CD97(S818);CD97(S831);CDC25C(S216);CDCA7L(S261);CDK13(T1056);CDK16(S138);CDK9(S347);CDV3(T182);CENPF(S276);CENPF(S3119);CEP170(S881);CEP55(S428);CEP57(S55);CEP97(S308);CHAF1A(S206);CHAMP1(S376);CHAMP1(S432);CHAMP1(S436);CHAMP1(S445);CHAMP1(S452);CHAMP1(S472);CHAMP1(S507);CHD4(S303);CHD8(S1978);CHD8(T1982);CIT(S1322);CLASP1(S636);CLASP2(S325);CLASP2(S529);CLASRP(S547);CLINT1(T308);CLK2(S142);CMTR1(S31);CNK3/IPCEF1(S892);CNP(S170);COL4A3BP(S373);CPSF7(S48);CREB1(S111);CREB1(S271);CSPP1(S901);CTAGE1(S616);CTAGE5(S647);CTPS1(S573);CTU2(S419);CYBA(T147);DACH1(S727);DAXX(S671);DBF4(S381);DBNL(T291);DDX21(S89);DDX3Y(S592);DENND4A(T1019);DENND4C(S1099);DGCR8(S271);DGCR8(S275);DGCR8(Y267);DIP2B(S259);DLG5(S1000);DLG5(T984);DLGAP5(S725);DNTTIP2(S434);DNTTIP2(T172);DOCK7(S898);DOCK7(S946);DOCK8(S451);DPYSL2(T509);DTL(S425);DYNC1LI1(S398);DYNC1LI1(S421);EEPD1(S21);EIF3E(S399);EIF4B(S207);EIF4ENIF1(S564);ELAVL1(S202);EML4(S144);EML4(S146);ENAH(T538);EP400(S722);EP400(S736);EPB41L1(S784);EPS15L1(S793);ERCC5(S384);ERRFI1(S461);ESF1(S198);EVL(S331);EZH2(S363);EZH2(T367);FADD(S194);FAM117B(S10);FAM122A(S143);FAM122A(S189);FAM129B(S665);FAM129B(S681);FAM129B(S696);FAM207A(T34);FAM53B(S179);FAM53C(S232);FAM76B(S193);FAM83B(S766);FAM83H(S914);FANCI(S1121);FARSA(S301);FBRSL1(T1010);FBXW9(S59);FGD6(S692);FIP1L1(S259);FLYWCH2(S21);FOXK1(S416);FOXK1(S420);FOXK1(S441);FOXO1(S329);FRMD3(S416);FTSJ3(T573);FUS(S462);FXR2(S601);FXR2(T411);GAB2(S141);GAGE13(S33);GAGE2A(S32);GAGE2B(S32);GAGE2D(S32);GAPVD1(S902);GATAD2A(T189);GATAD2B(S334);GATAD2B(S486);GBF1(S1061);GBF1(S1298);GFI1(S94);GIGYF2(S26);GJA1(S262);GNL3(S529);GPATCH2(S195);GRIP1(S847);GSK3B(S9);GTF2F1(S385);GTF2F1(T389);GTF2F1(T446);GTF3C2(S132);GTF3C2(S167);HCFC1(S598);HCFC1(S666);HDAC1(S406);HELB(S1050);HIC2(S348);HIST1H1E(T18);HJURP(S557);HMGA1(S36);HMGCS1(T490);HNRNPA1(S338);HNRNPA2B1(S344);HNRNPA3(S358);HNRNPC(S253);HNRNPLL(S61);HNRNPM(S528);HNRNPM(S618);HPS5(S534);HRNR(S903);HSPB1(S15);HSPB1(S82);HUWE1(S1084);IBTK(S1045);IGLL1(S58);INCENP(T292);INPP5D(T963);INTS12(S128);IPCEF1(S430);IRF2BP1(S421);IRF2BP2(S175);IRF2BP2(S318);IRF2BP2(S406);IRF2BPL(S519);ITGAL(S37);ITSN2(S884);ITSN2(S889);JADE3(S566);JMJD1C(S1223);JMJD1C(S641);JPT2(T76);KANK2(S172);KANK2(S175);KCAB2_HUMAN_Phospho (ST);KCNK2(S366);KHDRBS1(S20);KHDRBS1(T61);KIAA0319L(S978);KIAA1217(S357);KIAA1217(S361);KIAA1468(T143);KIAA1522(S858);KIAA1522(S862);KIAA1522(S929);KIF1A(S1094);KIF1A(S1528);KIF1A(S1532);KNOP1(S119);KPNA4(S60);KRT13(S427);KRT8(S36);L1TD1(S557);LAD1(S301);LAMTOR1(S27);LARP1(S1056);LARP1(S90);LARP1(T526);LAT2(S135);LAT2(S86);LEMD3(S187);LIMA1(S617);LIN28B(S203);LIN54(S310);LMNA(S390);LMNA(S628);LMNB1(S23);LMNB2(S37);LRCH1(S532);LRCH4(S520);LRRFIP1(S116);LRRFIP2(S324);LSM11(S21);LSR(S464);LSR(T453);LUZP1(S745);MACF1(S7330);MAML1(S360);MAP1A(S1675);MAP1A(S1776);MAP2(S1540);MAP2(S1653);MAP2(T1649);MAP3K20(S648);MAP7D1(S93);MARCKS(S163);MARK1(S588);MARK2(S456);MAST2(S876);MAZ(S361);MCM3(Y708);MCM3AP(S557);MCM4(S120);MDC1(T378);MEPCE(S217);MEPCE(T213);MFAP1(S116);MIA2(S1255);MIA3(S1741);MICAL3(S649);MICALL1(S391);MICALL1(S486);MICALL1(S640);MICALL2(S143);MICALL2(S153);MIS18BP1(S1042);MKI67(S2223);MLC1(S179);MLLT6(S378);MLLT6(S382);MORC2(S696);MORC2(S725);MPLKIP(S47);MPLKIP(T51);MPLKIP(Y45);MTA1(S386);MTA1(S449);MTA1(S522);MTA2(S435);MTFMT(S23);MTMR12(S564);MTMR3(S613);MTMR4(S961);MTOR(S2454);MTSS1L(S342);MYBBP1A(S11);MYC(S62);MYC(T58);MYCBP2(S3467);MYCN(S156);MZT2A(S139);MZT2B(S139);NAA10(S186);NAA30(S199);NAB1(S403);NAB2(S171);NADK(S48);NADK(S64);NASP(T390);NAV1(S808);NCAPD2(Y1325);NCL(T121);NCL(T76);NCOR1(S1980);NCOR1(S1981);NCOR2(S1547);NCOR2(S2424);NCOR2(S54);NDRG2(T334);NES(S768);NFATC2(S217);NFATC2(S814);NIFK(T238);NOLC1(S397);NOLC1(S508);NOLC1(S622);NOLC1(S643);NONO(T450);NOP16(S16);NOP2(S732);NOP53(S29);NOP58(S351);NSD1(S2471);NUCKS1(T179);NUFIP2(S230);NUMA1(S1862);NUMA1(S1887);NUMA1(T2000);NUMBL(S263);NUP153(S209);NUP210(S1877);NUP210(S1881);NUP210(T1844);NUP35(S66);OBSL1(S10);OSBPL8(S68);PABPN1(S150);PAGR1(S237);PARD3(S221);PARVA(S19);PATL1(S278);PBRM1(S12);PBRM1(S13);PBRM1(S14);PBX2(S330);PCBP1(S190);PCBP1(S231);PCM1(T79);PCM1(T82);PCNP(T139);PCYT1A(S315);PCYT1A(S347);PCYT1B(S315);PDCD6IP(S730);PDLIM2(S129);PDLIM4(S112);PDS5B(T1301);PDZD8(S521);PEA15(S116);PEAK1(S823);PFKL(S775);PGRMC1(S181);PHACTR1(S505);PHACTR2(T25);PHF3(S1614);PHF8(S880);PHKA2(S1043);PI4K2A(S51);PIK3AP1(S759);PKP4(S273);PKP4(S314);PLCB3(S926);PLEC(S1435);PLEKHA5(S937);PLEKHA5(T857);PLEKHA7(S903);PLEKHG4B(T727);PLK1(T214);PLPPR3(S353);PML(S505);POLA2(T127);POLD2(S15);POLM(S372);POM121(S298);POM121C(S275);POMZP3(S33);POTEE(S939);POTEF(S939);POTEKP(S239);PPFIBP1(S636);PPHLN1(S163);PPHLN1(S201);PPHLN1(T200);PPME1(S15);PPP1CA(T320);PPP1CC(T311);PPP1R13B(S681);PPP1R13L(S358);PPP1R9B(S100);PRAG1(S510);PRKDC(T1045);PRR12(S314);PRR36(T1082);PRRC2A(S1147);PRRC2A(S2113);PSMF1(S153);PTDSS2(S16);PXN(S85);R3HDM2(S349);RAB11FIP1(S529);RAD18(S103);RALGAPA1(T754);RALGAPB(T379);RALY(S135);RANBP2(S2454);RANBP2(S2900);RANBP2(T1396);RANBP3(S211);RANBP9(S477);RANBP9(S482);RASAL3(S18);RASAL3(S51);RASAL3(S72);RASGRP2(S391);RB1(S249);RB1(S788);RB1(T356);RB1(T821);RB1(T826);RB1(Y790);RBL1(S749);RBL1(T369);RBL2(S413);RBM10(S845);RBM15(S294);RBM15(S622);RBM15B(S265);RBM17(S169);RBM39(S97);RBM39(Y95);RBM6(S1025);RBMX(S208);RBMX(S249);RBMX(S352);RBMXL1(S208);RBMXL1(S249);RBMXL1(S88);RECQL5(S815);REPS1(S709);RFX7(S1028);RGPD1(S1463);RGPD2(S1471);RGPD3(S1479);RGPD4(S1479);RGPD5(S1478);RGPD8(S1478);RIF1(S1688);RIF1(S2205);RIPOR1(S351);RPA1(T180);RPL18(S161);RPL18(T158);RPRD2(S665);RPRD2(T732);RPS27(S78);RPS27L(S78);RRBP1(T1046);RRM2(T33);RRP15(T104);RRP1B(S735);RSL1D1(S392);RSL1D1(S396);RSL1D1(T465);SACS(S1779);SAFB2(S787);SALL2(S806);SAMD1(S161);SAMD4B(S172);SAP130(S442);SAPCD2(S157);SASH3(S21);SCML2(S267);SCRIB(S1348);SCRIB(S1448);SCRIB(S504);SEC16A(S1905);SEC31A(S799);SEPT9(S22);SET(S7);SF3B1(S129);SF3B1(T223);SF3B1(T227);SF3B1(T257);SF3B1(T303);SF3B1(T313);SF3B1(T426);SF3B1(T436);SFPQ(S33);SFSWAP(S909);SGO1(S468);SH3BP2(S427);SHANK2(S67);SHROOM3(T576);SIK3(T469);SIPA1L1(S1565);SLC4A1AP(S82);SLTM(S1002);SLTM(S551);SLTM(S553);SLX4(S1309);SLX4(S1333);SMARCA2(S588);SMARCAD1(S146);SMNDC1(S201);SNRK(S518);SNRNP200(S225);SNRNP70(S226);SNRPA1(T180);SNURF(S32);SNX17(S336);SNX17(S409);SPECC1(S55);SPEG(S2109);SRRM1(S695);SRRM2(S1499);SRRM2(S510);SRSF1(S199);SRSF1(S201);SRSF9(S216);SSB(S366);STAM(S156);STIM2(S523);STK10(S450);STK17A(S28);STMN1(S38);SUPT6H(T1523);SURF6(S138);SVIL(S968);SYNJ1(S1053);SYTL2(S344);TACC3(S25);TACC3(S250);TACC3(S317);TAF7(S201);TAOK1(S965);TBC1D1(S211);TBC1D9B(S435);TBX2(S653);TCF20(S574);TCF20(S966);TCOF1(S1227);TCOF1(S156);TCOF1(S503);TCOF1(T914);TELO2(S836);TEX2(S732);THAP4(S128);THOC5(S314);THRAP3(S248);THRAP3(S575);THRAP3(S928);TICRR(T1260);TJAP1(S320);TJAP1(T318);TJAP1(Y316);TJP1(S617);TJP2(S266);TK1(S231);TLN1(S425);TMPO(S306);TMPO(S354);TMX1(S270);TNIK(S764);TNIK(S766);TNKS1BP1(S1103);TNKS1BP1(S836);TNRC6C(S714);TOM1(S464);TOR1AIP1(S135);TP53BP2(S558);TPD52(S176);TPD52L2(S166);TPR(S379);TRA2A(T202);TRA2B(T201);TRA2B(T212);TRIM24(S654);TRIM71(S187);TRIP12(S312);TRPM7(S1477);TRPS1(S216);TRPS1(T751);TUBA1A(S48);TUBA1B(S48);TUBA1C(S48);TUBA3C(S48);TUBA3E(S48);TXLNG(S97);U2SURP(S37);UBE2O(T838);UBE4B(S65);UBE4B(T64);UCK1(S253);UNC13B(S367);UNC93B1(S547);UNC93B1(S550);UNG(T60);UPF3B(T169);USP10(S211);USP15(S242);USP20(S134);USP32(S1416);USP36(S546);USP36(S742);USP36(T653);USP6(S1214);USP7(S18);VCL(S290);VGLL4(S149);VPS13D(S1042);WBP11(S237);WDFY4(S3123);WIPF1(S340);WIZ(S1012);WT1(S273);XPO4(S521);XRCC1(S226);XRCC1(S229);XRCC1(T198);XRCC1(Y211);XRCC6(S477);YAP1(S289);YBX3(T67);YTHDC2(S1223);ZC3H11A(S132);ZC3H4(S907);ZCCHC8(S598);ZCCHC8(T479);ZCCHC8(T485);ZDHHC5(S425);ZFHX4(S2996);ZFP64(S547);ZFP91(S101);ZFP91(S103);ZFYVE26(S1764);ZMYM4(T217);ZNF24(S274);ZNF318(S1896);ZNF318(S501);ZNF462(S1251);ZNF574(S164);ZNF639(S88);ZNF687(S374);ZYX(S308)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CDK1</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>92</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(T142);AEBP2(S24);AGFG1(S181);AMFR(S542);ANKRD17(S2401);ANLN(S182);ANLN(T194);ARHGAP29(S1029);ASIC3(S37);ATXN2L(S424);BAG3(T285);BAZ1B(S349);CDCA2(S98);CDK14(S134);CENPF(S276);CHAMP1(S416);DCDC2(S270);DENND4A(S1256);DLG5(S1209);DNMT1(S127);DNMT1(T137);EHBP1L1(S285);EIF4B(S283);ERLIN1(S324);FGFR1OP(T170);FOXP1(S83);GRB10(S104);GTF2I(S210);GTF2I(T558);HAUS6(T584);HBS1L(T231);HCFC1(S666);HIST1H1B(S18);INCENP(S311);JPT2(S97);KIAA1522(S971);LARP6(S409);LINC00322(S226);MAP7D1(S399);MARK2(S456);MARK2(S619);MARK3(S469);MEF2D(S180);MPLKIP(S115);MYO9B(S1405);NCOR2(S956);ORC6(T195);PARVA(S19);PDCD4(S94);PDLIM5(S111);PI4KB(S266);PLCL2(S17);PLEKHA5(S885);PLEKHG3(S76);PLPPR3(S508);PPFIA3(S1164);PPL(S14);PPM1H(S221);PQBP1(S247);PRAG1(S889);PRRC2A(T1347);RAB11FIP1(S435);RAB40C(S268);RBSN(S429);REPIN1(S27);RPA1(T180);SATB1(S637);SHROOM3(S242);SKIV2L(S131);SLC9A3R1(S280);SNRK(S518);SNRPA1(T180);SNTB1(S87);SORBS3(S530);SRRM2(S2382);SRSF7(S165);STIM2(S523);TCOF1(S583);TET2(S1107);TRIM37(S771);UBE2O(S515);UCKL1(S56);WIPF2(S235);XPR1(S666);XRCC1(S226);XRCC1(S229);XRCC1(S241);XRCC1(T198);ZC3H11A(T321);ZFR(S1054);ZNF638(S1401);ZYX(S259)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CDK16</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>4</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>AHCTF1(S528);CTU2(S419);MARK2(S456);RBL2(S413)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>CDK17</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>19</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(S30);AMBRA1(S1205);CTU2(S419);ELAVL1(S202);EPB41L5(S436);HTT(S1199);IRS1(S374);LMNA(S628);MAP4(S928);MAP7D1(S399);MARK2(S456);MAST2(S1364);OTUD4(S416);PRAM1(S334);RANBP1(S60);RBL1(T369);RBL2(S413);SRRM1(S429);TRA2A(T202)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CDK2</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>537</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(T142);09/09/18 00:00:00(T49);ACD(S425);ADD1(S12);ADNP(S709);AEBP2(S24);AEBP2(S390);AFF4(S1043);AFF4(S1062);AFF4(S703);AGFG1(S181);AGFG1(T177);AHNAK(S177);AHNAK(S2397);AHNAK(S5731);AKAP13(S2563);AKAP3(S208);AMBRA1(S1205);AMFR(S542);ANK3(S4298);ANKLE2(S268);ANLN(S182);ANLN(S518);ANLN(T194);ANLN(T364);APPL1(S401);ARFGAP1(T135);ARHGAP17(S625);ARHGAP29(S1029);ARHGEF16(S174);ARHGEF26(S80);ARID1A(S301);ARID1A(S363);ARID3A(S362);ASF1B(T179);ASH1L(S1170);ASH1L(T1165);ATF7(S434);ATP13A1(S899);ATRIP(S224);ATXN2(S624);ATXN2(S684);ATXN2(T666);ATXN2L(S424);BAG3(S289);BAG3(T285);BAP18(S110);BAP18(S96);BAZ1A(T1547);BAZ1B(S349);BAZ2A(S1397);BCL9L(S1017);BCL9L(S999);BPTF(S1300);BPTF(S2098);BRD4(S1064);BRD4(S1117);BRIP1(S206);C12orf43(S179);C12orf45(S178);C16orf72(S167);CAD(T1884);CAMSAP3(S368);CBX5(S92);CBX8(S110);CBX8(S265);CCDC117(S53);CCNE2(S21);CD3EAP(S172);CD3EAP(S285);CDC25B(S375);CDCA2(S98);CDCA3(S68);CDCA5(S75);CDK12(T893);CDK13(S317);CDK14(S134);CENPC(S177);CENPF(S276);CENPF(S3094);CENPF(S3119);CHAF1A(T865);CHAMP1(S297);CHAMP1(S416);CHAMP1(S507);CHD1(S90);CLASP2(S952);CLASRP(S547);CLSPN(S775);CNOT2(S165);CNOT2(T93);CPEB2(S89);CPEB2(S92);CREB1(S271);CRMP1(S522);CTTN(T401);CTTN(Y421);CTU2(S419);CXXC1(S143);DAG1(T790);DCDC2(S270);DCP2(S284);DDX21(S71);DENND4A(S1256);DIDO1(S1019);DKC1(S21);DLG5(S1209);DLGAP5(S662);DMAP1(T445);DNM1L(S616);DNMT1(S127);DNMT1(T137);DNTTIP2(S117);DNTTIP2(S330);DOT1L(S786);DPYSL2(T509);DTL(S425);DTL(T429);DTNA(T504);DTNB(T468);DUS3L(T240);DYNC1LI1(S421);DYNC1LI2(S407);DYNC1LI2(S446);DYRK2(S30);E2F7(S825);E2F8(S71);ECSIT(Y302);EFHD2(S74);EHBP1L1(S285);EHMT1(S435);EIF4ENIF1(S120);ELAVL1(S202);EML3(T881);EPB41(S712);EPB41L5(S436);ERCC5(S384);ERLIN1(S324);ERRFI1(S461);ESCO1(S412);ESCO2(S75);ESF1(S198);FAM122A(S76);FAM122B(S115);FAM53C(S162);FBXO46(S293);FGFR1OP(T170);FIP1L1(S259);FLCN(S62);FLYWCH2(S21);FNBP1(S359);FOXK1(S213);FOXK1(S223);FOXK1(S416);FOXO4(S230);FOXP1(S83);FTSJ3(T573);GATAD2A(S340);GATAD2A(S546);GATAD2B(S486);GIGYF1(S756);GNL3L(S465);GRB10(S104);GSK3A(Y279);GSK3B(Y216);GTF2I(S210);GTF2I(T558);GTF3C1(S1653);GTF3C2(S132);GTSE1(S536);H2AFY(T129);HACD3(S135);HBS1L(T231);HCFC1(S666);HEY2(S39);HIRIP3(S27);HIST1H1B(S18);HJURP(S557);HMGA1(S36);HMGA1(S44);HMGA1(T53);HMGXB4(S497);HNRNPA2B1(S259);HNRNPLL(S61);HSH2D(S194);HSPH1(S809);HUWE1(S2534);INCENP(S275);INCENP(S311);INF2(S589);INTS10(S231);IRF2BP1(S436);JPT2(S97);KDM2A(T550);KIAA1217(S1806);KIAA1522(S342);KIAA1522(S979);KIF18B(S413);KIF20B(S1740);KIF4A(S1225);KIF4B(S1227);KLC2(S445);KMT2A(S3511);KMT2D(S2309);KPNA2(S62);LAMTOR1(S27);LEMD3(S187);LIG3(S210);LIMD2(S29);LIN54(S310);LMNA(S22);LMNA(S628);LMNB1(S391);LMNB1(S393);LMNB2(S405);LMNB2(S407);LRCH3(S419);LRCH4(S309);MAP2(S1540);MAP7D1(S399);MARK2(S456);MARK2(S619);MASTL(S370);MASTL(S453);MCM4(S120);MED1(S1223);MEF2D(S180);MEPCE(S254);MGA(S1208);MGA(S1457);MKI67(S1207);MKI67(S1937);MKI67(S2223);MKI67(S2344);MKI67(S648);MKI67(T2231);MKL2(S921);MLF2(S238);MPLKIP(S115);MPLKIP(S47);MPLKIP(T51);MPLKIP(Y45);MRGBP(S195);MSANTD2(S79);MSL3(S400);MSL3(T405);MTA1(S386);MTA1(S576);MTCL1(S1808);MTDH(S568);MYBBP1A(S11);MYBBP1A(S1163);MYBBP1A(S1290);MYO9B(S1405);MYO9B(S717);MZT2A(S139);MZT2B(S139);NAA10(S186);NAA30(S89);NAV1(S541);NAV2(S1245);NCL(T121);NCOA1(S395);NCOR2(S1487);NCOR2(S1786);NCOR2(S2404);NCOR2(S956);NELFE(S131);NELFE(S353);NFIC(S323);NFRKB(S1291);NIFK(S230);NIPBL(S306);NIPBL(S350);NOLC1(S397);NONO(T450);NOP2(S732);NSD2(S437);NUCKS1(S181);NUMA1(T2000);NUP107(S11);NUP133(S50);NUP210(T1844);NUP35(S73);ORC2(T116);ORC6(T195);OSBPL10(S201);PACS1(S495);PAICS(S27);PALM3(S303);PARVA(S19);PCM1(T79);PCM1(T82);PDCD4(S94);PDCD6IP(S730);PDLIM5(S111);PDLIM5(S360);PDXDC1(S718);PHC3(S315);PHF3(S283);PHLDB1(S419);PHRF1(S867);PI4KB(S266);PIAS1(S488);PIAS1(S503);PIKFYVE(S329);PKP2(S82);PLCB3(S934);PLCB3(T924);PLEKHA5(S607);PLEKHA5(S933);PLEKHA5(S937);PLEKHA5(T438);PLEKHA7(S903);PLEKHG3(S76);PLPPR3(S508);POU2F1(T270);PPFIA3(S1164);PPL(S14);PPM1H(S221);PPP1R13L(S526);PPP1R14B(S32);PPP4R2(S226);PPP4R3B(S840);PPP6R1(S759);PQBP1(S247);PRC1(T481);PRRC2A(T1347);PRRC2C(S779);PSMA5(S16);PSMF1(S153);RAB11FIP1(S435);RAB11FIP1(S528);RAB11FIP1(S529);RAB3IL1(S179);RAB40C(S268);RAD18(S103);RAD18(S99);RALBP1(S34);RALY(S135);RANBP2(S1456);RANBP2(S788);RANBP2(T1396);RANBP2(T1412);RANBP2(T2613);RASAL3(S72);RB1(S249);RB1(S612);RB1(S811);RB1(T601);RB1(T821);RB1(T826);RB1(Y606);RBBP6(S516);RBL1(S1041);RBL1(T369);RBL2(S1112);RBL2(S413);RBL2(T417);RBMX(S208);RBMX(S332);RBMXL1(S208);RBSN(S429);REPIN1(S27);RGPD1(S779);RGPD2(S787);RGPD3(S789);RGPD4(S789);RGPD5(S788);RGPD8(S788);RIF1(S1454);RIF1(S2161);RIF1(S2348);RIOX1(S109);RIPK3(S316);RPA1(T180);RPAIN(S18);RPS6KB2(S423);RRBP1(T1046);RREB1(S36);RREB1(S42);RRM2(S20);RRM2(T33);RRP15(T104);RRP1B(S513);RRP1B(S679);RRP1B(S680);RRP1B(S702);RRP1B(S706);RRP1B(S735);RSF1(S392);RSF1(S397);RSL1D1(S469);RSL1D1(T465);RTN3(S229);SAMD1(S161);SAP130(S442);SATB1(S637);SCFD1(S303);SCML2(S267);SCRIB(S1445);SEC61B(S14);SENP3(S181);SETDB1(S1066);SF3B1(T211);SF3B1(T223);SF3B1(T227);SF3B1(T436);SFPQ(S33);SHROOM3(S242);SIPA1L1(S1565);SIPA1L2(S148);SLAIN2(S391);SLAIN2(S63);SLC4A1AP(S82);SLC9A3R1(S280);SLX4(S1185);SLX4IP(S396);SMARCA5(S116);SMARCA5(T113);SNAPIN(S133);SNRK(S518);SNRPA1(T180);SNTB1(S87);SNTB2(S393);SORBS3(S530);SP2(S78);SPTY2D1(S471);SRCAP(S3148);SRRM2(S1014);SRRM2(S2382);SRRM2(T1531);SRRM2(T2289);SRSF11(S207);SRSF9(S211);STIM2(S523);STMN1(S25);SUGT1(S281);SURF6(T229);TACC3(S25);TACC3(S71);TAF9(T159);TANC2(S169);TAOK1(S421);TCF20(S1019);TCF20(S1335);TCF20(S966);TCF3(S379);TCOF1(S1257);TCOF1(S156);TCOF1(S583);TELO2(S836);THOC2(T1443);THRAP3(S253);TICRR(S1430);TICRR(S1433);TICRR(S923);TINF2(S330);TIPIN(T224);TLK1(S159);TLK2(S99);TLN1(S425);TNKS1BP1(S1297);TNKS1BP1(S1715);TNKS1BP1(S178);TNKS1BP1(S435);TNS3(S660);TOP2A(S1213);TP53BP1(S265);TRIM33(S862);TSC22D4(S279);TTF1(S65);TTF2(S883);TUBA1A(S48);TUBA1B(S48);TUBA1C(S48);TUBA3C(S48);TUBA3E(S48);U2SURP(S67);UBAP2L(S416);UBE4B(S65);UBE4B(S79);UBE4B(S83);UBE4B(T64);UCKL1(S56);UFD1(S247);USP20(S408);USP24(S1141);USP32(S1430);USP36(S546);USP36(S713);VCL(S290);VENTX(S6);VPS26B(S304);WBP11(S237);WIPI2(S413);WIZ(S1012);WIZ(S996);XRCC1(S226);XRCC1(S229);XRCC1(S241);XRCC1(S266);XRCC1(T198);XRCC1(Y211);YAP1(S131);YEATS2(S627);YTHDC2(S1221);ZBTB3(S549);ZBTB7A(S526);ZC3H11A(S132);ZC3H11A(T321);ZC3H13(S209);ZC3H13(S64);ZC3H4(S907);ZC3H4(S908);ZC3HAV1(S378);ZFP91(S101);ZFR(S1054);ZMYM2(S305);ZMYM4(T217);ZNF219(S684);ZNF239(S191);ZNF286A(S19);ZNF444(S232);ZNF444(S235);ZNF462(S1090);ZNF462(S688);ZNF552(S86);ZNF574(S164);ZNF587B(S87);ZNF609(S804);ZNF638(S1401);ZNF687(S433);ZNF814(S87);ZXDC(S34);ZYX(S259);ZYX(S267)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>CDK4</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>684</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(S30);09/09/18 00:00:00(T142);09/09/18 00:00:00(T49);AAK1(S14);ABI1(S216);ABI1(Y213);ABL2(S936);ABLIM1(S431);ABR(T74);ACIN1(T414);ACTA1(S241);ACTA1(S54);ACTA2(S241);ACTA2(S54);ACTB(S239);ACTB(S52);ACTBL2(S240);ACTC1(S241);ACTC1(S54);ACTG1(S239);ACTG1(S52);ACTG2(S240);ACTG2(S53);ADAM17(S791);ADD1(S12);ADD1(S431);ADNP(S709);AEBP2(S24);AFDN(S1721);AFF4(S1043);AFF4(S1058);AFF4(S32);AGFG1(S181);AGFG1(T177);AHCTF1(S528);AHDC1(S1064);AHDC1(S1507);AHNAK(S115);AHNAK(S177);AHNAK(S216);AHNAK(S3412);AHNAK(S3426);AHNAK(S41);AHNAK(S5731);AKAP11(S1580);AKAP11(S448);AKAP11(T1100);AKAP13(S2728);AMBRA1(S639);AMPD2(S100);ANKRD39(S153);ANKZF1(S675);ANLN(S182);ANLN(S518);ANLN(T194);ANLN(T364);ANP32B(T244);APPL1(S401);ARFGAP1(T135);ARFGAP2(S368);ARHGAP1(S44);ARHGAP1(S51);ARHGAP17(S625);ARHGAP21(S856);ARHGAP29(S1029);ARHGAP39(S407);ARHGEF11(S150);ARHGEF16(S174);ARHGEF17(S735);ARHGEF26(S80);ARID1A(S1604);ARID1A(S363);ARID1A(S730);ARID3B(S381);ARL6IP6(S80);ASF1B(T179);ATAD2(S327);ATAT1(S315);ATF1(S198);ATG2B(S1582);ATG2B(S1583);ATG2B(Y1577);ATN1(S661);ATN1(T653);ATRIP(S224);ATXN2(S684);ATXN2(T666);ATXN2L(S424);BAG3(S195);BAG3(S289);BAG3(T285);BAZ1B(S349);BCAM(S600);BCL11A(S328);BCL2L12(S113);BCL2L12(S121);BCL2L12(T117);BMS1(S552);BPTF(S1300);BRD4(S1117);BRD4(S1126);BRIP1(S956);BRSK2(S439);BRSK2(T459);BRSK2(T463);BUB1(S655);C16orf72(S167);C2CD5(S281);C2CD5(S662);C6orf106(S215);C6orf132(S449);C7orf50(S175);CABLES1(S291);CARHSP1(S41);CARMIL2(S1315);CCDC6(S240);CD97(S831);CDC42EP4(S292);CDCA2(S98);CDCA7L(S139);CDK13(T1056);CDK14(S134);CDK16(S138);CDK18(S117);CDK9(S347);CDV3(T182);CENPF(S276);CENPF(S3119);CENPF(T144);CEP170(S881);CEP55(S428);CEP97(S308);CHAF1A(S206);CHAMP1(S376);CHAMP1(S432);CHAMP1(S436);CHAMP1(S507);CHD4(S303);CIT(S1322);CLASP1(S1091);CLASP1(S636);CLASP2(S529);CLASRP(S547);CLINT1(T308);CNK3/IPCEF1(S892);CNTNAP4(S520);CPSF7(S48);CREB1(S111);CREB1(S271);CSPP1(S901);CTPS1(Y567);CTTN(Y421);CTU2(S419);DAXX(S671);DBF4(S381);DCDC2(S270);DDX21(S89);DGCR8(S271);DGCR8(S275);DGCR8(Y267);DIP2B(S259);DLG5(S1000);DLG5(S1209);DLG5(T984);DLGAP5(S725);DNMT1(S127);DNMT1(T137);DNTTIP2(S434);DOCK7(S898);DOCK7(S946);DPYSL2(T509);DPYSL3(T509);DYNC1LI1(S398);DYNC1LI1(S421);EHBP1L1(S285);EIF3E(S399);EIF4G2(S395);ELAVL1(S202);EML4(S144);EML4(S146);ENAH(T538);EP400(S722);EP400(S736);EPB41L1(S541);EPB41L1(S544);EPB41L1(S784);EPB41L5(S436);ERCC5(S384);ERLIN1(S324);ERRFI1(S461);ESF1(S198);EZH2(S363);EZH2(T367);FADD(S194);FAM122A(S143);FAM122A(S147);FAM122A(S189);FAM124A(S321);FAM129B(S665);FAM129B(S681);FAM129B(S696);FAM207A(T34);FAM83H(S914);FANCI(S1121);FBRSL1(T1010);FGD6(S692);FIP1L1(S259);FLYWCH2(S21);FOXK1(S420);FOXK1(S441);FOXP1(S83);FRMD3(S416);FTSJ3(S677);FTSJ3(T573);FXR2(T411);GAGE13(S33);GAGE2A(S32);GAGE2B(S32);GAGE2D(S32);GATAD2A(T189);GATAD2B(S334);GATAD2B(S486);GBF1(S1298);GIGYF2(S26);GJA1(S262);GNL3(S529);GRIP1(S847);GSE1(S710);GTF2F1(S385);GTF2F1(T389);GTF2I(S210);GTF2I(T558);GTF3C2(S132);GTF3C2(S167);HBS1L(T231);HCFC1(S598);HCFC1(S666);HDAC1(S406);HEATR6(S643);HIST1H1E(T18);HJURP(S557);HMGA1(S36);HMGA1(T53);HNRNPA1(S338);HNRNPA2B1(S344);HNRNPA3(S358);HNRNPC(S253);HNRNPLL(S61);HNRNPM(S528);HNRNPM(S618);HSPB1(S15);HSPB8(S24);HUWE1(S1084);IBTK(S1045);INCENP(T292);INPP5D(T963);IPCEF1(S430);IRF2BP1(S421);IRF2BP2(S175);IRF2BP2(S318);IRF2BP2(S406);IRF2BPL(S519);ITGAL(S37);ITSN2(S884);ITSN2(S889);IWS1(S398);IWS1(S400);JADE3(S566);JMJD1C(S1223);JMJD1C(S641);JPT2(S30);JPT2(S97);JPT2(T76);KANK2(S172);KANK2(S175);KIAA0319L(S978);KIAA0930(S304);KIAA1217(S357);KIAA1217(S361);KIAA1468(T143);KIAA1522(S342);KIAA1522(S545);KIAA1522(S858);KIAA1522(S862);KIAA1522(S929);KIAA1522(S979);KIF1A(S1094);KIF1A(S1528);KIF1A(S1532);KNOP1(S119);KPNA4(S60);KRT8(S410);L1TD1(S557);LAD1(S301);LAMTOR1(S27);LARP1(T526);LARP1(T649);LEMD3(S187);LIN28B(S203);LIN54(S310);LMNA(S628);LMNB1(S23);LMNB1(T20);LMNB2(S37);LSM11(S21);LSR(S464);LSR(T453);LUZP1(S745);MACF1(S7330);MAML1(S360);MAP1A(S1776);MAP2(S1540);MAP2(S1653);MAP2(T1649);MAP3K11(S524);MAP4K3(S616);MAP4K3(S618);MARCKS(S163);MARK2(S456);MARK2(S619);MAST2(S876);MAZ(S361);MCM3(Y708);MCM3AP(S557);MCM4(S120);MDC1(T378);MEF2D(S180);MEPCE(S217);MEPCE(T213);MFAP1(S116);MIA3(S1741);MICAL3(S649);MICALL1(S391);MICALL1(S486);MICALL1(S640);MICALL2(S143);MICALL2(S153);MICALL2(S249);MIS18BP1(S1042);MKI67(S1207);MKI67(S1937);MKI67(S2223);MKI67(S2299);MLC1(S179);MORC2(S696);MPDZ(S230);MPLKIP(S47);MPLKIP(T51);MPLKIP(Y45);MSH6(S41);MTA1(S386);MTA1(S449);MTA1(S522);MTA2(S435);MTBP(S755);MTFMT(S23);MTMR3(S613);MTSS1L(S342);MYC(S62);MYC(T58);MYCN(S156);MZT2A(S139);MZT2B(S139);NAA10(S186);NAA30(S89);NAB1(S403);NAB2(S171);NADK(S48);NADK(S64);NASP(T390);NAV1(S808);NAV2(S1800);NCAPD2(Y1325);NCL(T121);NCOR1(S1980);NCOR1(S1981);NCOR2(S1487);NCOR2(S1547);NCOR2(S54);NECAP2(S181);NFATC2(S217);NFIC(S333);NIFK(T238);NIPBL(S306);NOLC1(S397);NOLC1(S508);NOLC1(S622);NOLC1(T607);NOLC1(T610);NONO(T450);NOP53(S29);NOP58(S351);NPM1(S137);NPM1(S139);NSFL1C(S140);NUCKS1(T179);NUFIP2(S230);NUMA1(S1862);NUMA1(S1991);NUMA1(T2000);NUMBL(S263);NUP107(S11);NUP153(S209);NUP210(T1844);NUP35(S66);NYNRIN(S660);OBSL1(S10);ORC6(T195);PABPN1(S150);PAGR1(S237);PARVA(S19);PBRM1(S13);PBX2(S330);PCBP1(S190);PCM1(T79);PCM1(T82);PCNP(T139);PCYT1A(S315);PCYT1B(S315);PDCD6IP(S730);PDLIM2(S129);PDLIM5(S111);PDS5B(T1301);PEAK1(S823);PGRMC1(S181);PHACTR2(T25);PHF3(S1614);PHF8(S880);PHKA2(S1043);PHLDA2(S42);PHLDB1(S461);PHLDB2(S73);PI4KB(S266);PIAS1(S503);PKP4(S273);PKP4(S314);PLEC(S1435);PLEC(S4613);PLEKHA5(S933);PLEKHA5(S937);PLEKHA5(T857);PLEKHA7(S903);PLEKHG2(S1261);PLEKHG2(T1257);PLEKHG3(S76);PLEKHG4B(T727);PML(S505);POLA1(S190);POLA2(T127);POLD2(S15);POLM(S372);POM121(S298);POM121C(S275);POMZP3(S33);POTEE(S939);POTEF(S939);POTEKP(S239);PPFIA1(S1172);PPFIA3(S1164);PPFIBP1(S636);PPHLN1(S163);PPHLN1(S201);PPHLN1(T204);PPL(S14);PPM1H(S221);PPP1CA(T320);PPP1CC(T311);PPP1R13B(S681);PPP1R13L(S358);PPP1R13L(S395);PPP1R14B(S32);PRAG1(S510);PRAG1(S712);PRKDC(T1045);PRR12(S314);PRR36(T1082);PRRC2A(S1147);PRRC2A(T1347);PSMF1(S153);PXN(S85);R3HDM2(S349);RAB11FIP1(S435);RAB11FIP1(S529);RAB40C(S268);RAD18(S103);RALGAPB(T379);RALY(S135);RANBP3(S211);RAP1GAP2(S564);RB1(S249);RB1(S788);RB1(T821);RB1(T826);RB1(Y790);RBBP6(S516);RBBP8(S327);RBM15(S294);RBM17(S169);RBM27(T447);RBM39(S97);RBM39(Y95);RBM6(S1025);RBMX(S208);RBMX(S249);RBMXL1(S208);RBMXL1(S249);RBSN(S429);RECQL5(S815);REPS1(S709);RFX7(S1028);RIF1(S1688);RIF1(S2205);RPA1(T180);RPL18(S161);RPL18(T158);RPS6(S235);RPS6KB1(S441);RRBP1(T1046);RRM2(T33);RRP15(T104);RRP1B(S732);RSL1D1(T465);RUNX3(S214);SALL2(S806);SAMD1(S161);SAP130(S442);SCML2(S267);SCRIB(S1348);SCRIB(S1448);SCRIB(S1475);SCRIB(S504);SCRIB(S853);SEC16A(S136);SEC16A(S1786);SET(S7);SF3B1(S129);SF3B1(T223);SF3B1(T227);SF3B1(T303);SF3B1(T313);SF3B1(T426);SF3B1(T436);SFPQ(S33);SFRP2(S287);SFRP2(S289);SGO1(S468);SHANK2(S67);SHROOM3(T576);SIK3(T469);SIPA1L1(S1565);SLC4A1AP(S82);SLC9A3R1(S280);SMARCA2(S588);SMARCAD1(S146);SMNDC1(S201);SMTN(S341);SNRK(S518);SNRNP200(S225);SNRNP70(S226);SNRPA1(T180);SNRPC(S17);SNTB2(S393);SNTB2(S95);SNX17(S336);SNX17(S409);SNX17(S421);SORBS3(S530);SP2(S78);SPECC1(S55);SPEG(S2109);SPTAN1(S1190);SRRM2(S2382);SRRM2(S510);SRSF11(S207);SRSF9(S216);SSB(S366);STAM(S156);STIM2(S523);STK17A(S28);STMN1(S38);SUGT1(S281);SUPT6H(T1523);SURF6(S138);SYNJ1(S1053);SYTL2(S301);SYTL2(S344);TACC3(S25);TAF7(S201);TAOK1(S421);TBX2(S653);TCF20(S574);TCF20(S966);TCOF1(S156);TCOF1(S503);TCOF1(S583);TCOF1(T914);TELO2(S836);TFE3(S556);THAP4(S128);THOC5(S314);THRAP3(S248);THRAP3(S253);THRAP3(S575);THRAP3(S928);TJAP1(S320);TJAP1(T318);TJAP1(Y316);TJP2(S266);TK1(S231);TMPO(S306);TMPO(S354);TMPO(S424);TNIK(S764);TNIK(S766);TNKS1BP1(S1103);TNRC6C(S714);TNS1(T1173);TOM1(S464);TOM1L1(S323);TP53BP2(S558);TPR(S379);TPX2(T369);TRA2A(T202);TRA2B(T201);TRA2B(T212);TRIM33(S862);TRIM71(S187);TRIP12(S312);TRPM7(S1477);TRPS1(S216);TRPS1(T751);TUBA1A(S48);TUBA1B(S48);TUBA1C(S48);TUBA3C(S48);TUBA3E(S48);TXLNG(S97);UBAP2L(S605);UBE2O(T838);UBE4B(S65);UBE4B(T64);UCK1(S253);UCKL1(S56);UNC13B(S367);UNG(S64);UNG(T60);USP10(S211);USP15(S242);USP20(S134);USP32(S1416);USP36(S742);USP6(S1214);USP7(S18);VCL(S290);VGLL4(S149);WASHC2A(S704);WASHC2C(S702);XPO4(S521);XRCC1(S226);XRCC1(S229);XRCC1(T198);XRCC1(Y211);YAP1(S289);YBX3(T67);YTHDC2(S1223);ZC3H11A(S132);ZC3H4(S907);ZC3HAV1(S378);ZC3HC1(S321);ZCCHC8(T479);ZCCHC8(T485);ZDHHC5(S621);ZFHX4(S2996);ZFP64(S547);ZFP91(S103);ZFR(S1054);ZFYVE26(S1764);ZMYM4(T217);ZNF318(S1896);ZNF462(S1251);ZNF574(S164);ZNF639(S88);ZNF687(S374);ZYX(S308)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>CDK5</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>92</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(T142);AEBP2(S24);AGFG1(S181);AMFR(S542);ANKRD17(S2401);ANLN(S182);ANLN(T194);ARHGAP29(S1029);ASIC3(S37);ATXN2L(S424);BAG3(T285);BAZ1B(S349);CDCA2(S98);CDK14(S134);CENPF(S276);CHAMP1(S416);DCDC2(S270);DENND4A(S1256);DLG5(S1209);DNMT1(S127);DNMT1(T137);EHBP1L1(S285);EIF4B(S283);ERLIN1(S324);FGFR1OP(T170);FOXP1(S83);GRB10(S104);GTF2I(S210);GTF2I(T558);HAUS6(T584);HBS1L(T231);HCFC1(S666);HIST1H1B(S18);INCENP(S311);JPT2(S97);KIAA1522(S971);LARP6(S409);LINC00322(S226);MAP7D1(S399);MARK2(S456);MARK2(S619);MARK3(S469);MEF2D(S180);MPLKIP(S115);MYO9B(S1405);NCOR2(S956);ORC6(T195);PARVA(S19);PDCD4(S94);PDLIM5(S111);PI4KB(S266);PLCL2(S17);PLEKHA5(S885);PLEKHG3(S76);PLPPR3(S508);PPFIA3(S1164);PPL(S14);PPM1H(S221);PQBP1(S247);PRAG1(S889);PRRC2A(T1347);RAB11FIP1(S435);RAB40C(S268);RBSN(S429);REPIN1(S27);RPA1(T180);SATB1(S637);SHROOM3(S242);SKIV2L(S131);SLC9A3R1(S280);SNRK(S518);SNRPA1(T180);SNTB1(S87);SORBS3(S530);SRRM2(S2382);SRSF7(S165);STIM2(S523);TCOF1(S583);TET2(S1107);TRIM37(S771);UBE2O(S515);UCKL1(S56);WIPF2(S235);XPR1(S666);XRCC1(S226);XRCC1(S229);XRCC1(S241);XRCC1(T198);ZC3H11A(T321);ZFR(S1054);ZNF638(S1401);ZYX(S259)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>CDK6</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>138</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(S30);ADAM17(S791);AFF4(S487);AGAP2(S808);AGFG1(T177);AMBRA1(S1205);AMBRA1(S639);ANK1(S15);APPL1(S401);ARFGAP2(S432);ARHGAP17(S625);ARID1A(S1184);ATAD2(S327);BRD4(S1126);BUB1(S655);C2CD5(S662);CALU(S35);CALU(S44);CAMSAP1(S563);CDCA7L(S261);CEP170(S881);CHD1(S1677);DBNL(T291);DLG5(T1279);DOCK7(S898);DOCK8(S451);DYNC1LI1(S398);EEPD1(S21);EIF4EBP1(T82);EIF4G1(S1092);EPB41L1(S541);EPB41L1(S544);FGD6(S692);FZR1(S163);GAB2(S141);GAPVD1(S902);GPATCH2(S195);GTF3C2(S167);HNRNPA1(S338);HNRNPLL(S61);HNRNPM(S528);HNRNPM(S618);HSPB1(S82);HUWE1(S1084);ICE1(S255);IRF2BP2(S318);ISCU(S20);JPH4(S157);KIAA1551(S1358);KIF21A(S1239);LIMA1(S617);LIN54(S310);LRCH4(S520);MAP1A(S1675);MAP7D1(S399);MARK2(S456);MARK3(S469);MAST2(S876);MAZ(S361);MEPCE(S217);MEPCE(T213);MICALL1(S486);MICALL2(S249);MTA1(S386);MTA1(S639);MTBP(S755);MTX3(S284);MYO9B(S1405);NADK(S48);NADK(S64);NAV1(S808);NCKIPSD(T181);NOLC1(S397);NOLC1(S622);NUMA1(S1991);NUP210(S1881);NUP214(S1045);OSBPL8(S68);PARVA(S14);PCDH1(S949);PCM1(T79);PCM1(T82);PDLIM2(S129);PDZD8(S521);PEA15(S116);PFKL(S775);PLEKHA2(S349);PLK1(T214);PLPPR3(S353);PLPPR3(S508);PPM1H(S221);PPP1R9B(S100);PRKDC(T1045);R3HDM2(S349);RASAL3(S18);RB1(S795);RB1(T356);RB1(T821);RB1(T826);RBL1(S749);RBL1(T369);RBM10(S845);RBM39(Y95);RBMX(S249);RBMXL1(S249);RIF1(S1688);SEC16A(S136);SH3BP2(S427);SHROOM3(S242);SLC12A7(T980);SLC9A3R1(S280);SNTB1(S87);SPEG(S2109);SUPT6H(T1523);SVIL(S968);TACC3(S250);TAOK1(S421);TBC1D1(S211);TBC1D9B(S435);TCOF1(S1227);TCOF1(S503);TCOF1(T914);THRAP3(S248);THRAP3(S575);TMX1(S270);TNKS1BP1(S836);TOR1AIP1(S135);TPD52L2(S166);UNC13B(S367);USP36(T653);VGLL4(S149);XRCC6(S477);ZC3HAV1(S378);ZCCHC8(S598);ZFPM1(S786);ZMYND8(S547);ZNF24(S274);ZNF777(S47)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>CDK7</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>27</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>AMFR(S542);ATXN2L(S424);CDC25B(S375);CDK12(T893);CTU2(S419);DCUN1D5(S9);HIST1H1B(S18);HSH2D(S194);INCENP(S311);KHDRBS1(S20);PALM3(S303);RALY(S135);RB1(T601);RBM15(S292);RBM15B(S265);RBMX(S208);RBMXL1(S208);RBMXL1(S88);RPA1(T180);SAFB2(S787);SATB1(S637);SF3B1(T436);SLTM(S1002);SLTM(S551);SNRPA1(T180);SRSF9(S189);TCOF1(S156)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>CDK9</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>389</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(S30);09/09/18 00:00:00(T142);09/09/18 00:00:00(T49);ABI1(S216);ACTA1(S241);ACTA1(S54);ACTA2(S241);ACTA2(S54);ACTB(S239);ACTB(S52);ACTBL2(S240);ACTC1(S241);ACTC1(S54);ACTG1(S239);ACTG1(S52);ACTG2(S240);ACTG2(S53);ADAM17(S791);ADD1(S12);ADNP(S709);AFF4(S1043);AFF4(S1062);AGAP2(S808);AGFG1(T177);AHNAK(S177);AHNAK(S3412);AHNAK(S3426);AHNAK(S41);AHNAK(S5731);AKAP11(T1100);AMBRA1(S1205);ANKRD39(S153);ANLN(S182);ANLN(S518);ANLN(T194);ANLN(T364);APPL1(S401);ARFGAP1(T135);ARFGAP2(S432);ARHGAP17(S625);ARHGEF16(S174);ARHGEF26(S80);ARID1A(S1184);ARID1A(S363);ASF1B(T179);ATF1(S198);ATRIP(S224);ATXN2(S684);ATXN2(T666);ATXN2L(S424);BAG3(S195);BAG3(S289);BAG3(T285);BAP18(S110);BAZ1A(T1547);BAZ1B(S349);BMS1(S552);BPTF(S1300);BRD4(S1117);BRD4(S1126);BUB1(S655);C16orf72(S167);C2CD5(S662);C6orf106(S215);CALU(S35);CALU(S44);CAMSAP1(S563);CDCA7L(S139);CDCA7L(S261);CDK14(S134);CDK9(S347);CENPF(S276);CENPF(S3119);CENPF(T144);CEP170(S881);CEP55(S428);CHAMP1(S376);CHAMP1(S382);CHAMP1(S507);CLASP1(S1091);CLASRP(S547);CLINT1(T308);CNTNAP4(S520);CPSF7(S48);CREB1(S111);CTPS1(Y567);CTTN(Y421);CTU2(S419);DBNL(T291);DCDC2(S270);DDX21(S71);DLG5(S1209);DLGAP5(S725);DOCK7(S898);DOCK8(S451);DPYSL2(T509);DPYSL3(T509);DYNC1LI1(S398);DYNC1LI1(S421);DYRK2(S30);EEPD1(S21);EFHD2(S74);ELAVL1(S202);EP400(S722);EPB41L5(S436);ERRFI1(S461);ESF1(S198);EZH2(S363);FAM122A(S147);FAM129B(S696);FAM207A(T34);FBXW9(S59);FBXW9(T55);FGD6(S692);FIP1L1(S259);FLYWCH2(S21);FNBP1(S359);FOXP1(S83);FTSJ3(S677);FTSJ3(T573);G3BP2(T227);GAB2(S141);GAPVD1(S902);GATAD2B(S486);GNL3(S529);GPATCH2(S195);GSE1(S710);GSK3A(Y279);GSK3B(Y216);GTF3C2(S167);H2AFY(T129);HBS1L(T231);HCFC1(S666);HEATR6(S643);HIST1H1E(T18);HJURP(S557);HMGA1(S36);HMGA1(T53);HNRNPA1(S338);HNRNPA2B1(S344);HNRNPLL(S61);HNRNPM(S528);HNRNPM(S618);HSPB8(S24);HUWE1(S1084);IRF2BP1(S421);IRF2BP1(S436);IRF2BP2(S318);JPT1(T54);JPT2(S30);JPT2(S97);KANK2(S172);KIAA0319L(S978);KIAA1522(S342);KIAA1522(S545);KIAA1522(S979);KRT8(S410);LAD1(S301);LAMTOR1(S27);LARP1(T649);LEMD3(S187);LIMA1(S617);LIN54(S310);LMNB1(S23);LMNB1(T20);LMNB2(S37);LRCH4(S520);MAP1A(S1675);MAP4K3(S616);MAP4K3(S618);MAP7D1(S399);MARK2(S456);MAST2(S876);MAZ(S361);MCM4(S120);MEF2D(S180);MEPCE(S217);MEPCE(T213);MICALL1(S486);MKI67(S1207);MKI67(S1937);MKI67(S2299);MPLKIP(S47);MPLKIP(T51);MPLKIP(Y45);MSH6(S41);MTA1(S386);MTMR2(S58);MYC(S62);MYC(T58);MYO9B(S1405);MYO9B(S717);MZT2A(S139);MZT2B(S139);NAA10(S186);NAA30(S89);NADK(S48);NADK(S64);NAV1(S808);NCL(T121);NCOR2(S1487);NFIC(S333);NIFK(T238);NIPBL(S306);NOLC1(S397);NOLC1(S508);NOLC1(S622);NOLC1(T607);NOLC1(T610);NONO(T450);NOP2(S732);NPM1(S137);NPM1(S139);NUFIP2(S230);NUMA1(S1862);NUMA1(T2000);NUP107(S11);NUP210(S1881);NUP210(T1844);NUP35(S66);ORC6(T195);OSBPL8(S68);PABPN1(S150);PCBP1(S190);PCM1(T79);PCM1(T82);PCNP(T139);PDCD6IP(S730);PDLIM2(S129);PDLIM5(S111);PDZD8(S521);PEA15(S116);PFKL(S775);PHC3(S315);PHKA2(S1043);PHRF1(S867);PIAS1(S503);PLEKHA5(S933);PLEKHA5(S937);PLEKHA7(S903);PLEKHG2(S1261);PLEKHG2(T1257);PLEKHG3(S76);PLK1(T214);PLPPR3(S353);PLPPR3(S508);POLA1(S190);POTEE(S939);POTEF(S939);POTEKP(S239);PPFIA1(S1172);PPHLN1(S201);PPP1CA(T320);PPP1R13B(S681);PPP1R13L(S358);PPP1R14B(S32);PPP1R9B(S100);PRKDC(T1045);PRR36(T1082);PSMF1(S153);R3HDM2(S349);RAB11FIP1(S529);RAD18(S103);RALY(S135);RANBP2(T1396);RAP1GAP2(S564);RASAL3(S18);RB1(S249);RB1(T356);RB1(T821);RB1(T826);RBBP6(S516);RBBP8(S327);RBL1(S749);RBL1(S762);RBL1(T369);RBL2(S413);RBM10(S845);RBM17(S169);RBM39(Y95);RBMX(S249);RBMXL1(S249);RECQL5(S815);RFX7(S1028);RIF1(S1688);RPA1(T180);RPS6KB1(S441);RRBP1(T1046);RRM2(T33);RRP15(T104);RRP1B(S732);RSL1D1(T465);RUNX3(S214);SAP130(S442);SCML2(S267);SCRIB(S1348);SCRIB(S1445);SCRIB(S1448);SCRIB(S1475);SEC16A(S1786);SF3B1(T223);SF3B1(T227);SF3B1(T426);SF3B1(T436);SFPQ(S33);SH3BP2(S427);SHANK2(S67);SHROOM3(S242);SIPA1L1(S1565);SLAIN2(S391);SLC4A1AP(S82);SLC9A3R1(S280);SNRNP70(S226);SNRPA1(T180);SNTB1(S87);SNTB2(S393);SNX17(S421);SORBS3(S530);SP2(S78);SPEG(S2109);SPTAN1(S1190);SRRM2(S2382);SRRM2(T2289);SRSF11(S207);SRSF9(S211);SRSF9(S216);STIM2(S523);STK17A(S28);STMN1(S38);SUGT1(S281);SUPT6H(T1523);SVIL(S968);SYTL2(S301);TACC3(S25);TACC3(S250);TACC3(S71);TAOK1(S421);TBC1D1(S211);TBC1D9B(S435);TCF20(S966);TCOF1(S1227);TCOF1(S1257);TCOF1(S156);TCOF1(S503);TCOF1(T914);TELO2(S836);THRAP3(S248);THRAP3(S253);THRAP3(S575);TK1(S231);TMPO(S306);TMPO(S424);TMX1(S270);TNKS1BP1(S1297);TOR1AIP1(S135);TPD52L2(S166);TRIM33(S862);UBAP2L(S605);UFD1(S247);UNC13B(S367);UNG(S64);UNG(T60);USP32(S1416);USP36(S546);USP36(T653);USP6(S1214);VCL(S290);VGLL4(S149);WASHC2A(S704);WASHC2C(S702);WBP11(S237);WIZ(S1012);XRCC1(S229);XRCC1(T198);XRCC1(Y211);XRCC6(S477);ZC3H11A(S132);ZC3H4(S907);ZC3HAV1(S378);ZC3HC1(S321);ZCCHC8(S598);ZCCHC8(T479);ZCCHC8(T485);ZFR(S1054);ZMYM2(S305);ZMYM4(T217);ZNF24(S274);ZYX(S267);ZYX(S308)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>CDKL5</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>330</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(S30);ACIN1(T414);ADAM17(S791);ADD1(S431);AFAP1(S668);AFDN(S1318);AFF4(S1058);AFF4(S32);AGPS(S65);AHDC1(S1064);AHDC1(S1507);AMPD2(S100);ANP32B(T244);ARAP3(S1444);ARFGAP2(S368);ARHGAP1(S44);ARHGAP1(S51);ARHGAP21(S476);ARHGAP21(S856);ARHGEF11(S150);ARHGEF2(T152);ARID1A(S1604);ARID1A(S730);ARID3B(S381);ATG2B(S1582);ATG2B(S1583);ATG2B(Y1577);ATL1(S10);BCAM(S600);BCL11A(S328);BCL2L12(S113);BCL2L12(S121);BCL2L12(T117);BCL9(T315);BRD4(S1126);BRSK2(T459);BRSK2(T463);BTF3(S30);BUB1(S655);C2CD5(S281);C2CD5(S662);CABLES1(S291);CASP3(S26);CCDC6(S240);CCDC85C(S246);CDC42EP4(S118);CDC42EP4(T23);CDK12(S383);CDK12(S385);CDK13(T1056);CDK14(S24);CDV3(T182);CENPF(S276);CEP170(S881);CEP97(S308);CHAMP1(S432);CHAMP1(S436);CHD8(S1995);CIT(S1322);CLASP2(S529);CLASRP(S547);CNK3/IPCEF1(S892);CPSF7(S48);CRTC3(S370);CTNND1(S349);DAXX(S671);DBF4(S381);DBNL(T291);DDX21(S89);DGCR8(S271);DGCR8(S275);DGCR8(Y267);DOCK7(S898);DOCK7(S946);DVL3(S125);DYNC1LI1(S398);EIF3A(S1336);EIF4B(S207);EIF4G1(S1194);EML4(S144);ENAH(T538);EP400(S736);EPB41(S709);EPB41L1(S784);EPN2(S173);ERCC5(S384);ESS2(T386);EZH2(S363);EZH2(T367);FADD(S194);FANCI(S1121);FGD6(S692);FLYWCH2(S21);FOXK1(S420);FOXK1(S441);FRMD3(S416);FRS2(S211);FXR2(T411);GAB2(T391);GAGE13(S33);GAGE2A(S32);GAGE2B(S32);GAGE2D(S32);GAPVD1(S902);GIGYF2(S26);GJA1(S262);GON4L(S206);GTF2F1(S385);GTF2F1(T389);GTF3C2(S167);HCFC1(S598);HCFC1(S666);HDAC1(S406);HMGCR(S872);HNRNPC(S253);HNRNPLL(S61);HNRNPM(S528);HNRNPM(S618);HSPB1(S15);HUWE1(S1084);ICE1(S1712);IPCEF1(S430);IRF2BP1(S421);IRF2BP2(S175);ITGAL(S37);JADE3(S566);JMJD1C(S1223);JMJD1C(S641);KANK2(S172);KANK2(S175);KHDRBS1(S20);KIAA1217(S357);KIAA1468(T143);KIAA1522(S929);KIFC1(S351);KNOP1(S119);L1TD1(S557);LEMD3(S187);LIN28B(S203);LSM11(S21);LSR(S464);LSR(T453);LUC7L2(S18);LUZP1(S745);LZTS1(S233);MACF1(S7330);MAML1(S360);MAP1A(S1776);MAP2(S1555);MAP2(S1653);MAP2(T1649);MAP3K2(S153);MAP4(S928);MAP7D1(S113);MARCKS(S163);MAST2(S876);MAST3(S747);MAZ(S361);MCM3(Y708);MDC1(T378);MELK(S505);MELK(S529);MEPCE(S217);MEPCE(T213);MFAP1(S116);MFSD10(S271);MIA3(S1741);MTA1(S386);MTFMT(S23);MTFR1L(S238);MYCBP2(S2751);MYCN(S156);MYH10(S1937);NAB1(S403);NAB2(S171);NADK(S48);NADK(S64);NASP(T390);NAV1(S808);NCAPD2(Y1325);NCOR2(S1547);NDRG2(T334);NHSL1(S1233);NOLC1(S397);NOLC1(S622);NONO(T450);NOP53(S29);NUMA1(S1862);NUP35(S66);OSER1(S82);OSER1(S84);PABPN1(S150);PAK4(S163);PARD3(S717);PBRM1(S13);PBRM1(S14);PBX2(S330);PCM1(T79);PCM1(T82);PDLIM2(S129);PDS5A(T1208);PDS5B(T1301);PEAK1(S823);PHF3(S1614);PHF8(S880);PHKA2(S1043);PHLDB1(S334);PI4KB(S428);PKP4(S273);PKP4(S314);PLCG1(S1263);PLEKHG4B(T727);POLA2(T127);POLD2(S15);POLH(S380);POLM(S372);POLR2A(S1868);POLR2A(Y1860);POM121(S298);POM121C(S275);POMZP3(S33);PPFIBP1(S466);PPFIBP1(S636);PPHLN1(S201);PPIP5K2(S1074);PPP1CC(T311);PRKDC(T1045);PRR12(S314);PRR36(T1082);PTPN12(S449);R3HDM2(S349);RALGAPA1(S797);RALY(S135);RBL1(T369);RBM15B(S113);RBM15B(S265);RBM15B(T532);RBM39(S97);RBM39(Y95);RBMX(S249);RBMX(S352);RBMX(S88);RBMXL1(S249);RBMXL1(S88);REPS1(S709);RIF1(S1688);RIF1(S2205);RLIM(S228);RLIM(S230);RPL18(S161);RPL18(T158);RPS27(S78);RPS27L(S78);SAFB2(S787);SALL2(S806);SASH1(S90);SCAF1(S874);SCRIB(T475);SF3B1(S129);SF3B1(T223);SF3B1(T227);SF3B1(T303);SF3B1(T313);SF3B1(T426);SF3B1(T434);SF3B1(T436);SGO1(S468);SH3BP4(S296);SHANK2(S67);SHROOM2(T647);SIK3(S866);SLTM(S1002);SLTM(S551);SLTM(S553);SMARCAD1(S146);SMCR8(S489);SNRNP70(S226);SNX17(S409);SPECC1(S55);SPEG(S2109);SPTAN1(S1031);SRRM2(S510);SRSF4(S446);SSB(S366);SSSCA1(S78);STIM2(S680);STIM2(S719);STX17(S289);SUPT6H(T1523);TCF20(S574);TCOF1(S503);TCOF1(T914);THOC5(S314);THRAP3(S575);THRAP3(S928);TJAP1(S320);TJAP1(T318);TJAP1(Y316);TNIK(S766);TNKS1BP1(S429);TNRC6C(S714);TP53BP2(S558);TPR(S379);TRA2A(T202);TRA2B(T201);TRA2B(T212);TRIM71(S187);TUBA1A(S48);TUBA1B(S48);TUBA1C(S48);TUBA3C(S48);TUBA3E(S48);TXLNG(S97);UBE2O(T838);UBE4B(S65);UBE4B(T64);UCK1(S253);UNC13B(S367);XPO4(S521);XRCC1(S226);XRCC6(S477);YBX3(S293);ZC3H13(T364);ZC3H3(S571);ZFHX4(S2996);ZFP91(S103);ZMYND8(S425);ZNF462(S1251);ZNF574(S164);ZNF687(S374)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>CIT</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>950</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(S30);AAK1(S14);ABI1(S216);ABI1(Y213);ABLIM1(S431);ABR(T74);ACIN1(T414);ACTA1(S241);ACTA2(S241);ACTB(S239);ACTBL2(S240);ACTC1(S241);ACTG1(S239);ACTG2(S240);ADAM10(S740);ADAM10(Y741);ADAM17(S791);ADD1(S12);ADD1(S431);ADD1(S726);ADD2(S713);ADD3(S693);AFDN(S1173);AFDN(S1721);AFF4(S1043);AFF4(S1058);AFF4(S32);AFF4(S836);AGAP2(S808);AGFG1(T177);AHCTF1(S528);AHDC1(S1064);AHDC1(S1507);AHNAK(S115);AHNAK(S216);AHNAK(S3412);AHNAK(S3426);AHNAK(S5731);AHNAK(T490);AKAP11(S1580);AKAP11(S422);AKAP11(S448);AKAP13(S2728);AKT1S1(S183);AMBRA1(S639);ANAPC1(S355);ANKRD17(S2401);ANKS1A(S382);ANKZF1(S675);ANLN(S182);ANLN(S518);ANP32B(T244);APC(T1773);APPL1(S401);ARFGAP1(T135);ARFGAP2(S368);ARFGAP2(S432);ARHGAP1(S44);ARHGAP1(S51);ARHGAP17(S625);ARHGAP21(S856);ARHGAP39(S407);ARHGEF11(S1295);ARHGEF11(S150);ARHGEF11(S35);ARHGEF17(S735);ARHGEF18(S1111);ARHGEF2(S143);ARHGEF26(S80);ARID1A(S1184);ARID1A(S1604);ARID1A(S363);ARID1A(S730);ARID3B(S381);ARL6IP6(S80);ASF1B(T179);ATAD2(S327);ATG2B(S1582);ATG2B(S1583);ATG2B(Y1577);ATN1(S661);ATN1(T653);ATRIP(S224);ATXN2(S684);ATXN2(S857);ATXN2(S861);ATXN2(T666);BAG3(S289);BAG3(T285);BAIAP2(S366);BAP18(S110);BCAM(S600);BCAR1(S139);BCL11A(S328);BCL2L12(S113);BCL2L12(S121);BCL2L12(T117);BCOR(T486);BCR(S215);BCR(S459);BIN2(S259);BPTF(S1300);BRD4(S1117);BRD4(S1126);BRIP1(S956);BRSK2(T459);BRSK2(T463);BRWD1(S1943);BRWD1(S701);BUB1(S655);BUD23(S240);C16orf54(S194);C16orf72(S167);C2CD2L(S662);C2CD5(S281);C2CD5(S662);C6orf106(S215);C6orf132(S449);C7orf50(S175);CABLES1(S291);CAD(S1859);CALD1(S656);CALU(S35);CALU(S44);CAMSAP1(S563);CARMIL2(S1315);CASKIN1(S787);CAT(S515);CBL(S799);CBX8(S311);CCDC6(S240);CCDC9(S376);CCDC93(S305);CCL13(S44);CCNL1(S374);CD97(S818);CD97(S831);CDC25C(S216);CDCA7L(S261);CDCA8(S219);CDK13(T1056);CDK9(S347);CDV3(T182);CENPF(S276);CENPF(S3119);CENPT(S47);CEP170(S881);CEP55(S428);CEP57(S55);CEP97(S308);CHAF1A(S206);CHAMP1(S308);CHAMP1(S319);CHAMP1(S376);CHAMP1(S382);CHAMP1(S386);CHAMP1(S432);CHAMP1(S436);CHAMP1(S445);CHAMP1(S452);CHAMP1(S472);CHAMP1(S507);CHD1(S1689);CHD1L(T629);CHD4(S303);CHD8(S1978);CHD8(T1982);CHTF18(S871);CIT(S1322);CIZ1(T244);CLASP1(S636);CLASP2(S325);CLASP2(S529);CLASRP(S547);CLINT1(T308);CLK2(S142);CMTR1(S31);CNK3/IPCEF1(S892);CNP(S170);COL4A3BP(S373);CPSF7(S48);CREB1(S111);CREB1(S271);CSPP1(S901);CTAGE1(S616);CTAGE5(S647);CTPS1(S573);CTU2(S419);CYBA(T147);DACH1(S727);DAXX(S671);DBF4(S381);DBNL(T291);DDX21(S89);DDX3X(S606);DDX3Y(S592);DDX5(S480);DENND4A(T1019);DGCR8(S271);DGCR8(S275);DGCR8(Y267);DIP2B(S187);DIP2B(S259);DLG5(S1000);DLG5(T984);DLGAP5(S725);DNTTIP2(S434);DNTTIP2(T172);DOCK10(S12);DOCK2(S1705);DOCK2(S587);DOCK7(S898);DOCK7(S946);DOCK8(S451);DPPA4(T215);DPYSL2(T509);DSN1(S81);DTL(S425);DTL(S444);DYNC1LI1(S398);DYNC1LI1(S421);EAF2(S22);EEF2K(S72);EEF2K(S74);EEPD1(S21);EHMT2(S119);EIF3A(S882);EIF3E(S399);EIF3G(S42);EIF4EBP2(T70);EIF4ENIF1(S120);EIF4ENIF1(S564);EIF4G3(S495);ELL(S309);ELMSAN1(S461);EML4(S144);EML4(S146);ENAH(T538);EP400(S722);EP400(S736);EPB41L1(S784);EPS15L1(S793);ERCC5(S384);ERRFI1(S461);ESF1(S198);EZH2(S363);EZH2(T367);FADD(S194);FAM102A(S251);FAM117B(S10);FAM122A(S143);FAM122A(S189);FAM129B(S665);FAM129B(S681);FAM129B(S696);FAM207A(T34);FAM53B(S179);FAM76B(S193);FAM83B(S766);FAM83H(S914);FANCI(S1121);FARSA(S301);FBRSL1(T1010);FBXW9(S59);FBXW9(T55);FGD6(S692);FIP1L1(S259);FLYWCH2(S21);FOXK1(S416);FOXK1(S420);FOXK1(S441);FOXO1(S329);FOXO1(S430);FRMD3(S416);FTSJ3(T573);FUS(S462);FXR2(S601);FXR2(T411);GAB2(S141);GAGE13(S33);GAGE2A(S32);GAGE2B(S32);GAGE2D(S32);GAPVD1(S902);GATAD2A(T189);GATAD2B(S334);GATAD2B(S486);GBF1(S1061);GBF1(S1298);GCN1(S786);GFI1(S94);GGA3(S159);GIGYF2(S26);GJA1(S262);GNL3(S529);GOLGA4(S1248);GPATCH2(S195);GPN1(S314);GRIP1(S847);GSE1(S710);GTF2F1(S385);GTF2F1(T389);GTF2F1(T446);GTF3C2(S132);GTF3C2(S167);GTF3C2(S893);HABP4(S108);HCFC1(S598);HCFC1(S666);HCLS1(T308);HDAC1(S406);HDGF(S132);HDGFL2(S240);HELB(S1050);HELLS(S515);HIC2(S348);HJURP(S557);HMGA1(S36);HMGCS1(T490);HNRNPA1(S199);HNRNPA1(S338);HNRNPA1(S6);HNRNPA1(S95);HNRNPA1L2(S95);HNRNPA2B1(S344);HNRNPA3(S358);HNRNPC(S253);HNRNPK(S284);HNRNPLL(S61);HNRNPM(S528);HNRNPM(S618);HNRNPUL2(S161);HOMER3(S135);HPS5(S534);HRNR(S903);HSF1(S303);HSF1(S307);HSPB1(S15);HSPB1(S82);HUWE1(S1084);IBTK(S1045);IGLL1(S58);INCENP(S894);INCENP(T292);INPP5D(T963);INTS12(S128);IPCEF1(S430);IRF2BP1(S421);IRF2BP2(S175);IRF2BP2(S318);IRF2BP2(S406);IRF2BPL(S519);IRS1(T530);ITGAL(S37);ITPK1(S396);ITSN2(S884);ITSN2(S889);JADE1(S743);JADE3(S566);JMJD1C(S1223);JMJD1C(S641);JPT2(T76);KANK2(S172);KANK2(S175);KCAB2_HUMAN_Phospho (ST);KCNK2(S366);KHDRBS1(S20);KIAA0319L(S978);KIAA0930(S304);KIAA1217(S357);KIAA1217(S361);KIAA1468(T143);KIAA1522(S342);KIAA1522(S858);KIAA1522(S862);KIAA1522(S929);KIAA1522(S979);KIF1A(S1094);KIF1A(S1528);KIF1A(S1532);KIF4A(S801);KNOP1(S119);KPNA3(S60);KPNA4(S60);KRT13(S427);KRT8(S36);L1TD1(S557);LAD1(S301);LAMTOR1(S27);LARP1(S1056);LARP1(S766);LARP1(S90);LARP1(T526);LARP1(T649);LARP1(Y777);LAT2(S135);LAT2(S51);LAT2(S86);LEMD3(S187);LIMA1(S617);LIMD2(S29);LIN28B(S203);LIN54(S310);LMNA(S390);LMNB2(S37);LPIN1(S162);LRCH1(S532);LRCH4(S520);LRRC47(S431);LRRFIP1(S116);LRRFIP2(S324);LSM11(S21);LSP1(T244);LSR(S464);LSR(T453);LUZP1(S745);MACF1(S7330);MAML1(S360);MAP1A(S1675);MAP1A(S1776);MAP2(S1540);MAP2(S1653);MAP2(T1649);MAP3K11(S524);MAP4K4(S681);MAP7(S365);MAP7D1(S93);MARCKS(S163);MARF1(S1093);MARK1(S588);MARK3(S378);MARK3(S469);MAST2(S876);MAZ(S361);MCM3(Y708);MCM3AP(S557);MCM4(S120);MCM8(S630);MDC1(T378);MED1(T1051);MEPCE(S217);MEPCE(T213);MEX3B(S442);MFAP1(S116);MFSD10(S270);MIA2(S1255);MIA3(S1706);MIA3(S1740);MIA3(S1741);MICAL3(S649);MICALL1(S391);MICALL1(S486);MICALL1(S640);MICALL2(S143);MICALL2(S153);MIGA2(S276);MIS18BP1(S1042);MISP(T157);MISP3(S91);MKI67(S1207);MKI67(S2223);MKI67(S2299);MKL2(T548);MLC1(S179);MLLT6(S378);MLLT6(S382);MORC2(S696);MORC2(S725);MPLKIP(S47);MPLKIP(T51);MPLKIP(Y45);MTA1(S386);MTA1(S449);MTA1(S522);MTA2(S435);MTBP(S755);MTFMT(S23);MTM1(S18);MTMR12(S564);MTMR2(S58);MTMR3(S613);MTMR4(S961);MTOR(S2454);MTSS1L(S342);MTSS1L(S569);MYBBP1A(S11);MYC(T58);MYCBP2(S3467);MYCN(S156);MZT2A(S139);MZT2B(S139);NAA10(S186);NAA30(S199);NAB1(S403);NAB2(S171);NADK(S48);NADK(S64);NAF1(S315);NASP(T390);NAV1(S696);NAV1(S808);NCAPD2(Y1325);NCAPH(S87);NCL(T121);NCL(T76);NCOR1(S1980);NCOR1(S1981);NCOR2(S1547);NCOR2(S2269);NCOR2(S2424);NCOR2(S54);NECAP2(S181);NELFE(S131);NES(S768);NFATC2(S217);NFATC2(S814);NIPBL(S306);NOB1(S325);NOLC1(S397);NOLC1(S508);NOLC1(S622);NOLC1(S643);NOLC1(T188);NONO(T450);NOP16(S16);NOP2(S732);NOP53(S29);NOP58(S351);NPM1(S254);NR2C2(S46);NSD1(S2471);NUCKS1(T179);NUFIP2(S230);NUFIP2(S629);NUMA1(S1862);NUMA1(S1887);NUMA1(S2062);NUMA1(T2000);NUMBL(S263);NUP153(S209);NUP210(S1877);NUP210(S1881);NUP210(T1844);NUP35(S66);NUP98(S934);OBSL1(S10);OSBPL8(S68);PABPN1(S150);PAGR1(S237);PARD3(S221);PARVA(S19);PATL1(S278);PBRM1(S12);PBRM1(S13);PBX2(S330);PCBP1(S190);PCBP1(S231);PCBP2(S272);PCM1(T79);PCM1(T82);PCNP(T139);PCYT1A(S315);PCYT1A(S347);PCYT1B(S315);PDAP1(S176);PDCD6IP(S730);PDLIM2(S129);PDLIM4(S112);PDS5B(S1257);PDS5B(T1301);PDZD8(S521);PEA15(S116);PEAK1(S823);PFKL(S775);PGRMC1(S181);PHACTR1(S505);PHACTR2(T25);PHF3(S1614);PHF8(S880);PHKA2(S1043);PHLDA2(S42);PI4K2A(S51);PIAS1(S503);PIK3AP1(S759);PKP4(S273);PKP4(S314);PLCB3(S926);PLCB3(S934);PLCB3(T924);PLCH1(S1494);PLEC(S1435);PLEKHA5(S937);PLEKHA5(T857);PLEKHA7(S903);PLEKHG4B(T727);PLEKHN1(S611);PLK1(T214);PLPPR3(S353);PML(S505);PNISR(S211);PNPO(S241);POGZ(S1338);POLA1(S190);POLA2(T127);POLD2(S15);POLH(S379);POLM(S372);POM121(S298);POM121C(S275);POMZP3(S33);POTEE(S939);POTEF(S939);POTEKP(S239);PPFIA1(S693);PPFIBP1(S579);PPFIBP1(S636);PPHLN1(S163);PPHLN1(S172);PPHLN1(T200);PPIG(S356);PPIG(T358);PPIP5K2(S38);PPME1(S15);PPP1CC(T311);PPP1R13L(S358);PPP1R13L(S395);PPP1R9B(S100);PRAG1(S510);PRAM1(S484);PRDM2(S742);PRKAA2(S377);PRKDC(T1045);PRKRA(S18);PRPF38B(S5);PRR12(S314);PRR36(T1082);PRRC2A(S1147);PRRC2A(S2113);PSMF1(S153);PTDSS2(S16);PTGES3(S113);PTPN22(S325);PXN(S85);R3HDM2(S349);RAB11FIP1(S529);RAD18(S103);RALGAPB(T379);RALY(S135);RANBP2(S2454);RANBP2(S2900);RANBP2(T1396);RANBP3(S211);RANBP9(S477);RANBP9(S482);RAP1GAP(S484);RAP1GAP2(S564);RAPH1(S894);RASAL2(S635);RASAL3(S18);RASEF(S377);RASGRP2(S391);RAVER1(T463);RB1(S249);RB1(S788);RB1(T356);RB1(T821);RB1(T826);RB1(Y790);RBL1(S640);RBL1(S749);RBM10(S845);RBM14(T206);RBM15(S294);RBM15(S622);RBM17(S169);RBM23(S149);RBM39(S97);RBM39(Y95);RBM6(S1025);RBMX(S208);RBMX(S249);RBMX(S326);RBMXL1(S208);RBMXL1(S249);RBMXL1(S326);RBMXL1(S88);RECQL5(S815);REPS1(S709);RFC1(S69);RFC1(S71);RFC1(Y67);RFX7(S1028);RGPD1(S1463);RGPD2(S1471);RGPD3(S1479);RGPD4(S1479);RGPD5(S1478);RGPD8(S1478);RGS14(S218);RIF1(S1688);RIF1(S2205);RNF169(S403);RPA1(T180);RPL12(S38);RPL18(S161);RPL18(T158);RPL27A(S68);RPLP1(S101);RPLP2(S102);RPRD2(S593);RPRD2(S614);RPRD2(S665);RPRD2(T732);RPS27(S78);RPS27L(S78);RPS6(S235);RPS6(S240);RPS6KB1(S441);RPS6KB1(S452);RPTOR(S859);RRM2(S20);RRM2(T33);RRN3(S44);RRN3P2(S44);RRP15(T104);RRP1B(S732);RRP1B(S735);RSL1D1(S392);RSL1D1(S396);RSL1D1(T465);SACS(S1779);SALL2(S806);SAMD1(S161);SAMD4B(S172);SAP130(S442);SAPCD2(S157);SASH3(S21);SCML2(S267);SCRIB(S1348);SCRIB(S1448);SCRIB(S504);SEC16A(S1786);SEC16A(S1905);SEC31A(S799);SEPT9(S22);SERBP1(S203);SET(S7);SF3B1(S129);SF3B1(T211);SF3B1(T257);SF3B1(T303);SF3B1(T313);SFPQ(S33);SFSWAP(S909);SGO1(S468);SH3BP2(S427);SHANK2(S67);SHROOM3(T576);SIK3(T469);SIPA1L1(S1255);SIPA1L1(S1565);SLC4A1AP(S82);SLC4A2(S132);SLC7A6(S22);SLX4(S1309);SLX4(S1333);SMARCA2(S588);SMARCAD1(S146);SMARCC1(S350);SMG9(S32);SMNDC1(S201);SNRK(S518);SNRNP200(S225);SNRNP70(S226);SNRPA1(T180);SNURF(S32);SNX17(S336);SNX17(S409);SP2(S78);SPAM1(S78);SPECC1(S55);SPEG(S2109);SRRM1(S452);SRRM1(S695);SRRM2(S1499);SRRM2(S2382);SRRM2(S510);SRSF1(S199);SRSF1(S201);SRSF9(S216);SSB(S366);STAM(S156);STIM2(S523);STK10(S450);STK11IP(S599);STK11IP(S777);STK17A(S28);STK24(T184);STK25(T168);STK26(T172);STMN1(S38);SUPT5H(S666);SUPT6H(T1523);SURF6(S138);SVIL(S968);SYK(S297);SYNJ1(S1053);SYTL2(S344);TACC3(S25);TACC3(S250);TACC3(S317);TAF7(S201);TAGLN2(S185);TAGLN3(S185);TAOK1(S965);TAOK3(S324);TBC1D1(S211);TBC1D9B(S435);TBX2(S653);TCF20(S574);TCF20(S966);TCOF1(S1227);TCOF1(S1350);TCOF1(S156);TCOF1(S503);TCOF1(T914);TELO2(S836);TEX2(S732);THAP4(S128);THOC5(S314);THRAP3(S248);THRAP3(S575);THRAP3(S928);TICRR(T1260);TJAP1(S320);TJAP1(T318);TJAP1(Y316);TJP1(S617);TJP2(S266);TK1(S231);TLE3(S267);TLN1(S425);TMEM201(S454);TMPO(S306);TMPO(S354);TMX1(S270);TNIK(S764);TNIK(S766);TNKS1BP1(S1103);TNKS1BP1(S691);TNKS1BP1(S836);TNRC6C(S714);TNS1(T1173);TOM1(S464);TOR1AIP1(S135);TP53BP1(S1758);TP53BP2(S558);TPD52L2(S166);TPR(S379);TRA2A(T202);TRA2B(T201);TRA2B(T212);TRIM24(S654);TRIM71(S187);TRIP12(S312);TRIR(S114);TRPM7(S1477);TRPS1(S216);TRPS1(T751);TTK(S281);TUBA1A(S48);TUBA1B(S48);TUBA1C(S48);TUBA3C(S48);TUBA3E(S48);TXLNG(S97);U2SURP(S37);UBAP2L(S605);UBE2O(T838);UBE4B(S65);UBE4B(T64);UCK1(S253);UFD1(S299);ULK1(S638);UNC13B(S367);UNC93B1(S547);UNC93B1(S550);UNG(T60);UNK(S375);UPF3B(T169);USP10(S211);USP15(S242);USP20(S134);USP24(S1141);USP32(S1416);USP36(S546);USP36(S742);USP36(T653);USP6(S1214);USP6NL(S714);USP7(S18);UTP18(S46);VCL(S290);VGLL4(S149);VIM(S25);VIM(S26);VPS13D(S1042);WASHC2A(S704);WASHC2C(S702);WBP11(S237);WDFY4(S3123);WIPF1(S234);WIPF1(S276);WIPF1(S340);WIZ(S1012);WT1(S273);XPO4(S521);XRCC1(S226);XRCC1(S229);XRCC1(T198);XRCC1(Y211);XRCC6(S477);YAP1(S289);YBX3(T67);YTHDC2(S1223);ZC3H11A(S132);ZC3H4(S907);ZC3HC1(S321);ZCCHC8(S598);ZCCHC8(T479);ZCCHC8(T485);ZDHHC5(S425);ZDHHC5(S694);ZFHX4(S2996);ZFP64(S547);ZFP91(S101);ZFP91(S103);ZFR(S1054);ZFYVE26(S1764);ZMYM4(T217);ZMYND8(S457);ZNF24(S274);ZNF318(S1896);ZNF318(S501);ZNF462(S1251);ZNF574(S164);ZNF639(S88);ZNF687(S374);ZNF687(S433);ZYX(S308)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>CLK1</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>36</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(S30);AHCTF1(S528);ARFGAP2(S432);CNK3/IPCEF1(S892);COBLL1(S394);DBNL(T291);EIF4B(S283);FXR2(T411);GTF3C2(S167);IPCEF1(S430);KHDRBS1(S20);NADK(S48);NCOA5(S381);PBRM1(S13);PBRM1(S14);PCNP(T139);PKP4(S314);RALY(S135);RBM15(S292);RBM15(S622);RBM15B(S265);RBM39(S97);RBM39(Y95);RBMX(S326);RBMX(S352);RBMXL1(S326);RBMXL1(S88);RIPOR1(S351);RPA1(T180);SAFB2(S787);SHANK2(S67);SLTM(S1002);SLTM(S551);SLTM(S553);SNRPA1(T180);SRSF9(S189)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>CLK2</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>15</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>ADD1(S465);AHNAK(S5830);COBLL1(S394);EIF4B(S283);GTF3C2(S167);HSPB1(S82);KANK2(S172);KANK2(S175);KHDRBS1(S20);RBM15B(S265);RBMXL1(S88);SAFB2(S787);SLTM(S551);SLTM(S553);TMX1(S270)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>CLK4</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>9</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>COBLL1(S394);DBNL(T291);FAM102A(S189);KHDRBS1(S20);RBM15B(S265);RBMXL1(S88);SAFB2(S787);SLTM(S551);SLTM(S553)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>CSNK1E</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>883</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(T142);ABI1(T215);ABI2(S368);ABLIM1(S655);ABLIM1(S706);ACD(S425);ACIN1(S388);ADGRL2(S1275);ADNP(S709);AEBP2(S24);AEBP2(S390);AFDN(S1318);AFDN(T1330);AFF1(T372);AFF1(T376);AFF4(S1043);AFF4(S1062);AFF4(S703);AGAP1(S605);AGFG1(S181);AGO2(S387);AHNAK(S2397);AHNAK(S5448);AKAP13(S2563);AKAP2(S720);AKAP3(S208);AMFR(S542);ANK3(S4298);ANKLE2(S268);ANKRD17(S1696);ANKRD17(S2401);ANKS1A(S663);ANKS1A(S887);ANLN(S182);ANLN(T194);ANLN(T364);AP1M1(T154);ARFGAP1(T135);ARHGAP17(S162);ARHGAP17(T682);ARHGAP21(S1862);ARHGAP21(S856);ARHGAP29(S1029);ARHGAP4(S906);ARHGEF11(S255);ARHGEF11(S35);ARHGEF16(S107);ARHGEF2(S122);ARID1A(S301);ARID1A(S363);ARID1A(S604);ARID1A(S772);ARID3A(S119);ARID3A(S362);ARL6IP4(S239);ASAP2(S822);ASCC3(S2195);ASH1L(S1170);ASH1L(T1165);ATAD5(S306);ATAT1(S315);ATF7(S434);ATF7IP(S474);ATF7IP(S477);ATP13A1(S899);ATP1A1(S16);ATRIP(S224);ATXN2(S624);ATXN2L(S32);ATXN2L(S424);BAP18(S110);BAP18(S96);BAZ1A(T1547);BAZ1B(S349);BAZ2A(S1397);BCL9L(S1017);BCL9L(S999);BCOR(S488);BICRAL(S675);BPTF(S2098);BRAF(S365);BRCA1(S1524);BRD4(S1064);BRD4(S1117);BRIP1(S206);BRSK2(S393);BUB1B(S543);C12orf43(S179);C12orf45(S178);C17orf47(S195);C2CD2(S649);C9orf40(S69);C9orf78(T100);CAAP1(S312);CAD(T1884);CAMKV(T435);CAMSAP1(S793);CAMSAP3(S368);CAMSAP3(S814);CARD9(S425);CASKIN2(S711);CBX5(S92);CBX8(S110);CBX8(S265);CCDC117(S53);CCDC14(S798);CCDC86(S160);CCDC86(Y164);CCDC88A(S1820);CCNE2(S21);CCNL2(S369);CD2AP(S510);CD3EAP(S172);CD3EAP(S285);CDC25B(S323);CDC25B(S375);CDC42BPG(S1482);CDC42EP1(S350);CDC6(S106);CDCA2(S98);CDCA3(S68);CDCA5(S75);CDCA8(S219);CDK11A(S577);CDK11B(S589);CDK12(S32);CDK12(T893);CDK13(S317);CDK14(S134);CDK17(S180);CDK18(S117);CDK18(S132);CDK18(S14);CENPA(T21);CENPC(S177);CENPF(S276);CENPF(S3094);CENPF(S3119);CEP170(T1533);CEP170P1(T242);CEP76(S83);CFL1(S3);CGN(S149);CHAF1A(S206);CHAF1A(T865);CHAMP1(S297);CHAMP1(S416);CHAMP1(S507);CHD1(S90);CHD8(S2008);CLASP2(S952);CLSPN(S775);CNOT2(S101);CNOT2(S165);CNOT2(S170);CNOT2(T93);CPEB2(S89);CPEB2(S92);CPSF4(S202);CRAMP1(S1268);CREB1(S143);CREB1(S271);CRKL(Y207);CRMP1(S522);CRTC2(S613);CRTC3(S329);CSNK1D(S331);CTAGE5(S635);CTTN(T401);CXXC1(S143);DAB2IP(S747);DAG1(T790);DCDC2(S270);DCLRE1C(S518);DCP2(S284);DDX17(S571);DDX21(S71);DDX41(S21);DENND4A(S1256);DHX57(S77);DHX8(S460);DIDO1(S1019);DIP2B(S100);DKC1(S21);DLG5(S1115);DLG5(S1209);DLG5(S1232);DLG5(S1254);DLGAP5(S662);DMAP1(T445);DNM1L(S616);DNMT1(S127);DNMT1(T137);DNMT3B(S136);DNTTIP2(S117);DNTTIP2(S330);DOCK5(S1766);DOT1L(S786);DTL(S425);DTL(T429);DTNA(T504);DTNB(T468);DUS3L(T240);DUSP16(S612);DYNC1H1(S4368);DYNC1LI1(S421);DYNC1LI2(S407);DYNC1LI2(S446);DYRK2(S30);E2F7(S825);E2F8(S71);ECSIT(Y302);EDC4(S729);EEF1D(T147);EEF1G(T46);EEF2K(S72);EEF2K(S74);EEF2K(Y69);EFHD2(S74);EHBP1L1(S285);EHMT1(S435);EIF3A(S1188);EIF4ENIF1(S120);EIF4ENIF1(S752);EIF4G3(S232);EML3(T881);EML4(S146);ENAH(S531);EPB41(S560);EPB41(S712);EPS15(S563);EPS15(S796);ERCC5(S384);ERF(S327);ERLIN1(S324);ERRFI1(S461);ESCO1(S412);ESCO2(S75);ESF1(S198);ETV6(S203);EVPL(S2025);EXO1(S623);FAM120A(Y452);FAM122A(S76);FAM122B(S115);FAM122B(S119);FAM193A(S393);FAM193B(S785);FAM234B(S62);FAM53C(S122);FAM53C(S162);FAM83H(S1025);FAM83H(S647);FBXO46(S293);FGFR1OP(T170);FLCN(S62);FLNA(S2158);FNBP1(S359);FOXK1(S213);FOXK1(S223);FOXK1(S416);FOXK2(S373);FOXO4(S230);FOXP1(S83);FRYL(T1959);FTSJ3(T573);FUBP3(S569);FYB1(S46);GAPDH(S151);GATA3(S115);GATAD2A(S340);GATAD2A(S546);GATAD2B(S486);GIGYF1(S756);GLCCI1(S30);GNL3L(S465);GPATCH8(S738);GRAMD1B(S274);GRB10(S104);GSK3A(Y279);GSK3B(S25);GSK3B(S9);GSK3B(Y216);GTF2F1(T389);GTF2I(S210);GTF2I(T558);GTF3C1(S1653);GTF3C1(S1865);GTF3C2(S132);GTF3C2(S765);GTSE1(S536);H2AFY(T129);HACD3(S135);HBS1L(T231);HEY2(S39);HIPK1(T351);HIPK2(T360);HIRIP3(S27);HIST1H1B(S18);HMGA1(S36);HMGA1(S44);HMGA1(T53);HMGCS1(S516);HMGXB4(S497);HNRNPA2B1(S259);HNRNPLL(S61);HOXC9(S159);HSH2D(S194);HSP90AA1(S263);HSP90AB1(S226);HSP90AB3P(S205);HSPH1(S809);HTATSF1(S642);HUWE1(S2534);HUWE1(T2889);IFI16(S153);IKBKB(S672);INCENP(S275);INCENP(S311);INCENP(S481);INF2(S589);INTS10(S231);IRF2BP1(S436);IRF2BPL(S215);ITSN1(S315);IWS1(S235);IWS1(S237);JAZF1(T109);JAZF1(T113);JMJD1C(S2053);JPT2(S97);JUN(S63);KANSL1(S829);KANSL1(S839);KDM2A(T550);KIAA1217(S1806);KIAA1522(S971);KIDINS220(S1633);KIF18B(S413);KIF1A(S1548);KIF20B(S1740);KIF23(S902);KIF4A(S1225);KIF4B(S1227);KIFC1(S26);KLC2(S445);KMT2A(S3511);KMT2D(S2309);KMT2D(S3130);KPNA2(S62);KTN1(S75);LARP1(S766);LARP1(Y777);LIG1(S76);LIG1(T195);LIG3(S210);LIMD2(S29);LMNA(S22);LMNA(S628);LMNB1(S391);LMNB1(S393);LMNB2(S405);LMNB2(S407);LRCH3(S419);LRCH4(S309);LSM14A(S178);LSM14A(S183);LYST(S2627);MACF1(S7330);MAGED2(S265);MAP2(S1540);MAP3K11(S524);MAP3K21(S514);MAP3K9(S519);MAP4K2(S328);MAP7D1(S460);MAP9(S79);MARCKS(S167);MARK2(S619);MASTL(S370);MASTL(S453);MATK(S501);MCM3AP(S527);MCM4(S120);MCRIP2(S82);MED1(S1223);MED13(S890);MEF2D(S180);MEPCE(S254);MEX3B(S4);MGA(S1208);MGA(S1457);MIA2(S1243);MINK1(S733);MKI67(S1207);MKI67(S1937);MKI67(S2223);MKI67(S2344);MKI67(S648);MKI67(T2231);MKL2(S921);MLF2(S238);MNAT1(S279);MON1B(S59);MON1B(S61);MPHOSPH8(S403);MPHOSPH8(T89);MPLKIP(S115);MPLKIP(S47);MPRIP(S289);MPRIP(S292);MRGBP(S195);MSANTD2(S79);MSL3(S400);MSL3(T405);MTA1(S576);MTCL1(S1808);MTDH(S568);MTMR3(S647);MYB(S599);MYBBP1A(S11);MYBBP1A(S1163);MYBBP1A(S1290);MYC(S62);MYCN(S62);MYO18A(S102);MYO9B(S717);NAA30(S39);NAV1(S528);NAV1(S541);NAV1(S672);NAV1(S695);NAV2(S1245);NCL(T121);NCOA1(S395);NCOR1(S1472);NCOR2(S1487);NCOR2(S1786);NCOR2(S2404);NCOR2(S956);NDRG2(S332);NDRG3(S331);NDRG3(S334);NECTIN1(T391);NEDD4L(S448);NEDD4L(S487);NELFE(S131);NELFE(S353);NFATC2IP(S204);NFIC(S323);NFRKB(S1291);NIFK(S230);NIPBL(S306);NIPBL(S350);NMNAT1(S117);NOC2L(S49);NOL8(S432);NOLC1(S397);NONO(T450);NOP2(S732);NOP58(S502);NSD2(S437);NSMCE3(S64);NSRP1(S33);NSUN2(S456);NSUN2(S473);NUCKS1(S181);NUMA1(T2000);NUP133(S50);NUP35(S73);ORC2(T116);ORC6(T195);OSBPL10(S201);PACS1(S495);PAICS(S27);PAK1(S137);PAK2(T143);PAK4(S181);PAK4(T207);PALD1(S406);PALM3(S303);PARD3(S174);PARVA(S19);PATL1(T194);PCBP1(S173);PCDH18(T442);PCDH7(S1011);PCIF1(S144);PCYT1A(S343);PDCD4(S94);PDCD6IP(S730);PDE3B(S495);PDHA1(S232);PDHA1(S293);PDHA1(S300);PDHA2(S291);PDHA2(S298);PDLIM5(S111);PDLIM5(S360);PDS5B(S1358);PDXDC1(S718);PFKP(S386);PHACTR1(S505);PHC3(S315);PHC3(T609);PHF3(S283);PHIP(S1315);PHKA2(S729);PHLDB1(S419);PHLDB2(T404);PHRF1(S867);PI4KB(S266);PIAS1(S488);PIAS1(S503);PIKFYVE(S329);PKN1(S562);PKP2(S293);PKP2(S82);PKP4(S337);PKP4(S406);PLCB3(S934);PLCB3(T924);PLEKHA5(S607);PLEKHA5(S933);PLEKHA5(T438);PLEKHA6(S808);PLEKHG2(S450);PLEKHG2(T445);PLPPR3(S508);PML(S518);PML(S527);PNPO(S241);POU2F1(T270);PPFIA1(S666);PPFIA3(S1164);PPFIBP2(S387);PPL(S14);PPM1H(S124);PPM1H(S221);PPP1R12A(S903);PPP1R13L(S102);PPP1R13L(S526);PPP1R14B(S32);PPP4R2(S226);PPP4R3B(S840);PPP6R1(S759);PQBP1(S247);PRAG1(S889);PRAG1(S907);PRC1(T481);PRKD2(S214);PROSER1(S613);PROSER2(S179);PRPF38B(S268);PRPF38B(S5);PRPF40B(S764);PRRC2A(T1347);PRRC2C(S779);PRRC2C(T2673);PSMA5(S16);PSMF1(S153);PTPN13(S214);PTPN13(S908);PTPN22(S692);PXN(S258);RAB11FIP1(S435);RAB11FIP1(S528);RAB3IL1(S179);RAB40C(S268);RAD18(S103);RAD18(S99);RALBP1(S34);RALGPS2(S296);RANBP2(S1456);RANBP2(S2510);RANBP2(S788);RANBP2(S955);RANBP2(T1412);RANBP2(T2613);RAP1GAP2(S45);RAPGEF6(S1094);RAPH1(S539);RASAL2(S16);RASAL3(S72);RB1(S249);RB1(S612);RB1(S811);RB1(T601);RB1(Y606);RBL1(S1041);RBL2(S1112);RBL2(T417);RBM10(S797);RBM14(S256);RBM20(S644);RBM27(S120);RBMX(S208);RBMX(S332);RBMXL1(S208);RBSN(S429);RCOR1(S260);RCSD1(S116);RCSD1(S120);RFX7(S225);RFX7(S424);RGPD1(S1519);RGPD1(S779);RGPD2(S1527);RGPD2(S787);RGPD3(S1535);RGPD3(S789);RGPD4(S1535);RGPD4(S789);RGPD5(S1534);RGPD5(S788);RGPD8(S1534);RGPD8(S788);RIF1(S1454);RIF1(S1554);RIF1(S2161);RIF1(S2348);RIOK1(S22);RIOX1(S109);RIPK3(S316);RNF2(S168);ROR2(S449);RPA1(T180);RPAIN(S18);RPRD2(S374);RPRD2(T723);RPS6KB1(S427);RPS6KB2(S423);RRBP1(T1046);RREB1(S36);RREB1(S42);RRM2(S20);RRP1B(S513);RRP1B(S679);RRP1B(S680);RRP1B(S702);RRP1B(S706);RRP1B(S735);RSF1(S392);RSF1(S397);RSL1D1(S469);RSL1D1(T465);RTN3(S229);RYBP(S127);SAMD1(S161);SASH1(S407);SATB1(S637);SBNO1(T819);SCFD1(S303);SCML2(S267);SCRIB(S1445);SCRIB(S1508);SCYL3(T153);SEC24B(T329);SEC61B(S14);SEC62(T375);SENP3(S169);SENP3(S181);SERPING1(S198);SETDB1(S1066);SF3A1(S359);SF3B1(T211);SF3B1(T223);SF3B1(T227);SF3B1(T350);SF3B1(T436);SH2B3(S150);SH2D3A(S147);SH3BP4(S279);SH3GL1(S288);SH3KBP1(S230);SHC3(S474);SHCBP1(S42);SHROOM2(S193);SHROOM3(S242);SHROOM3(S664);SHROOM3(S816);SIPA1L2(S148);SIRT1(S27);SLAIN2(S391);SLAIN2(S63);SLC20A2(S256);SLC20A2(S259);SLC43A1(T256);SLC4A7(S556);SLC4A7(T559);SLC9A1(S703);SLC9A3R1(S280);SLX4(S1185);SLX4IP(S396);SMAD1(S463);SMAD1(S465);SMAD9(S465);SMAD9(S467);SMAP(S93);SMARCA5(S116);SMARCA5(T113);SMARCC2(S347);SMG8(T743);SMG8(Y746);SNAPIN(S133);SNIP1(S35);SNRK(S518);SNRPA1(T180);SNTB1(S87);SORBS3(S530);SP2(S78);SPTAN1(S1217);SPTBN2(S2384);SPTY2D1(S471);SRCAP(S3148);SRRM2(S1014);SRRM2(S1144);SRRM2(S1404);SRRM2(S2123);SRRM2(S2382);SRRM2(S322);SRRM2(T1531);SRRM2(T2289);SRRM2(T318);SRRM2(Y1145);SRSF11(S207);SRSF4(S450);SRSF9(S211);SSBP3(S347);STAT5A(S193);STAU1(S390);STIM1(S618);STIM2(S523);STK33(S470);STMN1(S25);SURF6(T229);SYMPK(S1243);SYNRG(S1075);SYT6(S187);SYT6(Y190);TACC3(S71);TAF9(T159);TANC2(S169);TBC1D22A(S167);TBKBP1(S365);TCF20(S1019);TCF20(S1335);TCF3(S379);TCF4(S372);TCOF1(S1257);TCOF1(S156);TCOF1(S583);TERF2IP(S154);TEX2(S266);THOC2(T1443);THRAP3(S253);TICRR(S1430);TICRR(S1433);TICRR(S923);TINF2(S330);TIPIN(T224);TJP1(S168);TJP1(S968);TJP3(S164);TLE4(S208);TLK1(S159);TLK2(S99);TLN1(S425);TNK2(T829);TNK2(Y827);TNKS1BP1(S1297);TNKS1BP1(S1715);TNKS1BP1(S178);TNKS1BP1(S435);TNKS1BP1(S872);TNKS1BP1(S983);TNRC6C(S714);TNS1(S1269);TNS3(S660);TOP2A(S1213);TOP2B(S1400);TP53BP1(S265);TP53BP1(S580);TPD52L1(S149);TRAF4(S426);TRAFD1(S470);TRAM1(S365);TRAPPC12(S184);TRIM33(S862);TRIO(S1724);TRMT2A(S602);TRUB1(T27);TSC1(S505);TSC22D4(S279);TSC22D4(S62);TTF1(S65);TTF2(S883);TTN(S1406);TUBA1A(S48);TUBA1B(S48);TUBA1C(S48);TUBA3C(S48);TUBA3E(S48);TVP23C(S223);U2SURP(S67);UBA1(S13);UBAP2L(S416);UBE4B(S65);UBE4B(S79);UBE4B(S83);UBE4B(T64);UCKL1(S56);UFD1(S247);UFD1(S299);UPF1(S1127);UPF3B(T169);USP1(S67);USP20(S408);USP24(S1141);USP32(S1423);USP32(S1430);USP36(S713);UTP20(T1741);UTP3(S365);UTP3(S368);VCPIP1(S747);VENTX(S6);VPS26B(S304);WDFY4(S3123);WDR20(S434);WDR44(S403);WEE1(T190);WIPI2(S413);WIZ(S996);XRCC1(S226);XRCC1(S229);XRCC1(S241);XRCC1(S266);XRCC1(T198);XRN2(S471);YAP1(S131);YBX1(Y162);YEATS2(S627);YTHDC2(S1221);ZBTB3(S549);ZBTB37(S164);ZBTB7A(S526);ZC3H11A(S132);ZC3H11A(T321);ZC3H13(S209);ZC3H13(S64);ZC3H13(S873);ZC3H4(S908);ZFC3H1(S949);ZFP91(S101);ZFR(S1054);ZKSCAN8(S12);ZMYM2(S305);ZNF106(S641);ZNF219(S684);ZNF239(S191);ZNF280D(S545);ZNF286A(S19);ZNF444(S232);ZNF444(S235);ZNF462(S1090);ZNF462(S688);ZNF513(S85);ZNF516(T930);ZNF518A(S655);ZNF552(S86);ZNF574(S164);ZNF587B(S87);ZNF609(S1055);ZNF609(S804);ZNF638(S1401);ZNF687(S433);ZNF814(S87);ZNRF2(S21);ZRANB2(S153);ZXDC(S34);ZYX(S259);ZYX(S267)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>CSNK2A2</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>35</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(T49);AHCTF1(S528);AKAP11(S422);AMFR(S542);ANAPC1(S355);ANLN(S182);ANLN(T194);ATXN2L(S424);CENPF(S3119);CNK3/IPCEF1(S892);FTSJ3(T573);FUS(S462);FXR2(T411);GTF3C2(S167);HIST1H1B(S18);HPS5(S534);INCENP(S311);IPCEF1(S430);NADK(S48);NUP107(S11);PBRM1(S13);PCNP(T139);PEA15(S116);PKP4(S314);RALY(S135);RBM39(S97);RBM39(Y95);RPA1(T180);RRM2(T33);SATB1(S637);SHANK2(S67);SNRPA1(T180);TELO2(S836);THRAP3(S253);UPF3B(T169)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>DYRK2</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>47</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>ABI1(Y213);ACIN1(T414);AHCTF1(S528);AKAP11(S422);ANAPC1(S355);ARHGEF18(S1111);CNK3/IPCEF1(S892);FAF1(S582);FARSA(S301);FUS(S462);FXR2(T411);GTF3C2(S167);HNRNPC(S253);HPS5(S534);IGLL1(S58);IPCEF1(S430);JPT2(T76);KIF4A(T1181);MAPK3(T207);MKI67(S1131);NADK(S48);NCL(T76);NUFIP2(S112);NUP210(S1877);PBRM1(S13);PCNP(T139);PEA15(S116);PHF8(S880);PIH1D1(S173);PKP4(S314);PLEKHG4B(T727);RANBP2(S1128);RBM15(S622);RBM39(S97);RBM39(Y95);RFC1(S71);RFC1(Y67);RGL2(T752);RRP1B(S458);SACS(S1779);SAPCD2(S157);SHANK2(S67);SPAG9(S733);TMEM201(S454);TMPO(S306);TNKS1BP1(S836);UPF3B(T169)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>EIF2AK1</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>37</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(S30);AHCTF1(S528);AMPD2(S100);ANKRD17(S2401);ASIC3(S37);BAG3(T285);CNK3/IPCEF1(S892);EIF4B(S283);FXR2(T411);GTF3C2(S167);IPCEF1(S430);IRF2BP2(S318);KIAA1522(S971);LARP6(S409);LINC00322(S226);MARK2(S456);MARK3(S469);NADK(S48);PBRM1(S13);PCNP(T139);PKP4(S314);PLCL2(S17);PLEKHA5(S885);PRAG1(S712);PRAG1(S889);RBM15(S622);RBM39(S97);RBM39(Y95);SCRIB(S1448);SHANK2(S67);SKIV2L(S131);SRSF7(S165);TRIM37(S771);UBE2O(S515);WIPF2(S235);XPR1(S666);ZC3HAV1(S378)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>ERN1</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1745</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>09/07/18 00:00:00(T228);09/09/18 00:00:00(S30);09/09/18 00:00:00(T142);AAK1(S14);AAK1(T606);ABCB11(S694);ABI1(S216);ABI1(Y213);ABI2(S368);ABL2(S936);ABLIM1(S431);ABLIM1(S640);ABR(T74);ACIN1(S657);ACIN1(T414);ACSL3(T107);ACTA1(S241);ACTA2(S241);ACTB(S239);ACTBL2(S240);ACTC1(S241);ACTG1(S239);ACTG2(S240);ACTL6A(S233);ADAM10(S740);ADAM10(Y741);ADAM17(S791);ADAMTS5(S264);ADD1(S12);ADD1(S431);ADD1(S726);ADD2(S600);ADD2(S713);ADD3(S681);ADD3(S693);ADNP(S709);AEBP2(S24);AFDN(S1721);AFDN(T1330);AFF4(S1043);AFF4(S1058);AFF4(S32);AFF4(S487);AGAP1(S422);AGAP1(S521);AGAP1(T836);AGAP2(S808);AGAP2(T809);AGFG1(S181);AGFG1(S293);AGFG1(T177);AHCTF1(S528);AHDC1(S1064);AHDC1(S1507);AHNAK(S115);AHNAK(S177);AHNAK(S216);AHNAK(S3412);AHNAK(S3426);AHNAK(S5763);AKAP1(S107);AKAP1(S445);AKAP11(S1580);AKAP11(S422);AKAP11(S448);AKAP12(S286);AKAP13(S2728);AKAP2(S121);AKAP8(S339);AKIRIN2(S21);AKT1S1(S88);ALMS1(T3036);ALX1(S69);AMBRA1(S1205);AMBRA1(S639);AMPD2(S100);ANAPC1(S355);ANK1(S15);ANKHD1(S1679);ANKMY1(S861);ANKRD17(S1709);ANKRD17(S19);ANKRD17(S2401);ANKRD2(S99);ANKS1A(S382);ANKZF1(S675);ANLN(S182);ANLN(S323);ANLN(S449);ANLN(S485);ANLN(S927);ANLN(T194);ANP32B(T244);AP1M1(T154);AP3B1(S276);APPL1(S401);APRT(S30);ARFGAP1(T135);ARFGAP2(S368);ARFGAP2(S432);ARFGEF2(S227);ARFGEF3(S2061);ARFGEF3(S2097);ARHGAP1(S44);ARHGAP1(S51);ARHGAP17(S162);ARHGAP17(S625);ARHGAP21(S856);ARHGAP29(S1029);ARHGAP39(S286);ARHGAP39(S366);ARHGAP39(S407);ARHGEF11(S150);ARHGEF11(S255);ARHGEF11(S35);ARHGEF16(S174);ARHGEF16(S208);ARHGEF17(S735);ARHGEF18(S1124);ARHGEF2(S137);ARID1A(S1184);ARID1A(S1604);ARID1A(S730);ARID1A(S772);ARID1A(T1206);ARID3B(S381);ARID3B(S89);ARL6IP6(S80);ARPP19(S104);ASCC3(S2195);ATAD2(S327);ATAT1(S315);ATF7(S434);ATF7IP(S474);ATF7IP(S477);ATG2B(S1582);ATG2B(S1583);ATG2B(Y1577);ATN1(S661);ATN1(T653);ATP2B1(S1193);ATXN2L(S32);ATXN2L(S424);ATXN2L(S559);AUTS2(S941);AXIN1(S77);B3GNT8(S37);BAG3(S289);BAG3(T285);BAIAP2L1(S261);BAIAP2L1(S414);BAZ1A(S1280);BAZ1B(S349);BCAM(S600);BCL11A(S205);BCL11A(S328);BCL2L12(S113);BCL2L12(S121);BCL2L12(T117);BCL7C(S126);BCL9L(S21);BCL9L(S750);BCLAF1(S397);BCR(S122);BCR(S459);BICRAL(S675);BIN1(S331);BIN2(S259);BIRC6(S577);BRD1(S128);BRD2(S633);BRD4(S1126);BRIP1(S128);BRIP1(S956);BRSK2(S439);BRSK2(T459);BRSK2(T463);BUB1(S655);BUD13(S325);C16orf54(S194);C2CD2L(S662);C2CD4C(S178);C2CD5(S281);C2CD5(S662);C6orf132(S449);C7orf50(S175);CABLES1(S291);CALU(S35);CALU(S44);CAMKV(T435);CAMSAP1(S563);CAMSAP1(S793);CAMSAP3(S1074);CAMSAP3(S1080);CAMSAP3(S814);CARD11(S512);CARHSP1(S30);CARHSP1(S41);CARMIL2(S1315);CASKIN2(S471);CASP8AP2(S567);CAT(S515);CBL(S799);CBX8(S311);CBY1(S9);CC2D1A(S455);CCAR2(S124);CCDC120(S358);CCDC6(S240);CCDC8(S261);CCDC86(T42);CCDC88B(S1379);CCDC88C(S227);CCDC9(S376);CCDC93(S305);CCL13(S44);CCNE1(S103);CCNK(S340);CCNL1(S342);CCNY(S25);CD244(S334);CD2AP(S458);CD97(S818);CD97(S831);CDAN1(S160);CDC25C(S216);CDC42BPA(S1651);CDC42EP4(S292);CDC6(S106);CDC6(S54);CDCA2(S98);CDCA3(S29);CDCA3(S87);CDCA7L(S261);CDK11A(S271);CDK11B(S283);CDK12(S423);CDK12(T1244);CDK12(T893);CDK13(T1056);CDK14(S134);CDK14(S78);CDK14(S95);CDK16(S138);CDK17(S137);CDK17(S9);CDK18(S117);CDK18(S74);CDK7(T170);CDK9(S347);CDV3(T182);CEBPE(S21);CENPF(S276);CENPF(T144);CENPO(S35);CEP131(S114);CEP170(S881);CEP192(S1514);CEP55(S428);CEP72(S237);CEP97(S308);CFL1(S3);CHAF1A(S206);CHAF1A(S772);CHAF1A(S775);CHAMP1(S308);CHAMP1(S319);CHAMP1(S376);CHAMP1(S416);CHAMP1(S432);CHAMP1(S436);CHAMP1(S445);CHAMP1(S452);CHAMP1(S472);CHAMP1(S507);CHD1(S1677);CHD4(S303);CHD8(S1978);CHD8(T1982);CIR1(S202);CIT(S1322);CIZ1(S838);CLASP1(S636);CLASP2(S325);CLASP2(S525);CLASP2(S529);CLASRP(S547);CLINT1(T308);CLK1(S337);CLK2(S142);CLNS1A(S102);CLSPN(S516);CMTR1(S31);CNK3/IPCEF1(S873);CNK3/IPCEF1(S892);CNN3(S296);CNNM3(S467);CNOT2(T93);CNP(S170);CNTNAP4(S520);COBL(S269);COBL(S347);COG2(T480);COIL(T303);COL19A1(S81);COL4A3BP(S373);COPA(S173);COPE(S13);CPSF7(S48);CPSF7(T203);CRAMP1(S1268);CREB1(S111);CREB1(S271);CRKL(Y198);CSNK1D(S331);CSNK1D(S350);CSNK1E(S363);CSPP1(S901);CSPP1(S966);CTAGE1(S616);CTAGE5(S647);CTDP1(S416);CTPS1(S573);CTPS2(S568);CTTN(S405);CTTN(Y421);CTTNBP2NL(S568);CTU2(S419);CXADR(S332);CYBA(T147);DACH1(S727);DAXX(S178);DAXX(S671);DBF4(S359);DBF4(S381);DBF4(T510);DBNL(T291);DBP(S86);DCDC2(S270);DCK(S74);DCLK1(S337);DCLRE1C(S518);DCP2(S284);DDX20(T552);DDX21(S89);DDX3Y(S592);DDX5(S480);DENND4A(S1240);DENND4A(S1256);DENND4A(S728);DENND4A(T1019);DENND4C(S1277);DENND4C(S1301);DENR(S73);DFFA(S315);DGCR8(S271);DGCR8(S275);DGCR8(Y267);DHX29(S200);DIDO1(S1040);DIP2B(S259);DKC1(S494);DLG5(S1000);DLG5(S1209);DLG5(T1279);DLG5(T984);DLGAP4(S666);DLGAP5(S725);DMAP1(T445);DMWD(S495);DNMT1(S127);DNMT1(T137);DNTTIP2(S434);DNTTIP2(T172);DOCK5(S1789);DOCK7(S30);DOCK7(S898);DOCK7(S946);DOCK8(S139);DOCK8(S451);DPF2(S244);DTL(S425);DYNC1LI1(S398);EAF2(S154);EEF1A1(Y29);EEF1A1P5(Y29);EEF1A2(Y29);EEF2K(S72);EEF2K(S74);EEF2K(Y69);EEPD1(S21);EHBP1(T378);EHBP1L1(S285);EIF2B1(S107);EIF3A(S1188);EIF3E(S399);EIF4B(S283);EIF4EBP1(T82);EIF4EBP3(S51);EIF4ENIF1(S5);EIF4ENIF1(S752);EIF4G1(S1092);EIF4G1(S1209);EIF4G2(S395);EIF4H(S21);EIF5B(S438);ELAVL1(S202);ELF2(T374);ELMO1(S344);ELOA(S413);ELP2(S122);EML4(S144);EML4(S146);EMSY(S1213);ENAH(T538);EP300(S1038);EP400(S1547);EP400(S722);EP400(S736);EPB41L1(S541);EPB41L1(S544);EPB41L1(S784);EPB41L2(S715);EPB41L3(S760);EPB41L3(S962);EPB41L4B(S390);EPB41L5(S436);EPB41L5(S550);EPS15(S814);EPS15L1(S793);EPX(S672);ERC1(S21);ERCC5(S384);ERCC6L(S1069);ERLIN1(S324);ERRFI1(S461);ESCO2(S75);ESS2(S292);ESS2(T110);ESS2(Y102);ETV6(S203);EVPL(S2025);EXOC2(S435);EZH2(S363);EZH2(T367);FADD(S194);FAM117B(S10);FAM117B(S457);FAM120A(Y452);FAM122A(S143);FAM122A(S189);FAM124A(S321);FAM129B(S665);FAM129B(S681);FAM129B(S696);FAM169A(S526);FAM171A1(S849);FAM193B(S785);FAM207A(T34);FAM53B(S118);FAM53B(S179);FAM53C(S162);FAM53C(S273);FAM76B(S193);FAM83B(S766);FAM83H(S523);FAM83H(S914);FANCI(S1121);FARP1(S340);FARP1(S427);FARSA(S301);FBRSL1(T1010);FBXW9(S59);FCHO2(S387);FERMT3(S497);FGD1(S82);FGD6(S692);FGFR1OP(T170);FIP1L1(S259);FOCAD(T543);FOXJ3(S223);FOXK1(S223);FOXK1(S257);FOXK1(S416);FOXK1(S420);FOXK1(S441);FOXK2(S398);FOXO1(S329);FOXP1(S83);FRMD3(S416);FUBP3(S296);FUBP3(S569);FUS(S462);FXR2(S601);FXR2(T411);FZR1(S163);G3BP2(S141);G3BP2(S149);GAB2(S141);GAB2(S623);GAGE13(S33);GAGE2A(S32);GAGE2B(S32);GAGE2D(S32);GAPVD1(S902);GATAD2A(T189);GATAD2B(S334);GATAD2B(S486);GBF1(S1061);GBF1(S1298);GEMIN2(S81);GEMIN5(S770);GFI1(S94);GFPT1(S261);GIGYF2(S26);GJA1(S262);GJA1(S325);GJA1(Y267);GLCCI1(S30);GLCCI1(T110);GMPS(T318);GNL3(S529);GON4L(S346);GORASP1(S220);GPAT3(S68);GPATCH2(S195);GPRIN1(S615);GPS1(S468);GRAMD1A(S263);GRAMD1B(S274);GRB10(S104);GRIP1(S847);GSE1(S826);GSE1(S828);GSE1(T433);GSK3B(S25);GSK3B(S9);GTF2F1(S385);GTF2F1(T389);GTF2F1(T446);GTF2I(S210);GTF2I(T558);GTF3C2(S132);GTF3C2(S167);GTF3C2(S893);GTPBP1(S580);HAUS6(T584);HBS1L(T231);HCFC1(S1205);HCFC1(S598);HCFC1(S666);HCLS1(S275);HCN4(S1059);HDAC1(S406);HDAC1(S421);HDAC1(S423);HDAC2(S422);HDAC2(S424);HDAC4(S266);HDAC5(S279);HDAC7(S358);HDAC7(S487);HDAC9(S240);HDGF(S133);HDGFL2(S366);HDGFL2(S369);HDGFL2(S370);HDGFL2(S664);HEATR6(S336);HECW1(S1344);HECW2(S1310);HELB(S1050);HIC2(S348);HIPK1(T351);HIPK2(T360);HIPK4(S337);HMGCS1(T490);HMGN1(S25);HNRNPA1(S338);HNRNPA1(S6);HNRNPA1(S95);HNRNPA1L2(S95);HNRNPA2B1(S212);HNRNPA2B1(S225);HNRNPA2B1(S259);HNRNPA2B1(S344);HNRNPA3(S358);HNRNPC(S253);HNRNPK(S284);HNRNPLL(S61);HNRNPM(S528);HNRNPM(S618);HPS5(S534);HRNR(S903);HSP90AA1(S399);HSP90AB1(S391);HSP90AB3P(S333);HSPB1(S15);HSPB1(S199);HSPB1(S82);HSPB1(S98);HSPH1(S809);HUWE1(S1084);HUWE1(S1907);HUWE1(S3127);HUWE1(T2889);HYLS1(S297);IBTK(S1045);ICE1(S255);IGLL1(S58);IKBKB(S672);INCENP(T292);INPP5D(T963);INTS10(S231);INTS12(S128);INTS3(S994);INTS3(S998);IPCEF1(S411);IPCEF1(S430);IRF2BP1(S421);IRF2BP2(S175);IRF2BP2(S318);IRF2BP2(S360);IRF2BP2(S406);IRF2BPL(S215);IRF2BPL(S519);IRS1(S1078);IRS1(S329);IRS1(T351);IRS2(S1176);ISCU(S20);ITGAL(S37);ITSN1(S315);ITSN2(S884);ITSN2(S889);IWS1(S248);IWS1(S250);IWS1(S398);IWS1(S400);JADE3(S566);JMJD1C(S1223);JMJD1C(S641);JMY(S115);JPH1(S216);JPH4(S157);JPT1(S131);JPT2(S97);JPT2(T76);KANK2(S172);KANK2(S175);KANSL1(S249);KANSL1(S991);KANSL1(S994);KCAB2_HUMAN_Phospho (ST);KCNK2(S366);KIAA0319L(S978);KIAA0754(S25);KIAA0930(S304);KIAA1217(S1794);KIAA1217(S357);KIAA1217(S361);KIAA1468(T143);KIAA1522(S327);KIAA1522(S342);KIAA1522(S858);KIAA1522(S862);KIAA1522(S929);KIAA1522(S971);KIAA1522(S979);KIAA1551(S1358);KIF13B(S1644);KIF15(S568);KIF1A(S1094);KIF1A(S1528);KIF1A(S1532);KIF21A(S1212);KIF21A(S1239);KIF21B(S1241);KIF21B(T1237);KIFC1(S26);KIFC1(S351);KLF3(S250);KMT2A(S2098);KMT2A(S2151);KMT2C(S46);KNOP1(S119);KPNA4(S60);KRT13(S427);KRT18(S30);KRT8(S36);KRT80(S451);KSR1(S334);L1TD1(S557);L3MBTL3(S608);LAD1(S301);LAMTOR1(S27);LARP1(S1056);LARP1(S90);LARP1(T526);LARP1(T649);LARP4(S583);LARP4(S722);LARP4(T389);LARP6(S409);LASP1(T104);LAT2(S135);LAT2(S51);LAT2(S86);LATS1(S464);LCP2(S207);LEMD3(S187);LEO1(S546);LIG3(S242);LIMA1(S132);LIMA1(S362);LIMA1(S609);LIMA1(S617);LIMK1(S298);LIMK1(S310);LIN28B(S203);LIN54(S310);LMNA(S390);LMNA(S628);LMNB1(T20);LMNB2(S37);LRCH1(S532);LRCH1(T568);LRCH4(S457);LRCH4(S520);LRP6(S1490);LRRFIP1(S116);LRRFIP2(S324);LRRTM4(S195);LSM11(S21);LSM14A(S183);LSM14B(S165);LSP1(S189);LSR(S464);LSR(S510);LSR(T453);LUZP1(S745);LYSMD2(S24);MACF1(S7330);MAGED2(S191);MAML1(S360);MAP1A(S1675);MAP1A(S1776);MAP1B(S1501);MAP1B(S1512);MAP1S(S640);MAP1S(T638);MAP2(S1540);MAP2(S1653);MAP2(T1649);MAP3K1(S1018);MAP3K11(S507);MAP3K11(S524);MAP3K8(S141);MAP4(T521);MAP4(T942);MAP4K3(S616);MAP4K4(S639);MAP7D1(S93);MAP7D3(S433);MARCKS(S163);MARCKS(S167);MARK1(S588);MARK2(S456);MARK2(S486);MARK2(S619);MARK3(S469);MARK3(S585);MARK3(S587);MAST2(S1381);MAST2(S876);MASTL(S619);MATR3(S598);MAZ(S361);MCM3(S704);MCM3(Y708);MCM3AP(S557);MCRIP2(S82);MDC1(T378);MED1(S1207);MED1(S953);MED1(T1215);MED13(S890);MEF2D(S180);MEF2D(S251);MEPCE(S217);MEPCE(T213);MFAP1(S116);MFAP1(S132);MFAP1(S133);MFGE8(S42);MFSD2B(S494);MGA(S2088);MGA(S3020);MGRN1(S524);MIA2(S1255);MIA3(S1741);MICAL3(S649);MICALL1(S295);MICALL1(S391);MICALL1(S486);MICALL1(S578);MICALL1(S621);MICALL1(S640);MICALL2(S143);MICALL2(S153);MICALL2(S249);MID1(S96);MIS18BP1(S1042);MISP(S394);MISP3(S91);MKI67(S2223);MKI67(S584);MLC1(S179);MLLT6(S378);MLLT6(S382);MMACHC(S275);MNAT1(S279);MOB1A(T35);MOB1B(T35);MOK(S298);MOK(T291);MON1B(S59);MON1B(S61);MORC2(S696);MORC2(S725);MPDZ(S230);MPHOSPH8(S403);MPLKIP(S115);MPLKIP(T51);MPLKIP(Y45);MPND(T76);MROH6(S9);MSANTD3(S274);MSH4(S902);MTA1(S386);MTA1(S449);MTA1(S522);MTA1(S576);MTA1(S639);MTA2(S435);MTBP(S639);MTBP(S755);MTCL1(S43);MTCL1(S87);MTFMT(S23);MTMR3(S613);MTMR4(S961);MTOR(S2454);MTSS1L(S342);MTX3(S284);MUC16(S12130);MYBBP1A(S11);MYBBP1A(S1267);MYC(S62);MYC(T58);MYCBP2(S3467);MYCN(S156);MYCN(S62);MYO10(S1883);MYO9B(S1267);MYO9B(S1331);MZT2A(S139);MZT2B(S139);NAA25(S691);NAA30(S199);NAA30(S39);NAA30(S89);NAB1(S403);NAB2(S171);NADK(S48);NADK(S64);NAF1(S315);NAP1L4(S125);NASP(S480);NASP(T390);NAV1(S1000);NAV1(S1382);NAV1(S754);NAV1(S760);NAV1(S808);NAV2(S1559);NAV2(S1800);NCAPD2(Y1325);NCKAP5L(S473);NCKIPSD(T181);NCL(S145);NCL(S153);NCL(S184);NCL(S206);NCOA2(S565);NCOA3(S1330);NCOA5(T460);NCOR1(S1980);NCOR1(S1981);NCOR2(S1018);NCOR2(S1487);NCOR2(S1547);NCOR2(S2424);NCOR2(S54);NCOR2(S956);NDC1(S500);NECAP2(S181);NECTIN1(T391);NELFA(S233);NES(S475);NES(S476);NES(S768);NEXN(S243);NF1(S1140);NFATC1(S278);NFATC1(S282);NFATC2(S217);NFATC2(S814);NFIA(S287);NFIC(S473);NFIX(S265);NHSL1(S1386);NIPBL(S318);NKTR(S379);NKTR(S463);NLN(S485);NMT1(S47);NOL6(S283);NOL8(S268);NOL8(S890);NOL8(T888);NOLC1(S397);NOLC1(S456);NOLC1(S508);NOLC1(S622);NOLC1(S643);NONO(T450);NOP16(S16);NOP53(S29);NOP58(S351);NOS1AP(S266);NPFFR2(S54);NPM1(S137);NPM1(S260);NSD1(S2471);NSD2(S421);NSFL1C(S140);NSRP1(S33);NSUN2(S456);NSUN2(S473);NUCKS1(S113);NUCKS1(S181);NUCKS1(T179);NUFIP2(S230);NUMA1(S1862);NUMA1(S1887);NUMA1(S1991);NUMBL(S263);NUP153(S209);NUP210(S1848);NUP210(S1877);NUP210(S1881);NUP214(S1045);NUP35(S55);NUP35(S66);NUP35(T273);NUP98(S1043);NYNRIN(S660);OBSL1(S10);OBSL1(S1671);OR8J2(S137);ORC2(T226);ORC6(T195);OSBPL11(S181);OSBPL8(S68);OSBPL9(S326);OTUD7B(S464);P2RX7(S470);P2RX7(T467);PA2G4(S363);PABPN1(S150);PACS1(S495);PAGR1(S237);PAK4(T207);PALD1(S406);PALLD(S1116);PALLD(S1118);PALLD(S1121);PALM3(S155);PALM3(T151);PAPOLA(T23);PAPOLG(S599);PARD3(S174);PARD3(S220);PARD3(S221);PARG(S137);PARN(S619);PARVA(S10);PARVA(S14);PARVA(S19);PATL1(S278);PAXX(S148);PBRM1(S12);PBRM1(S13);PBX2(S330);PCBP1(S173);PCBP1(S190);PCBP1(S231);PCBP1(S262);PCBP2(S189);PCDH1(S949);PCDH1(S962);PCDHB13(S69);PCDHB8(S69);PCGF6(S115);PCM1(S1958);PCM1(S776);PCM1(S779);PCM1(T79);PCM1(T82);PCNP(T139);PCNT(S2355);PCYT1A(S315);PCYT1A(S347);PCYT1B(S315);PDCD4(S94);PDCD6IP(S730);PDLIM2(S129);PDLIM4(S112);PDLIM5(S111);PDLIM5(S313);PDS5B(S1358);PDS5B(T1301);PDZD2(S1270);PDZD4(S564);PDZD8(S521);PEAK1(S823);PER2(S977);PFKL(S775);PGAM1(S118);PGAM4(S118);PGRMC1(S181);PHACTR1(S505);PHACTR2(S443);PHACTR2(S445);PHACTR2(S471);PHACTR2(T25);PHACTR2(T452);PHACTR2(Y451);PHACTR4(S131);PHACTR4(S443);PHF3(S1614);PHF6(S154);PHF8(S880);PHKA2(S1043);PHLDA2(S144);PHLDA2(S42);PHLDB1(S461);PHLDB1(S470);PHLDB2(S73);PHOX2A(S208);PHRF1(S1124);PHRF1(S1202);PI4K2A(S51);PI4KB(S266);PIK3AP1(S759);PKN1(S562);PKP4(S273);PKP4(S314);PKP4(S337);PKP4(S406);PLCB3(S926);PLCH1(S1060);PLCL2(S17);PLEC(S1435);PLEC(S4613);PLEKHA2(S349);PLEKHA5(S140);PLEKHA5(S568);PLEKHA5(S885);PLEKHA5(S933);PLEKHA5(T857);PLEKHA7(S612);PLEKHG3(S76);PLEKHG4B(T727);PLEKHO2(S390);PLIN3(S130);PLK1(T214);PLPPR3(S353);PLPPR3(S508);PML(S505);PML(S527);PNISR(S211);PNN(S100);POLA2(T127);POLD2(S15);POLD3(S307);POLM(S372);POLR2A(S1875);POM121(S298);POM121(S435);POM121B(S19);POM121C(S275);POM121C(S412);POMZP3(S33);POTEE(S939);POTEF(S939);POTEKP(S239);PPAN(S359);PPFIA1(S1172);PPFIA3(S1164);PPFIBP1(S636);PPHLN1(S163);PPHLN1(S205);PPHLN1(T200);PPHLN1(T204);PPIP5K1(S964);PPL(S14);PPM1H(S221);PPME1(S15);PPP1CA(T320);PPP1CC(T311);PPP1R12A(S903);PPP1R12C(S509);PPP1R13L(S102);PPP1R13L(S358);PPP1R13L(S395);PPP1R14B(S32);PPP1R35(S87);PPP1R35(T84);PPP1R3D(S74);PPP1R3D(S78);PPP1R9B(S100);PPP4R2(S159);PPP4R2(S226);PPP4R3A(S741);PPP4R3A(S774);PQBP1(S247);PRAG1(S510);PRAG1(S712);PRAG1(S889);PRAM1(S298);PRDM2(S1484);PRKCD(S645);PRKCD(T141);PRKD1(S549);PRKD1(S742);PRKD3(S735);PRKDC(S2612);PRKDC(S3205);PRKDC(T1045);PRPF4B(S277);PRPF4B(S292);PRPF4B(S294);PRPF4B(S852);PRPF4B(Y849);PRPF6(T266);PRR11(S40);PRR12(S314);PRR15(S49);PRR36(T1082);PRR5(S11);PRRC2A(S1147);PRRC2A(S2113);PRRC2A(S761);PRRC2A(T1347);PRRC2B(S1691);PSD4(S118);PSMD1(T273);PSMD2(S16);PSMF1(S153);PSPC1(S477);PTDSS2(S16);PTGES3(S113);PTPN13(S2032);PTPN22(S692);PTS(S19);PTTG1(S165);PTTG2(S165);PWP1(S50);PXN(S258);PXN(S85);PXN(Y118);PYCR2(S304);QSER1(S1348);QSER1(T1341);R3HDM2(S349);RAB11FIP1(S435);RAB12(S21);RAB3IL1(S168);RAB40C(S268);RABGEF1(S302);RABGEF1(S607);RAD51AP1(S120);RALGAPA2(S1629);RALGAPB(T379);RALGPS2(S308);RALGPS2(S329);RANBP2(S2454);RANBP2(S2900);RANBP2(S788);RANBP3(S108);RANBP3(S211);RANBP9(S477);RANBP9(S482);RAPGEF1(S311);RAPGEF2(S1080);RASAL3(S18);RASGRP2(S391);RB1(S788);RB1(S795);RB1(S807);RB1(T356);RB1(T821);RB1(T826);RB1(Y790);RBBP6(S1697);RBBP6(S516);RBBP8(T315);RBL1(S749);RBL1(S988);RBL1(T369);RBL1(T385);RBL2(S413);RBL2(S639);RBM10(S797);RBM10(S845);RBM12B(S638);RBM14(S520);RBM15(S128);RBM15(S294);RBM15B(S552);RBM17(S169);RBM27(T447);RBM39(S97);RBM39(Y95);RBM6(S1025);RBMX(S208);RBMX(S249);RBMX2(S188);RBMXL1(S208);RBMXL1(S249);RBMXL1(S88);RBPMS(T118);RBSN(S429);RCSD1(S116);RCSD1(S120);RECQL5(S815);REPS1(S709);REXO4(S15);RFTN1(S61);RFX7(S1028);RFX7(S225);RFX7(S424);RGL2(T752);RGPD1(S1463);RGPD1(S779);RGPD2(S1471);RGPD2(S787);RGPD3(S1479);RGPD3(S789);RGPD4(S1479);RGPD4(S789);RGPD5(S1478);RGPD5(S21);RGPD5(S788);RGPD8(S1478);RGPD8(S21);RGPD8(S788);RHBDF2(S113);RICTOR(S1284);RIF1(S1454);RIF1(S1688);RIF1(S2205);RIF1(T1047);RIOK1(S22);RIPOR1(S349);RIPOR1(S351);ROBO1(S1055);ROBO2(S1156);RPL18(S161);RPL18(T158);RPL34(S12);RPRD2(S665);RPRD2(S769);RPRD2(S965);RPRD2(T732);RPS6(S235);RPS6KA3(S369);RPUSD2(S68);RREB1(S1320);RREB1(S161);RREB1(S42);RRP1B(S735);RSF1(S1277);RSF1(S1282);RSF1(T1278);RSF1(T1305);RSF1(Y1281);RSL1D1(S392);RSL1D1(S396);RSL1D1(T415);RSRC2(S32);RTKN(S543);RTN3(S229);RUFY1(S620);RUNX1(S21);SACS(S1779);SALL2(S806);SALL3(T935);SAMD1(S161);SAMD4B(S172);SAMD4B(S628);SASH3(S21);SCAF8(S617);SCML2(S267);SCRIB(S1306);SCRIB(S1348);SCRIB(S1448);SCRIB(S504);SCRIB(S853);SEC16A(S136);SEC16A(S1905);SEC16A(S391);SEC16A(T19);SEC31A(S799);SEC61A1(S408);SEMA6A(T761);SENP1(S170);SENP6(S350);SEPT9(S22);SET(S28);SET(S7);SETDB1(S1066);SETX(S1663);SF3B1(S129);SF3B1(T244);SF3B1(T303);SF3B1(T313);SF3B2(S307);SFMBT2(T762);SFPQ(S33);SFRP2(S287);SFRP2(S289);SFSWAP(S909);SGO1(S461);SGO1(S468);SH2D3C(S440);SH2D5(S231);SH3BP1(S586);SH3BP1(S598);SH3BP1(S612);SH3BP1(S613);SH3BP1(T626);SH3BP2(S278);SH3BP2(S427);SHANK1(S948);SHANK2(S1069);SHANK2(S452);SHANK2(S67);SHC3(S474);SHROOM2(S422);SHROOM3(S242);SHROOM3(S439);SHROOM3(S816);SHROOM3(S913);SHROOM3(T576);SIK3(T469);SIN3A(S1112);SIPA1L1(S1087);SIRT1(S172);SIRT1(S27);SLAIN2(S48);SLC12A7(T30);SLC12A7(T980);SLC13A4(S246);SLC4A1AP(S82);SLC4A7(S556);SLC6A15(S687);SLC7A6OS(S308);SLC9A3R1(S280);SLX4(S1044);SLX4(S1309);SLX4(S1333);SMAP2(S219);SMARCA2(S588);SMARCA4(S695);SMARCAD1(S146);SMARCC2(S283);SMARCC2(T548);SMC3(S1083);SMCR8(S498);SMNDC1(S201);SMTN(S32);SMTN(S341);SNAP23(S110);SNAPC4(S599);SNIP1(S35);SNRK(S518);SNRNP200(S225);SNRNP70(S226);SNRPC(S17);SNTB1(S219);SNTB1(S87);SNTB2(S393);SNTB2(S95);SNURF(S32);SNX1(S188);SNX17(S336);SNX17(S409);SNX17(S437);SNX17(S440);SNX2(S277);SNX8(S456);SNX8(T452);SOGA1(S1017);SORBS3(S530);SOWAHC(S213);SP110(S380);SP3(S73);SPATA19(S148);SPECC1(S55);SPECC1(S847);SPEG(S2109);SPIRE1(T509);SPRY2(S142);SPRY4(S125);SPTBN1(S2341);SRF(S224);SRGAP1(S932);SRRM1(S391);SRRM1(S431);SRRM1(S695);SRRM1(S738);SRRM2(S1329);SRRM2(S1404);SRRM2(S1499);SRRM2(S2071);SRRM2(S2123);SRRM2(S2272);SRRM2(S2382);SRRM2(S322);SRRM2(S323);SRRM2(S358);SRRM2(S398);SRRM2(S510);SRRM2(S774);SRRM2(S952);SRRM2(S954);SRRM2(T1492);SRRM2(T1531);SRRM2(T2058);SRRM2(T2061);SRRM2(T2069);SRRM2(T315);SRSF1(S199);SRSF1(S201);SRSF1(S205);SRSF11(S434);SRSF7(S192);SRSF9(S216);SSB(S366);STAM(S156);STAMBPL1(S242);STAU2(S486);STIM1(S575);STIM1(S618);STIM2(S523);STK10(S417);STK10(S438);STK10(S450);STK11IP(S470);STK17A(S28);STK33(S470);STMN1(S38);STRN(S245);STRN(T143);STRN(Y135);STUB1(S23);SUGT1(S281);SUPT6H(T1523);SURF6(S138);SVIL(S968);SYN1(S427);SYN1(S551);SYN1(S553);SYNJ1(S1053);SYNJ2(S1124);SYTL2(S344);SZRD1(S74);TACC3(S250);TACC3(S317);TAF4B(S595);TAF6(S634);TAF6(S636);TAF7(S201);TALDO1(S237);TANC1(S67);TANC2(S1977);TAOK1(S421);TAOK1(S9);TAOK1(S965);TARDBP(S292);TBC1D1(S211);TBC1D10B(S22);TBC1D10B(S678);TBC1D10B(T152);TBC1D13(S184);TBC1D22A(S167);TBC1D2B(S155);TBC1D5(S522);TBC1D5(S554);TBC1D5(S730);TBC1D9B(S435);TBKBP1(S365);TBX2(S653);TC2N(S168);TCF20(S559);TCF20(S574);TCOF1(S1227);TCOF1(S1257);TCOF1(S503);TCOF1(S583);TCOF1(S906);TCOF1(T914);TCOF1(T983);TDRD12(S211);TERF2IP(S154);TET2(S1107);TEX2(S266);TEX2(S732);TFDP1(S23);TFE3(S548);TFE3(S556);THAP4(S128);THOC2(T1443);THOC5(S314);THOP1_HUMAN_Phospho (ST);THRAP3(S248);THRAP3(S575);THRAP3(S928);TICRR(T1260);TJAP1(S320);TJAP1(T318);TJAP1(T60);TJAP1(Y316);TJP1(S617);TJP1(S968);TJP2(S266);TJP3(S591);TK1(S231);TLE1(T312);TLE3(S263);TLK2(S771);TLN1(S425);TMEM185A(S333);TMEM185B(S333);TMEM201(S466);TMF1(S328);TMPO(S224);TMPO(S306);TMPO(S354);TMX1(S270);TNIK(S548);TNIK(S764);TNIK(S766);TNK2(Y827);TNKS1BP1(S1103);TNKS1BP1(S1620);TNKS1BP1(S1621);TNKS1BP1(S1715);TNRC6C(S714);TNS1(S1269);TNS1(T1173);TOM1(S464);TOM1L1(S323);TOR1AIP1(S135);TOR1AIP1(S143);TP53BP1(S1678);TP53BP1(S294);TP53BP1(S398);TP53BP2(S558);TPD52L2(S166);TPD52L2(S21);TPR(S379);TPX2(T369);TRA2A(T202);TRA2B(T201);TRA2B(T212);TRAFD1(S470);TRAP1(S401);TRAPPC12(S184);TRIM24(S654);TRIM71(S187);TRIO(S1724);TRIP12(S312);TRMT2A(S602);TRPM7(S1477);TRPS1(S216);TRPS1(T751);TRPV3(S372);TSC2(S1155);TTC7A(S182);TTYH3(S496);TUBA1A(S48);TUBA1B(S48);TUBA1C(S48);TUBA3C(S48);TUBA3E(S48);TVP23C(S223);TXLNG(S97);U2SURP(S37);U2SURP(S67);UBAP2L(S471);UBAP2L(S609);UBE2O(S515);UBE2O(T838);UBE4B(S65);UBE4B(T64);UBR4(S2718);UCK1(S253);UCKL1(S56);UHRF1(S287);UIMC1(S140);ULK1(S477);UNC13B(S367);UNC93B1(S547);UNC93B1(S550);UNG(T60);UPF3B(T169);USP1(S67);USP10(S211);USP14(S143);USP15(S242);USP20(S134);USP28(S1053);USP32(S1423);USP33(S439);USP36(S742);USP36(S952);USP36(T653);USP6NL(S396);USP7(S18);UTF1(S245);UTF1(S54);UTP18(S121);UTP18(S206);VCL(S290);VCL(S346);VCP(S770);VEZT(S696);VGLL4(S149);VPS13C(T1437);VPS13D(S1042);VPS72(S127);VRTN(S432);WAC(S511);WAC(T457);WASF1(S310);WDCP(S690);WDFY4(S3123);WDR20(S434);WDR44(S50);WDR62(S33);WEE1(S139);WIPF1(S340);WIPF2(S235);WIPF3(S149);WNK1(S2121);WNK3(S1095);WT1(S273);WWP2(S211);XPO4(S521);XRCC1(S226);XRCC1(S229);XRCC1(S241);XRCC1(T198);XRCC1(T202);XRCC1(Y211);XRCC4(S237);XRCC6(S477);YAP1(S289);YBX3(T67);YTHDC2(S1223);YTHDC2(S1279);YTHDF1(S291);ZBTB17(S120);ZBTB7B(S487);ZC3H11A(T321);ZC3H14(S515);ZC3H18(S67);ZC3H18(S74);ZC3H18(T796);ZC3H3(S571);ZC3H4(S1110);ZC3HAV1(S378);ZCCHC8(S598);ZCCHC8(T479);ZCCHC8(T485);ZDHHC18(S19);ZDHHC5(S425);ZDHHC5(S621);ZEB1(S679);ZFHX4(S2996);ZFP36L1(S54);ZFP64(S547);ZFP91(S101);ZFP91(S103);ZFPM1(S786);ZFR(S1054);ZFYVE19(S463);ZFYVE26(S1764);ZMYM4(S242);ZMYND8(S444);ZMYND8(S486);ZMYND8(S488);ZMYND8(S547);ZNF106(S641);ZNF221(S486);ZNF224(S548);ZNF24(S274);ZNF318(S1896);ZNF318(S501);ZNF326(S56);ZNF462(S1251);ZNF462(S455);ZNF507(S545);ZNF516(S852);ZNF516(T930);ZNF552(S86);ZNF574(S164);ZNF609(S1055);ZNF622(S143);ZNF638(S1401);ZNF639(S60);ZNF639(S88);ZNF687(S374);ZNF777(S47);ZNF800(S336);ZNF814(S87);ZNRF2(S135);ZSCAN29(S153);ZYX(S259);ZYX(S308);ZZEF1(S1518)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>FYN</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>288</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>AAK1(T653);AFAP1(S668);AFDN(S1318);AFDN(T1330);AGAP3(S538);AGPS(S65);AMBRA1(S1205);AMPD2(S100);ANKRD17(S2401);AP1M1(T154);ARHGAP17(S162);ARHGAP21(S476);ARHGAP45(S23);ARHGEF11(S255);ARHGEF2(T152);ARHGEF9(S502);ARPC1B(T315);ASCC3(S2195);ATF7(S434);ATF7IP(S474);ATF7IP(S477);ATL1(S10);ATXN2L(S32);BCL9(T315);BICRAL(S675);BTF3(S30);C17orf53(S332);CAMKV(T435);CAMSAP1(S793);CAMSAP3(S814);CASP3(S26);CCDC85C(S246);CCNY(S83);CDC42EP4(S118);CDC42EP4(T23);CDC6(S106);CDK12(S383);CDK12(S385);CDK14(S24);CDK14(S78);CDK16(S119);CDK17(S146);CDK18(S117);CHD4(S1531);CHD8(S1995);CIC(S173);COL4A3BP(S373);CRAMP1(S1268);CRTC3(S370);CRTC3(S62);CSNK1D(S331);CTNND1(S349);DCLK1(S332);DCLRE1C(S518);DOCK7(S888);DOPEY2(S681);DVL3(S125);EEF2K(S72);EEF2K(S74);EEF2K(Y69);EGLN1(S125);EIF3A(S1188);EIF3A(S1336);EIF4ENIF1(S752);EIF4G1(S1194);EPB41(S709);EPN2(S173);EPS15L1(S593);ESS2(T386);ESYT1(S627);ETV6(S203);EVPL(S2025);FAM120A(Y452);FAM193B(S785);FOXK1(S223);FRS2(S211);FYTTD1(S16);GAB2(T391);GAPVD1(S902);GLCCI1(S30);GON4L(S206);GPRIN1(S389);GRAMD1B(S274);GTF2F1(T389);HIPK1(T351);HIPK1(Y352);HIPK2(T360);HIPK2(Y361);HMGA1(S44);HMGCR(S872);HSH2D(S194);HTT(S1199);HUWE1(T2889);ICE1(S1712);IGLL1(S62);IKBKB(S672);INSRR(S72);IRS1(S374);ITSN1(S315);ITSN1(S978);KIF21A(S855);KIFC1(S26);KIFC1(S351);LSM14B(S165);LUC7L2(S18);LUC7L2(S347);LZTS1(S233);MAP2(S1555);MAP3K1(S292);MAP3K11(S524);MAP3K2(S153);MAP3K20(S727);MAP4(S928);MAP7D1(S113);MAP7D1(S399);MARCKS(S167);MARK1(S394);MARK2(S456);MARK3(S400);MAST2(S1364);MAST3(S747);MED13(S890);MELK(S505);MELK(S529);MFSD10(S271);MNAT1(S279);MON1B(S59);MON1B(S61);MPHOSPH8(S403);MTA1(S576);MTFR1L(S103);MTFR1L(S238);MYC(S62);MYCBP2(S2749);MYCBP2(S2751);MYCN(S62);MYH10(S1937);MYO7B(S689);MYOF(S1915);NAA30(S39);NAB2(S193);NECTIN1(T391);NFX1(Y48);NHSL1(S1233);NINL(S585);NSRP1(S33);NSUN2(S456);NSUN2(S473);NUP214(S1023);OSER1(S82);OSER1(S84);OTUD4(S416);PAK1(S144);PAK4(S163);PAK4(S181);PAK4(T207);PALD1(S406);PALM3(S303);PAPOLG(S708);PARD3(S174);PARD3(S717);PDHA1(S232);PDS5A(T1208);PDS5B(S1358);PHACTR1(S505);PHLDB1(S334);PI4KB(S428);PKN1(S562);PKP2(S289);PKP2(S329);PKP4(S337);PKP4(S406);PLCG1(S1263);PLEKHA5(S471);PLEKHA5(S885);POLH(S380);POLR2A(S1868);POLR2A(Y1860);PPFIBP1(S466);PPHLN1(S133);PPIP5K2(S1074);PPP1R12A(S445);PPP1R12A(S903);PPP1R13L(S102);PRAG1(S889);PRAM1(S334);PRPF6(S279);PRPF6(T275);PRRC2A(S1386);PRRC2C(S1544);PTPN12(S449);PTPN14(S642);RABEP1(S377);RALGAPA1(S797);RANBP1(S60);RAP1GAP2(S564);RB1(S249);RB1(T601);RBL1(S640);RBL1(T369);RBL2(S413);RBM10(S797);RBM15(S700);RBM15B(S113);RBM15B(S267);RBM15B(T532);RBMX(S208);RBMX(S326);RBMX(S332);RBMX(S88);RBMXL1(S208);RCSD1(S116);RCSD1(S120);RFX7(S225);RFX7(S424);RICTOR(S1284);RLIM(S228);RLIM(S230);RNF39(S244);RREB1(S42);SAFB(S604);SASH1(S813);SASH1(S90);SCAF1(S874);SCAMP2(S320);SCRIB(T475);SF3B1(T434);SH3BP4(S296);SH3PXD2B(S291);SHC3(S474);SHROOM2(T647);SHROOM3(S816);SIK3(S866);SIPA1(S839);SIRT1(S27);SLC4A10(S238);SLC4A7(S233);SLC4A7(S556);SLTM(S553);SMAP2(S240);SMARCA4(S610);SMCR8(S489);SNIP1(S35);SPAG9(S730);SPAG9(S733);SPP2(S182);SPTAN1(S1031);SRRM1(S429);SRRM2(S1404);SRRM2(S1458);SRRM2(S322);SRSF4(S446);SSSCA1(S78);STIM2(S680);STIM2(S719);STK33(S470);STX17(S289);TBKBP1(S365);TCOF1(S156);TEX2(S266);THRAP3(S232);TMEM201(S441);TNKS1BP1(S429);TNKS1BP1(S983);TNS1(S1269);TP53BP1(S1317);TRA2A(T202);TRAFD1(S470);TRAPPC12(S184);TRIO(S1724);TTC28(S2224);TVP23C(S223);ULK1(S556);ULK1(S719);USP1(S67);USP32(S1423);VASN(S284);YBX3(S293);ZC3H13(T364);ZC3H3(S571);ZC3HAV1(S335);ZC3HAV1(Y348);ZMYND8(S425);ZNF106(S641);ZNF516(T930);ZNF552(S86);ZNF609(S1055);ZNF814(S87)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>GAK</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>5</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(S30);GTF3C2(S167);NADK(S48);PCNP(T139);RBM39(Y95)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>GSK3A.B</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>AGFG1(T177)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>HIPK3</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>78</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(S30);ACTA1(S241);ACTA2(S241);ACTB(S239);ACTBL2(S240);ACTC1(S241);ACTG1(S239);ACTG2(S240);ADAM10(Y741);ADD1(S465);AHCTF1(S528);AKAP11(S422);AMPD2(S100);ANAPC1(S355);ANLN(S927);ARFGAP2(S432);ARHGEF38(S553);CAMSAP1(S629);CCNK(S340);CDK12(S383);CDK12(S385);CDK17(S137);CDK9(S347);CHD1L(T629);CHEK1(S280);CLASP2(S585);CRKL(Y207);DBNL(T291);DLG5(S1232);DNTTIP2(S117);EIF4B(S283);EPB41L1(S784);F11R(S284);FUS(S462);HPS5(S534);KIAA1522(S971);LRMP(S363);LRRFIP1(S116);MAP7D1(S254);MED1(T1051);MICALL2(S153);MSH6(S309);NCAPG(S674);NOB1(S352);NOP16(S16);NUMBL(S263);PCNP(T139);PININ_HUMAN_Phospho (ST);PLEKHA5(S885);POTEE(S939);POTEF(S939);POTEKP(S239);PPFIA1(S666);PPHLN1(S163);PREX1(S319);PTPN1(S378);R3HDM1(S381);RAB31(S35);RALGAPB(T379);RBMXL1(S88);RHBDD1(S291);RICTOR(S1284);RPA1(T180);RPS27(S78);RPS27L(S78);SAFB2(S787);SCAF1(T976);SHANK2(S67);SNRPA1(T180);SPAG9(S733);SPN(S291);STX7(S131);TBC1D13(S184);TNS2(S1003);TRAPPC12(S184);UBAP2L(S470);UPF3B(T169);VIM(S25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>IRAK1</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>586</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(S30);AAK1(S14);ABI1(S216);ABI1(Y213);ABLIM1(S431);ABR(T74);ACTA1(S241);ACTA2(S241);ACTB(S239);ACTBL2(S240);ACTC1(S241);ACTG1(S239);ACTG2(S240);ADAM10(S740);ADAM10(Y741);ADAM17(S791);ADD1(S12);ADD1(S726);ADD2(S713);ADD3(S693);ADNP(S709);AFDN(S1721);AFF4(S1043);AGAP2(S808);AGFG1(T177);AHCTF1(S528);AHNAK(S115);AHNAK(S177);AHNAK(S216);AHNAK(S3412);AHNAK(S3426);AHNAK(S5731);AKAP1(S107);AKAP11(S1580);AKAP11(S422);AKAP11(S448);AKAP13(S2728);AMBRA1(S1205);AMBRA1(S639);AMPD2(S100);ANAPC1(S355);ANKRD17(S2401);ANKS1A(S382);ANKZF1(S675);APPL1(S401);ARFGAP1(T135);ARFGAP2(S432);ARHGAP17(S625);ARHGAP39(S407);ARHGEF11(S35);ARHGEF16(S174);ARHGEF17(S735);ARHGEF18(S1111);ARHGEF26(S80);ARID1A(S1184);ARID1A(S1604);ARL6IP6(S80);ASF1B(T179);ATAD2(S327);ATAT1(S315);ATG2B(S1582);ATG2B(S1583);ATG2B(Y1577);ATN1(S661);ATN1(T653);ATXN2(S684);ATXN2(T666);ATXN2L(S424);BAG3(S289);BAG3(T285);BAP18(S110);BCL11A(S328);BCR(S459);BIN2(S259);BPTF(S1300);BRIP1(S956);C16orf54(S194);C16orf72(S167);C2CD2L(S662);C2CD5(S281);C6orf132(S449);C7orf50(S175);CALU(S35);CALU(S44);CAMSAP1(S563);CARHSP1(S41);CARMIL2(S1315);CAT(S515);CBL(S799);CBX8(S311);CCDC6(S240);CCDC9(S376);CCDC93(S305);CCL13(S44);CD97(S818);CD97(S831);CDC25C(S216);CDCA7L(S261);CDK18(S117);CDK9(S347);CENPF(S3119);CEP170(S881);CEP55(S428);CHAF1A(S206);CHAMP1(S376);CHAMP1(S445);CHAMP1(S452);CHAMP1(S472);CHAMP1(S507);CHD4(S303);CHD8(S1978);CHD8(T1982);CLASP1(S636);CLASP2(S325);CLASRP(S547);CLINT1(T308);CLK2(S142);CMTR1(S31);CNP(S170);COL4A3BP(S373);CPSF7(S48);CREB1(S111);CREB1(S271);CSPP1(S901);CTAGE1(S616);CTAGE5(S647);CTPS1(S573);CTU2(S419);CYBA(T147);DACH1(S727);DBF4(S381);DBNL(T291);DBP(S86);DDX3Y(S592);DENND4A(T1019);DIP2B(S259);DLG5(S1000);DLG5(T984);DLGAP5(S725);DNTTIP2(S434);DNTTIP2(T172);DOCK8(S451);DPYSL2(T509);DTL(S425);DYNC1LI1(S398);EEPD1(S21);EIF3E(S399);EIF4G2(S395);ELAVL1(S202);EML4(S146);EP400(S722);EPS15L1(S793);ERRFI1(S461);ESF1(S198);EZH2(T367);FADD(S194);FAM117B(S10);FAM122A(S143);FAM122A(S189);FAM129B(S665);FAM129B(S681);FAM129B(S696);FAM207A(T34);FAM53B(S179);FAM76B(S193);FAM83B(S766);FAM83H(S914);FARSA(S301);FBRSL1(T1010);FBXW9(S59);FIP1L1(S259);FLYWCH2(S21);FOXK1(S416);FOXK1(S420);FOXO1(S329);FTSJ3(T573);FUS(S462);FXR2(S601);GAB2(S141);GAPVD1(S902);GATAD2A(T189);GATAD2B(S334);GATAD2B(S486);GBF1(S1061);GBF1(S1298);GFI1(S94);GIGYF2(S26);GNL3(S529);GPATCH2(S195);GRIP1(S847);GTF2F1(T446);GTF3C2(S132);HCFC1(S666);HELB(S1050);HIC2(S348);HJURP(S557);HMGCS1(T490);HNRNPA1(S338);HNRNPA2B1(S344);HNRNPA3(S358);HNRNPM(S528);HNRNPM(S618);HPS5(S534);HRNR(S903);HSPB1(S82);IBTK(S1045);IGLL1(S58);INCENP(T292);INPP5D(T963);INTS12(S128);IRF2BP2(S318);IRF2BP2(S406);IRF2BPL(S519);ITSN2(S884);ITSN2(S889);JPT1(S131);JPT2(T76);KCAB2_HUMAN_Phospho (ST);KCNK2(S366);KIAA0319L(S978);KIAA0930(S304);KIAA1217(S361);KIAA1522(S342);KIAA1522(S858);KIAA1522(S862);KIAA1522(S929);KIAA1522(S979);KIF1A(S1094);KIF1A(S1528);KIF1A(S1532);KPNA4(S60);KRT13(S427);KRT18(S30);KRT8(S36);LAD1(S301);LAMTOR1(S27);LARP1(S1056);LARP1(S90);LARP1(T526);LAT2(S135);LAT2(S86);LCP2(S207);LEMD3(S187);LIMA1(S617);LIN54(S310);LMNA(S390);LMNA(S628);LMNB2(S37);LRCH1(S532);LRCH1(T568);LRCH4(S520);LRRFIP1(S116);LRRFIP2(S324);LSR(S464);MAP1A(S1675);MAP2(S1540);MAP3K11(S524);MAP7D1(S93);MARK1(S588);MARK2(S456);MARK3(S469);MAZ(S361);MCM3AP(S557);MCM4(S120);MIA2(S1255);MIA3(S1741);MICAL3(S649);MICALL1(S391);MICALL1(S486);MICALL1(S578);MICALL1(S640);MICALL2(S143);MICALL2(S153);MICALL2(S249);MIS18BP1(S1042);MKI67(S2223);MLC1(S179);MLLT6(S378);MLLT6(S382);MOB1A(T35);MOB1B(T35);MORC2(S696);MORC2(S725);MPDZ(S230);MPLKIP(S47);MTA1(S386);MTA1(S449);MTA1(S522);MTA2(S435);MTMR3(S613);MTMR4(S961);MTOR(S2454);MTSS1L(S342);MYBBP1A(S11);MYC(T58);MYCBP2(S3467);MZT2A(S139);MZT2B(S139);NAA10(S186);NAA30(S199);NAA30(S89);NCL(T121);NCL(T76);NCOR1(S1980);NCOR1(S1981);NCOR2(S1487);NCOR2(S1547);NCOR2(S2424);NCOR2(S54);NDC1(S500);NECAP2(S181);NES(S768);NFATC1(S278);NFATC1(S282);NFATC2(S217);NFATC2(S814);NOLC1(S397);NOLC1(S508);NOLC1(S643);NOP16(S16);NOP2(S732);NOP58(S351);NSD1(S2471);NUCKS1(T179);NUFIP2(S230);NUMA1(S1862);NUMA1(S1887);NUMA1(T2000);NUMBL(S263);NUP153(S209);NUP210(S1877);NUP210(S1881);NUP210(T1844);NUP35(S66);NYNRIN(S660);OBSL1(S10);ORC6(T195);OSBPL8(S68);PABPN1(S150);PAGR1(S237);PARD3(S221);PARVA(S19);PATL1(S278);PBRM1(S12);PCBP1(S190);PCBP1(S231);PCM1(T79);PCM1(T82);PCNP(T139);PCYT1A(S315);PCYT1A(S347);PCYT1B(S315);PDCD6IP(S730);PDLIM4(S112);PDLIM5(S111);PDZD8(S521);PEA15(S116);PFKL(S775);PGRMC1(S181);PHACTR2(T25);PHLDA2(S42);PHLDB1(S461);PI4K2A(S51);PIK3AP1(S759);PKP4(S314);PLCB3(S926);PLEC(S1435);PLEC(S4613);PLEKHA5(S933);PLEKHA5(S937);PLEKHA5(T857);PLEKHA7(S612);PLEKHA7(S903);PLEKHG3(S76);PLK1(T214);PLPPR3(S353);PML(S505);POLA2(T127);POTEE(S939);POTEF(S939);POTEKP(S239);PPHLN1(S163);PPHLN1(T200);PPME1(S15);PPP1R13L(S358);PPP1R13L(S395);PPP1R14B(S32);PPP1R9B(S100);PPP4R3A(S774);PRAG1(S510);PRKCD(T141);PRR11(S40);PRR36(T1082);PRRC2A(S1147);PRRC2A(S2113);PSMF1(S153);PTDSS2(S16);PXN(S85);RAB12(S21);RAB40C(S268);RALGAPB(T379);RANBP2(S2454);RANBP2(S2900);RANBP2(T1396);RANBP3(S211);RANBP9(S477);RANBP9(S482);RASAL3(S18);RASGRP2(S391);RB1(S249);RB1(S788);RB1(S795);RB1(T356);RB1(T821);RB1(T826);RB1(Y790);RBBP6(S516);RBL1(S749);RBL1(T369);RBL1(T385);RBL2(S413);RBM10(S845);RBM15(S294);RBM17(S169);RBM27(T447);RBM6(S1025);RBMX(S208);RBMXL1(S208);RBMXL1(S88);RECQL5(S815);REPS1(S709);RFX7(S1028);RGPD1(S1463);RGPD2(S1471);RGPD3(S1479);RGPD4(S1479);RGPD5(S1478);RGPD8(S1478);RIF1(S1454);RPRD2(S665);RPRD2(T732);RRM2(T33);RRP15(T104);RRP1B(S735);RSL1D1(S392);RSL1D1(S396);RSL1D1(T465);SACS(S1779);SAMD1(S161);SAMD4B(S172);SAPCD2(S157);SASH3(S21);SCML2(S267);SCRIB(S1348);SCRIB(S1448);SCRIB(S504);SCRIB(S853);SEC16A(S136);SEC16A(S1905);SEC31A(S799);SEPT9(S22);SET(S7);SF3B1(T257);SFSWAP(S909);SH3BP2(S427);SHANK2(S67);SHROOM3(T576);SIK3(T469);SIPA1L1(S1565);SLC4A1AP(S82);SLX4(S1309);SLX4(S1333);SMARCA2(S588);SMNDC1(S201);SMTN(S341);SNRK(S518);SNRNP200(S225);SNRNP70(S226);SNRPC(S17);SNTB2(S393);SNTB2(S95);SNURF(S32);SNX17(S336);SP3(S73);SRRM1(S695);SRRM2(S1499);SRSF1(S199);SRSF1(S201);SRSF9(S216);STAM(S156);STIM2(S523);STK10(S450);STK17A(S28);STMN1(S38);SURF6(S138);SVIL(S968);SYNJ1(S1053);SYTL2(S344);TACC3(S25);TACC3(S250);TACC3(S317);TAF6(S634);TAF6(S636);TAF7(S201);TAOK1(S421);TAOK1(S965);TBC1D1(S211);TBC1D2B(S155);TBC1D9B(S435);TBX2(S653);TCF20(S966);TCOF1(S1227);TCOF1(S1257);TCOF1(S156);TELO2(S836);TEX2(S732);THAP4(S128);THRAP3(S248);TICRR(T1260);TJP1(S617);TJP2(S266);TK1(S231);TLN1(S425);TMPO(S306);TMPO(S354);TMX1(S270);TNIK(S764);TNIK(S766);TNKS1BP1(S1103);TNS1(T1173);TOM1(S464);TOM1L1(S323);TOR1AIP1(S135);TPD52L2(S166);TPX2(T369);TRIM24(S654);TRIP12(S312);TRPM7(S1477);TRPS1(S216);TRPS1(T751);U2SURP(S37);ULK1(S477);UNC93B1(S547);UNC93B1(S550);UNG(T60);UPF3B(T169);USP10(S211);USP15(S242);USP20(S134);USP36(S546);USP36(S742);USP36(T653);USP7(S18);VCL(S290);VGLL4(S149);VPS13D(S1042);WBP11(S237);WDFY4(S3123);WIPF1(S340);WIZ(S1012);WT1(S273);XRCC1(S226);XRCC1(S229);XRCC1(T198);XRCC1(Y211);XRCC6(S477);YAP1(S289);YBX3(T67);YTHDC2(S1223);ZC3H11A(S132);ZC3HAV1(S378);ZCCHC8(S598);ZCCHC8(T479);ZCCHC8(T485);ZDHHC5(S425);ZDHHC5(S621);ZFP64(S547);ZFP91(S101);ZFP91(S103);ZFYVE26(S1764);ZMYND8(S547);ZNF24(S274);ZNF318(S1896);ZNF318(S501);ZNF639(S88);ZYX(S308)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>JAK3</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>2</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>HSPB1(S82);TMX1(S270)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>KIT</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>247</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>ABI1(S231);ABLIM1(S655);ABLIM1(S706);ACIN1(S729);AHCTF1(S528);ANKS1A(S663);AP1M1(T154);APC(T1773);ARHGAP15(S43);ARHGAP17(S162);ARHGAP21(S1862);ARHGAP21(S856);ARHGEF11(S255);ARID1A(S604);ARL6IP4(S239);ASCC3(S2195);ATAD5(S306);ATF7(S434);ATF7IP(S474);ATF7IP(S477);ATG9A(S828);ATP1A1(S16);ATXN2L(S32);BCOR(S488);BRAF(S365);BUB1B(S543);C17orf47(S195);CAAP1(S312);CAMKV(T435);CAMSAP1(S793);CCDC14(S798);CCDC86(S160);CCDC86(Y164);CCNL2(S330);CCNL2(S369);CD2AP(S510);CDCA8(S219);CDK11A(S577);CDK11B(S589);CDK12(S32);CEP76(S83);CHAF1A(S206);CHD8(S2008);CLNS1A(S195);CNOT2(S101);CPSF4(S202);CRAMP1(S1268);CREB1(S143);CRKL(Y207);CRTC2(S613);CRTC3(S329);DCLRE1C(S518);DDX41(S21);DDX54(S782);EDC4(S729);EEF1G(T46);EIF4ENIF1(S752);EIF4G3(S232);EML4(S146);EP300(S1038);EPB41(S560);EPS15(S563);EPS15(S796);ETV6(S203);EVPL(S2025);EXO1(S623);FAF1(S582);FAM120A(Y452);FAM193B(S785);FARSA(S301);FERMT3(S8);FLNA(S2158);FOXK1(S223);FRYL(T1959);GLCCI1(S30);GPATCH8(S738);GRAMD1B(S274);GTF2F1(T389);GTF3C1(S1865);GTF3C2(S765);HDAC1(S421);HDAC1(S423);HDAC2(S422);HDAC2(S424);HSP90AA1(S263);HSP90AB1(S226);HSP90AB3P(S205);HTATSF1(S642);HUWE1(T2889);IGLL1(S58);IKBKB(S672);INCENP(S481);INPPL1(S151);ITSN1(S315);IWS1(S720);JADE1(S703);KANSL1(S829);KANSL1(S839);KIF23(S902);KLF3(S92);KTN1(S75);LIG1(S76);LIG1(T195);LYST(S2627);MACF1(S7330);MARCKS(S167);MCM3AP(S527);MED1(S664);MED13(S890);MNAT1(S279);MON1B(S59);MON1B(S61);MPHOSPH8(T89);MPRIP(S289);MPRIP(S292);MSH6(S41);MTA1(S576);MTMR3(S647);MYH9(S1943);MYO9B(S1267);MYO9B(T1271);NAA30(S39);NIPBL(S280);NMNAT1(S117);NOC2L(S49);NOL8(S432);NOP58(S502);NSRP1(S33);NSUN2(S456);NUP210(S1877);PCBP1(S173);PCIF1(S144);PCYT1A(S343);PDE7A(S113);PDE7B(S74);PHC3(T609);PHIP(S1315);PHKA2(S729);PKN1(S562);PKP4(S337);PKP4(S406);PML(S518);PNPO(S241);PPFIBP2(S387);PPM1H(S124);PPP1R12A(S903);PRKD2(S214);PROSER1(S613);PROSER2(S179);PRPF38B(S5);PSD4(S118);PSIP1(S177);PSRC1(S98);RAD18(S322);RANBP2(S2510);RASAL2(S16);RBM10(S797);RBM14(S256);RBM15(S670);RCOR1(S260);RCSD1(S116);RCSD1(S120);RFX7(S424);RGPD1(S1519);RGPD2(S1527);RGPD3(S1535);RGPD4(S1535);RGPD5(S1534);RGPD8(S1534);RPRD2(S374);RREB1(S42);RTF1(S697);SACS(S1779);SCAF11(S798);SCYL3(T153);SEC24B(T329);SEC62(T375);SERPING1(S198);SF3A1(S359);SH3GL1(S288);SHC3(S474);SHCBP1(S42);SHROOM3(S816);SIPA1L1(S1585);SLC43A1(T256);SLC4A7(S556);SLC9A1(S703);SLX4(S1044);SMARCC2(S347);SMG8(T743);SMG8(Y746);SNIP1(S35);SNTB1(S389);SNX17(S333);SRRM1(S391);SRRM2(S1144);SRRM2(S1320);SRRM2(S1329);SRRM2(S1404);SRRM2(S322);SRRM2(T318);SRRM2(Y1145);STAT5A(S193);STAU1(S390);STK10(S392);STK33(S470);STK4(S414);SYMPK(S1243);SYT6(S187);SYT6(Y190);TACC3(S71);TALDO1(S237);TBC1D10B(T697);TBC1D22A(S167);TCF4(S372);TCOF1(T983);TEX2(S266);THRAP3(S232);TJP3(S164);TLE4(S208);TLK2(S99);TNRC6C(S714);TP53BP1(S1618);TP53BP1(S580);TRAFD1(S470);TRAM1(S365);TRAPPC12(S184);TRIO(S1724);TSC22D4(S62);TVP23C(S223);USP1(S67);USP32(S1423);UTP20(T1741);VCPIP1(S747);WDR44(S403);XRN2(S471);XRN2(S499);XRN2(S501);ZC3H11A(S132);ZNF106(S641);ZNF280D(S545);ZNF516(T930);ZNF552(S86);ZNF609(S1055);ZNF814(S87);ZNRF2(S21);ZRANB2(S153)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>LATS1</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>199</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>ACIN1(S825);ACLY(S455);AHNAK(S5830);ALDH1A3(S95);ALKBH5(S361);ANK3(S1459);ANKRD2(S99);ARHGEF12(S1288);ARHGEF16(S107);ARHGEF17(S420);ARHGEF6(S684);ARPP19(S104);ASAP2(S822);AUTS2(S941);BAD(S99);BAG6(S113);BAIAP2(S261);BAIAP2(S366);BCL9(S917);BCL9L(S750);BTF3(S30);C2CD5(S260);CAD(S1406);CAD(S1859);CAMSAP1(S629);CARHSP1(S52);CDC25B(S323);CDC42EP1(S192);CDC5L(T396);CDK12(T893);CDK17(S180);CDK18(S132);CDK18(S14);CENPF(S3150);CEP170B(S421);CFL1(S3);CLASP1(S636);COBLL1(S394);CPA6(S60);CRIP2(S115);CSNK1D(S382);DAPK3(S312);DDX17(S571);DENND4C(S989);DENND5B(S1076);DIP2B(S100);ECD(S205);EHBP1L1(S310);EIF2B1(S105);EIF2B1(S107);EML3(S176);EPB41L1(S510);EPX(S670);EPX(S672);ERBIN(S1168);ESS2(T386);FAM102B(S228);FAM117A(S145);FAM117B(S273);GAB2(S210);GOLGA4(S71);GPN1(S338);GPSM2(S565);GSK3A(S21);GTF2I(S412);GTF3C2(S167);HDAC1(S421);HDAC1(S423);HDGFL2(S454);HMGCR(S872);HSPB1(S82);ID2(S5);ID2B(S5);IRS2(S577);ITPR3(S1832);ITSN1(S978);JPH1(S216);JPT1(S28);KAZN(S387);KHDRBS1(S20);KIDINS220(S1633);KIF21A(S855);KIFC1(S349);KIFC1(S351);KLC2(S610);KRT8(S43);LARP1(S1056);LARP4B(S498);LASP1(S146);LIMD2(S29);LRRTM4(S195);LUZP1(S995);MAP3K2(S153);MAP4K4(S900);MAPRE2(S200);MARCKS(S167);MARCKS(S170);MARCKSL1(S104);MEPCE(S152);MFSD10(S270);MFSD2B(S491);MPRIP(S993);MRGBP(S195);MTA1(T564);MTFR1L(S103);MTMR12(S564);MTSS1L(S601);MYL12A(S19);MYL12B(S20);MYL9(S20);NASP(S705);NAV1(S528);NEK6(S206);NFATC1(S245);NFATC2(S326);NPY1R(S368);NUP214(S678);NUP214(T670);OSBPL5(S12);PALLD(S893);PDAP1(S176);PDYN(S101);PGM5(S510);PHACTR1(S505);PHACTR4(S590);PHACTR4(S628);PHC3(S823);PHIP(S1315);PI4K2A(S462);PI4KB(S511);PIK3CD(T226);PITPNM1(T665);POLH(S379);PPHLN1(Y162);PPP1R12A(S445);PRAM1(S473);PRMT9(S81);PRRC2A(S1386);PXN(Y88);RASAL3(S865);RBM14(S618);RIF1(S1542);RPL15(S34);RPL24(S149);RPL34(S12);RPS6(S235);RPS6KB1(S427);RPS6KB1(S441);RREB1(S1238);RRP9(S293);SCAMP3(S32);SEC22B(S137);SERBP1(S203);SF3A1(S329);SFPQ(S33);SH3BP1(S612);SH3BP1(S613);SH3BP2(S278);SH3KBP1(S410);SH3PXD2B(S291);SLAIN2(S391);SLTM(S1014);SLTM(S551);SLTM(S553);SNRNP200(S225);SRRM2(S771);SSH3(S37);STAT5A(S780);STIM2(S680);STK4(S414);SUGP2(S315);SYNRG(S1075);TBC1D15(S70);TMCC2(S438);TMCC3(S216);TMEM163(S12);TMEM201(S441);TMX1(S270);TNKS1BP1(S429);TP53BP2(S698);TPR(T2116);TRA2A(T202);TRIM33(S1119);TRPV3(S372);UBE2O(S515);ULK1(S556);VIPAS39(S121);VRTN(S432);WDR20(S434);YAP1(T110);YBX1(S209);YRDC(S37);ZC3H11A(S758);ZC3H14(S343);ZC3H3(S569);ZC3H3(S571);ZNF185(S64);ZNF687(S1118);ZNRF1(S123)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>LATS2</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>3</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>EIF4EBP2(T37);EIF4EBP2(T41);EIF4EBP2(Y34)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>LIMK1.2</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>169</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>AFDN(T1330);AFF4(S1043);AKIRIN2(S21);AKT1S1(T246);ALDH5A1(S121);ANKHD1(S1679);ANKRD17(S2401);ANKRD2(S99);ANLN(S182);ANLN(T194);AP1M1(T154);ARHGAP17(S162);ARHGEF11(S255);ARID1A(S772);ASCC3(S2195);ASIC3(S37);ASIC3(S39);ATF7(S434);ATF7IP(S474);ATF7IP(S477);ATXN2L(S32);AUTS2(S941);BAIAP2L1(S261);BCL9L(S750);BICRAL(S675);CAMKV(T435);CAMSAP1(S793);CAMSAP3(S814);CANX(S554);CDC6(S106);CDK18(S117);CFL1(S3);CHAF1A(S206);CRAMP1(S1268);CRTC3(S62);CSNK1D(S331);DCLRE1C(S518);DDX17(S571);DIP2B(S100);DUSP27(S965);EEF2K(S72);EEF2K(S74);EEF2K(Y69);EIF2B1(S105);EIF2B1(S107);EIF3A(S1188);EIF4ENIF1(S752);EPX(S670);EPX(S672);ETV6(S203);EVPL(S2025);FAM120A(Y452);FAM189A1(S18);FAM193B(S785);FAM47A(S258);FBXL15(S262);FOXK1(S223);GLCCI1(S30);GRAMD1B(S274);GSK3B(S25);GSK3B(S9);GTF2F1(T389);HDAC1(S421);HDAC1(S423);HDAC2(S422);HDAC2(S424);HIPK1(T351);HIPK2(T360);HNRNPK(S284);HUWE1(T2889);IKBKB(S672);IRF2BPL(S215);ITSN1(S315);JUN(S63);KAZN(S387);KIFC1(S26);KIFC1(S349);KIFC1(S351);LINC00322(S226);LINC00322(S228);LRRTM4(S195);MAP3K11(S524);MARCKS(S167);MCRIP2(S82);MED13(S890);MFSD10(S270);MNAT1(S279);MON1B(S59);MON1B(S61);MPHOSPH8(S403);MTA1(S576);MTSS1L(S300);MYC(S62);MYCN(S62);MYO9B(S1405);NAA30(S39);NCOR2(S215);NECTIN1(T391);NSRP1(S33);NSUN2(S456);NSUN2(S473);PAK4(T207);PALD1(S406);PARD3(S174);PAWR(S259);PDS5B(S1358);PHACTR1(S505);PKN1(S562);PKP4(S337);PKP4(S406);POLH(S379);PPP1R12A(S903);PPP1R13L(S102);PRAG1(S889);PTPN22(S692);PXN(S258);PXN(Y118);RAB3IP(S157);RBL2(S662);RBM10(S797);RCSD1(S116);RCSD1(S120);RFX7(S225);RFX7(S424);RIOK1(S22);RPS6(S235);RREB1(S42);SAMD4B(S628);SH3BP1(S612);SH3BP1(S613);SH3BP2(S278);SHC3(S474);SHROOM3(S816);SIRT1(S27);SKIV2L(S131);SKIV2L(S133);SLC4A7(S556);SNIP1(S35);SRRM2(S1404);SRRM2(S322);SRSF7(S165);SRSF7(S167);STK33(S470);TBKBP1(S365);TEX2(S266);TNS1(S1269);TRAFD1(S470);TRAPPC12(S184);TRIM37(S771);TRIM37(S773);TRIO(S1724);TRPV3(S372);TVP23C(S223);USP1(S67);USP32(S1423);VRTN(S432);WDR20(S434);XPR1(S666);XPR1(S668);ZC3H3(S569);ZC3H3(S571);ZNF106(S641);ZNF516(T930);ZNF552(S86);ZNF609(S1055);ZNF75A(S286);ZNF75D(S490);ZNF814(S87);ZSCAN10(S6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>MAP2K1</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>163</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>ABR(T74);AFF2(S790);AGPS(S65);AHNAK(S5110);APC(S1360);ARFIP1(S132);ARHGAP25(S362);ARID3A(S362);ASIC3(S39);ATXN2L(S496);AUTS2(S1233);BAG6(S1081);BCAR1(S428);BRWD1(S696);C17orf47(S195);CAD(S1900);CAMSAP1(S1080);CARMIL1(S1094);CC2D1A(T204);CCDC130(S332);CCDC43(Y135);CDCA5(S75);CENPJ(S260);CEP350(S2115);CLASP1(T798);CRMP1(S522);CROCC(S512);CTTN(T401);DENND1A(S523);DIP2B(S100);DIP2B(S53);DPYSL3(S539);EIF5B(S113);EIF5B(S214);EPB41L1(S510);EPB41L3(T469);ERF(S327);ERF(S532);ETV3(S139);ETV3(S159);F11R(S284);FAM83H(S892);FARP2(T22);GAB2(T391);GOLGA5(S116);GTF2I(S412);HID1(S593);HMGXB4(S197);INCENP(S143);INF2(S589);IRS1(S374);IRS2(S1203);JMJD1C(S639);JMJD1C(S641);JMJD1C(S652);KIF21B(S1149);LIMA1(S15);LINC00322(S228);LPIN1(S162);LRRC47(S431);LRWD1(S212);MACF1(S4496);MAP2K2(T394);MAP4(S280);MAPK1(T185);MAPK1(Y187);MAPK3(T202);MAPK3(T207);MAPK3(Y204);MARCKSL1(S93);MARCKSL1(T85);MASTL(S370);MAVS(S222);MCM3(T722);MCM3(Y708);MDC1(S376);MED1(S1156);MED24(S873);MTMR4(S961);MYC(S62);MYC(T58);NFIX(S265);NIPBL(S280);NPM1(S70);OSBPL8(S810);PAK4(T207);PAPOLG(S708);PDCD4(S457);PDLIM7(S217);PHF3(S283);PINX1(T164);PJA1(S265);PKMYT1(S143);PPP1R13L(S187);PPP1R3F(S547);PPP1R9B(S100);PPP4R2(S226);PPP6R1(S759);PPP6R3(S525);PRC1(S4);PREX1(S319);PTPN12(S435);PTPN14(S760);PUM1(S209);QRICH1(S345);RABEP1(S377);RAP1GAP(S484);RB1(S612);RB1(Y606);RFTN1(S199);RIF1(S1454);RNF214(S501);RPL17(S142);RPL28(S115);RPS6KA1(S363);RPS6KA1(T733);RUNX1(S21);SASH1(S90);SEC22B(S137);SHANK2(S877);SIPA1L1(S1549);SIRT1(S172);SKIV2L(S133);SLC9A1(S703);SNTB1(S87);SRRM1(S429);SRRM2(S1083);SRRM2(S1539);SRRM2(S1925);SRRM2(T1927);SRRM2(T2289);SRSF11(S207);STXBP5(S759);TBC1D4(S588);TCF3(S379);TCOF1(S583);TIPIN(T224);TJP3(S368);TJP3(S371);TLK1(T38);TNS3(S363);TNS3(S776);TP53BP1(S366);TPR(S2155);TRIM37(S773);TRMT44(S78);UBAP1(S146);UBE2O(S515);VCL(S290);VCPIP1(S747);VPS8(S1338);VWA7(S461);WASHC2A(S288);WASHC2C(S288);WIPF2(S267);WRNIP1(S65);WRNIP1(S75);ZC3H13(T364);ZC3H14(S343);ZDHHC5(S621);ZFP36L1(S334);ZFP36L2(S490);ZNF106(S641)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>MAP2K2</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>11</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>AHNAK(S5110);ARFIP1(S132);DENND1A(S523);EPB41L1(S510);ERF(S327);F11R(S284);LPIN1(S162);PAK4(T207);PAPOLG(S708);PREX1(S319);SLC9A1(S703)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>MAP2K4</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>2</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>DENND4A(S1256);SAMD4B(S628)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>MAP3K1</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>958</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(S30);09/09/18 00:00:00(T142);ABCF1(S228);ABI1(S216);ABI1(T215);ABI1(Y213);ABI2(S368);ABL1(S718);ABLIM1(S655);ABLIM1(S706);ACIN1(S388);ADAM17(S791);ADGRL2(S1275);AFDN(S1318);AFDN(T1330);AFF1(T372);AFF1(T376);AFF4(S1043);AFF4(S1062);AFF4(S487);AGAP1(S605);AGAP1(T836);AGAP2(S808);AGO2(S387);AHDC1(S1064);AHNAK(S3412);AHNAK(S3426);AHNAK(S511);AHNAK(S5448);AIF1L(S134);AKAP2(S720);AMBRA1(S1205);AMER1(S246);AMPD2(S100);ANK1(S15);ANKRD17(S1696);ANKRD17(S2045);ANKRD17(S2401);ANKRD26(S23);ANKS1A(S663);ANKS1A(S887);AP1M1(T154);AP3D1(S829);APPL1(S401);ARFGAP2(S368);ARFGAP2(S432);ARFIP1(S132);ARHGAP17(S162);ARHGAP17(S625);ARHGAP17(T682);ARHGAP21(S1862);ARHGAP21(S856);ARHGAP4(S906);ARHGAP4(S930);ARHGEF10(S373);ARHGEF10(S379);ARHGEF11(S255);ARHGEF11(S35);ARHGEF16(S107);ARHGEF2(S122);ARHGEF2(S163);ARID1A(S1184);ARID1A(S604);ARID1A(S772);ARID3A(S119);ARL6IP4(S239);ASAP2(S822);ASCC3(S2195);ATAD2B(S83);ATAD5(S306);ATAT1(S315);ATF7(S434);ATF7IP(S474);ATF7IP(S477);ATG2A(S1263);ATN1(S34);ATP1A1(S16);ATRX(S704);ATXN2L(S32);BAZ1A(T1547);BCLAF1(S559);BCOR(S488);BCR(S463);BICRAL(S674);BICRAL(S675);BRAF(S365);BRCA1(S1497);BRCA1(S1524);BRD4(S1126);BUB1(S655);BUB1B(S543);BUD13(S299);C17orf47(S195);C1orf226(S258);C2CD2(S649);C2CD4C(S273);C2CD5(S662);C9orf40(S69);C9orf78(T100);CAAP1(S312);CALU(S35);CALU(S44);CAMKV(T435);CAMSAP1(S563);CAMSAP1(S793);CAMSAP3(S814);CARD9(S425);CARMIL1(S968);CASK(S589);CASKIN2(S711);CAST(S243);CCDC14(S798);CCDC86(S160);CCDC86(Y164);CCDC88A(S1820);CCDC88A(S237);CCDC9(S80);CCNL2(S369);CCNT2(S601);CCZ1(S76);CCZ1B(S76);CD2AP(S510);CD5L(S292);CDC25B(S323);CDC42BPG(S1482);CDC42EP1(S350);CDC42EP4(S142);CDC6(S106);CDCA7L(S261);CDCA8(S219);CDK11A(S577);CDK11B(S589);CDK12(S32);CDK13(S525);CDK14(S134);CDK17(S180);CDK18(S117);CDK18(S132);CDK18(S14);CDK9(S347);CENPA(T21);CENPC(S73);CENPF(S276);CENPN(S282);CEP170(S881);CEP170(T1533);CEP170P1(T242);CEP55(S428);CEP76(S83);CFDP1(S250);CFL1(S3);CGN(S149);CHAF1A(S206);CHAF1A(S775);CHAMP1(S376);CHAMP1(S507);CHAMP1(S87);CHD1(S1677);CHD1(T1700);CHD8(S2008);CIZ1(S838);CLINT1(T308);CNOT2(S101);CNOT2(S170);COBL(S269);COBL(S815);COL4A3BP(S132);COL4A3BP(S373);CPSF4(S202);CPSF7(S48);CRAMP1(S1268);CREB1(S111);CREB1(S143);CRKL(Y207);CRTC1(S153);CRTC1(S172);CRTC1(T149);CRTC2(S613);CRTC3(S329);CRTC3(S62);CSNK1D(S331);CSTF2(S524);CTAGE1(S616);CTAGE5(S635);CTAGE5(S647);CTPS1(S562);DAB2IP(S747);DBNL(T291);DBP(S161);DCAF12(S15);DCDC2(S270);DCLK1(S330);DCLRE1C(S518);DCP1B(S275);DDX17(S571);DDX3X(S594);DDX41(S21);DDX42(S185);DDX51(S83);DENND5A(S193);DHX57(S77);DHX8(S460);DIP2B(S100);DLG5(S1115);DLG5(S1232);DLG5(S1254);DLG5(T1279);DLGAP5(S725);DNAJC6(S570);DNMT3B(S136);DOCK2(T1797);DOCK5(S1766);DOCK7(S1438);DOCK7(S898);DOCK8(S451);DUSP15(S192);DUSP16(S612);DYNC1H1(S4368);DYNC1LI1(S398);DYNC1LI1(S465);DYNC1LI1(S468);DYNC1LI1(T512);DYRK2(S30);EDC4(S729);EEF1D(T147);EEF1G(T46);EEF2K(S72);EEF2K(S74);EEF2K(Y69);EEPD1(S21);EFHD2(S74);EHMT2(S232);EIF2B4(S130);EIF3A(S1188);EIF3A(S882);EIF3F(S258);EIF4B(S406);EIF4EBP1(S65);EIF4EBP1(S83);EIF4EBP1(T82);EIF4ENIF1(S752);EIF4G1(S1077);EIF4G1(S1092);EIF4G3(S232);EML4(S146);ENAH(S531);EP400(S722);EPB41(S560);EPN3(S264);EPS15(S563);EPS15(S796);EPS15L1(S793);ERF(S327);ERRFI1(S461);ETV6(S203);EVPL(S2025);EXO1(S623);FAM120A(Y452);FAM129B(S696);FAM169A(S635);FAM169A(S637);FAM189A2(S275);FAM193A(S393);FAM193B(S785);FAM193B(S9);FAM207A(T34);FAM234B(S62);FAM53C(S122);FAM76B(S193);FAM83H(S1025);FAM83H(S647);FGD1(S116);FGD6(S692);FLNA(S2158);FNBP1(S359);FOXK1(S223);FOXK2(S373);FOXK2(S61);FRYL(T1959);FYB1(S46);FZR1(S163);GAB2(S141);GAPDH(S151);GAPVD1(S902);GATA3(S115);GATAD2B(S486);GIGYF2(S139);GIGYF2(S236);GLCCI1(S30);GNL3(S529);GON4L(S1896);GPATCH2(S195);GPATCH8(S738);GPRIN1(S229);GRAMD1B(S274);GSE1(S826);GSE1(S828);GSK3B(S25);GSK3B(S9);GTF2F1(T389);GTF3C1(S1865);GTF3C2(S167);GTF3C2(S765);GTF3C2(S901);GTPBP4(S558);H2AFY(T129);HCFC1(S666);HDGFL3(S121);HDGFL3(S122);HEATR1(S1190);HECTD1(S1567);HELLS(S503);HIPK1(T351);HIPK2(T360);HIVEP2(S433);HMCN2(S2897);HMGA1(S36);HMGCS1(S516);HNRNPA1(S338);HNRNPA2B1(S344);HNRNPD(S82);HNRNPLL(S61);HNRNPM(S528);HNRNPM(S618);HNRNPUL1(S718);HOXC9(S159);HSP90AA1(S263);HSP90AB1(S226);HSP90AB3P(S205);HSPB1(S82);HSPH1(T815);HTATSF1(S409);HTATSF1(S481);HTATSF1(S642);HUWE1(S1084);HUWE1(T2889);ICE1(S255);IFI16(S153);IKBKB(S672);IL17RA(S708);INCENP(S481);INPP5F(S907);INPP5J(S278);INTS12(S128);IQSEC1(S180);IRF2BP1(S436);IRF2BP1(S453);IRF2BP2(S318);IRF2BPL(S215);IRS2(S308);ISCU(S20);ITSN1(S315);IWS1(S235);IWS1(S237);JAZF1(T109);JAZF1(T113);JMJD1C(S2053);JMJD1C(T1187);JPH4(S157);JUN(S63);KANSL1(S829);KANSL1(S839);KIAA0319L(S978);KIAA1522(S971);KIAA1551(S1358);KIAA1671(S1499);KIDINS220(S1633);KIF1A(S1548);KIF21A(S1239);KIF23(S902);KIFC1(S26);KLC2(S445);KMT2D(S3130);KTN1(S75);LAD1(S301);LAD1(S356);LARP1(S546);LCOR(S42);LDB1(S265);LIG1(S76);LIG1(T195);LIMA1(S617);LIMK1(S298);LIMK1(S310);LMNB2(S37);LRCH3(S324);LRCH4(S520);LRRC17(S28);LSM14A(S178);LSM14A(S183);LYST(S2627);MACF1(S7330);MAGED2(S265);MAP1A(S1675);MAP1B(S1252);MAP3K11(S507);MAP3K11(S524);MAP3K21(S514);MAP3K9(S519);MAP4(S1000);MAP4(S358);MAP4(S636);MAP4(T354);MAP4K2(S328);MAP7(S209);MAP7D1(S460);MAP7D3(T186);MAP9(S79);MARCKS(S167);MARK1(S588);MARK3(S583);MARK3(S585);MAST2(S1256);MAST2(S876);MASTL(S320);MATK(S501);MAVS(S258);MAZ(S302);MAZ(S361);MCM3AP(S527);MCRIP2(S82);MED1(S1223);MED13(S890);MEPCE(S152);MEPCE(S217);MEPCE(T213);MEX3B(S4);MGA(S2924);MGMT(S201);MIA2(S1243);MIA2(S1255);MICALL1(S486);MICALL2(S249);MINK1(S733);MKI67(S579);MKI67(T401);MNAT1(S279);MON1B(S59);MON1B(S61);MORC2(S730);MOV10(S969);MPHOSPH8(S403);MPHOSPH8(T89);MPRIP(S289);MPRIP(S292);MSH6(S309);MTA1(S386);MTA1(S576);MTA1(S639);MTBP(S755);MTMR3(S647);MTX3(S284);MYB(S599);MYC(S281);MYC(S62);MYC(T58);MYCBP2(S2315);MYCN(S62);MYH9(S1943);MYO18A(S102);MYO9B(S717);NAA30(S39);NADK(S48);NADK(S64);NAP1L4(T51);NAV1(S1265);NAV1(S528);NAV1(S672);NAV1(S695);NAV1(S808);NCKIPSD(T181);NCOA3(S857);NCOR1(S1472);NCOR2(S2016);NDRG2(S332);NDRG3(S331);NDRG3(S334);NECTIN1(T391);NEDD4L(S448);NEDD4L(S487);NEO1(S1214);NES(S320);NFATC2IP(S204);NFIX(S301);NMNAT1(S117);NOC2L(S49);NOL8(S432);NOLC1(S397);NOLC1(S508);NOLC1(S622);NOLC1(S623);NOMO2(S1205);NOMO3(S1205);NOP2(S67);NOP58(S502);NSD1(S2471);NSFL1C(S140);NSFL1C(S272);NSMCE3(S64);NSRP1(S33);NSUN2(S456);NSUN2(S473);NUCKS1(S19);NUCKS1(S61);NUFIP2(S230);NUMA1(S169);NUMA1(S1862);NUMA1(T2000);NUP155(S992);NUP210(S1848);NUP210(S1852);NUP210(S1874);NUP210(S1881);NUP214(S1045);NUP35(S66);NUP50(S221);OBSL1(T1669);OSBPL11(S181);OSBPL8(S68);OTUD4(S416);PABPN1(S150);PAK1(S137);PAK2(T143);PAK4(S181);PAK4(T207);PALD1(S406);PARD3(S174);PARVA(S14);PATL1(S184);PATL1(T194);PAXX(S148);PCBP1(S173);PCBP1(S190);PCDH1(S949);PCDH18(T442);PCDH7(S1011);PCIF1(S144);PCM1(S804);PCM1(T79);PCM1(T82);PCNP(T139);PCYT1A(S329);PCYT1A(S343);PDAP1(S176);PDCD6IP(S730);PDE3B(S495);PDHA1(S232);PDHA1(S293);PDHA1(S300);PDHA2(S291);PDHA2(S298);PDLIM2(S129);PDLIM5(S360);PDS5B(S1358);PDZD8(S521);PFKL(S775);PFKP(S386);PHACTR1(S505);PHACTR2(S235);PHC3(S315);PHC3(T609);PHIP(S1315);PHIP(S676);PHKA2(S729);PHLDB2(T404);PHRF1(S867);PIK3AP1(Y570);PKN1(S562);PKP2(S293);PKP4(S337);PKP4(S406);PLCG1(S815);PLEKHA2(S349);PLEKHA6(S808);PLK1(T214);PLPPR3(S353);PLPPR3(S508);PML(S518);PML(S527);PNN(S66);PNPO(S241);PPFIA1(S666);PPFIBP2(S387);PPM1H(S124);PPM1H(S221);PPP1R12A(S903);PPP1R12B(S694);PPP1R13L(S102);PPP1R13L(S187);PPP1R13L(S358);PPP1R18(S125);PPP1R9B(S100);PPP2R5D(S89);PPP2R5D(S90);PRAG1(S745);PRAG1(S889);PRAG1(S907);PRAM1(S204);PRKAA1(S356);PRKAR2A(S99);PRKCD(S304);PRKD2(S214);PRKDC(T1045);PROSER1(S613);PROSER2(S179);PRPF38B(S268);PRPF38B(S5);PRPF40B(S764);PRRC2C(T2673);PSMD1(T270);PSMF1(S153);PTK2(S722);PTK2(S910);PTPN12(S449);PTPN13(S1033);PTPN13(S214);PTPN13(S908);PTPN13(S938);PTPN22(S449);PTPN22(S692);PTPN7(S44);PUM1(S209);PXN(S106);PXN(S258);PXN(Y118);R3HDM2(S349);RAB12(S21);RAB31(S35);RABGEF1(S302);RAD18(S99);RAI1(S1358);RALBP1(S34);RALGAPA1(T754);RALGPS2(S296);RANBP2(S1128);RANBP2(S1835);RANBP2(S2510);RANBP2(S955);RAP1GAP2(S45);RAPGEF6(S1094);RAPH1(S539);RARG(S43);RASAL2(S16);RASAL2(S758);RASAL3(S18);RB1(S612);RB1(T356);RB1(T821);RBL1(S640);RBL1(S749);RBL1(S988);RBL1(T369);RBM10(S797);RBM10(S845);RBM14(S256);RBM15(S259);RBM17(S169);RBM20(S644);RBM27(S120);RBM39(Y95);RBMX(S249);RBMX(S332);RBMXL1(S249);RCOR1(S260);RCSD1(S116);RCSD1(S120);RECQL5(S815);RFX7(S1028);RFX7(S225);RFX7(S424);RGPD1(S1519);RGPD2(S1527);RGPD3(S1535);RGPD4(S1535);RGPD5(S1534);RGPD5(T19);RGPD8(S1534);RGPD8(T19);RIF1(S1008);RIF1(S1554);RIF1(S1688);RIOK1(S22);RIPK2(S363);RNF2(S168);ROBO2(T1154);ROR2(S449);RPA1(T180);RPRD2(S374);RPRD2(T723);RPS6KB1(S441);RPS6KB2(S423);RREB1(S42);RRM2(T33);RRP1B(S245);RSF1(S473);RUBCN(S388);RYBP(S127);SAFB(S443);SAFB2(S444);SAP130(S442);SASH1(S407);SBNO1(T819);SCAF11(S796);SCARF2(S651);SCARF2(S653);SCML2(S267);SCRIB(S1348);SCRIB(S1445);SCRIB(S1508);SCYL3(T153);SEC16A(S136);SEC24B(T329);SEC62(T375);SERPING1(S198);SF3A1(S359);SF3B1(T207);SF3B1(T211);SF3B1(T313);SF3B1(T350);SF3B2(T780);SH2B3(S150);SH2D3A(S147);SH3BP2(S427);SH3BP4(S279);SH3GL1(S288);SH3KBP1(S230);SHANK1(T946);SHANK2(S67);SHANK2(S96);SHC3(S474);SHCBP1(S42);SHROOM2(S193);SHROOM3(S242);SHROOM3(S664);SHROOM3(S816);SIK3(S866);SIRT1(S27);SLAIN2(S345);SLAIN2(S391);SLBP(S111);SLC12A4(T926);SLC12A6(T991);SLC12A7(T926);SLC12A7(T980);SLC13A4(T244);SLC20A2(S256);SLC20A2(S259);SLC43A1(T256);SLC4A7(S556);SLC4A7(T559);SLC9A1(S703);SLC9A3R1(S280);SMAD1(S463);SMAD1(S465);SMAD9(S465);SMAD9(S467);SMAP(S93);SMAP2(S231);SMARCC2(S304);SMARCC2(S347);SMC3(S1085);SMG8(T743);SMG8(Y746);SNIP1(S35);SNRPA1(S178);SNRPA1(T180);SNTB1(S87);SOX13(S386);SOX2(S250);SP110(S244);SPAM1(S78);SPEG(S2109);SPIN1(S39);SPN(T341);SPTAN1(S1217);SPTBN2(S2384);SRRM1(S597);SRRM1(S694);SRRM1(T872);SRRM2(S1144);SRRM2(S1404);SRRM2(S1691);SRRM2(S1694);SRRM2(S1925);SRRM2(S2115);SRRM2(S2123);SRRM2(S2272);SRRM2(S2581);SRRM2(S322);SRRM2(T1492);SRRM2(T1927);SRRM2(T2289);SRRM2(T2316);SRRM2(T318);SRRM2(Y1145);SRSF2(S191);SRSF2(S26);SRSF4(S448);SRSF4(S450);SRSF9(S211);SRSF9(S216);SSBP3(S347);STAT5A(S193);STAU1(S390);STIM1(S618);STIM2(S523);STK11IP(S761);STK17A(S28);STK33(S470);STMN1(S38);SUCO(S1081);SUGP2(T281);SUPT6H(T1523);SVIL(S968);SYMPK(S1243);SYNRG(S1075);SYT6(S187);SYT6(Y190);TACC3(S25);TACC3(S250);TACC3(S71);TBC1D1(S211);TBC1D10B(T148);TBC1D13(S184);TBC1D14(S295);TBC1D22A(S167);TBC1D9B(S435);TBKBP1(S365);TCF4(S372);TCF4(S92);TCOF1(S1227);TCOF1(S503);TCOF1(T914);TERF2IP(S154);TEX10(T29);TEX2(S266);THRAP3(S248);THRAP3(S575);THRAP3(S939);THYN1(S14);TJAP1(S320);TJAP1(T318);TJAP1(Y316);TJP1(S168);TJP1(S899);TJP1(S968);TJP3(S164);TK1(S231);TLE4(S208);TMEM131(S1604);TMX1(S270);TNK2(T829);TNK2(Y827);TNKS1BP1(S1297);TNKS1BP1(S178);TNKS1BP1(S836);TNKS1BP1(S872);TNKS1BP1(S983);TNRC18(S1644);TNRC6C(S714);TNS1(S1269);TNS1(T1173);TOM1(S462);TOP2B(S1400);TOPORS(S98);TOR1AIP1(S135);TOR1AIP1(S315);TP53BP1(S1430);TP53BP1(S1618);TP53BP1(S580);TPD52L1(S149);TPD52L2(S166);TPX2(S486);TRAF4(S426);TRAFD1(S470);TRAM1(S365);TRAPPC12(S184);TRIM24(S687);TRIO(S1724);TRIP12(S997);TRIP12(T941);TRMT2A(S602);TRO(S155);TRUB1(T27);TSC1(S505);TSC22D4(S62);TTN(S1406);TVP23C(S223);TXLNG(S105);UBA1(S13);UCK1(S253);UFD1(S299);UNC13B(S367);UPF1(S1127);UPF3B(T169);USP1(S67);USP15(S225);USP32(S1423);USP36(S611);USP36(S682);USP36(T653);UTP20(T1741);UTP3(S365);UTP3(S368);VCPIP1(S747);VCPIP1(S768);VGLL4(S149);WAC(S470);WAC(T462);WASHC2A(S522);WASL(Y256);WDFY4(S3123);WDR20(S434);WDR3(T247);WDR44(S403);WDR44(S96);WDR48(T343);WDR62(S1144);WEE1(T190);WRNIP1(S153);WTAP(S290);WWTR1(S90);XPC(S347);XRCC6(S477);XRN2(S448);XRN2(S471);YAP1(S367);YBX1(Y162);YBX3(S346);YEATS2(S627);ZBTB37(S164);ZC3H11A(S132);ZCCHC17(S114);ZCCHC8(S598);ZCCHC8(T479);ZCCHC8(T485);ZCCHC8(T496);ZFC3H1(S949);ZFPM1(S786);ZKSCAN8(S12);ZMYM2(S305);ZNF106(S641);ZNF148(S665);ZNF24(S274);ZNF280D(S545);ZNF318(S1971);ZNF513(S85);ZNF516(T930);ZNF518A(S655);ZNF552(S86);ZNF609(S1055);ZNF649(S474);ZNF777(S47);ZNF814(S87);ZNRF2(S21);ZRANB2(S153);ZYX(S267);ZYX(S308)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>MAP3K11</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>68</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(S30);ADD1(S465);AFF4(S1043);AKIRIN2(S21);ALKBH5(S361);ANKHD1(S1679);ANKRD17(S2401);ANKRD2(S99);ANLN(S182);ANLN(T194);ASIC3(S37);AUTS2(S941);BAG3(T285);BAIAP2L1(S261);BCL9L(S750);CDC42SE1(S74);COBLL1(S394);DBNL(T291);DCUN1D5(S9);DENND4C(S1277);DENND4C(S1301);EIF4B(S283);ERCC6L(S820);FAM189A1(S20);FBXL15(S264);FXR2(S566);GTF3C2(S167);HAUS6(T584);HDAC1(S421);HDAC1(S423);HDAC2(S422);HDAC2(S424);HNRNPK(S284);KHDRBS1(S20);KIAA1522(S971);LARP6(S409);LINC00322(S226);LRRTM4(S195);MARK2(S456);MARK3(S469);MTMR1(S43);PLCL2(S17);PLEKHA5(S885);PPHLN1(Y162);PRAG1(S889);PXN(Y118);R3HDM1(S381);RAB3IP(S159);RICTOR(S1284);SAFB2(S787);SAMD4B(S628);SCRIB(S1448);SH3BP1(S612);SH3BP1(S613);SH3BP2(S278);SKIV2L(S131);SLTM(S551);SLTM(S553);SRSF7(S165);TET2(S1107);TRIM37(S771);TRPV3(S372);UBE2O(S515);VANGL1(T47);VRTN(S432);WIPF2(S235);XPR1(S666);ZSCAN10(S8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>MAP3K15</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>39</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(S30);AHCTF1(S528);AKAP11(S422);ANAPC1(S355);ARFGAP2(S432);ARHGEF18(S1111);CDK12(S383);CDK12(S385);CNK3/IPCEF1(S892);CRKL(Y207);DBNL(T291);FUS(S462);FXR2(T411);GPATCH8(S1033);GTF3C2(S167);HPS5(S534);IPCEF1(S430);KHDRBS1(S20);KIF15(T1144);LRMP(S363);NADK(S48);NCAPG(S674);NOB1(S352);OTUD5(S64);PBRM1(S13);PCNP(T139);PEA15(S116);PKP4(S314);RBM15(S622);RBM15B(S265);RBM39(S97);RBM39(Y95);RBMX(S326);RBMXL1(S326);SHANK2(S67);SLTM(S551);SRRM1(S234);UPF3B(T169);ZC3H15(S360)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>MAP3K2</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>19</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>AKIRIN1(S22);C2CD2L(S411);COL4A3BP(S373);FAM109A(S213);FAM53B(S268);FLNC(S2624);JMJD1C(S2053);KNOP1(T310);PCDH18(T442);PLEKHA6(S808);RAPGEF1(S311);RBM17(S169);SF3B1(T434);SRRM1(T718);TBC1D5(S522);TRAFD1(S470);TSC22D4(S62);TWISTNB(S316);XRN2(S471)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>MAP3K3</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>50</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>AGAP2(T809);ARFGAP2(S368);ATL1(S10);BCL9L(S813);C17orf53(S332);CDC42EP4(T23);DLGAP4(S666);DOCK7(S888);EPB41(T710);EPB41L5(S436);FAM102A(S189);FARP2(S389);FEZ1(S298);HECTD1(S1387);HMGN1(S25);INSRR(S72);IRS1(S374);KIF21A(S855);LIMA1(S15);LRRC41(S308);MAP3K2(S153);MAP7D1(S254);MAPRE1(S155);MYO7B(S689);NBN(S432);NCBP1(S22);OSBP(S240);PAK2(T143);PAPOLG(S708);PLEKHA5(S471);PXN(Y88);RAP1GAP2(S564);RBM15(S292);RBMX(S326);SEPT9(S30);SF3B1(T261);SIK3(S866);SPP2(S182);SRSF4(S113);SRSF5(S117);SRSF6(S119);SRSF9(S189);TBC1D10B(S687);TBX2(S657);TNS2(S1003);TNS3(S363);TRIM33(S1119);VASN(S284);VIPAS39(S121);ZMYND8(S425)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>MAP4K4</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1073</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(S30);AAK1(S14);ABI1(S216);ABI1(T215);ABI1(Y213);ABI2(S368);ABLIM1(S431);ABLIM1(S655);ABLIM1(S706);ABR(T74);ACIN1(S388);ACIN1(T414);ACTA1(S241);ACTA2(S241);ACTB(S239);ACTBL2(S240);ACTC1(S241);ACTG1(S239);ACTG2(S240);ADAM10(S740);ADAM10(Y741);ADAM17(S791);ADD1(S12);ADD1(S431);ADD1(S726);ADD2(S713);ADD3(S693);ADGRL2(S1275);AFDN(S1318);AFDN(S1721);AFDN(T1330);AFF1(T372);AFF1(T376);AFF4(S1043);AFF4(S1058);AFF4(S32);AGAP1(S605);AGAP2(S808);AGO2(S387);AHCTF1(S528);AHDC1(S1064);AHDC1(S1507);AHNAK(S115);AHNAK(S216);AHNAK(S3412);AHNAK(S3426);AHNAK(S5448);AKAP11(S1580);AKAP11(S422);AKAP11(S448);AKAP13(S2728);AKAP2(S720);AMBRA1(S639);AMPD2(S100);ANAPC1(S355);ANKRD17(S1696);ANKRD17(S2401);ANKS1A(S382);ANKS1A(S663);ANKS1A(S887);ANKZF1(S675);ANP32B(T244);AP1M1(T154);APPL1(S401);ARFGAP2(S368);ARFGAP2(S432);ARHGAP1(S44);ARHGAP1(S51);ARHGAP17(S162);ARHGAP17(S625);ARHGAP17(T682);ARHGAP21(S1862);ARHGAP21(S856);ARHGAP4(S906);ARHGEF11(S150);ARHGEF11(S255);ARHGEF11(S35);ARHGEF16(S107);ARHGEF17(S735);ARHGEF2(S122);ARID1A(S1184);ARID1A(S1604);ARID1A(S604);ARID1A(S730);ARID1A(S772);ARID3A(S119);ARID3B(S381);ARL6IP4(S239);ARL6IP6(S80);ARVCF(S887);ASAP2(S822);ASCC3(S2195);ATAD2(S327);ATAD5(S306);ATAT1(S315);ATF7(S434);ATF7IP(S474);ATF7IP(S477);ATG2B(S1582);ATG2B(S1583);ATG2B(Y1577);ATN1(S661);ATN1(T653);ATP1A1(S16);ATXN2L(S32);BCAM(S600);BCL11A(S328);BCL2L12(S113);BCL2L12(S121);BCL2L12(T117);BCOR(S488);BCR(S459);BICRAL(S675);BIN2(S259);BRAF(S365);BRCA1(S1524);BRD4(S1126);BRIP1(S956);BRSK2(T459);BRSK2(T463);BUB1(S655);BUB1B(S543);C16orf54(S194);C17orf47(S195);C2CD2(S649);C2CD2L(S662);C2CD5(S281);C2CD5(S662);C6orf132(S449);C7orf50(S175);C9orf40(S69);C9orf78(T100);CAAP1(S312);CABLES1(S291);CALU(S35);CALU(S44);CAMKV(T435);CAMSAP1(S563);CAMSAP1(S793);CAMSAP3(S814);CARD9(S425);CARMIL2(S1315);CASKIN2(S711);CAT(S515);CBL(S799);CBX8(S311);CCDC14(S798);CCDC6(S240);CCDC86(S160);CCDC86(Y164);CCDC88A(S1820);CCDC9(S376);CCDC93(S305);CCL13(S44);CCNL2(S369);CD2AP(S510);CD97(S818);CD97(S831);CDC25B(S323);CDC25C(S216);CDC42BPG(S1482);CDC42EP1(S350);CDC6(S106);CDCA7L(S261);CDCA8(S219);CDK11A(S577);CDK11B(S589);CDK12(S32);CDK13(T1056);CDK16(S138);CDK17(S180);CDK18(S117);CDK18(S132);CDK18(S14);CDK9(S347);CDV3(T182);CENPA(T21);CENPF(S276);CEP170(S881);CEP170(T1533);CEP170P1(T242);CEP55(S428);CEP76(S83);CEP97(S308);CFL1(S3);CGN(S149);CHAF1A(S206);CHAMP1(S376);CHAMP1(S432);CHAMP1(S436);CHAMP1(S445);CHAMP1(S452);CHAMP1(S472);CHAMP1(S507);CHD4(S303);CHD8(S1978);CHD8(S2008);CHD8(T1982);CIT(S1322);CLASP1(S636);CLASP2(S325);CLASP2(S360);CLASP2(S529);CLASRP(S547);CLINT1(T308);CLK2(S142);CMTR1(S31);CNK3/IPCEF1(S892);CNOT2(S101);CNOT2(S170);CNP(S170);COL4A3BP(S373);CPSF4(S202);CPSF7(S48);CRAMP1(S1268);CREB1(S111);CREB1(S143);CREB1(S271);CRKL(Y207);CRTC2(S613);CRTC3(S329);CSNK1D(S331);CSPP1(S901);CSTF2(S524);CTAGE1(S616);CTAGE5(S635);CTAGE5(S647);CTPS1(S573);CTU2(S419);CYBA(T147);DAB2IP(S747);DACH1(S727);DAXX(S671);DBF4(S381);DBNL(T291);DCLRE1C(S518);DDX17(S571);DDX21(S89);DDX3Y(S592);DDX41(S21);DENND4A(T1019);DGCR8(S271);DGCR8(S275);DGCR8(Y267);DHX57(S77);DHX8(S460);DIP2B(S100);DIP2B(S259);DLG5(S1000);DLG5(S1115);DLG5(S1232);DLG5(S1254);DLG5(T984);DLGAP5(S725);DNMT3B(S136);DNTTIP2(S434);DNTTIP2(T172);DOCK5(S1766);DOCK7(S898);DOCK7(S946);DOCK8(S451);DTL(S425);DUSP16(S612);DYNC1H1(S4368);DYNC1LI1(S398);EDC4(S729);EEF1D(T147);EEF1G(T46);EEF2K(S72);EEF2K(S74);EEF2K(Y69);EEPD1(S21);EIF3A(S1188);EIF3E(S399);EIF4ENIF1(S752);EIF4G3(S232);EML4(S144);EML4(S146);ENAH(S531);ENAH(T538);EP400(S722);EP400(S736);EPB41(S560);EPB41L1(S784);EPS15(S563);EPS15(S796);EPS15L1(S793);ERCC5(S384);ERF(S327);ERRFI1(S461);ETV6(S203);EVPL(S2025);EXO1(S623);EZH2(S363);EZH2(T367);FADD(S194);FAM117B(S10);FAM120A(Y452);FAM122A(S143);FAM122A(S189);FAM129B(S665);FAM129B(S681);FAM129B(S696);FAM193A(S393);FAM193B(S785);FAM207A(T34);FAM234B(S62);FAM53B(S179);FAM53C(S122);FAM76B(S193);FAM83B(S766);FAM83H(S1025);FAM83H(S647);FAM83H(S914);FANCI(S1121);FARSA(S301);FBRSL1(T1010);FBXW9(S59);FGD1(S116);FGD6(S692);FIP1L1(S259);FLNA(S2158);FOXK1(S223);FOXK1(S416);FOXK1(S420);FOXK1(S441);FOXK2(S373);FOXO1(S329);FRMD3(S416);FRYL(T1959);FUS(S462);FXR2(S601);FXR2(T411);FYB1(S46);GAB2(S141);GAGE13(S33);GAGE2A(S32);GAGE2B(S32);GAGE2D(S32);GAPDH(S151);GAPVD1(S902);GATA3(S115);GATAD2A(T189);GATAD2B(S334);GATAD2B(S486);GBF1(S1061);GBF1(S1298);GFI1(S94);GIGYF2(S26);GIPC1(S232);GJA1(S262);GLCCI1(S30);GNL3(S529);GPATCH2(S195);GPATCH8(S738);GRAMD1B(S274);GRIP1(S847);GSK3B(S25);GSK3B(S9);GTF2F1(S385);GTF2F1(T389);GTF2F1(T446);GTF3C1(S1865);GTF3C2(S132);GTF3C2(S167);GTF3C2(S765);HCFC1(S598);HCFC1(S666);HDAC1(S406);HELB(S1050);HIC2(S348);HIPK1(T351);HIPK2(T360);HMGCS1(S516);HMGCS1(T490);HNRNPA1(S338);HNRNPA2B1(S344);HNRNPA3(S358);HNRNPC(S253);HNRNPLL(S61);HNRNPM(S528);HNRNPM(S618);HOXC9(S159);HPS5(S534);HRNR(S903);HSP90AA1(S263);HSP90AB1(S226);HSP90AB3P(S205);HSPB1(S15);HSPB1(S82);HTATSF1(S642);HUWE1(S1084);HUWE1(T2889);IBTK(S1045);IFI16(S153);IGLL1(S58);IKBKB(S672);INCENP(S481);INCENP(T292);INPP5D(T963);INTS12(S128);IPCEF1(S430);IRF2BP1(S421);IRF2BP2(S175);IRF2BP2(S318);IRF2BP2(S406);IRF2BPL(S215);IRF2BPL(S519);ITGAL(S37);ITSN1(S315);ITSN2(S884);ITSN2(S889);IWS1(S235);IWS1(S237);JADE3(S566);JAZF1(T109);JAZF1(T113);JMJD1C(S1223);JMJD1C(S2053);JMJD1C(S641);JPT1(S131);JPT2(T76);JUN(S63);KANK2(S172);KANK2(S175);KANSL1(S829);KANSL1(S839);KCAB2_HUMAN_Phospho (ST);KCNK2(S366);KIAA0319L(S978);KIAA1217(S357);KIAA1217(S361);KIAA1468(T143);KIAA1522(S858);KIAA1522(S862);KIAA1522(S929);KIAA1522(S971);KIDINS220(S1633);KIF1A(S1094);KIF1A(S1528);KIF1A(S1532);KIF1A(S1548);KIF23(S902);KIFC1(S26);KMT2D(S3130);KNOP1(S119);KPNA4(S60);KRT13(S427);KRT8(S36);KTN1(S75);L1TD1(S557);LAD1(S301);LAMTOR1(S27);LARP1(S1056);LARP1(S90);LARP1(T526);LAT2(S135);LAT2(S86);LEMD3(S187);LIG1(S76);LIG1(T195);LIMA1(S617);LIN28B(S203);LIN54(S310);LMNA(S390);LMNB2(S37);LRCH1(S532);LRCH4(S520);LRRFIP1(S116);LRRFIP2(S324);LSM11(S21);LSM14A(S178);LSM14A(S183);LSR(S464);LSR(T453);LUZP1(S745);LYST(S2627);MACF1(S7330);MAGED2(S265);MAML1(S360);MAP1A(S1675);MAP1A(S1776);MAP2(S1540);MAP2(S1653);MAP2(T1649);MAP3K11(S524);MAP3K21(S514);MAP3K9(S519);MAP4K2(S328);MAP7D1(S460);MAP7D1(S93);MAP9(S79);MARCKS(S163);MARCKS(S167);MARK1(S588);MAST2(S876);MATK(S501);MAZ(S361);MCM3(Y708);MCM3AP(S527);MCM3AP(S557);MCRIP2(S82);MDC1(T378);MED13(S890);MEPCE(S217);MEPCE(T213);MEX3B(S4);MFAP1(S116);MIA2(S1243);MIA2(S1255);MIA3(S1741);MICAL3(S649);MICALL1(S391);MICALL1(S486);MICALL1(S640);MICALL2(S143);MICALL2(S153);MINK1(S733);MIS18BP1(S1042);MKI67(S2223);MLC1(S179);MLLT6(S378);MLLT6(S382);MNAT1(S279);MON1B(S59);MON1B(S61);MORC2(S696);MORC2(S725);MPHOSPH8(S403);MPHOSPH8(T89);MPRIP(S289);MPRIP(S292);MSH6(S309);MTA1(S386);MTA1(S449);MTA1(S522);MTA1(S576);MTA2(S435);MTBP(S755);MTFMT(S23);MTMR3(S613);MTMR3(S647);MTMR4(S961);MTOR(S2454);MTSS1L(S342);MYB(S599);MYBBP1A(S11);MYC(S62);MYC(T58);MYCBP2(S3467);MYCN(S156);MYCN(S62);MYO18A(S102);N4BP3(S211);NAA30(S199);NAA30(S39);NAB1(S403);NAB2(S171);NADK(S48);NADK(S64);NASP(T390);NAV1(S528);NAV1(S672);NAV1(S695);NAV1(S808);NCAPD2(Y1325);NCBP3(S25);NCOR1(S1472);NCOR1(S1980);NCOR1(S1981);NCOR2(S1547);NCOR2(S2424);NCOR2(S54);NDRG2(S332);NDRG3(S331);NDRG3(S334);NECTIN1(T391);NEDD4L(S448);NEDD4L(S487);NES(S768);NFATC2(S217);NFATC2(S814);NFATC2IP(S204);NMNAT1(S117);NOC2L(S49);NOL8(S432);NOLC1(S397);NOLC1(S508);NOLC1(S622);NOLC1(S643);NONO(T450);NOP16(S16);NOP53(S29);NOP58(S351);NOP58(S502);NSD1(S2471);NSMCE3(S64);NSRP1(S33);NSUN2(S456);NSUN2(S473);NUCKS1(T179);NUFIP2(S230);NUMA1(S1862);NUMA1(S1887);NUMA1(S2062);NUMBL(S263);NUP153(S209);NUP210(S1877);NUP210(S1881);NUP35(S66);OBSL1(S10);OSBPL8(S68);PABPN1(S150);PAGR1(S237);PAK1(S137);PAK2(T143);PAK4(S181);PAK4(T207);PALD1(S406);PARD3(S174);PARD3(S221);PARVA(S19);PATL1(S278);PATL1(T194);PBRM1(S12);PBRM1(S13);PBX2(S330);PCBP1(S173);PCBP1(S190);PCBP1(S231);PCDH18(T442);PCDH7(S1011);PCIF1(S144);PCM1(T79);PCM1(T82);PCNP(T139);PCYT1A(S315);PCYT1A(S343);PCYT1A(S347);PCYT1B(S315);PDCD6IP(S730);PDE3B(S495);PDHA1(S232);PDHA1(S293);PDHA1(S300);PDHA2(S291);PDHA2(S298);PDLIM2(S129);PDLIM4(S112);PDS5B(S1358);PDS5B(T1301);PDZD8(S521);PEAK1(S823);PFKL(S775);PFKP(S386);PGRMC1(S181);PHACTR1(S505);PHACTR2(T25);PHC3(T609);PHF3(S1614);PHF8(S880);PHIP(S1315);PHKA2(S1043);PHKA2(S729);PHLDB2(T404);PI4K2A(S51);PIK3AP1(S759);PIK3AP1(Y570);PKN1(S562);PKP2(S293);PKP4(S273);PKP4(S314);PKP4(S337);PKP4(S406);PLCB3(S926);PLEC(S1435);PLEKHA5(T857);PLEKHA6(S808);PLEKHG4B(T727);PLK1(T214);PLPPR3(S353);PML(S505);PML(S518);PML(S527);PNPO(S241);POLA2(T127);POLD2(S15);POLM(S372);POM121(S298);POM121C(S275);POMZP3(S33);POTEE(S939);POTEF(S939);POTEKP(S239);PPFIA1(S666);PPFIBP1(S636);PPFIBP2(S387);PPHLN1(S163);PPHLN1(T200);PPM1H(S124);PPME1(S15);PPP1CC(T311);PPP1R12A(S903);PPP1R13L(S102);PPP1R13L(S358);PPP1R9B(S100);PRAG1(S510);PRAG1(S889);PRAG1(S907);PRKD2(S214);PRKDC(T1045);PROSER1(S613);PROSER2(S179);PRPF38B(S268);PRPF38B(S5);PRPF40B(S764);PRR12(S314);PRR36(T1082);PRRC2A(S1147);PRRC2A(S2113);PRRC2C(T2673);PSMF1(S153);PTDSS2(S16);PTPN13(S214);PTPN13(S908);PTPN22(S692);PXN(S258);PXN(S85);R3HDM2(S349);RALGAPA1(T754);RALGAPB(T379);RALGPS2(S296);RANBP2(S2454);RANBP2(S2510);RANBP2(S2900);RANBP2(S955);RANBP3(S211);RANBP9(S477);RANBP9(S482);RAP1GAP2(S45);RAPGEF6(S1094);RAPH1(S539);RASAL2(S16);RASAL3(S18);RASGRP2(S391);RB1(S788);RB1(T356);RB1(Y790);RBL1(S749);RBM10(S797);RBM10(S845);RBM14(S256);RBM15(S294);RBM17(S169);RBM20(S644);RBM27(S120);RBM39(S97);RBM39(Y95);RBM6(S1025);RBMX(S208);RBMX(S249);RBMXL1(S208);RBMXL1(S249);RBMXL1(S88);RCOR1(S260);RCSD1(S116);RCSD1(S120);RECQL5(S815);REPS1(S709);RFX7(S1028);RFX7(S225);RFX7(S424);RGPD1(S1463);RGPD1(S1519);RGPD2(S1471);RGPD2(S1527);RGPD3(S1479);RGPD3(S1535);RGPD4(S1479);RGPD4(S1535);RGPD5(S1478);RGPD5(S1534);RGPD8(S1478);RGPD8(S1534);RIF1(S1554);RIF1(S1688);RIF1(S2205);RIOK1(S22);RNF2(S168);ROR2(S449);RPL18(S161);RPL18(T158);RPLP1(S101);RPLP1(S104);RPLP2(S102);RPLP2(S105);RPRD2(S374);RPRD2(S665);RPRD2(T723);RPRD2(T732);RPS6KB2(S423);RREB1(S42);RRP1B(S735);RSL1D1(S392);RSL1D1(S396);RYBP(S127);SACS(S1779);SALL2(S806);SAMD1(S161);SAMD4B(S172);SASH1(S407);SASH3(S21);SBNO1(T819);SCML2(S267);SCRIB(S1348);SCRIB(S1448);SCRIB(S1508);SCRIB(S504);SCYL3(T153);SEC16A(S1905);SEC24B(T329);SEC31A(S799);SEC62(T375);SEPT9(S22);SERPING1(S198);SET(S7);SF3A1(S359);SF3B1(S129);SF3B1(T261);SF3B1(T303);SF3B1(T313);SF3B1(T350);SFSWAP(S909);SGO1(S468);SH2B3(S150);SH2D3A(S147);SH3BP2(S427);SH3BP4(S279);SH3GL1(S288);SH3KBP1(S230);SHANK2(S67);SHC3(S474);SHCBP1(S42);SHROOM2(S193);SHROOM3(S664);SHROOM3(S816);SHROOM3(T576);SIK3(T469);SIRT1(S27);SLC20A2(S256);SLC20A2(S259);SLC43A1(T256);SLC4A7(S556);SLC4A7(T559);SLC9A1(S703);SLX4(S1309);SLX4(S1333);SMAD1(S463);SMAD1(S465);SMAD9(S465);SMAD9(S467);SMAP(S93);SMARCA2(S588);SMARCAD1(S146);SMARCC2(S347);SMG8(T743);SMG8(Y746);SMG9(S32);SMNDC1(S201);SNIP1(S35);SNRK(S518);SNRNP200(S225);SNRNP70(S226);SNURF(S32);SNX17(S336);SNX17(S409);SP3(S73);SPECC1(S55);SPEG(S2109);SPTAN1(S1217);SPTBN2(S2384);SRRM1(S695);SRRM2(S1144);SRRM2(S1404);SRRM2(S1499);SRRM2(S2123);SRRM2(S322);SRRM2(S510);SRRM2(T318);SRRM2(Y1145);SRSF1(S199);SRSF1(S201);SRSF4(S450);SRSF9(S216);SSB(S366);SSBP3(S347);STAM(S156);STAT5A(S193);STAU1(S390);STIM1(S618);STIM2(S523);STK10(S450);STK17A(S28);STK33(S470);STMN1(S38);SUPT6H(T1523);SURF6(S138);SVIL(S968);SYMPK(S1243);SYNJ1(S1053);SYNRG(S1075);SYT6(S187);SYT6(Y190);SYTL2(S344);TACC3(S250);TACC3(S317);TAF6(S634);TAF6(S636);TAF7(S201);TAOK1(S965);TBC1D1(S211);TBC1D22A(S167);TBC1D9B(S435);TBKBP1(S365);TBX2(S653);TCF20(S574);TCF4(S372);TCOF1(S1227);TCOF1(S503);TCOF1(T914);TERF2IP(S154);TEX2(S266);TEX2(S732);THAP4(S128);THOC5(S314);THRAP3(S248);THRAP3(S575);THRAP3(S928);TICRR(T1260);TIMELESS(S1087);TJAP1(S320);TJAP1(T318);TJAP1(Y316);TJP1(S168);TJP1(S617);TJP1(S968);TJP2(S266);TJP3(S164);TK1(S231);TLE3(S267);TLE4(S208);TLN1(S425);TMPO(S306);TMPO(S354);TMX1(S270);TNIK(S764);TNIK(S766);TNK2(T829);TNK2(Y827);TNKS1BP1(S1103);TNKS1BP1(S872);TNKS1BP1(S983);TNRC6C(S714);TNS1(S1269);TNS1(T1173);TOM1(S464);TOP2B(S1400);TOR1AIP1(S135);TP53BP1(S580);TP53BP2(S558);TPD52L1(S149);TPD52L2(S166);TPR(S379);TRA2A(T202);TRA2B(T201);TRA2B(T212);TRAF4(S426);TRAFD1(S470);TRAM1(S365);TRAPPC12(S184);TRIM24(S654);TRIM71(S187);TRIO(S1724);TRIP12(S312);TRMT2A(S602);TRPM7(S1477);TRPS1(S216);TRPS1(T751);TRUB1(T27);TSC1(S505);TSC22D4(S62);TTN(S1406);TUBA1A(S48);TUBA1B(S48);TUBA1C(S48);TUBA3C(S48);TUBA3E(S48);TVP23C(S223);TXLNG(S97);U2SURP(S37);UBA1(S13);UBE2O(T838);UBE4B(S65);UBE4B(T64);UCK1(S253);UFD1(S299);UNC13B(S367);UNC93B1(S547);UNC93B1(S550);UNG(T60);UPF1(S1127);UPF3B(T169);USP1(S67);USP10(S211);USP15(S242);USP20(S134);USP32(S1423);USP36(S742);USP36(T653);USP7(S18);UTP20(T1741);UTP3(S365);UTP3(S368);VCL(S290);VCPIP1(S747);VGLL4(S149);VPS13D(S1042);WDFY4(S3123);WDR20(S434);WDR44(S403);WEE1(T190);WIPF1(S340);WT1(S273);XPO4(S521);XRCC1(S226);XRCC1(T198);XRCC6(S477);XRN2(S471);YAP1(S289);YBX1(Y162);YBX3(T67);YTHDC2(S1223);ZBTB37(S164);ZCCHC8(S598);ZCCHC8(T479);ZCCHC8(T485);ZDHHC5(S425);ZFC3H1(S949);ZFHX4(S2996);ZFP64(S547);ZFP91(S101);ZFP91(S103);ZFYVE26(S1764);ZKSCAN8(S12);ZMYM2(S305);ZNF106(S641);ZNF24(S274);ZNF280D(S545);ZNF318(S1896);ZNF318(S501);ZNF462(S1251);ZNF513(S85);ZNF516(T930);ZNF518A(S655);ZNF552(S86);ZNF574(S164);ZNF609(S1055);ZNF639(S88);ZNF687(S374);ZNF814(S87);ZNRF2(S21);ZRANB2(S153);ZYX(S308)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>MAP4K5</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>917</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>09/02/18 00:00:00(S218);AAK1(S637);AAK1(T653);AATF(S320);AATF(S321);ABI1(T215);ABI1(Y213);ABI2(S368);ABLIM1(S655);ABLIM1(S706);ACIN1(S388);ACSS2(S267);ADD1(S726);ADD2(S713);ADD3(S693);ADGRA1(S8);ADGRL2(S1275);ADNP(S953);ADNP(S955);ADRM1(T217);AFDN(S1318);AFDN(T1330);AFF1(T372);AFF1(T376);AGAP1(S605);AGAP1(T836);AGO2(S387);AHNAK(S3412);AHNAK(S5448);AKAP1(S445);AKAP2(S720);AKT1S1(T246);ALMS1(S3802);AMPD2(S76);ANKHD1(S1670);ANKRD17(S1696);ANKRD17(S1940);ANKRD17(S2401);ANKRD30B(S806);ANKS1A(S663);ANKS1A(S887);ANLN(S362);ANXA2(T19);ANXA2P2(T19);AP1M1(T154);AP3B2(S272);AP3B2(Y270);APBA2(S11);ARAF(S157);ARFGEF2(S240);ARFGEF2(T244);ARFIP1(S132);ARHGAP17(S162);ARHGAP17(S674);ARHGAP17(T682);ARHGAP21(S1862);ARHGAP21(S856);ARHGAP29(S521);ARHGAP39(S248);ARHGAP4(S906);ARHGAP5(S1218);ARHGEF11(S255);ARHGEF11(S35);ARHGEF16(S107);ARHGEF16(S578);ARHGEF17(S420);ARHGEF2(S122);ARHGEF6(S488);ARHGEF6(S684);ARHGEF7(S518);ARHGEF9(S502);ARID1A(S382);ARID1A(S604);ARID1A(S772);ARID1B(S502);ARID3A(S119);ARL6IP4(S239);ARPP19(S62);ASAP2(S822);ASCC3(S2195);ASH1L(S1748);ATAD5(S306);ATAT1(S315);ATF7(S434);ATF7IP(S474);ATF7IP(S477);ATP13A1(S899);ATP13A3(S817);ATP1A1(S16);ATRX(S1527);ATXN2L(S32);BAIAP2(S366);BAIAP2L1(T257);BASP1(S164);BBX(S844);BCL11A(S630);BCL11A(S718);BCL2L12(S242);BCL9(S1044);BCLAF1(S222);BCOR(S488);BICRA(S1413);BICRAL(S675);BIN1(S298);BOD1L1(T2480);BOLA1(S123);BRAF(S365);BRCA1(S1189);BRCA1(S1191);BRCA1(S1524);BRSK1(S563);BRSK2(S489);BUB1B(S543);C11orf94(S77);C17orf47(S195);C19orf47(S151);C2CD2(S649);C9orf40(S69);C9orf78(S261);C9orf78(T100);CAAP1(S312);CALD1(T730);CAMKK2(S511);CAMKV(T435);CAMSAP1(S793);CAMSAP3(S368);CAMSAP3(S814);CANX(S583);CARD9(S425);CASKIN2(S711);CBL(S619);CCDC14(S798);CCDC86(S160);CCDC86(S91);CCDC86(Y164);CCDC88A(S1820);CCNK(S9);CCNL2(S369);CCNY(S83);CD2AP(S510);CD3EAP(S27);CDC25B(S323);CDC42BPG(S1482);CDC42EP1(S350);CDC6(S106);CDCA5(S75);CDCA8(S219);CDK1(T14);CDK10(T196);CDK11A(S577);CDK11A(T583);CDK11B(S589);CDK12(S32);CDK12(T514);CDK13(T871);CDK16(S138);CDK17(S180);CDK17(S75);CDK18(S117);CDK18(S132);CDK18(S14);CDK18(S98);CDK18(T154);CDK2(T14);CDK3(T14);CEBPZ(S629);CENPA(T21);CENPF(S1750);CEP170(T1533);CEP170P1(T242);CEP57(S55);CEP76(S83);CFL1(S3);CGN(S149);CHAF1A(S206);CHAF1B(S538);CHAMP1(S603);CHD1(S90);CHD8(S2008);CHD8(S2046);CHD8(T1982);CLASP2(S892);CLINT1(S299);CLSPN(S1289);CNNM3(S700);CNNM4(S664);CNOT2(S101);CNOT2(S170);CPSF4(S202);CPT1C(S549);CRAMP1(S1268);CREB1(S143);CRKL(Y207);CRTC2(S613);CRTC3(S329);CRTC3(S62);CSNK1D(S331);CSTF2(S524);CSTF3(S691);CTAGE5(S635);CTNND1(Y865);CTTN(T411);CYBRD1(S260);DAB2IP(S747);DAXX(S495);DCLRE1C(S518);DCP1A(S525);DCP1B(S511);DDX17(S571);DDX41(S21);DGCR8(S271);DGCR8(S95);DHX57(S77);DHX8(S460);DIP2B(S100);DLG5(S1115);DLG5(S1232);DLG5(S1254);DNMT3B(S136);DOCK5(S1766);DOCK7(S864);DONSON(S9);DOT1L(S1001);DTL(T196);DTL(T429);DUSP16(S612);DYNC1H1(S4368);EBAG9(S36);EDC4(S729);EEF1B2(S95);EEF1D(T147);EEF1G(T46);EEF2K(S72);EEF2K(S74);EEF2K(Y69);EIF3A(S1188);EIF3A(S584);EIF3E(S399);EIF4A3(T163);EIF4ENIF1(S577);EIF4ENIF1(S752);EIF4G3(S230);EIF4G3(S232);EML4(S146);EMSY(S209);ENAH(S125);ENAH(S531);ENSA(S67);EPB41(S560);EPB41L1(S510);EPB41L2(S562);EPS15(S563);EPS15(S796);EPS15L1(S108);ERF(S327);ERRFI1(S302);ETNK2(T322);ETV6(S203);EVPL(S2025);EXO1(S623);EZH2(T367);FAM117B(S16);FAM120A(Y452);FAM122A(S76);FAM122B(S119);FAM126B(S430);FAM171A1(S422);FAM193A(S393);FAM193B(S785);FAM234B(S62);FAM53B(S167);FAM53B(S268);FAM53C(S122);FAM83G(S760);FAM83H(S1025);FAM83H(S647);FAM83H(S998);FAM98B(S261);FANCI(S407);FBXO28(S344);FLI1(S241);FLNA(S2158);FLNC(S2233);FNBP1(S497);FNBP1L(S295);FNBP1L(S489);FOXK1(S213);FOXK1(S223);FOXK2(S373);FRY(T1956);FRYL(T1959);FUBP3(S569);FXR1(S409);FYB1(S46);GAB2(S210);GAPDH(S151);GAS2L1(S394);GATA3(S115);GDI2(S61);GEMIN2(S81);GLCCI1(S223);GLCCI1(S30);GLCCI1(S406);GPATCH2(S54);GPATCH4(S128);GPATCH8(S738);GRAMD1B(S274);GRIN3B(S634);GSK3B(S25);GSK3B(S9);GTF2F1(T389);GTF3C1(S1653);GTF3C1(S1865);GTF3C2(S765);HDAC5(S661);HDGFL2(S652);HERC2(S1539);HIPK1(T351);HIPK2(T360);HIRIP3(S530);HIRIP3(S87);HMGCS1(S516);HNRNPC(S260);HOXC9(S159);HR(S6);HRNR(S903);HSP90AA1(S263);HSP90AB1(S226);HSP90AB1(S255);HSP90AB2P(S177);HSP90AB3P(S205);HTATSF1(S642);HUWE1(S3816);HUWE1(T2889);IFI16(S153);IKBKB(S672);ILF3(S62);IMPDH2(S122);IMPDH2(S416);INCENP(S142);INCENP(S312);INCENP(S481);INTS1(T83);INVS(S617);IRF2BPL(S215);IRF2BPL(S519);IRF3(S175);IRS2(S915);ITSN1(S315);ITSN1(S978);IWS1(S235);IWS1(S237);JAZF1(T109);JAZF1(T113);JMJD1C(S2053);JPH1(S475);JPT1(S131);JUN(S63);KANSL1(S829);KANSL1(S839);KDM1B(S17);KHSRP(S181);KIAA0319L(S978);KIAA1143(S115);KIAA1522(S858);KIAA1522(S862);KIAA1522(S971);KIAA1522(T162);KIAA1671(S1488);KIDINS220(S1633);KIF13B(S1410);KIF1A(S1548);KIF23(S902);KIFC1(S26);KLC1(S460);KMT2A(S2098);KMT2D(S3130);KTN1(S75);L3MBTL2(S683);L3MBTL2(S689);LAMTOR1(S98);LAS1L(S617);LAT2(Y136);LEMD3(S144);LIG1(S141);LIG1(S51);LIG1(S76);LIG1(T195);LINC01549(S26);LLGL2(S1000);LSM14A(S178);LSM14A(S183);LYST(S2627);MACF1(S7330);MAGED2(S265);MAGOH(S106);MAGOHB(S108);MAP1S(S657);MAP3K11(S507);MAP3K11(S524);MAP3K21(S514);MAP3K3(T353);MAP3K9(S519);MAP4K2(S328);MAP4K4(S900);MAP7D1(S311);MAP7D1(S460);MAP9(S79);MAPRE2(S200);MARCKS(S167);MARK3(S583);MARK3(S601);MATK(S501);MCM3AP(S527);MCRIP2(S82);MDC1(S495);MDC1(S498);MECP2(S229);MED13(S890);MEX3B(S4);MIA2(S1243);MIIP(S303);MINK1(S733);MIS18BP1(S365);MLF2(S238);MLXIPL(S614);MNAT1(S279);MON1B(S59);MON1B(S61);MPDZ(S1595);MPHOSPH8(S403);MPHOSPH8(T89);MPRIP(S289);MPRIP(S292);MSH6(S254);MTA1(S576);MTBP(S755);MTCL1(S549);MTFR1L(S238);MTMR3(S647);MTOR(S2454);MTSS1L(T391);MYB(S599);MYBPC3(T307);MYC(S62);MYCN(S62);MYO18A(S102);N4BP3(S211);NAA30(S39);NAB1(S183);NAV1(S1265);NAV1(S528);NAV1(S648);NAV1(S672);NAV1(S695);NAV2(S1059);NCOA3(S640);NCOR1(S1472);NCOR1(S2120);NCOR1(T2396);NCOR2(S1982);NCOR2(S215);NCOR2(S2424);NDRG2(S332);NDRG3(S331);NDRG3(S334);NECTIN1(S422);NECTIN1(T391);NEDD4L(S448);NEDD4L(S487);NEO1(S1214);NES(S325);NES(S548);NFATC2IP(S204);NFIC(S333);NFIC(S339);NFIX(S301);NHS(T401);NIPBL(S2658);NLN(S485);NME1(T94);NME2(T94);NME2P1(T79);NMNAT1(S117);NOC2L(S49);NOL4L(S130);NOL8(S432);NOLC1(S698);NOP2(S181);NOP2(S786);NOP2(T185);NOP58(S502);NOP58(S514);NSD2(S421);NSFL1C(S114);NSMCE3(S64);NSRP1(S33);NSUN2(S456);NSUN2(S473);NUMA1(S2062);NUMB(S634);NUP160(S1157);NUP98(S839);ORC1(S199);OSBPL10(S201);PAK1(S115);PAK1(S137);PAK2(T143);PAK4(S181);PAK4(T207);PALD1(S406);PARD3(S144);PARD3(S174);PATL1(T194);PAWR(S259);PCBP1(S173);PCBP1(S264);PCDH18(T442);PCDH7(S1011);PCDHA13(S356);PCDHA4(S356);PCF11(T1530);PCIF1(S144);PCM1(S960);PCM1_HUMAN_Phospho (ST);PCYT1A(S315);PCYT1A(S343);PCYT1B(S315);PDE3B(S495);PDHA1(S232);PDHA1(S293);PDHA1(S300);PDHA2(S291);PDHA2(S298);PDS5B(S1358);PFKP(S386);PGM2(S165);PGM2L1(S175);PHACTR1(S505);PHACTR4(S628);PHC3(T609);PHIP(S1315);PHKA2(S729);PHLDB1(S430);PHLDB2(T404);PI4KB(S266);PIK3AP1(Y570);PIKFYVE(S307);PITPNM1(S621);PJA2(S309);PKN1(S562);PKP2(S293);PKP4(S337);PKP4(S406);PLEKHA6(S808);PLPPR3(S353);PML(S518);PML(S527);PNPO(S241);POGZ(S445);POM121(S269);POM121C(S246);PPA2(S317);PPFIA1(S666);PPFIA4(S684);PPFIBP2(S387);PPHLN1(S163);PPM1H(S124);PPP1R12A(S903);PPP1R13L(S102);PPP1R7(S37);PPP6R3(S525);PPP6R3(S617);PPP6R3(S853);PRAG1(S889);PRAG1(S907);PREX1(S1182);PRKAA1(S184);PRKAA2(S173);PRKAR1B(S83);PRKD2(S214);PROSER1(S613);PROSER2(S179);PRPF38B(S268);PRPF38B(S5);PRPF40B(S764);PRPF4B(S852);PRRC2A(S1386);PRRC2A(S456);PRRC2A(S761);PRRC2B(T225);PRRC2C(T2673);PRRC2C(T2682);PTK2(S722);PTPN13(S214);PTPN13(S240);PTPN13(S890);PTPN13(S908);PTPN14(S642);PTPN2(S304);PTPN21(S660);PTPN22(S692);PTPRK(S856);PTPRK(Y858);PTPRZ1(S2056);PXN(S119);PXN(S258);PXN(Y88);RAD18(S322);RAD54B(S14);RAF1(T234);RALGPS2(S296);RALY(S135);RANBP2(S2510);RANBP2(S788);RANBP2(S955);RANBP3(S211);RAP1GAP2(S45);RAPGEF1(T216);RAPGEF2(S585);RAPGEF6(S1094);RAPH1(S539);RASAL2(S16);RASAL2(S18);RBBP6(S873);RBL2(S662);RBM10(S723);RBM10(S797);RBM14(S256);RBM15(S741);RBM20(S644);RBM27(S120);RBMX(S88);RCOR1(S260);RCOR1(S460);RCSD1(S116);RCSD1(S120);RFC1(S156);RFX7(S225);RFX7(S424);RGPD1(S1519);RGPD1(S779);RGPD2(S1527);RGPD2(S787);RGPD3(S1535);RGPD3(S789);RGPD4(S1535);RGPD4(S789);RGPD5(S1534);RGPD5(S788);RGPD8(S1534);RGPD8(S788);RIF1(S1554);RIF1(S1707);RIF1(S2161);RIOK1(S22);RIPK2(S363);RNF2(S168);RNF214(S500);RNPS1(S251);ROR2(S449);RPAP3(S121);RPLP1(S101);RPLP1(S104);RPLP2(S102);RPLP2(S105);RPRD2(S374);RPRD2(T723);RRAS2(S186);RREB1(S231);RREB1(S42);RSL1D1(S392);RSL1D1(S396);RTN3(S229);RYBP(S127);SALL2(S641);SALL4(S756);SAMHD1(T592);SASH1(S407);SBNO1(T819);SCAF11(S608);SCNM1(S183);SCRIB(S1508);SCRIB(T1549);SCYL3(T153);SDK2(S2014);SEC24B(T329);SEC31A(S527);SEC62(T375);SENP7(S443);SENP7(S444);SERBP1(S203);SERPING1(S198);SF3A1(S359);SF3B1(T223);SF3B1(T227);SF3B1(T350);SFN(S45);SH2B3(S150);SH2D3A(S147);SH3BP4(S279);SH3GL1(S288);SH3KBP1(S230);SHARPIN(S131);SHC3(S474);SHCBP1(S42);SHROOM2(S1116);SHROOM2(S193);SHROOM2(S208);SHROOM3(S664);SHROOM3(S816);SIN3A(S1112);SIN3A(T266);SIN3B(S273);SIPA1L1(S1255);SIPA1L1(S1549);SIPA1L1(S1649);SIPA1L1(S1650);SIPA1L3(S1364);SIRT1(S27);SLC16A1(S461);SLC20A2(S256);SLC20A2(S259);SLC22A17(S515);SLC2A3(S485);SLC43A1(T256);SLC4A1AP(S466);SLC4A7(S556);SLC4A7(T559);SLC9A1(S703);SMAD1(S463);SMAD1(S465);SMAD9(S465);SMAD9(S467);SMAP(S93);SMARCAD1(S79);SMARCC2(S347);SMC3(S1085);SMG8(T743);SMG8(Y746);SNIP1(S35);SNRNP70(S320);SORBS2(S278);SOWAHD(S22);SPAG9(S733);SPTAN1(S1217);SPTBN1(S2358);SPTBN2(S2384);SQSTM1(S328);SRCAP(S274);SREK1IP1(T146);SRGAP1(S1029);SRRM1(S260);SRRM1(S402);SRRM1(S549);SRRM1(S551);SRRM1(T406);SRRM2(S1144);SRRM2(S1404);SRRM2(S2121);SRRM2(S2123);SRRM2(S2581);SRRM2(S322);SRRM2(S377);SRRM2(S440);SRRM2(T1003);SRRM2(T318);SRRM2(T400);SRRM2(Y1145);SRRT(S67);SRSF1(S199);SRSF1(S201);SRSF4(S450);SRSF9(S204);SSBP3(S347);STAT5A(S193);STAU1(S390);STIM1(S618);STK33(S470);SUPT5H(S666);SURF6(S138);SYAP1(T248);SYMPK(S1243);SYNRG(S1075);SYNRG(S473);SYT6(S187);SYT6(Y190);TAF2(S1185);TAF6(S634);TAF6(S636);TAF9(T144);TANC2(S1458);TANC2(T434);TAX1BP1(S666);TBC1D10B(S658);TBC1D10B(S661);TBC1D22A(S167);TBKBP1(S365);TCF12(S79);TCF4(S372);TERF2IP(S154);TEX2(S266);TIAM1(S1407);TJP1(S1579);TJP1(S168);TJP1(S968);TJP3(S164);TLE3(S263);TLE3(S267);TLE4(S208);TLE4(S292);TMC6(S63);TMEM163(S12);TMEM201(S443);TMEM41B(T18);TMEM9(S137);TMPO(T160);TNIK(S707);TNK2(T829);TNK2(Y827);TNKS1BP1(S872);TNKS1BP1(S893);TNKS1BP1(S983);TNRC18(S1925);TNRC6C(S714);TNS1(S1269);TNS1(T1173);TNS3(S874);TOMM70(S91);TOP2B(S1400);TP53BP1(S1068);TP53BP1(S1320);TP53BP1(S580);TP53BP1(S831);TPD52L1(S149);TRA2A(T202);TRAF4(S426);TRAFD1(S470);TRAM1(S365);TRAPPC12(S184);TRIM16(S36);TRIO(S1724);TRIT1(S443);TRMT2A(S602);TRPS1(S1081);TRPS1(S1085);TRUB1(T27);TSC1(S505);TSC22D4(S62);TTN(S1406);TVP23C(S223);UBA1(S13);UBE2J1(S266);UFD1(S299);ULK3(S240);UNC80(S3073);UPF1(S1127);UPF3B(T169);USP1(S67);USP11(S648);USP18(T87);USP32(S1423);USP41(T87);UTP20(T1741);UTP3(S365);UTP3(S368);VCPIP1(S747);VDAC1(S104);VDAC2(S115);WDFY3(S2278);WDFY4(S3123);WDR20(S434);WDR44(S403);WEE1(T190);WIZ(S1151);WNK1(S2370);XRN2(S471);YBX1(S209);YBX1(Y162);YTHDC1(S424);YWHAB(S47);YWHAE(S46);YWHAG(S46);YWHAH(S46);YWHAQ(S45);YWHAZ(S45);ZBTB37(S164);ZBTB7A(S549);ZC3H13(S873);ZC3H15(S381);ZDH18_HUMAN_Phospho (ST);ZDHHC5(T348);ZFC3H1(S949);ZFP36L2(S438);ZFPM1(S909);ZKSCAN8(S12);ZMYM2(S305);ZMYND8(S406);ZNF106(S641);ZNF219(S16);ZNF280D(S545);ZNF318(S2035);ZNF326(S270);ZNF513(S85);ZNF516(T930);ZNF518A(S655);ZNF552(S86);ZNF609(S1055);ZNF638(S605);ZNF649(S474);ZNF687(S266);ZNF687(S271);ZNF814(S87);ZNF84(S128);ZNRF2(S21);ZRANB2(S120);ZRANB2(S153)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>MAPK1.3</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>471</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>09/02/18 00:00:00(S218);2 Phospho (ST);AAK1(S14);AAK1(S21);AATF(S321);ABCA2(S1238);ABCF1(S105);ABCF1(S228);ABCF1(T108);ADD1(S431);ADD1(S436);AHNAK(S5110);AHNAK(S5731);AHNAK(S5841);AKAP2(S748);ANAPC4(S779);ANK2(S3823);ANK3(S4298);ANKRD13D(S465);ANKRD13D(T469);ANKS1A(S647);ANLN(S792);APBB1IP(S526);ARFGEF2(S624);ARFGEF2(T626);ARHGAP39(S251);ARHGEF17(S420);ATAD1(S322);ATF7IP(S673);ATXN2(S861);BAG3(T406);BCL11A(T208);BCLAF1(S183);BCLAF1(S385);BCOR(T1145);BCR(S459);BRIP1(S1032);C11orf84(S148);C1orf174(S189);C1orf198(S37);CAMK1D(T184);CASC3(S363);CAST(S243);CCAR2(S678);CCDC43(T139);CCDC43(Y135);CCDC86(S58);CCDC86(S66);CCDC86(S69);CD2BP2(S49);CD3EAP(S285);CDC20(T70);CDC25A(S18);CDC42EP1(S143);CDCA5(S75);CDK13(S358);CDK13(S360);CDK13(T871);CDKL5(S407);CDS2(S33);CDYL(S216);CEBPE(S181);CHD8(S1420);CHD8(S1424);CLCC1(S438);CLDN10(S203);CLK1(S341);CLK4(S339);CNK3/IPCEF1(S873);CREBBP(S121);CRKL(S107);CRTC1(S153);CTAGE5(S594);CTPS1(S575);CTTN(S405);CTTN(T411);CTTNBP2NL(S560);CTTNBP2NL(S568);DAP(S51);DCLK1(T336);DCP1A(S62);DDX41(S23);DENND4A(S1256);DENND4C(S989);DGCR8(S275);DGKH_HUMAN_3 Phospho (ST);DLG1(S122);DLGAP5(S690);DNTTIP2(S88);DNTTIP2(T188);DNTTIP2(T87);DOT1L(S902);DOT1L(T900);DPF2(S200);DPPA4(T215);DVL3(S125);DYNC1LI2(S194);EEF1AKMT2(S21);EEF1B2(S106);EEF1B2(Y79);EEF1D(S162);EHBP1(S432);EHBP1L1(S1257);ELAC2(S213);EMD(S141);ERF_HUMAN_2 Phospho (ST);ERRFI1(S374);ETV1(S97);ETV3(S139);ETV3(S159);FAM117B(S10);FAM177A1(S70);FAM177A1(T71);FAM177A1(Y69);FAM234B(S62);FAM83B(S764);FAM83H(S998);FAM84B(T289);FBXO46(S240);FIP1L1(S500);FLI1(S241);FLNA(S2152);FOXO3(S284);FOXO3(S55);FRMD4A(S800);GIGYF2(S30);GLCCI1(S406);GMIP(S914);GMPS(S332);GOLGA4(S1248);GON4L(S1426);GPHN(S188);GPHN(S194);GPHN(T198);GPN1(S338);GSE1(S857);GTF3C1(S1856);GTF3C2(S901);HBS1L(T231);HELZ(S1620);HERC2(S2928);HIRIP3(S104);HJURP(S557);HMGA1(S102);HMGA1(S103);HNRNPU(S59);HSPH1(T815);IGF2BP1(S181);IGLL1(S62);IPCEF1(S411);IRF2BP2(S175);IRX2(S317);ITPKB(S43);IWS1(S80);IWS1(S82);JPT1(S131);KCNK2(S385);KDM2B(S497);KDM2B(T493);KDM2B(T495);KDM2B(Y490);KIF1A(S1370);KIF21A(S1271);KIF21A(S1274);KIF21A(S1304);KIF21A(S1307);KLHDC4(S418);KMT2B(S1092);KMT2B(S1095);KMT2D(S2274);KPNA4(S60);KRT18(S399);KRT19(S395);L1TD1(S737);LAD1(S394);LARP1(S627);LARP1(S631);LARP1(T376);LASP1(T68);LEMD2(S499);LIMA1(S230);LIMA1(S686);LIMK1(S302);LLGL2(S480);LTBP1(S1413);LYSMD2(S33);MAP1B(S1427);MAP1B(S1438);MAP1B(S1443);MAP1B(S937);MAP1B(T1317);MAP1B(T1341);MAP2(S1787);MAP2(S1790);MAP3K2(S239);MAP7D1(S116);MAPK1(Y187);MAPT(S713);MAST2(S1254);MCM3(S711);MCM3(T722);MCM3(Y708);MCM9(S1088);MDC1(S780);MED1(S664);MEPCE(S217);MEX3A(S428);MEX3C(S540);MEX3C(T541);MFAP1(S116);MFAP1(S52);MFAP1(S53);MGA(S2088);MIA2(S1202);MKI67(T401);MKL2(S921);MPLKIP(S115);MPLKIP(T51);MPLKIP(Y45);MYC(S62);MYC(T58);MYCBP2(T1587);MYCN(S62);MYCN(T58);MYO18A(S102);NAB2(S6);NASP(T477);NCAPG(S674);NCOR1(S158);NCOR2(S2065);NCOR2(S215);NCOR2(S2404);NCOR2(T1391);NFATC2(S236);NFATC2(S243);NGDN(S142);NGDN(S143);NHS(S1329);NRIP1(S356);NUCB1(S369);NUFIP1(S338);NUFIP1(S340);NUFIP1(S342);NUP50(S221);OSBPL8(S314);OSTM1(S322);PACSIN3(S383);PAPOLG(S708);PARN(S619);PCBP1(S231);PCNP(S119);PDLIM2(S197);PDS5B(S1358);PDZD2(S1270);PHACTR4(S118);PHF6(S154);PHKA2(S1015);PHKA2(S1044);PHLDB1(S518);PHLDB1(T516);PHLDB2(S513);PHRF1(S1229);PLCB3(S934);PLCB3(T924);PLEKHG3(T964);PNISR(S311);PNISR(S313);PNISR(S321);POLA1(S186);POM121(S395);POM121(S396);POM121C(S372);PPIG(S256);PPIG(S257);PPP1R12A(S871);PPP1R2(T89);PPP4R3B(S840);PPP6R1(S531);PPP6R1(S759);PPP6R3(S523);PRCC(S267);PRICKLE2(S546);PRKAA2(S491);PRPF38B(S527);PRPF38B(S529);PRPF4B(S87);PRPF4B(S93);PRR5(S310);PSMD1(S315);PSMD1(T311);PUM1(T112);PWWP2B(S447);Phospho (ST);QRICH1(S345);RABL6(S640);RABL6(S641);RAD54B(S14);RAI14(S286);RALY(S239);RANBP2(S948);RANBP2(S955);RANBP3(S101);RAP1GAP2(S608);RB1(S37);RBM10(S89);RBM15(S670);RBM15(S674);RBM15B(S562);RBMX(S189);RBMXL1(S189);RBMXL1(S88);RCSD1(S68);REPS1(S392);RFC1(S108);RFC1(T110);RFTN1(S199);RIC8A(S436);RIC8A(T441);RIOK2(S337);RPAP3(S116);RPAP3(S119);RPL27A(S68);RPP30(S251);RPS6KA1(S363);RPS6KA3(T365);RREB1(S36);RREB1(S42);RRP1B(S453);RRP1B(S736);RRP8(S62);RRP8(S64);RSF1(T628);RSL1D1(S469);SAC3D1(S402);SAFB(S604);SAFB2(S832);SALL1(S586);SALL1(S590);SALL1(S593);SAMD4B(S628);SART1(S448);SCML2(S511);SCRIB(S1348);SCRIB(S1378);SCRIB(S1439);SCRIB(T1342);SCRIB(T826);SEC16A(S1786);SERBP1(S234);SET(S161);SETSIP(S171);SF3A1(S329);SF3A1(S359);SF3A1(T374);SGTA(S77);SGTA(T81);SIPA1L1(S1649);SIPA1L1(S1650);SKA3(S110);SKA3(S152);SLC4A1AP(S466);SLC9A3R1(S280);SMARCAD1(S124);SMARCAD1(S127);SMARCC1(T398);SMC4(S22);SMC4(S28);SMN1(S28);SNX17(S333);SOGA1(S1303);SON(S1026);SON(S1784);SPATA5L1(S610);SPP1(S63);SPTBN2(S2171);SQSTM1(S224);SQSTM1(S332);SRRM1(S260);SRRM2(S1014);SRRM2(S1501);SRRM2(S1502);SRRM2(S377);SRRM2(S846);SRRM2(T400);SRRM2(T848);SRSF10(S131);SRSF11(S434);SSFA2(S1040);SSH1(S897);STAU1(S390);STAU2(S455);STK17A(S28);SVIL(S221);SYCE2(S188);TACC2(S2317);TACC2(S2321);TACC2(S2359);TACC3(S177);TBKBP1(S372);TBKBP1(S400);TCOF1(S1227);TCOF1(S156);TEX10(T29);TEX2(S266);THRAP3(S232);TJAP1(S345);TJP1(S125);TJP2(S1159);TLN1(S425);TMF1(S72);TNKS1BP1(S1158);TNKS1BP1(S1297);TNKS1BP1(S435);TOM1(S462);TOMM70(S110);TOMM70(S91);TOP2B(S1400);TOP2B(S1522);TOP2B(S1524);TOR1AIP1(S157);TPR(S2155);TPR(T2116);TPR(T650);TPX2(T369);TRA2B(T201);TRA2B(T212);TRIM28(S50);TRPS1(S127);TWISTNB(S304);UBAP1(S146);UBE2E3(T15);UHRF1BP1L(S414);UHRF1BP1L(S418);UIMC1(S44);UIMC1(S46);USP20(S373);USP20(T377);USP36(S952);UTP3(S37);UTP3(Y43);VCAN(S2116);VRK3(S83);WAPL(S221);WAPL(S226);WAPL(S77);WASHC2A(S158);WASHC2A(S160);WASHC2C(S158);WASHC2C(S160);WDHD1(S868);WIPF2(S267);XRN1(S1645);XRN2(S499);XRN2(S501);YBX3(S346);YLPM1(S756);YTHDC2(S1221);ZC3H11A(S758);ZC3H4(S1108);ZC3H4(S1110);ZC3H4(S1269);ZMYM3(S267);ZMYM4(S122);ZNF106(S1304);ZNF281(S651);ZNF318(S40);ZNF609(S358);ZNF639(S60);ZNF768(S90);ZNF768(S97);ZRANB2(S120)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>MAPK14</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>1037</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>AATF(S316);AATF(S320);AATF(S321);ABCF1(S105);ABCF1(S228);ABCF1(T108);ABI1(S231);ABI1(T215);ABI1(Y213);ABI2(S368);ABLIM1(S655);ABLIM1(S706);ACIN1(S388);ACIN1(S838);ACIN1(T682);ADAD2(S522);ADGRL2(S1275);ADNP(S953);AFAP1(S683);AFDN(S1238);AFDN(S1318);AFDN(S216);AFDN(T1330);AFF1(T372);AFF1(T376);AGAP1(S605);AGO2(S387);AHNAK(S5448);AKAP12(S627);AKAP12(S629);AKAP2(S121);AKAP2(S720);AMPH(S262);AMPH(S268);AMPH(S272);AMPH(T260);ANK2(T3797);ANKLE2(S866);ANKRD17(S1696);ANKRD17(S2401);ANKS1A(S663);ANKS1A(S887);ANKS1A(T318);ANLN(S485);AP1M1(T154);AP3B1(S276);APC(S1371);APC(S2674);APIP(S87);ARFGAP2(S201);ARFGEF2(S624);ARFGEF2(T626);ARFIP1(S132);ARGLU1(S46);ARHGAP11A(S285);ARHGAP17(S162);ARHGAP17(T682);ARHGAP21(S1862);ARHGAP21(S856);ARHGAP4(S906);ARHGEF11(S251);ARHGEF11(S255);ARHGEF11(S35);ARHGEF16(S107);ARHGEF2(S122);ARHGEF26(S304);ARID1A(S1184);ARID1A(S1204);ARID1A(S604);ARID1A(S772);ARID3A(S119);ARL6IP4(S239);ARPC2_HUMAN;ASAP2(S822);ASCC3(S2195);ATAD5(S306);ATAT1(S315);ATF7(S434);ATF7IP(S474);ATF7IP(S477);ATG2B(S497);ATN1(S101);ATP1A1(S16);ATRX(S677);ATXN2(S667);ATXN2(S758);ATXN2(S784);ATXN2(S863);ATXN2L(S32);ATXN2L(S634);ATXN7L3(S281);BCL2L12(S113);BCL2L12(S121);BCL2L12(T117);BCL7C(S126);BCL7C(T118);BCL9(S35);BCL9L(S1004);BCLAF1(S222);BCLAF1(S282);BCLAF1(S397);BCOR(S1290);BCOR(S488);BICRAL(S675);BRAF(S365);BRCA1(S1524);BRPF1(S860);BRSK2(S382);BRWD1(S2018);BRWD1(S2020);BUB1B(S543);BUD13(S325);BYSL(S98);C11orf84(S148);C17orf47(S195);C2CD2(S649);C5orf30(S25);C7orf50(S175);C9orf40(S69);C9orf78(T100);CAAP1(S312);CAMK1D(T184);CAMKV(T435);CAMSAP1(S793);CAMSAP3(S814);CANX(S554);CANX(S564);CAPN15(S335);CARD9(S425);CARHSP1(S30);CASKIN2(S711);CASKIN2(S946);CBARP(S299);CBX8(S110);CBX8(S256);CCDC14(S798);CCDC14(T376);CCDC86(S160);CCDC86(S47);CCDC86(Y164);CCDC88A(S1820);CCDC88A(S230);CCNK(S9);CCNL2(S369);CD2AP(S510);CD2BP2(S195);CD3EAP(S490);CDC25B(S323);CDC42BPG(S1482);CDC42EP1(S143);CDC42EP1(S350);CDC42EP1(T145);CDC42EP2(S141);CDC42EP2(T137);CDC42EP4(T23);CDC6(S106);CDCA8(S219);CDK1(T14);CDK11A(S577);CDK11A(T739);CDK11B(S589);CDK11B(T751);CDK12(S32);CDK17(S180);CDK18(S117);CDK18(S132);CDK18(S14);CDK2(T14);CDK3(T14);CDV3(Y190);CENPA(T21);CENPF(S3094);CEP170(S1019);CEP170(T1023);CEP170(T1533);CEP170P1(T242);CEP76(S83);CFL1(S3);CGN(S149);CGN(S332);CHAF1A(S206);CHAMP1(S282);CHAMP1(S379);CHAMP1(S382);CHAMP1(S386);CHAMP1(S432);CHAMP1(S436);CHD4(S1531);CHD8(S2008);CHERP(S817);CHERP(T819);CLNS1A(S102);CNOT2(S101);CNOT2(S170);COPRS(S66);CPSF4(S202);CRAMP1(S1268);CREB1(S143);CRKL(Y207);CRTC2(S613);CRTC3(S329);CSNK1D(S331);CTAGE5(S590);CTAGE5(S594);CTAGE5(S596);CTAGE5(S635);CTDP1(S416);CTDP1(S839);CTNNA1(S641);CTTN(S405);CTTN(T411);CXXC5(S80);DAB2IP(S747);DAP(S51);DAXX(S415);DBN1(S381);DCLRE1C(S518);DCP1B(S275);DDA1(S33);DDX17(S571);DDX41(S21);DDX41(S23);DDX42(S96);DDX42(Y183);DDX51(S83);DEK(S72);DENR(S73);DGCR8(S377);DHX29(S200);DHX57(S77);DHX8(S460);DIDO1(S1456);DIP2B(S100);DKC1(S451);DKC1(S494);DLG5(S1115);DLG5(S1232);DLG5(S1254);DLG5(S1795);DLGAP4(S666);DNM1(S619);DNM2(S619);DNMT3B(S136);DOCK5(S1766);DOCK7(S180);DOCK7(S439);DOK3(T336);DUS3L(S277);DUSP16(S612);DUSP16(S627);DYNC1H1(S4368);DYNC1LI2(S446);EDC4(S729);EEF1D(T147);EEF1G(T46);EEF2K(S72);EEF2K(S74);EEF2K(Y69);EHBP1(S428);EIF2B4(S130);EIF3A(S1188);EIF4EBP1(S83);EIF4EBP3(T31);EIF4EBP3(T32);EIF4EBP3(Y20);EIF4ENIF1(S752);EIF4G3(S232);EIF5B(S135);EIF5B(S137);EML4(S146);EML4(T897);EML4(T899);ENAH(S531);EP300(S1038);EPB41(S560);EPS15(S563);EPS15(S796);EPS15L1(S108);ERCC6L(S820);ERF(S327);ESYT1(S820);ETV6(S203);EVPL(S2025);EXO1(S623);FAM120A(Y452);FAM193A(S393);FAM193B(S785);FAM234B(S62);FAM53C(S122);FAM53C(S232);FAM53C(S234);FAM76B(S193);FAM83B(S466);FAM83H(S1025);FAM83H(S647);FAM83H(S7);FAM83H(S8);FAM83H(S936);FARSA(S301);FBXO46(S293);FGD6(S692);FIP1L1(S500);FKBP15(S346);FLNA(S2158);FMN2(S295);FNBP4(S116);FOXK1(S223);FOXK2(S373);FOXO1(S293);FOXO1(S298);FOXO1(S303);FRYL(T1959);FTH1(S183);FXR1(S406);FXR1(S409);FXR1(S485);FXR2(S603);FYB1(S46);GAB2(S141);GAGE13(S33);GAGE2A(S32);GAGE2B(S32);GAGE2D(S32);GAPDH(S151);GATA3(S115);GIT1(Y598);GJA1(S306);GJA1(S314);GLCCI1(S30);GOLGA4(S1248);GPATCH8(S738);GPS1(S468);GRAMD1B(S274);GREB1(S1193);GSK3B(S25);GSK3B(S9);GTF2F1(T389);GTF2I(S679);GTF3C1(S1865);GTF3C2(S765);HARS2(S67);HCFC1(S1507);HDGF(S132);HDGF(S133);HDGFL2(S366);HDGFL2(S369);HDGFL2(S370);HEATR1(S1190);HELB(S1050);HID1(S653);HIPK1(T351);HIPK2(T360);HIRIP3(S223);HMGA1(S99);HMGCS1(S516);HNRNPA2B1(S212);HNRNPC(S138);HNRNPC(S253);HOXC9(S159);HSD17B4(S318);HSH2D(S298);HSP90AA1(S263);HSP90AB1(S226);HSP90AB3P(S205);HSPB1(S15);HSPB1(S82);HTATSF1(S642);HUWE1(S2888);HUWE1(T2889);ICE1(S939);IFI16(S153);IKBKB(S672);IL17RA(S708);INCENP(S481);INCENP(S828);INCENP(S831);INCENP(T832);INPP5D(S1039);INPP5F(S907);INVS(S617);IQSEC1(S107);IRF2BPL(S215);ITSN1(S315);ITSN1(S559);IWS1(S235);IWS1(S237);IWS1(S720);JAZF1(T109);JAZF1(T113);JMJD1C(S2053);JPH1(S162);JPT1(T54);JUN(S63);KANK2(S323);KANSL1(S829);KANSL1(S839);KDM1A(S69);KDM5C(S1359);KHNYN(S353);KHNYN(S359);KIAA0754(S25);KIAA0930(S324);KIAA1143(S50);KIAA1468(S170);KIAA1522(S971);KIDINS220(S1633);KIF18B(S468);KIF1A(S1548);KIF21B(S1241);KIF23(S902);KIFC1(S26);KIT(S943);KLC2(S610);KLF3(S250);KMT2D(S3130);KMT2D(T382);KPNA4(S60);KRI1(S628);KRI1(S639);KRT18(S30);KTN1(S75);L1TD1(S557);LARP1(S143);LARP1(S327);LARP1(S627);LARP1(S90);LCA5(S306);LENG1(S59);LIG1(S76);LIG1(T195);LSM14A(S178);LSM14A(S183);LSP1(S193);LYSMD2(S33);LYST(S2627);MACF1(S7330);MAF1(S60);MAGED2(S265);MAP1B(S1208);MAP1B(S1322);MAP1B(S1438);MAP1B(S1443);MAP1B(S614);MAP1B(S831);MAP1B(S832);MAP1B(T1317);MAP1B(T1341);MAP3K11(S524);MAP3K21(S514);MAP3K9(S519);MAP4(S358);MAP4(S624);MAP4K2(S328);MAP4K4(S900);MAP7D1(S460);MAP9(S79);MAPT(S721);MARCKS(S167);MARK2(S498);MATK(S501);MBD3(S86);MCM3(S672);MCM3(T674);MCM3AP(S527);MCM7(S121);MCRIP2(S82);MDC1(S329);MDC1(S986);MDC1(S988);MDC1(S995);MED13(S890);MED22(S173);MEX3B(S4);MFAP1(S116);MFAP1(S118);MIA2(S1198);MIA2(S1202);MIA2(S1204);MIA2(S1243);MIER1(S488);MINK1(S733);MINK1(S778);MINK1(S782);MINK1(S993);MKI67(S2105);MKI67(S2466);MKRN2(S139);MNAT1(S279);MON1B(S59);MON1B(S61);MORC3(S771);MORC3(Y773);MPHOSPH8(S403);MPHOSPH8(T89);MPRIP(S220);MPRIP(S289);MPRIP(S292);MSL1(S66);MTA1(S576);MTCL1(S1812);MTCL1(S1814);MTDH(S298);MTMR3(S647);MYB(S599);MYC(S62);MYCBP2(S3440);MYCN(S156);MYCN(S62);MYO18A(S102);MYO9B(S1267);MYO9B(S1405);NAA30(S39);NAV1(S528);NAV1(S672);NAV1(S695);NAV2(S1559);NCBP3(S25);NCKIPSD(S122);NCL(S184);NCL(S206);NCOR1(S1472);NCOR1(S172);NCOR2(S1018);NCOR2(S2057);NCOR2(S2065);NCOR2(S215);NDRG2(S332);NDRG3(S331);NDRG3(S334);NECTIN1(T391);NEDD4L(S448);NEDD4L(S487);NELFE(S51);NFATC2IP(S204);NGRN(S41);NHS(S1329);NIPBL(S274);NIPBL(S280);NLN(S485);NMNAT1(S117);NMT1(S47);NOC2L(S49);NOL8(S432);NOP2(S181);NOP2(S786);NOP2(T185);NOP58(S351);NOP58(S502);NOVA1(S157);NPM1(S260);NSMCE3(S64);NSRP1(S33);NSUN2(S456);NSUN2(S473);NUCKS1(S214);NUP210(S1852);NUP210(Y1855);NUP214(S1023);NUPL2(S106);ORC1(S258);OSBP(S190);OSBP(S193);OTUD4(S1023);OTUD4(S1024);OTUD5(S165);PACSIN2(S313);PAK1(S137);PAK1(T185);PAK2(T143);PAK4(S181);PAK4(T207);PALD1(S406);PALLD(S893);PARD3(S144);PARD3(S174);PARN(S557);PATL1(T194);PCBP1(S173);PCBP2(S173);PCDH18(T442);PCDH7(S1011);PCIF1(S144);PCM1(S93);PCYT1A(S343);PDE3B(S495);PDHA1(S232);PDHA1(S293);PDHA1(S300);PDHA2(S291);PDHA2(S298);PDS5B(S1358);PDZD8(S521);PFAS(S569);PFKFB3(T463);PFKP(S386);PGM2(S165);PHACTR1(S505);PHAX(S368);PHC1(S645);PHC3(T609);PHIP(S1315);PHKA2(S729);PHLDB2(T404);PHRF1(S936);PIKFYVE(S307);PIKFYVE(T477);PITPNM1(S621);PKN1(S562);PKP2(S293);PKP3(S331);PKP4(S337);PKP4(S406);PLCH1(S1060);PLEKHA3(T246);PLEKHA5(S855);PLEKHA6(S251);PLEKHA6(S808);PML(S518);PML(S527);PNN(S66);PNPO(S241);POLA1(S186);POLA2(T127);POLDIP2(T292);POLR2A(S1843);POM121C(S372);PPAN(S359);PPFIA1(S666);PPFIBP1(T603);PPFIBP2(S387);PPM1H(S124);PPP1R12A(S862);PPP1R12A(S903);PPP1R12C(S509);PPP1R13L(S102);PPP1R9B(S100);PPP6R3(S617);PRAG1(S889);PRAG1(S907);PRKAB1(S40);PRKAR2A(S99);PRKD2(S214);PRKRA(S18);PRMT3(S25);PRMT3(S27);PROSER1(S613);PROSER2(S179);PRPF38B(S268);PRPF38B(S5);PRPF40B(S764);PRPF4B(S427);PRRC2B(S1682);PRRC2B(S1683);PRRC2C(T2673);PSMB10(S229);PSRC1(S140);PTGES3(S113);PTPN12(S603);PTPN12(S606);PTPN12(S608);PTPN13(S214);PTPN13(S908);PTPN22(S692);PTPN6(S534);PTPN6(Y536);PXN(S258);PXN(Y118);QSER1(S615);RAB11FIP1(S202);RAB31(S35);RABEP1(T408);RABL6(S596);RABL6(T599);RAD18(S99);RAD9A(S277);RALBP1(S92);RALBP1(S93);RALGPS2(S296);RANBP2(S2246);RANBP2(S2510);RANBP2(S955);RANBP2(T2613);RANBP3(S108);RAP1GAP2(S45);RAPGEF6(S1094);RAPH1(S539);RASAL2(S16);RB1(S807);RBL2(S639);RBM10(S797);RBM10(S89);RBM12B(S839);RBM14(S256);RBM15(S670);RBM15(S674);RBM20(S644);RBM27(S120);RBM34(S28);RBM5(S624);RBMX(S249);RBMX2(S273);RBMXL1(S249);RCOR1(S260);RCSD1(S116);RCSD1(S120);REPS1(S162);REPS1(S166);REPS1(S170);REPS1(S392);REPS1(T173);RETREG3(S258);RETREG3(S260);RFC1(S69);RFC1(S71);RFC1(Y67);RFX1(S204);RFX7(S225);RFX7(S424);RGPD1(S1519);RGPD2(S1527);RGPD3(S1271);RGPD3(S1535);RGPD4(S1271);RGPD4(S1535);RGPD5(S1270);RGPD5(S1534);RGPD8(S1270);RGPD8(S1534);RHBDF2(S177);RIC8A(T441);RIC8A(Y435);RIF1(S1554);RIF1(S1688);RIF1(T1047);RIOK1(S22);RIOK2(S337);RIOK3(S125);RIOK3(S127);RIOK3(S128);RIPK2(S357);RNF2(S168);ROR2(S449);RPAP3(S121);RPL18A(S71);RPL5(S286);RPRD2(S374);RPRD2(S930);RPRD2(T723);RPS27(S27);RPS27L(S27);RPTOR(S877);RREB1(S1219);RREB1(S1225);RREB1(S42);RRP12(S1080);RRP1B(S735);RSF1(T1305);RYBP(S127);S100A13(S32);SASH1(S407);SBNO1(T819);SCAF11(S798);SCRIB(S1306);SCRIB(S1309);SCRIB(S1348);SCRIB(S1508);SCRIB(S835);SCYL3(T153);SDCCAG3(S247);SEC24B(T329);SEC62(T375);SENP3_HUMAN_Phospho (ST);SERPING1(S198);SETD1B(S1283);SF3A1(S329);SF3A1(S359);SF3B1(T350);SF3B2(S307);SFSWAP(S909);SH2B3(S150);SH2D3A(S147);SH3BP4(S279);SH3GL1(S288);SH3KBP1(S230);SHC3(S474);SHCBP1(S42);SHROOM2(S1173);SHROOM2(S193);SHROOM2(T1168);SHROOM3(S1497);SHROOM3(S664);SHROOM3(S816);SHROOM3(S910);SIK3(S551);SIK3(S866);SIRT1(S172);SIRT1(S27);SKA3(S103);SLBP(S114);SLC20A2(S256);SLC20A2(S259);SLC43A1(T256);SLC4A1AP(S466);SLC4A7(S556);SLC4A7(T559);SLC9A1(S703);SLTM(S553);SLX4(T1315);SLX4(T1320);SMAD1(S463);SMAD1(S465);SMAD9(S465);SMAD9(S467);SMAP(S93);SMARCA4(S610);SMARCAD1(S98);SMARCC1(T398);SMARCC2(S347);SMG8(T743);SMG8(Y746);SNIP1(S35);SNIP1(S52);SNRNP200(S225);SON(S1783);SON(S1784);SPP1(S303);SPP1(S62);SPP1(S63);SPTAN1(S1217);SPTBN1(S2169);SPTBN2(S2384);SQSTM1(S224);SRCAP(S349);SRF(S224);SRRM1(S389);SRRM1(S431);SRRM1(S463);SRRM1(S465);SRRM1(S694);SRRM1(S769);SRRM1(S775);SRRM1(S781);SRRM2(S1083);SRRM2(S1144);SRRM2(S1404);SRRM2(S1499);SRRM2(S1501);SRRM2(S1502);SRRM2(S1691);SRRM2(S1694);SRRM2(S1925);SRRM2(S2100);SRRM2(S2118);SRRM2(S2123);SRRM2(S2426);SRRM2(S322);SRRM2(S351);SRRM2(S437);SRRM2(S952);SRRM2(S954);SRRM2(T1927);SRRM2(T318);SRRM2(T848);SRRM2(Y1145);SRSF4(S448);SRSF4(S450);SRSF6(S314);SSBP3(S347);ST17A_HUMAN_Phospho (ST);STAT5A(S193);STAT5B(S193);STAU1(S390);STAU2(S455);STIM1(S618);STK33(S470);STRBP(S466);STRBP(S470);STRN(S245);STX17(S289);SUGP1(S485);SUZ12(S546);SYMPK(S1243);SYNRG(S1075);SYNRG(S752);SYT6(S187);SYT6(Y190);SYTL2(S535);TACC3(S317);TAF6(S634);TBC1D22A(S167);TBC1D4(S318);TBC1D4(S588);TBC1D4(S754);TBC1D4(T752);TBKBP1(S365);TBKBP1(S385);TBKBP1(S415);TCF20(S559);TCF4(S372);TCOF1(S1227);TCOF1(S583);TELO2(S836);TERF2IP(S154);TEX2(S266);TGFB1I1(S194);THRAP3(S624);THRAP3(S928);TJAP1(S345);TJP1(S125);TJP1(S168);TJP1(S968);TJP2(S1159);TJP2(S702);TJP3(S164);TLE4(S208);TLN2(S461);TMCC1(S382);TMPO(S67);TMPO(T74);TNK2(T829);TNK2(Y827);TNKS1BP1(S429);TNKS1BP1(S836);TNKS1BP1(S872);TNKS1BP1(S983);TNRC6C(S714);TNS1(S1269);TOMM70(S110);TOMM70(S91);TOP2A(S1393);TOP2B(S1400);TOP2B(S1522);TOP2B(S1524);TOX4(S174);TOX4(S182);TOX4(T175);TP53BP1(S523);TP53BP1(S580);TP53BP1(S831);TP53BP1(Y522);TPD52(S171);TPD52L1(S149);TRA2A(S86);TRA2A(T88);TRAF4(S426);TRAFD1(S470);TRAM1(S365);TRAPPC10(S711);TRAPPC12(S184);TRERF1(S758);TRERF1(T767);TRIO(S1724);TRIP12(T941);TRMT2A(S602);TRRAP(S2077);TRUB1(T27);TSC1(S505);TSC22D4(S62);TTF1(S487);TTN(S1406);TVP23C(S223);UBA1(S13);UBR5(S1549);UBR5(T637);UCK1(S253);UFD1(S299);UGDH(T91);UIMC1(S44);UIMC1(S46);UPF1(S1127);UPF3B(T169);URI1(T373);USP1(S67);USP10(S576);USP16(S552);USP20(S132);USP20(S134);USP32(S1423);USP7(S18);UTP11(S241);UTP14A(S407);UTP18(S121);UTP18(S124);UTP20(T1741);UTP3(S365);UTP3(S368);VCAN(S2116);VCPIP1(S747);VPS4B(S102);WDFY4(S3123);WDR20(S434);WDR44(S403);WDR48(S335);WDR70(S638);WEE1(T190);WIPF1(S340);XRCC6(S477);XRN1(S1645);XRN2(S471);XRN2(S499);XRN2(S501);YAP1(S276);YAP1(S289);YAP1(S367);YBX1(Y162);YBX3(S370);YY1(S247);ZBTB21(S435);ZBTB37(S164);ZC3H13(S325);ZC3H13(S77);ZC3H18(S67);ZC3H18(S74);ZC3H4(S1114);ZC3HC1(S354);ZDHHC20(S305);ZEB2(S1122);ZFC3H1(S352);ZFC3H1(S949);ZFP91(S103);ZFPM1(S909);ZKSCAN8(S12);ZNF106(S641);ZNF106(T1372);ZNF280D(S545);ZNF281(T888);ZNF513(S85);ZNF516(T930);ZNF518A(S655);ZNF552(S86);ZNF609(S1055);ZNF687(S1191);ZNF687(S1211);ZNF814(S87);ZNRF2(S145);ZNRF2(S21);ZRANB2(S153)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>MAPK9</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>172</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>AGFG1(T177);AMBRA1(S1205);ARFGAP1(T135);ARHGAP17(S625);ARID1A(S363);ATP13A1(S899);ATRIP(S224);ATXN2(S624);ATXN2L(S424);BAP18(S110);BAZ1A(T1547);BAZ1B(S349);BRD4(S1117);CBX8(S110);CDCA3(S29);CHAMP1(S382);CHAMP1(S416);CLASP2(S952);CPEB2(S89);CPEB2(S92);CREB1(S271);CRMP1(S522);DDX21(S71);DENND4A(S1256);DTL(T429);EFHD2(S74);ESF1(S198);EZH2(S363);FARSA(S301);FBXW9(S59);FBXW9(T55);FGFR1OP(T170);FLYWCH2(S21);FTSJ3(T573);G3BP2(T227);GATAD2A(S340);GATAD2A(S546);GRB10(S104);GSK3A(Y279);GSK3B(Y216);GTF2I(T558);GTSE1(S536);H2AFY(T129);HCFC1(S666);HIRIP3(S27);HIST1H1E(T18);HJURP(S557);HMGA1(S36);HMGA1(T53);HMGXB4(S497);HNRNPA2B1(S259);HNRNPLL(S61);HSH2D(S194);HSPH1(S809);IGLL1(S58);INF2(S589);JPT1(T54);JPT2(S97);KIF18B(S413);KMT2A(S3511);LAMTOR1(S27);LIN54(S310);LMNB1(S23);LMNB1(S391);LMNB2(S405);LRCH3(S419);MARK2(S456);MCM4(S120);MEPCE(T213);MKI67(S1207);MKI67(S2223);MKI67(S2344);MKI67(T2231);MPLKIP(S115);MPLKIP(T51);MPLKIP(Y45);MRGBP(S195);MTMR2(S58);MYBBP1A(S1290);MYO9B(S1405);MYO9B(S717);NAV2(S1245);NCL(T121);NCOR2(S956);NFIC(S323);NFRKB(S1291);NOLC1(S397);NONO(T450);NOP2(S732);NUMA1(T2000);NUP210(S1877);ORC2(T116);ORC6(T195);PALM3(S303);PDCD4(S94);PHC3(S315);PHKA2(S1043);PHRF1(S867);PI4KB(S266);PIAS1(S488);PLEKHA5(T438);PLPPR3(S508);PPP1R14B(S32);PPP6R1(S759);PQBP1(S247);PRRC2C(S779);PSMF1(S153);RAB40C(S268);RAD18(S103);RANBP2(T1396);RB1(T601);RBL1(S1041);RBL1(S762);RBL1(T369);RBL2(S1112);RBL2(S413);RBMX(S208);RBMXL1(S208);REPIN1(S27);RRP1B(S732);RSF1(S392);RSF1(S397);SACS(S1779);SAMD1(S161);SATB1(S637);SCFD1(S303);SCML2(S267);SF3B1(T223);SF3B1(T227);SHROOM3(S242);SLAIN2(S63);SNRK(S518);SNTB1(S87);SP2(S78);SPTY2D1(S471);SRCAP(S3148);SRRM2(S2382);SRSF11(S207);SURF6(T229);TAF9(T159);TCF20(S1335);TCOF1(S1257);TCOF1(S156);THOC2(T1443);THRAP3(S253);TICRR(S923);TP53BP1(S265);TTF1(S65);TTF2(S883);TUBA1A(S48);TUBA1B(S48);TUBA1C(S48);TUBA3C(S48);TUBA3E(S48);UFD1(S247);USP36(S546);WBP11(S237);WIPI2(S413);WIZ(S1012);WIZ(S996);XRCC1(S226);XRCC1(S229);XRCC1(S241);XRCC1(S266);XRCC1(T198);ZC3H11A(T321);ZC3H4(S908);ZNF574(S164);ZNF587B(S87);ZNF638(S1401);ZYX(S259);ZYX(S267)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>MAPKAPK2</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>44</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>AFF1(T372);AFF1(T376);AGAP1(S605);AKT1S1(T246);ANKRD17(S2401);ASAP2(S822);C2CD2(S649);C9orf78(T100);CANX(S564);CNOT2(S170);CRKL(Y207);DDX17(S571);DHX57(S77);DLG5(S1232);EEF2K(S72);EEF2K(S74);EEF2K(Y69);EHMT2(S232);F11R(S284);FAM53C(S122);HAUS6(T584);IRS2(S577);KMT2D(S3130);MPHOSPH8(S403);MTMR14(S530);MYC(S62);MYCN(S62);NCOR1(S1472);NDRG3(S334);NOL8(S432);PAK2(S58);PATL1(T194);PRAG1(S889);RFC1(S71);RFC1(Y67);RNF2(S168);RREB1(S1167);RRP1B(S458);SLC4A7(T559);TSC1(S505);UPF3B(T169);ZC3HAV1(T273);ZNRF2(S21);ZRANB2(S153)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>MARK2</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>14</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>AHNAK(S5830);BAIAP2(S366);BTF3(S30);CDC42EP4(S118);CIC(S173);DCLK1(S332);EGLN1(S125);EIF3A(S882);HMGCR(S872);LUC7L2(S18);MPRIP(S993);MTFR1L(S103);PPP1R12A(S445);SH3PXD2B(S291)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>MARK3</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>328</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>AAK1(T653);ADAM17(S791);AFAP1(S668);AFDN(S1318);AGAP3(S538);AGPS(S65);AHCTF1(S1142);AHNAK(S5739);AJUBA(S263);AKAP13(S1559);AKAP13(S1929);ALKBH5(S361);AMPD2(S100);ARFGAP2(S368);ARHGAP21(S476);ARHGAP45(S23);ARHGEF2(T152);ARHGEF6(S684);ATG2A(S498);ATL1(S10);BAD(S99);BAG6(S1081);BAIAP2(S366);BAZ1B(S1468);BCL9(T315);BCL9L(S750);BTF3(S30);C1orf198(S175);C1orf226(S18);CAD(S1406);CAMSAP3(S431);CASC1(S504);CASP3(S26);CBL(S486);CCDC85C(S246);CCSER1(S448);CDC25B(S230);CDC25B(S238);CDC25B(S375);CDC42EP4(S118);CDC42EP4(T23);CDK12(S383);CDK12(S385);CDK12(T893);CDK14(S24);CDK17(S180);CGN(S149);CHD4(S1531);CHD8(S1995);CIC(S173);COIL(T303);COL4A3BP(S373);CRIP2(S115);CRTC1(S153);CRTC3(S370);CTNND1(S349);DBNL(T291);DCLK1(S332);DLGAP4(T975);DVL3(S125);EGLN1(S125);EHBP1L1(S310);EIF3A(S1188);EIF3A(S1336);EIF3A(S882);EIF4B(S207);EIF4ENIF1(S564);EIF4G1(S1187);EIF4G1(S1194);ELAVL1(S202);EML3(S176);EPB41(S709);EPB41L1(S510);EPN2(S173);ESS2(T386);ESYT1(S627);FAM102A(S189);FAM102B(S228);FAM117A(S29);FERMT3(S15);FNBP4(S18);FRMD6(S522);FRMD6(S525);FRS2(S211);FYTTD1(S16);GAB1(S419);GAB2(S141);GAB2(T391);GAPVD1(S902);GOLGA4(S71);GON4L(S206);GSK3A(S21);GTF2I(S412);GTF3C2(S167);GTSE1(S575);HIPK1(Y352);HIPK2(Y361);HMGA1(S44);HMGCR(S872);HNRNPA2B1(S149);HSH2D(S194);ICE1(S1712);IGLL1(S62);IQSEC1(S180);IRS2(S306);JUP(S665);KHDRBS1(S20);KIF13B(S1410);KIF21A(S855);KIFC1(S351);KLC2(S582);KLC2(S610);KRT8(S43);LARP1(S824);LINC00337(S30);LSM14B(S165);LUC7L2(S18);LUC7L2(S347);LZTS1(S233);MACF1(S7279);MAP2(S1555);MAP3K1(S292);MAP3K2(S153);MAP3K20(S727);MAP3K4(S1274);MAP4(S1073);MAP4(S928);MAP7D1(S113);MARK3(S400);MAST2(S148);MAST3(S747);MELK(S505);MELK(S529);MEPCE(S152);MFSD10(S271);MINK1(S733);MISP(S394);MKI67(T1557);MPRIP(S993);MTA1(T564);MTFR1L(S103);MTFR1L(S238);MTMR12(S564);MVB12A(S170);MYCBP2(S2749);MYCBP2(S2751);MYH10(S1937);MYOF(S1915);NAB2(S193);NCBP1(S22);NCOA3(Y574);NCOR1(S70);NFX1(Y48);NHSL1(S1233);NKTR(T1155);NUP214(S678);NUP214(T670);OSBP(S379);OSER1(S82);OSER1(S84);PAK1(S144);PAK4(S163);PALM3(S303);PARD3(S717);PBRM1(S13);PBRM1(S14);PDHA1(S300);PDHA2(S298);PDS5A(T1208);PHACTR1(S505);PHAX(S368);PHLDB1(S334);PI4KB(S428);PIGT(S235);PITPNM1(T665);PKD2(S832);PKP2(S329);PLCG1(S1263);POLH(S380);POLM(S12);POLR2A(S1868);POLR2A(S1878);POLR2A(S1910);POLR2A(Y1860);PPFIBP1(S466);PPFIBP1(S601);PPHLN1(S133);PPIP5K2(S1074);PPP1CA(T320);PPP1R12A(S445);PPP1R35(S87);PPP1R35(T84);PPP1R9B(S100);PRC1(S4);PRPF6(S279);PRPF6(T275);PRRC2A(S1386);PRRC2C(S1544);PTK2(S716);PTPN12(S435);PTPN12(S449);PTPN14(S760);PUM1(S124);RABEP1(S377);RABEP2(S193);RALGAPA1(S797);RALY(S135);RANBP1(S60);RASAL3(S51);RASAL3(S865);RB1(T601);RBBP6(S873);RBL1(S640);RBL1(T369);RBM15(S700);RBM15B(S113);RBM15B(S265);RBM15B(S267);RBM15B(T532);RBM23(S140);RBM23(S142);RBMX(S208);RBMX(S326);RBMX(S332);RBMX(S352);RBMX(S88);RBMXL1(S208);REEP4(S152);RLIM(S228);RLIM(S230);RPA1(T180);RPL28(S115);RPS14(S139);RPS27(S78);RPS27L(S78);SAFB(S601);SAFB(S604);SAMD1(T107);SASH1(S90);SCAF1(S874);SCAF11(S796);SCRIB(T475);SDAD1(S585);SF3B1(T261);SF3B1(T434);SF3B1(T436);SGPP1(S101);SH3BP4(S296);SH3KBP1(S410);SH3PXD2B(S291);SHROOM2(T647);SIK3(S866);SIPA1(S839);SLAIN2(S413);SLC4A10(S238);SLC4A7(S233);SLTM(S1014);SLTM(S553);SMAP2(S240);SMARCA4(S610);SMARCD1(S206);SMARCD2(S229);SMARCD3(S181);SMCR8(S489);SNRPA1(T180);SPAG9(S730);SPAG9(S733);SPECC1(S914);SPTAN1(S1031);SRRM2(S1458);SRSF10(S133);SRSF4(S113);SRSF4(S446);SRSF5(S117);SRSF6(S119);SSH3(S37);SSSCA1(S78);STIM2(S680);STIM2(S719);STK4(S414);STX17(S289);STXBP5(S759);SURF6(T229);TBC1D1(S237);TBC1D4(S588);TCOF1(S156);THRAP3(S232);TJP1(S968);TJP2(T462);TJP3(S369);TJP3(S371);TJP3(S591);TMEM201(S441);TNKS1BP1(S429);TNKS1BP1(S983);TP53BP1(S1317);TRA2A(T202);TRA2B(T201);TRA2B(T212);TRAF4(S426);TRAPPC10(S711);TRIM11(S85);TRIP10(S296);ULK1(S556);ULK1(S719);USP32(S1416);USP54(S1036);USP6(S1214);UTP20(T1741);VIPAS39(S121);WASHC2A(S728);WASHC2C(S726);WDR44(T163);YBX3(S293);YEATS2(S536);ZC3H13(T364);ZC3H3(S571);ZC3HAV1(S257);ZC3HAV1(S335);ZC3HAV1(T273);ZC3HAV1(Y348);ZC3HC1(S354);ZMYND8(S425);ZNF136(S405);ZNF185(S64);ZNF408(T322);ZNF609(S1055);ZP2(S454)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>MAST1</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>107</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>ACIN1(S838);AHCTF1(S528);AKAP11(S1580);AKAP11(S422);AKAP11(S448);ANAPC1(S355);ANP32B(T244);ARHGEF17(S735);ARHGEF18(S1111);ATAD2(S327);ATN1(S661);ATN1(T653);BRIP1(S956);C7orf50(S175);CALU(S35);CALU(S44);CCDC9(S376);CDC25C(S216);CEP55(S428);CHAMP1(S376);CIT(S1322);CMTR1(S31);CNK3/IPCEF1(S892);DNTTIP2(T172);DOCK7(S946);EAF2(S22);EIF4B(S283);EPB41L1(S784);FAM122A(S189);FAM129B(S696);FIP1L1(S259);FUS(S462);FXR2(T411);GAB2(S141);GATAD2B(S486);GIGYF2(S26);GTF3C2(S167);HCFC1(S666);HNRNPA2B1(S344);HPS5(S534);HSPB1(S15);INCENP(T292);INTS12(S128);IPCEF1(S430);IRF2BP2(S318);KCAB2_HUMAN_Phospho (ST);LMNB2(S37);LSR(S464);LSR(T453);MAP7(S365);MDC1(T378);MED1(T1051);MKI67(S584);MTMR3(S613);MTMR3(Y614);MYC(T58);NADK(S48);NCOR2(S2424);NOLC1(S643);NOP58(S351);NUMA1(S1862);OSBPL8(S68);PAGR1(S237);PBRM1(S13);PCBP1(S190);PCNP(T139);PCYT1A(S315);PCYT1B(S315);PDZD8(S521);PEA15(S116);PKP4(S314);PLEKHA5(T857);PML(S505);POLM(S372);PPP1R9B(S100);PXN(S85);RAF1(S259);RALY(S135);RANBP2(S2900);RB1(T356);RBM15(S294);RBM15(S622);RBM39(S97);RBM39(Y95);RPRD2(T732);SCRIB(S1348);SEC31A(S799);SF3B1(T303);SFSWAP(S909);SHANK2(S67);SLX4(S1028);SNRNP200(S225);SNURF(S32);STMN1(S38);SYNJ1(S1053);THOC5(S314);THRAP3(S575);THRAP3(S928);TLE3(S267);TLN1(S425);TMEM238(S175);UBE2O(T838);UPF3B(T169);USP10(S211);VCL(S290);VGLL4(S149);ZFP64(S547)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>MELK</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>317</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(S30);09/09/18 00:00:00(T142);AAK1(T653);ABI2(S368);ABLIM1(S706);ADAM17(S791);AFAP1(S668);AFDN(S1318);AFF4(S487);AGAP3(S538);AGPS(S65);AHNAK(S5739);AJUBA(S263);AKAP13(S1559);AKAP13(S1929);ALKBH5(S361);AMBRA1(S1205);AMPD2(S100);ANLN(S485);ARFGAP2(S368);ARFGAP2(S432);ARHGAP21(S476);ARHGAP45(S23);ARHGEF2(T152);ARHGEF6(S684);ARPC1B(T315);ATG2A(S498);ATL1(S10);BAG6(S1081);BAIAP2(S366);BCL9(T315);BTF3(S30);C1orf198(S175);CASC1(S504);CASP3(S26);CASP8AP2(S567);CBL(S486);CCDC85C(S246);CCSER1(S448);CDC25B(S230);CDC25B(S238);CDC25B(S375);CDC42EP4(S118);CDC42EP4(T23);CDC42SE1(S74);CDK12(S383);CDK12(S385);CDK12(T893);CDK14(S24);CDK14(S78);CHD4(S1531);CHD8(S1995);CIC(S173);CRTC1(S153);CRTC3(S370);CRTC3(S62);CTNND1(S349);CTU2(S419);DBNL(T291);DCLK1(S332);DENND4A(S1256);DENND4C(S1099);DLGAP4(T975);DVL3(S125);EGLN1(S125);EIF3A(S1188);EIF3A(S1336);EIF3A(S882);EIF4B(S207);EIF4G1(S1092);EIF4G1(S1194);ELAVL1(S202);EPB41(S709);EPB41L5(S436);EPN2(S173);ESS2(T386);ESYT1(S627);FAM102A(S189);FAM117A(S29);FAM53C(S232);FERMT3(S15);FRMD6(S522);FRMD6(S525);FRS2(S211);FUBP3(S569);FYTTD1(S16);GAB2(S141);GAB2(T391);GAPVD1(S902);GON4L(S206);GRAMD1A(S263);GTF2I(S412);GTSE1(S575);HID1(S593);HIPK1(Y352);HIPK2(Y361);HMGA1(S44);HMGCR(S872);HSH2D(S194);HSPB1(S82);HTT(S1199);ICE1(S1712);IGLL1(S62);IQSEC1(S180);IRS1(S1145);IRS1(S374);JPH1(S216);JUP(S665);KHDRBS1(S20);KIF13B(S1410);KIF21A(S855);KIFC1(S351);KLC2(S610);LARP1(S824);LINC00337(S30);LMNA(S628);LSM14B(S165);LUC7L2(S18);LUC7L2(S347);LZTS1(S233);MACF1(S7279);MAP2(S1555);MAP3K1(S292);MAP3K2(S153);MAP3K20(S727);MAP3K4(S1274);MAP4(S928);MAP7D1(S113);MAP7D1(S399);MARK2(S456);MARK3(S400);MAST2(S1364);MAST3(S747);MELK(S505);MELK(S529);MFSD10(S271);MKI67(T1557);MPRIP(S993);MTA1(S639);MTFR1L(S103);MTFR1L(S238);MVB12A(S170);MYCBP2(S2749);MYCBP2(S2751);MYH10(S1937);MYOF(S1915);NAB2(S193);NAV1(S1265);NCBP1(S22);NCOA3(S857);NCOA3(Y574);NDRG2(T334);NFX1(Y48);NHSL1(S1233);NLN(S485);NOP58(S351);NUP214(S1023);OSER1(S82);OSER1(S84);OTUD4(S416);PAK4(S163);PALM3(S303);PARD3(S717);PBRM1(S13);PBRM1(S14);PCM1(S1958);PDHA1(S232);PDS5A(T1208);PHAX(S368);PHLDA2(S144);PHLDB1(S334);PI4KB(S428);PIGT(S235);PKD2(S832);PKP2(S329);PLCG1(S1263);POLH(S380);POLM(S12);POLR2A(S1868);POLR2A(S1878);POLR2A(S1910);POLR2A(Y1860);PPFIBP1(S466);PPFIBP1(S601);PPHLN1(S133);PPIP5K2(S1074);PPP1R12A(S445);PPP1R12A(S554);PPP1R35(S87);PPP1R35(T84);PPP1R9B(S100);PRAM1(S334);PRC1(S4);PREX1(S1182);PRPF6(S279);PRPF6(T275);PRRC2A(S1386);PRRC2C(S1544);PTK2(S716);PTPN12(S435);PTPN12(S449);PTPN14(S760);PUM1(S124);R3HDM1(S381);RABEP1(S377);RABEP2(S193);RALGAPA1(S797);RANBP1(S60);RAPGEF6(S1237);RAPGEF6(S1241);RASAL3(S51);RB1(S249);RB1(T601);RBL1(S640);RBL1(T369);RBL2(S413);RBM15(S700);RBM15B(S113);RBM15B(S265);RBM15B(S267);RBM15B(T532);RBM23(S140);RBM23(S142);RBMX(S208);RBMX(S326);RBMX(S332);RBMX(S352);RBMX(S88);RBMXL1(S208);RICTOR(S1284);RLIM(S228);RLIM(S230);RPL28(S115);RPS14(S139);SAFB(S601);SAFB(S604);SAMD1(T107);SASH1(S90);SCAF1(S874);SCAF11(S796);SCAMP2(S320);SCRIB(T475);SF3B1(T261);SF3B1(T434);SF3B1(T436);SGPP1(S101);SH3BP4(S296);SH3PXD2B(S291);SHROOM2(T647);SIK3(S866);SIPA1(S839);SLAIN2(S413);SLC4A10(S238);SLC4A7(S233);SLTM(S1014);SLTM(S551);SLTM(S553);SMAP2(S240);SMARCA4(S610);SMARCD1(S206);SMARCD2(S229);SMARCD3(S181);SMCR8(S489);SPAG9(S730);SPAG9(S733);SPTAN1(S1031);SRRM1(S429);SRRM2(S1458);SRSF10(S133);SRSF4(S113);SRSF4(S446);SRSF5(S117);SRSF6(S119);SSH3(S37);SSSCA1(S78);STIM2(S680);STIM2(S719);STX17(S289);SURF6(T229);SVIL(S968);TBC1D1(S237);TBC1D22A(S167);TCOF1(S156);THRAP3(S232);TJP1(S968);TJP2(T462);TJP3(S369);TJP3(S371);TJP3(S591);TMEM201(S441);TNKS1BP1(S429);TNKS1BP1(S983);TNS3(S363);TP53BP1(S1317);TRA2A(T202);TRAF4(S426);TRAFD1(S470);TRAPPC10(S711);TRIM11(S85);TRIP10(S296);TTC28(S2224);ULK1(S556);ULK1(S719);USP54(S1036);UTP20(T1741);YBX3(S293);ZC3H13(T364);ZC3H3(S571);ZC3HAV1(S257);ZC3HAV1(S335);ZC3HAV1(T273);ZC3HAV1(Y348);ZMYM4(S242);ZMYND8(S425);ZNF136(S405);ZNF408(T322);ZNF609(S1055)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>MINK1</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>1007</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>09/06/18 00:00:00(T418);09/07/18 00:00:00(T426);09/09/18 00:00:00(S30);09/09/18 00:00:00(T142);AAK1(S14);ABCF1(S140);ABI1(S216);ABI1(S231);ABI1(Y213);ABI2(S368);ABL1(S569);ABLIM1(S431);ABLIM1(S655);ABLIM1(S706);ABR(T74);ACIN1(T414);ACTA1(S241);ACTA2(S241);ACTB(S239);ACTBL2(S240);ACTC1(S241);ACTG1(S239);ACTG2(S240);ADAD2(S522);ADAM10(S740);ADAM10(Y741);ADAM17(S791);ADD1(S12);ADD1(S431);ADD1(S726);ADD2(S713);ADD3(S693);AEBP2(S390);AFDN(S1721);AFF4(S1043);AFF4(S1058);AFF4(S32);AFF4(S487);AFF4(S836);AGAP2(S808);AHCTF1(S528);AHDC1(S1064);AHDC1(S1507);AHNAK(S115);AHNAK(S216);AHNAK(S3412);AHNAK(S3426);AKAP11(S1580);AKAP11(S422);AKAP11(S448);AKAP13(S1565);AKAP13(S2728);ALDH5A1(S122);AMBRA1(S1205);AMBRA1(S639);AMOTL2(S183);ANAPC1(S355);ANKRD17(S2401);ANKRD34A(S291);ANKS1A(S382);ANKS1A(S887);ANKZF1(S675);ANLN(S485);ANLN(S661);ANP32B(T244);APPL1(S401);ARFGAP1(S361);ARFGAP2(S368);ARFGAP2(S432);ARHGAP1(S44);ARHGAP1(S51);ARHGAP17(S625);ARHGAP21(S856);ARHGAP29(S499);ARHGAP29(S930);ARHGEF11(S150);ARHGEF11(S35);ARHGEF17(S735);ARHGEF26(S98);ARID1A(S1184);ARID1A(S1600);ARID1A(S1604);ARID1A(S363);ARID1A(S730);ARID3B(S381);ARL6IP6(S80);ARVCF(T642);ASIC3(S37);ATAD2(S327);ATAD2B(S318);ATF1(S198);ATF7IP(S113);ATG2B(S1582);ATG2B(S1583);ATG2B(Y1577);ATN1(S661);ATN1(T653);BCAM(S600);BCAR3(S317);BCL11A(S328);BCL2L12(S113);BCL2L12(S121);BCL2L12(T117);BCL9L(S915);BCLAF1(S183);BCLAF1(S274);BCR(S459);BICRA(S1413);BIN2(S259);BRD4(S1064);BRD4(S1126);BRIP1(S956);BRSK2(S423);BRSK2(T459);BRSK2(T463);BUB1(S655);BUD23(S240);C11orf95(S408);C16orf54(S194);C19orf47(S151);C2CD2L(S662);C2CD5(S281);C2CD5(S662);C6orf132(S449);C7orf50(S175);CABLES1(S291);CAD(S1859);CALU(S35);CALU(S44);CAMSAP1(S563);CAMSAP2(S464);CAMSAP3(S431);CARMIL2(S1315);CASP8AP2(S567);CAT(S515);CBL(S619);CBL(S799);CBX8(S311);CBY1(S20);CCDC130(S332);CCDC18(S1355);CCDC6(S240);CCDC6(T434);CCDC9(S376);CCDC93(S305);CCL13(S44);CCNK(S9);CCNY(T75);CCNYL1(T97);CCZ1(S368);CCZ1B(S368);CD2AP(T87);CD97(S818);CD97(S831);CDC25C(S216);CDC42EP4(S80);CDCA7L(S261);CDK1(T161);CDK11A(T583);CDK12(S383);CDK12(S385);CDK13(T1056);CDK14(S78);CDK9(S347);CDV3(T182);CENPF(S276);CENPF(S2996);CEP170(S881);CEP55(S428);CEP97(S308);CHAF1A(S206);CHAMP1(S308);CHAMP1(S319);CHAMP1(S376);CHAMP1(S432);CHAMP1(S436);CHAMP1(S445);CHAMP1(S452);CHAMP1(S472);CHAMP1(S507);CHD1L(T629);CHD2(S1728);CHD4(S303);CHD8(S1978);CHD8(T1982);CHEK1(S280);CHTF18(S64);CIT(S1322);CLASP1(S636);CLASP2(S325);CLASP2(S529);CLASRP(S547);CLCC1(S532);CLIC6(S293);CLINT1(S299);CLINT1(T308);CLINT1(Y293);CLK2(S142);CLK3(S283);CMTR1(S31);CNK3/IPCEF1(S892);CNP(S170);CNTROB(S62);COL4A3BP(S373);CPSF7(S48);CREB1(S111);CREB1(S271);CRKL(Y207);CRTC2(S178);CRTC3(S329);CSPP1(S901);CTAGE1(S616);CTAGE5(S647);CTNNAL1(S538);CTNND1(S230);CTNND1(T906);CTPS1(S573);CTU2(S419);CUX1(S1218);CYBA(T147);DACH1(S727);DAP(S51);DAXX(S671);DBF4(S381);DBNL(T291);DCAF12(S15);DCP1B(S275);DDX21(S89);DDX3Y(S592);DENND4A(S1256);DENND4A(T1019);DGCR8(S271);DGCR8(S275);DGCR8(Y267);DIP2B(S259);DLG5(S1000);DLG5(S1254);DLG5(S1795);DLG5(T984);DLGAP5(S725);DNAAF2(T703);DNAJB6(S277);DNM1(S619);DNM2(S619);DNTTIP2(S434);DNTTIP2(T172);DOCK7(S898);DOCK7(S946);DOCK8(S451);DTL(S425);DUSP27(S966);DYNC1LI1(S398);DYNC1LI1(T513);EDC3(S131);EEF2(T57);EEF2K(S72);EEF2K(S74);EEPD1(S21);EIF2B1(S107);EIF3A(S584);EIF3E(S399);EIF4B(S406);EIF4EBP1(T41);EIF4EBP2(T46);EIF4EBP2(Y34);EIF4G1(S1092);EIF4G3(S230);EML4(S144);EML4(S146);ENAH(S531);ENAH(T538);EP400(S722);EP400(S736);EPB41L1(S784);EPS15L1(S793);EPX(S672);ERCC5(S384);ERRFI1(S461);ETV4(S140);EVL(S331);EVL(S369);EZH2(S363);EZH2(T367);FADD(S194);FAM102B(S228);FAM117A(S193);FAM117B(S10);FAM122A(S143);FAM122A(S189);FAM129B(S665);FAM129B(S681);FAM129B(S696);FAM207A(T34);FAM47A(S259);FAM53B(S179);FAM53C(S232);FAM53C(S234);FAM76B(S193);FAM83B(S766);FAM83H(S914);FANCI(S1121);FARSA(S301);FBRSL1(T1010);FBXW9(S59);FGD6(S692);FIP1L1(S259);FLNB(S1505);FNBP1(S296);FNBP1L(S501);FNDC3A(S203);FNDC3A(S206);FNDC3B(S208);FOXK1(S416);FOXK1(S420);FOXK1(S441);FOXO1(S329);FRMD3(S416);FRMD4A(S604);FUS(S462);FXR2(S601);FXR2(T411);GAB2(S141);GAGE13(S33);GAGE2A(S32);GAGE2B(S32);GAGE2D(S32);GAPVD1(S902);GATAD2A(T189);GATAD2B(S334);GATAD2B(S486);GBF1(S1061);GBF1(S1298);GFI1(S94);GIGYF2(S236);GIGYF2(S26);GIT1(S592);GJA1(S262);GNL3(S529);GORASP2(T415);GPATCH2(S195);GPATCH8(S1033);GRAMD1A(S263);GRIP1(S847);GSE1(S909);GSK3B(S25);GSK3B(S9);GTF2F1(S385);GTF2F1(T389);GTF2F1(T446);GTF3C2(S132);GTF3C2(S167);HCFC1(S598);HCFC1(S666);HCLS1(T308);HDAC1(S406);HECTD1(S1387);HELB(S1050);HIC2(S348);HID1(S653);HMGCS1(T490);HNRNPA1(S199);HNRNPA1(S338);HNRNPA2B1(S344);HNRNPA3(S358);HNRNPAB(S242);HNRNPC(S253);HNRNPK(S379);HNRNPLL(S61);HNRNPM(S365);HNRNPM(S528);HNRNPM(S618);HNRNPU(S271);HPS5(S534);HRNR(S903);HSPB1(S15);HSPB1(S82);HUWE1(S1084);HUWE1(S2534);HUWE1(T2889);IBTK(S1045);IGLL1(S58);INCENP(T292);INPP5D(T963);INTS12(S128);IPCEF1(S430);IQSEC1(S107);IRF2BP1(S421);IRF2BP2(S175);IRF2BP2(S318);IRF2BP2(S406);IRF2BPL(S519);IRS2(S915);ITGAL(S37);ITSN1(S559);ITSN2(S884);ITSN2(S889);JADE3(S566);JMJD1C(S1223);JMJD1C(S641);JPH1(S216);JPT2(T76);JUN(S63);KANK2(S172);KANK2(S175);KANSL3(S535);KAT7(S57);KCAB2_HUMAN_Phospho (ST);KCNK2(S366);KCTD12(S185);KDM3A(S445);KHDRBS1(S20);KHDRBS1(T33);KHSRP(T100);KIAA0319L(S978);KIAA1217(S357);KIAA1217(S361);KIAA1468(T143);KIAA1522(S858);KIAA1522(S862);KIAA1522(S929);KIAA1551(S1358);KIAA1551(S715);KIAA1671(S1224);KIDINS220(S1411);KIDINS220(Y1416);KIF1A(S1094);KIF1A(S1528);KIF1A(S1532);KIFC1(S351);KMT2B(S2348);KNOP1(S119);KPNA4(S60);KRT13(S427);KRT8(S330);KRT8(S36);L1TD1(S173);L1TD1(S557);LAD1(S301);LAMTOR1(S27);LARP1(S1056);LARP1(S90);LARP1(T526);LARP7(S337);LARP7(T338);LAT2(S135);LAT2(S86);LEMD2(S82);LEMD3(S187);LIMA1(S617);LIN28B(S203);LIN54(S310);LIN54(S314);LINC00322(S226);LMNA(S390);LMNB2(S37);LRCH1(S532);LRCH4(S520);LRMP(S363);LRRFIP1(S116);LRRFIP1(S120);LRRFIP2(S324);LSM11(S10);LSM11(S21);LSM14A(S178);LSM14A(S183);LSR(S464);LSR(T453);LTBP1(Y1422);LUZP1(S745);LUZP1(T441);LZTS1(S209);MACF1(S7330);MAGOH(S106);MAGOHB(S108);MAML1(S360);MAP1A(S1675);MAP1A(S1776);MAP2(S1540);MAP2(S1653);MAP2(T1649);MAP3K2(S239);MAP4(S1073);MAP7D1(S93);MAPKAP1(S510);MARCKS(S163);MARK1(S588);MARK2(S619);MARVELD2(S120);MAST2(S1032);MAST2(S74);MAST2(S876);MAZ(S361);MCM3(Y708);MCM3AP(S557);MDC1(T378);MEPCE(S217);MEPCE(T213);MEX3B(S442);MEX3D(S514);MFAP1(S116);MFSD10(S271);MFSD2B(S494);MIA2(S1255);MIA3(S1741);MICAL3(S649);MICALL1(S391);MICALL1(S486);MICALL1(S640);MICALL2(S143);MICALL2(S153);MIS18BP1(S1042);MIS18BP1(S594);MISP(S394);MKI67(S2223);MLC1(S179);MLLT6(S378);MLLT6(S382);MORC2(S696);MORC2(S725);MSANTD2(S27);MTA1(S386);MTA1(S449);MTA1(S522);MTA1(S639);MTA2(S435);MTFMT(S23);MTMR3(S613);MTMR4(S961);MTOR(S2448);MTOR(S2454);MTSS1L(S342);MTX3(S284);MYBBP1A(S11);MYC(T58);MYCBP2(S3467);MYCN(S156);MYO9B(S1405);MYO9B(T1271);NAA15(S759);NAA30(S199);NAB1(S403);NAB2(S171);NAB2(S479);NACA(S166);NACA(S2029);NADK(S48);NADK(S64);NASP(T390);NAV1(S808);NAV2(S1559);NAV2(S1808);NCAPD2(Y1325);NCOR1(S1980);NCOR1(S1981);NCOR2(S1331);NCOR2(S1547);NCOR2(S1783);NCOR2(S2424);NCOR2(S54);NDRG2(S332);NDRG2(T330);NDRG2(T334);NELFA(T212);NES(S768);NEXN(S160);NFATC2(S217);NFATC2(S814);NLN(S485);NMNAT1(S117);NOB1(S352);NOLC1(S397);NOLC1(S508);NOLC1(S622);NOLC1(S643);NONO(T450);NOP16(S16);NOP53(S29);NOP58(S351);NPM1(S260);NPM1(S70);NSD1(S2471);NSF(S437);NSFL1C(S114);NSRP1(S33);NUCKS1(T179);NUFIP2(S230);NUMA1(S1862);NUMA1(S1887);NUMBL(S263);NUP153(S209);NUP210(S1877);NUP210(S1881);NUP35(S66);OBSL1(S10);OSBP(S190);OSBP(S193);OSBPL8(S68);PABPN1(S150);PAGR1(S237);PAK4(S148);PANK2(S189);PARD3(S221);PARVA(S19);PATL1(S278);PBRM1(S12);PBRM1(S13);PBX2(S330);PCBP1(S190);PCBP1(S231);PCBP2(S272);PCM1(S1958);PCM1(T79);PCM1(T82);PCNP(T139);PCYT1A(S315);PCYT1A(S347);PCYT1B(S315);PDCD6IP(S730);PDLIM2(S129);PDLIM4(S112);PDS5B(T1301);PDZD8(S521);PEAK1(S823);PFKL(S775);PGK1(S203);PGRMC1(S181);PHACTR2(T25);PHF3(S1614);PHF8(S880);PHIP(S677);PHKA2(S1043);PHLDA2(S144);PI4K2A(S51);PIK3AP1(S759);PIK3C2A(S338);PIK3CD(T226);PIK3R4(T927);PKP2(S82);PKP3(S331);PKP4(S273);PKP4(S314);PLCB3(S926);PLEC(S1435);PLEKHA5(T857);PLEKHA6(S867);PLEKHG4B(S729);PLEKHG4B(T727);PLK1(T214);PLPPR3(S353);PML(S505);PODXL(S519);POLA2(T127);POLD2(S15);POLH(S380);POLM(S372);POM121(S298);POM121C(S275);POMZP3(S33);POTEE(S939);POTEF(S939);POTEKP(S239);PPFIBP1(S540);PPFIBP1(S636);PPHLN1(S163);PPHLN1(T200);PPIG(S356);PPME1(S15);PPP1CC(T311);PPP1R13L(S358);PPP1R9B(S100);PRAG1(S510);PRAG1(S782);PRKD1(S205);PRKD1(S208);PRKDC(T1045);PRKRA(S18);PRPF4B(S852);PRPF4B(Y849);PRR12(S314);PRR36(T1082);PRRC2A(S1147);PRRC2A(S2113);PRRC2C(S1568);PSMF1(S153);PTDSS2(S16);PTPN1(S378);PTPN22(S414);PTPN22(T450);PUM1(S209);PXN(S85);R3HDM2(S349);RABL6(S359);RAF1(S642);RALB(S6);RALGAPB(T379);RANBP2(S2454);RANBP2(S2900);RANBP3(S108);RANBP3(S211);RANBP9(S477);RANBP9(S482);RAPGEF2(S585);RASAL2(S634);RASAL2(S635);RASAL3(S18);RASGRP2(S391);RAVER1(T463);RB1(S788);RB1(T356);RB1(Y790);RBL1(S749);RBL1(T369);RBM10(S845);RBM14(S618);RBM15(S294);RBM15(Y266);RBM15B(S265);RBM15B(S562);RBM17(S169);RBM39(S97);RBM39(Y95);RBM6(S1025);RBMX(S208);RBMX(S249);RBMX(S326);RBMX(S352);RBMXL1(S208);RBMXL1(S249);RBMXL1(S326);RBMXL1(S88);RECQL5(S815);REPS1(S709);REXO4(S15);RFX1(S204);RFX7(S1028);RGPD1(S1463);RGPD2(S1471);RGPD3(S1479);RGPD4(S1479);RGPD5(S1478);RGPD8(S1478);RICTOR(S1284);RIF1(S1688);RIF1(S2205);RIF1(T1047);RPGR(S518);RPL18(S161);RPL18(T158);RPL5(S286);RPRD2(S665);RPRD2(T732);RPS10(S146);RPS10P5(S157);RPS14(T140);RPS27(S11);RPS27(S78);RPS27L(S78);RPS28(S23);RRP1B(S735);RSL1D1(S392);RSL1D1(S396);SACS(S1779);SALL2(S806);SAMD1(S161);SAMD4B(S172);SARNP(S163);SASH3(S21);SCFD1(S303);SCML2(S267);SCRIB(S1348);SCRIB(S1448);SCRIB(S504);SCYL3(S707);SDAD1(S585);SEC16A(S1194);SEC16A(S1905);SEC31A(S799);SEPT9(S22);SET(S7);SF3B1(S129);SF3B1(T303);SF3B1(T313);SFSWAP(S909);SGO1(S468);SH3BP2(S427);SH3BP4(S246);SH3BP5L(S362);SHANK2(S67);SHC3(S474);SHROOM3(S1497);SHROOM3(T576);SHTN1(S506);SIK3(S551);SIK3(T469);SIPA1L3(S1364);SKIV2L(S131);SLAIN2(S377);SLC20A2(Y389);SLC9A1(S703);SLTM(S1014);SLTM(S551);SLX4(S1309);SLX4(S1333);SMARCA2(S588);SMARCAD1(S146);SMG7(S781);SMNDC1(S201);SND1(S426);SNRK(S518);SNRNP200(S225);SNRNP70(S226);SNURF(S32);SNX17(S336);SNX17(S409);SOWAHD(S67);SPECC1(S55);SPECC1(S914);SPEG(S2109);SPEN(S1918);SPEN(T2421);SPN(S291);SRPK1(S309);SRRM1(S234);SRRM1(S695);SRRM2(S1499);SRRM2(S323);SRRM2(S377);SRRM2(S435);SRRM2(S510);SRRM2(S774);SRRM2(S876);SRRM2(T1413);SRRM2(T400);SRRT(S74);SRSF1(S199);SRSF1(S201);SRSF9(S216);SSB(S366);ST6GALNAC4(S298);STAM(S156);STIM2(S523);STK10(S450);STK17A(S28);STK3(T174);STK4(T177);STMN1(S38);STX7(S131);SUPT6H(T1523);SURF6(S138);SVIL(S968);SYNJ1(S1053);SYTL2(S344);SZRD1(S107);TACC1(S276);TACC3(S250);TACC3(S317);TAF7(S201);TAGLN2(S185);TAGLN3(S185);TANC2(S169);TAOK1(S965);TATDN2(S80);TBC1D1(S211);TBC1D10B(S658);TBC1D10B(S661);TBC1D10B(T697);TBC1D22A(S167);TBC1D4(S588);TBC1D9B(S435);TBX2(S653);TCF20(S574);TCOF1(S1227);TCOF1(S1378);TCOF1(S503);TCOF1(T914);TEX2(S732);THAP4(S128);THOC5(S314);THRAP3(S248);THRAP3(S575);THRAP3(S928);THYN1(S14);TICRR(T1260);TJAP1(S320);TJAP1(T318);TJAP1(Y316);TJP1(S617);TJP2(S266);TK1(S231);TLN1(S425);TMPO(S306);TMPO(S354);TMX1(S270);TMX2(S288);TNIK(S764);TNIK(S766);TNKS1BP1(S1103);TNRC18(S1644);TNRC6C(S714);TNS2(S1003);TOM1(S464);TOR1AIP1(S135);TP53BP2(S121);TP53BP2(S558);TPD52L2(S166);TPR(S379);TRA2B(T201);TRA2B(T212);TRAFD1(S470);TRIM24(S654);TRIM37(S771);TRIM71(S187);TRIP12(S312);TRIR(S114);TRIT1(S443);TRMT1L(S707);TRPM7(S1477);TRPS1(S216);TRPS1(T751);TSC2(S1448);TSC22D4(S24);TUBA1A(S48);TUBA1B(S48);TUBA1C(S48);TUBA3C(S48);TUBA3E(S48);TXLNG(S97);U2SURP(S37);UBAP2L(S605);UBE2C(S23);UBE2O(T838);UBE4B(S65);UBE4B(T64);UCK1(S253);UFD1(S299);UNC13B(S367);UNC93B1(S547);UNC93B1(S550);UNG(S23);UNG(T60);UPF3B(T169);USP10(S211);USP15(S242);USP20(S134);USP36(S682);USP36(S742);USP36(T653);USP7(S18);VASP(S239);VCL(S290);VCL(S755);VGLL4(S149);VIM(S25);VPS13D(S1042);WASHC2A(S1180);WASHC2C(S1157);WASHC2D(S147);WDFY4(S3123);WDR44(S561);WIPF1(S340);WIPI2(S413);WT1(S273);WWC3(S563);XPO4(S521);XPR1(S666);XRCC1(S226);XRCC1(T198);XRCC6(S477);YAP1(S164);YAP1(S289);YBX3(T67);YTHDC2(S1223);ZBTB21(S983);ZC3H15(S360);ZC3H3(S571);ZC3H4(S1114);ZCCHC8(S598);ZCCHC8(T479);ZCCHC8(T485);ZDHHC5(S425);ZFHX4(S2996);ZFP36L1(S334);ZFP36L2(S438);ZFP36L2(S490);ZFP64(S547);ZFP91(S101);ZFP91(S103);ZFYVE26(S1764);ZKSCAN8(S12);ZMYM4(S242);ZNF106(S893);ZNF24(S274);ZNF318(S136);ZNF318(S1896);ZNF318(S501);ZNF462(S1251);ZNF574(S164);ZNF592(S691);ZNF609(S578);ZNF639(S88);ZNF687(S374);ZNF75A(S287);ZNF75D(S491);ZSCAN5A(S296);ZSCAN5B(S295);ZYX(S308);ZYX(S344)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>MKNK2</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>26</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>CAMK1D(T184);DENND4A(S1256);DLG5(S1795);ERRFI1(S374);HID1(S653);KIF21A(S1304);KIF21A(S1307);MPLKIP(S115);MYC(S62);MYCN(S62);NEXN(S160);POM121C(S372);PTPN22(S414);RANBP3(S101);RAP1GAP2(S608);RPS10(S146);RPS10P5(S157);SAMD4B(S628);SF3A1(S329);SKA3(S110);SNX17(S333);SRRM2(S1501);SRRM2(S1502);XRN2(S499);XRN2(S501);ZMYM4(S122)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>MTOR</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>84</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>ALDH5A1(S121);ASAP2(S822);ASIC3(S39);C5orf30(S167);CAD(S1859);CCNL1(S338);CD2AP(S234);CD2AP(T236);DDX17(S571);DTNA(S662);DUSP27(S965);EEF2K(S72);EEF2K(S74);EEF2K(Y69);EHBP1L1(S310);EIF2B1(S105);EIF2B1(S107);EIF4EBP1(S65);EIF4EBP1(T41);EIF4EBP1(T46);EIF4EBP1(Y34);EIF4EBP2(T37);EIF4EBP2(T41);EIF4EBP2(T46);EIF4EBP2(T70);EIF4EBP2(Y34);EMSY(S209);EPX(S670);EPX(S672);FAM47A(S258);GRB10(S104);GRB10(S476);GSK3A(S21);GSK3B(S9);HCLS1(T308);HDGFL2(S454);HIPK1(Y352);HIPK2(Y361);IRS2(S620);IWS1(S720);KIFC1(S349);KIFC1(S351);LAMTOR1(S98);LARP1(S766);LARP1(Y777);LIMA1(S230);LINC00322(S228);MAF1(S60);MEPCE(S152);MFSD10(S270);MFSD2B(S491);MPG(S35);MTMR14(S530);NDRG3(S331);PATL1(S184);PATL1(T194);PCBP1(S264);PCBP2(S272);PCNP(S147);POGZ(S746);POLH(S379);PPP1R12C(S427);PRKAA2(S377);PUM1(S209);RAP1GAP2(S564);RBM14(S618);REPS1(T173);RPS6(S235);RPS6KB1(S441);SKIV2L(S133);SRRM2(S771);SRSF7(S167);TRIM33(S1119);TRIM37(S773);TTK(S436);WRNIP1(S75);XPR1(S668);YBX1(S209);ZC3H3(S569);ZC3H3(S571);ZNF609(S467);ZNF687(S1118);ZNF75A(S286);ZNF75D(S490)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>PAK1</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>460</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(S30);AAK1(T653);ABCF1(S140);ACACA(S80);ACIN1(S825);ADAM17(S791);ADGRL2(S1275);AEBP2(S390);AFAP1(S668);AFDN(S1318);AFF1(T372);AFF1(T376);AGAP3(S538);AGPS(S65);AHCTF1(S528);AHNAK(S5739);AJUBA(S263);AKAP1(S151);AKAP13(S1559);AKAP13(S1929);ALKBH5(S361);AMPD2(S100);AMPD2(S190);ARFGAP2(S368);ARFGEF2(S227);ARFIP1(S132);ARHGAP21(S476);ARHGAP21(T441);ARHGAP35(S1150);ARHGAP45(S23);ARHGEF11(S1413);ARHGEF16(S578);ARHGEF2(T152);ARHGEF6(S684);ARHGEF9(S502);ARPC1B(T315);ASAP1(S839);ATG2A(S498);ATL1(S10);AXIN1(S77);BAG3(T285);BAG6(S1081);BAIAP2(S366);BCAR3(S290);BCL11A(S630);BCL9(T315);BCL9L(S1017);BTF3(S30);C17orf53(S332);C1orf198(S175);CAD(S1406);CAD(S1900);CANX(S583);CAPRIN1(S21);CASC1(S504);CASC4(S233);CASP3(S26);CBL(S486);CCDC85C(S246);CCNY(S83);CCSER1(S448);CD2AP(S458);CDC25B(S230);CDC25B(S238);CDC25B(S375);CDC42EP4(S118);CDC42EP4(T23);CDC42SE1(S74);CDK12(S383);CDK12(S385);CDK12(T893);CDK14(S24);CDK16(S119);CDK17(S137);CDK17(S146);CDK17(S180);CEP350(S2115);CHD4(S1531);CHD8(S1995);CIC(S173);CRKL(Y207);CRTC1(S153);CRTC2(S178);CRTC2(S70);CRTC3(S370);CTAGE5(S594);CTAGE5(S596);CTAGE5(S635);CTNND1(S349);DBN1(S272);DCLK1(S332);DIP2B(S100);DIP2B(S53);DLG5(S1254);DLGAP4(T975);DOCK5(S1766);DOCK7(S888);DSP(S2209);DVL3(S125);EGLN1(S125);EIF3A(S1188);EIF3A(S1336);EIF3A(S584);EIF3A(S882);EIF4G1(S1092);EIF4G1(S1194);EIF4G2(S17);EIF5B(S214);ENAH(T538);EPB41(S709);EPN2(S173);ERF(S327);ESS2(T386);ESYT1(S627);ETV3(S159);EVL(S331);F11R(S284);FAM102A(S189);FAM102B(S228);FAM117A(S29);FAM117B(S136);FAM193A(S1144);FERMT3(S15);FGD1(S50);FNDC3A(S203);FRMD6(S522);FRMD6(S525);FRS2(S211);FYTTD1(S16);FZD6(S629);GAB1(S419);GAB2(S141);GAB2(T391);GAPVD1(S902);GNL1(S51);GON4L(S206);GTF2I(S412);GTSE1(S575);HCFC1(S669);HIPK1(Y352);HIPK2(Y361);HJURP(S486);HMGA1(S44);HMGCR(S872);HMGXB4(S197);HSH2D(S194);HSPB1(S82);ICE1(S1712);ID2(S14);IGLL1(S62);INSRR(S72);INTS1(S13);IQSEC1(S180);JPH1(S216);JPH1(S452);JUN(S63);JUP(S182);JUP(S665);KDM2A(S731);KDM5A(S1331);KIF13B(S1410);KIF21A(S855);KIFC1(S351);KLC2(S610);KMT2A(S2151);KRT8(S43);LAD1(S301);LARP1(S824);LIMD2(S29);LINC00337(S30);LSM14B(S165);LSR(S436);LSR(S493);LUC7L2(S18);LUC7L2(S347);LZTS1(S233);MACF1(S7279);MAP2(S1555);MAP3K1(S292);MAP3K2(S153);MAP3K20(S727);MAP3K4(S1274);MAP4(S928);MAP4(S941);MAP7D1(S113);MAPK1(T185);MAPK1(Y187);MAPK3(T202);MAPK3(Y204);MARCKSL1(S93);MARK3(S400);MARK3(S419);MAST3(S747);MAVS(S222);MCM3(S711);MCM3(T722);MELK(S505);MELK(S529);MEPCE(S152);METTL3(S30);MFSD10(S271);MGA(S1208);MGA(S1457);MIA2(S1202);MIA2(S1204);MIA2(S1243);MICAL3(S1310);MKI67(S2223);MKI67(T1557);MLPH(S552);MPRIP(S993);MSH6(S14);MTFR1L(S103);MTFR1L(S238);MTMR12(S564);MTUS1(S1268);MVB12A(S170);MYCBP2(S2749);MYCBP2(S2751);MYH10(S1937);MYH9(S1943);MYO18A(S102);MYO7B(S689);MYOF(S1915);N4BP3(S211);NAB2(S193);NAV1(S695);NCBP1(S22);NCOA3(S857);NCOA3(Y574);NCOR1(S992);NFIL3(S301);NFX1(Y48);NHSL1(S1233);NUCB1(S369);ORC1(S273);OSBPL6(S344);OSBPL8(S810);OSER1(S82);OSER1(S84);PAK2(S141);PAK4(S163);PALM3(S303);PAPOLG(S708);PARD3(S717);PBRM1(S13);PBRM1(S14);PDS5A(T1208);PGRMC1(S57);PHAX(S368);PHF3(S283);PHIP(S1315);PHLDB1(S334);PI4KB(S428);PIGT(S235);PIK3AP1(S737);PIKFYVE(S329);PKD2(S832);PKMYT1(S143);PKP4(S447);PLCG1(S1263);PLEKHA5(S568);PLEKHG3(T964);POLH(S380);POLM(S12);POLR2A(S1868);POLR2A(S1878);POLR2A(S1910);POLR2A(Y1860);POM121(S435);POM121B(S19);POM121C(S412);PPFIBP1(S466);PPFIBP1(S601);PPHLN1(S133);PPIG(S687);PPIP5K2(S1074);PPP1R10(S313);PPP1R12A(S445);PPP1R13L(S187);PPP1R35(S87);PPP1R35(T84);PPP1R9B(S100);PRC1(S4);PREX1(S1182);PRPF6(S279);PRPF6(T275);PRRC2A(S1386);PRRC2C(S1544);PSIP1(S177);PTK2(S716);PTPN12(S435);PTPN12(S449);PTPN14(S760);PTPRZ1(S2056);PUM1(S124);PUM2(S82);RAB31(S35);RABEP1(S377);RALGAPA1(S797);RALGAPA1(T754);RANBP1(S60);RANBP2(S955);RAP1GAP(S484);RAP1GAP2(S564);RASAL3(S51);RB1(S612);RB1(T601);RB1(Y606);RBL1(S640);RBL1(T369);RBM15(S700);RBM15B(S113);RBM15B(S265);RBM15B(S267);RBM15B(T532);RBM23(S140);RBM23(S142);RBMX(S208);RBMX(S326);RBMX(S332);RBMX(S352);RBMX(S88);RBMXL1(S208);REEP3(S152);REEP4(S152);RICTOR(S1284);RLIM(S228);RLIM(S230);RNF214(S176);RPL28(S115);RPS14(S139);RPUSD2(S68);SACS(S2511);SAFB(S601);SAFB(S604);SALL1(S1119);SALL3(S633);SAMD1(T107);SASH1(S813);SASH1(S90);SASH3(S26);SASS6(S510);SATB1(S633);SCAF1(S874);SCAF11(S796);SCRIB(T475);SDAD1(S585);SDK2(S1982);SEC16A(S1181);SF3B1(T261);SF3B1(T434);SF3B1(T436);SGO1(S461);SGPP1(S101);SH3BP4(S296);SH3PXD2B(S291);SHANK2(S877);SHROOM2(T647);SIK3(S866);SIPA1(S839);SLAIN2(S413);SLBP(T123);SLC4A10(S238);SLC4A7(S233);SLTM(S1014);SLTM(S553);SLX4(S1309);SLX4(S1333);SLX4(S1469);SLX4IP(S396);SMAP2(S240);SMARCA4(S610);SMARCA5(S116);SMARCD1(S206);SMARCD2(S229);SMARCD3(S181);SMCR8(S489);SPAG9(S730);SPAG9(S733);SPP2(S182);SPTAN1(S1031);SRRM2(S1458);SRRM2(S1539);SRRM2(S2115);SRSF10(S133);SRSF4(S113);SRSF4(S446);SRSF5(S117);SRSF6(S119);SSH3(S37);SSSCA1(S78);STIM2(S680);STIM2(S719);STX17(S289);SURF6(T229);TACC1(S276);TBC1D1(S237);TBC1D4(S588);TBC1D5(S522);TCF20(S1335);TCOF1(S156);THRAP3(S232);TICRR(S923);TJP1(S968);TJP2(T462);TJP3(S369);TJP3(S371);TJP3(S591);TLN1(S2040);TMEM201(S441);TMPO(S306);TNKS1BP1(S429);TNKS1BP1(S983);TNS3(S363);TOP2A(S1213);TOR1AIP1(T220);TP53BP1(S1317);TP53BP1(S366);TPD52L1(S149);TPD52L2(S166);TRA2A(T202);TRAF4(S426);TRAM1(S365);TRAPPC10(S711);TRAPPC12(S184);TRIM11(S85);TRIP10(S296);UBE2O(S515);ULK1(S556);ULK1(S623);ULK1(S719);USP14(Y136);USP32(S1416);USP54(S1036);USP6(S1214);UTP20(T1741);VASN(S284);VCPIP1(S747);WASHC2A(S728);WASHC2C(S726);WNK1(S2032);YAP1(S289);YBX3(S293);YEATS2(S575);ZC3H13(T364);ZC3H3(S571);ZC3HAV1(S257);ZC3HAV1(S335);ZC3HAV1(T273);ZC3HAV1(Y348);ZFP36L1(S334);ZFP36L2(S490);ZMYND8(S425);ZNF136(S405);ZNF185(S64);ZNF408(T322);ZNF609(S1055);ZNF639(S88);ZXDC(S34)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>PAK2</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>46</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(S30);ADAM10(S740);AHCTF1(S528);ARFGAP2(S432);ARFIP1(S132);ARHGEF18(S1111);ATAD2(S327);BIN2(S259);C2CD5(S281);CD97(S818);CHD8(S1978);CLASP2(S529);CPSF7(S48);CRTC2(S70);DDX3Y(S592);ENAH(T538);EZH2(T367);FOXK1(S420);GTF2F1(S385);HNRNPA3(S358);HSPB1(S82);JPH1(S216);KANK2(S172);KANK2(S175);LRRFIP2(S324);LSM11(S21);MAP7D1(S93);MAST2(S876);NAA30(S199);NUP210(S1877);PBX2(S330);PRAG1(S510);RANBP2(T1396);RBM15(S622);RBM17(S169);RBMX(S332);RRP1B(S735);THAP4(S128);TJP1(S617);TMPO(S306);TMX1(S270);WIPF1(S340);WNK1(S2032);ZDHHC5(S425);ZFHX4(S2996);ZNF639(S88)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>PAK3</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>484</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>09/07/18 00:00:00(T426);ABCF1(S140);ABCF1(S22);ABCF1(T108);ABI1(Y213);ABLIM1(S452);ACIN1(S825);ADD2(S613);ADGRL2(S1275);AEBP2(S390);AFF1(T372);AFF1(T376);AFF4(S1043);AFF4(S487);AGAP1(S605);AHCTF1(S528);AHNAK(S115);AHNAK(S5731);AHNAK(S5763);AHNAK(S5841);AKAP1(S151);ALKBH5(S361);AMPD2(S190);ANKRD17(S2047);ANKRD2(S99);ANLN(S182);ANLN(T194);ARAF(S157);ARFGAP2(S368);ARFGEF2(S227);ARFIP1(S132);ARHGAP35(S1150);ARHGEF17(S420);ARHGEF6(S684);ARPP19(S62);ASAP2(S822);ASMTL(S239);ATF7(S434);AXIN1(S77);BAIAP2L1(S261);BAIAP2L1(T257);BASP1(S164);BCAM(S600);BCL11A(S630);BCL7C(S126);BCL7C(T118);BCL9L(S1017);BCLAF1(S287);BMS1(S625);CAD(S1859);CAD(S1900);CALD1(S759);CANX(S583);CAPRIN1(S21);CASC4(S233);CBFA2T3(S459);CCDC86(S102);CCDC86(S47);CD248(T60);CDC20(S160);CDC20(T157);CDK11A(S72);CDK11A(T739);CDK11B(S72);CDK11B(T751);CDK12(S274);CDK12(S276);CDK13(T1147);CDK17(S137);CEP350(S2115);CGN(S149);CHAF1A(S772);CLASP2(S892);CLIP1(S204);CNOT2(T93);COG3(T534);CRAMP1(S1201);CRKL(Y207);CRTC1(S172);CRTC1(T149);CRTC2(S178);CRTC2(S70);CTAGE5(S594);CTAGE5(S596);CTAGE5(S635);CTNND1(T906);CTTN(T401);CUX1(S1215);CWF19L2(S479);CYBRD1(S260);DAXX(S178);DBN1(S272);DDX17(S571);DDX21(S89);DDX41(S23);DENND4C(S989);DGCR8(S377);DIP2B(S100);DIP2B(S53);DLG5(S1254);DMXL2(S1400);DNMT1(S714);DNTTIP2(S151);DOCK5(S1766);DOPEY2(S597);DTL(S485);DTL(S623);DTL(T429);DYNC1LI1(S465);DYNC1LI1(S468);EFHD2(S74);EIF3A(S1188);EIF3A(S584);EIF3B(S85);EIF4EBP1(S65);EIF4EBP3(S51);EIF4EBP3(T32);EIF4EBP3(Y20);EIF4G1(S15);EIF4G2(S17);EIF4G3(S230);EIF5B(S214);EMD(S173);EML4(T899);EMSY(S209);EMSY(T207);ENAH(T538);ENSA(S67);ERF(S327);ESS2(T386);ESYT2(S688);ESYT2(S739);ETV3(S159);EVL(S331);F11R(S284);FAM104A(S21);FAM117B(S136);FAM193A(S1144);FAM193A(S393);FAM193A(S985);FAM208B(S1025);FGD1(S50);FLI1(S39);FNDC3A(S203);FNDC3A(S213);FOXO3(S284);FRMD4B(S778);FUBP3(S569);FZD6(S629);GFI1(S98);GLCCI1(S30);GLCCI1(S406);GMIP(S919);GMIP(S923);GMPS(T318);GNL1(S51);GOLGA4(S266);GON4L(S206);GTF3C1(S1068);GTPBP4(S558);HCFC1(S669);HEATR6(S337);HELZ(S1620);HMGXB4(S197);HNRNPA1(S95);HNRNPA1L2(S95);HNRNPA2B1(S212);HNRNPM(S618);HNRNPU(S271);HNRNPU(S59);HP1BP3(S156);HSPB1(S82);HTATSF1(S409);INTS1(S13);ITPR3(S1832);ITSN1(S559);JPH1(S216);JPH1(S452);JPT1(S28);JUN(S63);JUP(S182);KDM1A(S166);KDM2A(S731);KDM5A(S1331);KIF4A(T1181);KMT2A(S2151);KRI1(S171);KRT18(S7);KRT8(S477);LAD1(S301);LARP1(S766);LARP1(T649);LARP1(Y777);LIMD1(S272);LIMD2(S29);LRCH4(S515);LRCH4(S520);LRMP(S131);LRRTM4(S195);LRRTM4(S197);LSR(S436);LUC7L2(T17);MAML1(S360);MAP4(S941);MAPK1(T185);MAPK1(Y187);MAPK3(T202);MAPK3(Y204);MARCKS(S167);MARCKSL1(S93);MARK3(S419);MARK3(S585);MAVS(S222);MCM3(S711);MCM3(T722);MCM7(S121);MED1(S1481);MED1(S1482);MEPCE(S152);METTL3(S50);MGA(S1208);MGA(S1457);MIA2(S1202);MIA2(S1204);MIA2(S1243);MICAL3(S1310);MICAL3(S649);MKI67(S2223);MKI67(S308);MLPH(S552);MORC3(S765);MPLKIP(S115);MRGBP(S195);MSH6(S256);MTDH(S308);MTUS1(S1268);MYH9(S1943);MYSM1(S218);NAB1(S407);NAV1(S391);NAV1(S695);NBEAL2(S2743);NCOR1(S992);NCOR2(S1018);NCOR2(S215);NCOR2(S2269);NEDD1(S516);NES(S471);NFIL3(S301);NOP14(S96);NSD1(S2471);NSD2(T115);NUCKS1(S19);NUP107(T46);NUP35(S55);NUP50(S208);OSBPL3(S304);OSBPL6(S344);OSBPL8(S810);PAK4(S148);PAPOLG(S599);PAPOLG(S708);PAXBP1(S557);PAXBP1(S558);PCM1(S960);PDE3B(S495);PGM3(S64);PGRMC1(S57);PHAX(S368);PHF3(S1763);PHF3(S283);PHIP(S1315);PHRF1(S936);PIK3AP1(S737);PIKFYVE(S329);PKMYT1(S143);PKP4(S447);PLCB2(S964);PLD1(S629);PLEKHA5(S568);PLEKHG3(T964);PNISR(S311);PNISR(S313);PNISR(S321);POGZ(S746);POLR2A(S1917);POM121(S435);POM121B(S19);POM121C(S412);PPFIA1(S1172);PPHLN1(S161);PPHLN1(S163);PPHLN1(Y162);PPIG(S687);PPP1R10(S313);PPP1R12A(S871);PPP1R13L(S187);PPP1R7(S27);PPP1R7(S37);PPP1R9A(S840);PRPF38B(S527);PRPF38B(S529);PSD4(S134);PSEN1(S43);PSIP1(S177);PTPRZ1(S2056);PUM1(S98);PUM2(S82);PWWP2B(S447);PXN(S303);RAB11FIP1(S202);RAB31(S35);RANBP2(S3207);RANBP2(S955);RANBP3(S125);RAP1GAP(S484);RB1(S612);RB1(Y606);RBBP7(S99);RBM15(S292);RBM15B(S265);RBM23(S128);RBM4B(S86);RBMX(S332);RBMX2(S273);RCSD1(S68);REPS1(T539);RICTOR(S1284);RIF1(S1542);RIF1(S1554);RNF214(S176);RNF223(S19);RNF31(S466);RPP30(S251);RPRD2(S930);RPRD2(T763);RPS6KB1(S427);RRBP1(S1277);RSF1(S570);RSF1(S622);RUNX1(T14);SACS(S2511);SAFB(S601);SALL1(S1119);SALL3(S633);SAMD1(T107);SASH3(S26);SASS6(S510);SATB1(S633);SBNO1(T819);SCAF11(S802);SCNM1(S183);SDK2(S1982);SEC16A(S1178);SEC16A(S1181);SERBP1(S203);SETD1A(S470);SETD2(T749);SF3A1(S359);SF3B1(T267);SF3B1(T436);SFSWAP(S909);SGO1(S461);SH3BP1(S598);SH3BP1(S612);SH3BP1(S613);SH3KBP1(S410);SHANK2(S877);SHROOM3(S890);SIPA1L1(S1433);SIRT1(S27);SLBP(T123);SLBP(T62);SLX4(S1309);SLX4(S1333);SLX4(S1469);SLX4IP(S396);SMARCA5(S116);SNRK(S518);SOX5(S109);SPAG9(S733);SPECC1L(S868);SPTBN2(T2200);SRRM1(T718);SRRM2(S1539);SRRM2(S1857);SRRM2(S2115);SRRM2(S2581);SRRM2(S323);SRRM2(S846);STAT5A(S193);STEAP3(S17);STIM1(S575);STK10(S438);STK11IP(S470);STK11IP(S761);STK4(S414);SUDS3(S237);TACC1(S276);TAF6(S634);TAF6(S636);TANC2(T434);TBC1D5(S522);TCF20(S574);THRAP3(S698);TICRR(S923);TJP2(S979);TLE3(S286);TMC6(S63);TMCC2(S438);TMCC3(S216);TMEM201(S441);TMPO(S159);TMPO(S306);TMPO(S66);TMPO(S67);TMPO(T160);TNIK(S688);TNKS1BP1(S435);TNS3(S363);TOP2A(S1213);TOPORS(S585);TOR1AIP1(T220);TOX4(S182);TP53BP1(S222);TP53BP1(S366);TPD52L1(S149);TRA2B(T201);TRA2B(T212);TRAM1(S365);TRAPPC12(S184);TRMT1(S625);TRPV3(S372);TRPV3(S374);TUBB(S75);TUBB2A(S75);TUBB2B(S75);TUBB3(S75);UBA1(S816);UBA1(S820);UBE2O(S515);ULK1(S623);UNC93B1(S547);UNC93B1(S550);UNG(T60);UNK(S385);UPF3B(T169);USP14(Y136);UTP3(S37);VCPIP1(S747);VRTN(S432);WAC(S511);WAPL(S221);WAPL(S226);WASHC2A(S1001);WASHC2C(S978);WASHC4(S1157);WIPF1(T218);WNK1(S2032);WWC3(T909);YAP1(S289);YEATS2(S575);ZC3H11A(S758);ZC3H14(S343);ZC3H14(S620);ZC3H18(S532);ZC3HAV1(S275);ZC3HAV1(S494);ZC3HC1(S359);ZDHHC5(S554);ZEB1(S679);ZFAND5(S58);ZFHX4(S2996);ZFP36L1(S334);ZFP36L2(S490);ZHX3(S946);ZNF106(S1304);ZNF185(S64);ZNF574(S298);ZNF608(S895);ZNF609(S467);ZNF639(S88);ZNRF2(S21);ZXDC(S34)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>PAK4</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>38</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>ALKBH5(S361);ARHGAP35(S1150);C17orf53(S332);C1orf226(S18);CAD(S1406);CD2AP(S458);CDK17(S180);DOCK7(S888);EIF4ENIF1(S564);FAM102B(S228);GAB1(S419);GSK3A(S21);ID2(S14);INSRR(S72);IQSEC1(S180);KIF21A(S855);KRT8(S43);MEPCE(S152);MTMR12(S564);MYO18A(S102);MYO7B(S689);NCBP1(S22);PAPOLG(S708);RALGAPA1(T754);RAP1GAP2(S564);REEP4(S152);SPP2(S182);TBC1D4(S588);TNS3(S363);USP32(S1416);USP6(S1214);VASN(S284);WASHC2A(S728);WASHC2C(S726);ZC3HAV1(S335);ZNF185(S64);ZNF609(S1055);ZP2(S454)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>PDGFRB</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>788</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>09/02/18 00:00:00(S218);2 Phospho (ST);AAK1(S14);AAK1(S21);AATF(S320);AATF(S321);ABCA2(S1238);ABCF1(S105);ABCF1(S228);ABCF1(T108);ABI1(T215);ABI2(S368);ABLIM1(S655);ABLIM1(S706);ACIN1(S388);ADD1(S431);ADD1(S436);ADGRL2(S1275);AFDN(S1318);AFDN(T1330);AFF1(T372);AFF1(T376);AGAP1(S605);AGO2(S387);AHNAK(S5110);AHNAK(S5448);AHNAK(S5731);AHNAK(S5841);AKAP2(S720);ANAPC4(S779);ANK2(S3823);ANK3(S4298);ANKRD13D(S465);ANKRD13D(T469);ANKRD17(S1696);ANKRD17(S2401);ANKS1A(S647);ANKS1A(S663);ANKS1A(S887);ANLN(S792);AP1M1(T154);APBB1IP(S526);ARFGEF2(S624);ARFGEF2(T626);ARHGAP17(S162);ARHGAP17(T682);ARHGAP21(S1862);ARHGAP21(S856);ARHGAP39(S251);ARHGAP4(S906);ARHGEF11(S255);ARHGEF11(S35);ARHGEF16(S107);ARHGEF17(S420);ARHGEF2(S122);ARID1A(S604);ARID1A(S772);ARID3A(S119);ARL6IP4(S239);ASAP2(S822);ASCC3(S2195);ATAD1(S322);ATAD5(S306);ATAT1(S315);ATF7(S434);ATF7IP(S474);ATF7IP(S477);ATF7IP(S673);ATP1A1(S16);ATXN2(S861);ATXN2L(S32);BAG3(T406);BCLAF1(S183);BCLAF1(S282);BCLAF1(S385);BCOR(S488);BCOR(T1145);BCR(S459);BICRAL(S675);BRAF(S365);BRCA1(S1524);BRIP1(S1032);BUB1B(S543);C11orf84(S148);C17orf47(S195);C1orf174(S189);C1orf198(S37);C2CD2(S649);C9orf40(S69);C9orf78(T100);CAAP1(S312);CAMK1D(T184);CAMKV(T435);CAMSAP1(S793);CAMSAP3(S814);CARD9(S425);CASC3(S363);CASKIN2(S711);CAST(S243);CCAR2(S678);CCDC14(S798);CCDC43(T139);CCDC43(Y135);CCDC86(S160);CCDC86(S66);CCDC86(S69);CCDC86(Y164);CCDC88A(S1820);CCNL2(S369);CD2AP(S510);CD2BP2(S49);CD3EAP(S285);CDC20(T70);CDC25A(S18);CDC25B(S323);CDC42BPG(S1482);CDC42EP1(S143);CDC42EP1(S350);CDC6(S106);CDCA8(S219);CDK11A(S577);CDK11B(S589);CDK12(S32);CDK13(T871);CDK17(S180);CDK18(S117);CDK18(S132);CDK18(S14);CDS2(S33);CDYL(S216);CENPA(T21);CEP170(T1533);CEP170P1(T242);CEP76(S83);CFL1(S3);CGN(S149);CHAF1A(S206);CHD8(S1420);CHD8(S1424);CHD8(S2008);CLDN10(S203);CNK3/IPCEF1(S873);CNOT2(S101);CNOT2(S170);CPSF4(S202);CRAMP1(S1268);CREB1(S143);CREBBP(S121);CRKL(S107);CRKL(Y207);CRTC2(S613);CRTC3(S329);CSNK1D(S331);CTAGE5(S594);CTAGE5(S635);CTPS1(S575);CTTN(T411);DAB2IP(S747);DAP(S51);DCLK1(T336);DCLRE1C(S518);DCP1A(S62);DDX17(S571);DDX41(S21);DDX41(S23);DENND4A(S1256);DENND4C(S989);DGCR8(S271);DGCR8(S275);DGKH_HUMAN_3 Phospho (ST);DHX57(S77);DHX8(S460);DIP2B(S100);DLG1(S122);DLG5(S1115);DLG5(S1232);DLG5(S1254);DLGAP5(S690);DNMT3B(S136);DNTTIP2(T188);DNTTIP2(T87);DOCK5(S1766);DOT1L(S902);DOT1L(T900);DPF2(S200);DPPA4(T215);DUSP16(S612);DYNC1H1(S4368);DYNC1LI2(S194);EDC4(S729);EEF1AKMT2(S21);EEF1B2(S106);EEF1B2(Y79);EEF1D(S162);EEF1D(T147);EEF1G(T46);EEF2K(S72);EEF2K(S74);EEF2K(Y69);EHBP1(S432);EHBP1L1(S1257);EIF3A(S1188);EIF4ENIF1(S752);EIF4G3(S232);ELAC2(S213);EMD(S141);EML4(S146);ENAH(S531);EPB41(S560);EPS15(S563);EPS15(S796);ERF(S327);ETV3(S139);ETV3(S159);ETV6(S203);EVPL(S2025);EXO1(S623);FAM117B(S10);FAM120A(Y452);FAM177A1(S70);FAM177A1(T71);FAM177A1(Y69);FAM193A(S393);FAM193B(S785);FAM234B(S62);FAM53C(S122);FAM83H(S1025);FAM83H(S647);FAM84B(T289);FBXO46(S240);FIP1L1(S500);FLI1(S241);FLNA(S2152);FLNA(S2158);FOXK1(S223);FOXK2(S373);FOXO3(S284);FOXO3(S55);FRMD4A(S800);FRYL(T1959);FYB1(S46);GAPDH(S151);GATA3(S115);GLCCI1(S30);GLCCI1(S406);GMPS(S332);GOLGA4(S1248);GON4L(S1426);GPATCH8(S738);GPHN(S188);GPHN(S194);GPHN(T198);GPN1(S338);GRAMD1B(S274);GSE1(S857);GSK3B(S25);GSK3B(S9);GTF2F1(T389);GTF3C1(S1856);GTF3C1(S1865);GTF3C2(S765);GTF3C2(S901);HBS1L(T231);HERC2(S2928);HIPK1(T351);HIPK2(T360);HIRIP3(S104);HMGA1(S102);HMGA1(S103);HMGCS1(S516);HNRNPU(S59);HOXC9(S159);HSP90AA1(S263);HSP90AB1(S226);HSP90AB3P(S205);HSPH1(T815);HTATSF1(S642);HUWE1(T2889);IFI16(S153);IGF2BP1(S181);IGLL1(S62);IKBKB(S672);INCENP(S481);IPCEF1(S411);IRF2BPL(S215);IRX2(S317);ITSN1(S315);IWS1(S235);IWS1(S237);IWS1(S80);IWS1(S82);JAZF1(T109);JAZF1(T113);JMJD1C(S2053);JUN(S63);KANSL1(S829);KANSL1(S839);KCNK2(S385);KIAA1522(S971);KIDINS220(S1633);KIF1A(S1370);KIF1A(S1548);KIF21A(S1271);KIF21A(S1274);KIF23(S902);KIFC1(S26);KLHDC4(S418);KMT2B(S1092);KMT2B(S1095);KMT2D(S2274);KMT2D(S3130);KPNA4(S60);KRT18(S399);KRT19(S395);KTN1(S75);L1TD1(S737);LARP1(S627);LARP1(S631);LASP1(T68);LEMD2(S499);LIG1(S76);LIG1(T195);LIMA1(S230);LIMA1(S686);LIMK1(S302);LLGL2(S480);LLGL2(S961);LSM14A(S178);LSM14A(S183);LTBP1(S1413);LYSMD2(S33);LYST(S2627);MACF1(S7330);MAGED2(S265);MAP1B(S1427);MAP1B(S1443);MAP1B(S937);MAP1B(T1317);MAP1B(T1341);MAP2(S1787);MAP2(S1790);MAP3K11(S524);MAP3K2(S239);MAP3K21(S514);MAP3K9(S519);MAP4K2(S328);MAP7D1(S116);MAP7D1(S460);MAP9(S79);MAPK1(Y187);MAPT(S713);MARCKS(S167);MAST2(S1254);MATK(S501);MCM3(S711);MCM3(T722);MCM3(Y708);MCM3AP(S527);MCM9(S1088);MCRIP2(S82);MDC1(S780);MED1(S664);MED13(S890);MEX3A(S428);MEX3B(S4);MEX3C(S540);MEX3C(T541);MFAP1(S116);MFAP1(S52);MFAP1(S53);MGA(S2088);MIA2(S1202);MIA2(S1243);MINK1(S733);MKI67(T401);MKL2(S921);MNAT1(S279);MON1B(S59);MON1B(S61);MPHOSPH8(S403);MPHOSPH8(T89);MPLKIP(S115);MPRIP(S289);MPRIP(S292);MTA1(S576);MTBP(S755);MTMR3(S647);MYB(S599);MYC(S62);MYCN(S62);MYO18A(S102);NAA30(S39);NAB2(S6);NAV1(S528);NAV1(S672);NAV1(S695);NCOR1(S1472);NCOR1(S158);NCOR2(S2065);NCOR2(S215);NCOR2(S2404);NCOR2(T1391);NDRG2(S332);NDRG3(S331);NDRG3(S334);NECTIN1(T391);NEDD4L(S448);NEDD4L(S487);NFATC2(S236);NFATC2(S243);NFATC2IP(S204);NGDN(S142);NGDN(S143);NHS(S1329);NMNAT1(S117);NOC2L(S49);NOL8(S432);NOP58(S502);NSMCE3(S64);NSRP1(S33);NSUN2(S456);NSUN2(S473);NUFIP1(S338);NUFIP1(S340);NUFIP1(S342);OSBPL8(S314);OSTM1(S322);PACSIN3(S383);PAK1(S137);PAK2(T143);PAK4(S181);PAK4(T207);PALD1(S406);PAPOLG(S708);PARD3(S174);PARN(S619);PATL1(T194);PCBP1(S173);PCDH18(T442);PCDH7(S1011);PCIF1(S144);PCNP(S119);PCYT1A(S343);PDE3B(S495);PDHA1(S232);PDHA1(S293);PDHA1(S300);PDHA2(S291);PDHA2(S298);PDS5B(S1358);PFKP(S386);PHACTR1(S505);PHACTR4(S118);PHC3(T609);PHF6(S154);PHIP(S1315);PHKA2(S1044);PHKA2(S729);PHLDB1(S518);PHLDB1(T516);PHLDB2(S513);PHLDB2(T404);PHRF1(S1229);PKN1(S562);PKP2(S293);PKP4(S337);PKP4(S406);PLEKHA6(S808);PML(S518);PML(S527);PNISR(S311);PNISR(S313);PNISR(S321);PNPO(S241);POLA1(S186);POM121(S395);POM121(S396);POM121C(S372);PPFIA1(S666);PPFIBP2(S387);PPIG(S256);PPIG(S257);PPM1H(S124);PPP1R12A(S871);PPP1R12A(S903);PPP1R13L(S102);PPP1R2(T89);PPP4R3B(S840);PPP6R1(S759);PPP6R3(S523);PRAG1(S889);PRAG1(S907);PRCC(S267);PRICKLE2(S546);PRKD2(S214);PROSER1(S613);PROSER2(S179);PRPF38B(S268);PRPF38B(S5);PRPF38B(S527);PRPF38B(S529);PRPF40B(S764);PRPF4B(S87);PRPF4B(S93);PRR5(S310);PRRC2C(T2673);PSMD1(S315);PSMD1(T311);PTPN13(S214);PTPN13(S908);PTPN14(S465);PTPN22(S692);PUM1(T112);PXN(S258);Phospho (ST);QRICH1(S345);RABL6(S640);RABL6(S641);RAD54B(S14);RALGPS2(S296);RALY(S239);RANBP2(S2510);RANBP2(S955);RAP1GAP2(S45);RAPGEF6(S1094);RAPH1(S539);RASAL2(S16);RB1(S37);RBM10(S797);RBM10(S89);RBM14(S256);RBM15(S670);RBM15(S674);RBM15B(S562);RBM20(S644);RBM27(S120);RBMX(S189);RBMXL1(S189);RBMXL1(S88);RCOR1(S260);RCSD1(S116);RCSD1(S120);RCSD1(S68);REPS1(S392);RFC1(S108);RFC1(T110);RFTN1(S199);RFX7(S225);RFX7(S424);RGPD1(S1519);RGPD2(S1527);RGPD3(S1535);RGPD4(S1535);RGPD5(S1534);RGPD8(S1534);RIC8A(S436);RIC8A(T441);RIF1(S1554);RIOK1(S22);RIOK2(S337);RNF2(S168);ROR2(S449);RPAP3(S116);RPAP3(S119);RPAP3(S121);RPRD2(S374);RPRD2(T723);RREB1(S42);RRP1B(S453);RRP8(S62);RRP8(S64);RSF1(T628);RYBP(S127);SAC3D1(S402);SAFB2(S832);SASH1(S407);SBNO1(T819);SCML2(S511);SCRIB(S1378);SCRIB(S1439);SCRIB(S1508);SCYL3(T153);SEC24B(T329);SEC62(T375);SERPING1(S198);SET(S161);SETSIP(S171);SF3A1(S329);SF3A1(S359);SF3A1(T374);SF3B1(T350);SGTA(S77);SGTA(T81);SH2B3(S150);SH2D3A(S147);SH3BP4(S279);SH3GL1(S288);SH3KBP1(S230);SHC3(S474);SHCBP1(S42);SHROOM2(S193);SHROOM3(S664);SHROOM3(S816);SIPA1L1(S1649);SIPA1L1(S1650);SIRT1(S27);SLC20A2(S256);SLC20A2(S259);SLC43A1(T256);SLC4A1AP(S466);SLC4A7(S556);SLC4A7(T559);SLC9A1(S703);SMAD1(S463);SMAD1(S465);SMAD9(S465);SMAD9(S467);SMAP(S93);SMARCAD1(S124);SMARCAD1(S127);SMARCC1(T398);SMARCC2(S347);SMC4(S22);SMC4(S28);SMG8(T743);SMG8(Y746);SMN1(S28);SNIP1(S35);SNX17(S333);SOGA1(S1303);SON(S1026);SON(S1784);SOX2(S250);SPATA5L1(S610);SPP1(S63);SPTAN1(S1217);SPTBN2(S2171);SPTBN2(S2384);SQSTM1(S224);SQSTM1(S332);SRRM2(S1014);SRRM2(S1144);SRRM2(S1404);SRRM2(S1501);SRRM2(S1502);SRRM2(S2123);SRRM2(S322);SRRM2(S377);SRRM2(S846);SRRM2(T318);SRRM2(T400);SRRM2(T848);SRRM2(Y1145);SRSF10(S131);SRSF11(S434);SRSF4(S450);SSBP3(S347);SSFA2(S1040);SSH1(S897);STAT5A(S193);STAU1(S390);STAU2(S455);STIM1(S618);STK17A(S28);STK33(S470);SVIL(S221);SYCE2(S188);SYMPK(S1243);SYNRG(S1075);SYT6(S187);SYT6(Y190);TACC2(S2317);TACC2(S2321);TACC3(S177);TBC1D22A(S167);TBKBP1(S365);TBKBP1(S372);TBKBP1(S400);TCF4(S372);TCOF1(S1227);TERF2IP(S154);TEX10(T29);TEX2(S266);TJAP1(S345);TJP1(S125);TJP1(S168);TJP1(S968);TJP2(S1159);TJP3(S164);TLE4(S208);TLN1(S425);TMF1(S72);TNK2(T829);TNK2(Y827);TNKS1BP1(S1158);TNKS1BP1(S1297);TNKS1BP1(S435);TNKS1BP1(S872);TNKS1BP1(S983);TNRC6C(S714);TNS1(S1269);TOMM70(S110);TOMM70(S91);TOP2B(S1400);TOP2B(S1522);TOP2B(S1524);TOR1AIP1(S157);TP53BP1(S580);TPD52L1(S149);TPX2(T369);TRAF4(S426);TRAFD1(S470);TRAM1(S365);TRAPPC12(S184);TRIM28(S50);TRIO(S1724);TRMT2A(S602);TRPS1(S1085);TRPS1(S127);TRUB1(T27);TSC1(S505);TSC22D4(S62);TTN(S1406);TVP23C(S223);TWISTNB(S304);UBA1(S13);UFD1(S299);UHRF1BP1L(S414);UHRF1BP1L(S418);UIMC1(S44);UIMC1(S46);UPF1(S1127);UPF3B(T169);USP1(S67);USP20(S373);USP20(T377);USP32(S1423);USP36(S952);UTP20(T1741);UTP3(S365);UTP3(S368);UTP3(S37);UTP3(Y43);VCAN(S2116);VCPIP1(S747);VRK3(S83);WAPL(S77);WASHC2A(S158);WASHC2A(S160);WASHC2C(S158);WASHC2C(S160);WDFY4(S3123);WDHD1(S868);WDR20(S434);WDR44(S403);WEE1(T190);WIPF2(S267);XRN1(S1645);XRN2(S471);XRN2(S499);XRN2(S501);YBX1(Y162);YBX3(S346);ZBTB37(S164);ZC3H11A(S758);ZC3H4(S1108);ZC3H4(S1110);ZC3H4(S1269);ZFC3H1(S949);ZKSCAN8(S12);ZMYM3(S267);ZMYM4(S122);ZNF106(S1304);ZNF106(S641);ZNF280D(S545);ZNF281(S651);ZNF318(S40);ZNF513(S85);ZNF516(T930);ZNF518A(S655);ZNF552(S86);ZNF609(S1055);ZNF609(S358);ZNF639(S60);ZNF814(S87);ZNRF2(S21);ZRANB2(S120);ZRANB2(S153)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>PHKG2</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>52</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(S30);AHCTF1(S528);AKAP11(S422);ANAPC1(S355);ARFGAP2(S432);ARHGEF2(S174);CDC42SE1(S74);CNK3/IPCEF1(S892);COBLL1(S394);DBNL(T291);DCUN1D5(S9);ERCC6L(S820);FUS(S462);FXR2(T411);GTF3C2(S167);HPS5(S534);IPCEF1(S430);IQSEC1(S180);KHDRBS1(S20);NADK(S48);NCOA5(S381);NUCB1(S369);PAK4(S181);PAPOLG(S708);PBRM1(S13);PBRM1(S14);PCNP(T139);PEA15(S116);PKP4(S314);PPHLN1(S133);PRAG1(S148);R3HDM1(S381);RALY(S135);RBBP6(S873);RBM15(S292);RBM15(S700);RBM15B(S265);RBM15B(S267);RBM39(S97);RBM39(Y95);RBMXL1(S88);RICTOR(S1284);RPA1(T180);SAFB2(S787);SHANK2(S67);SLTM(S1002);SLTM(S551);SLTM(S553);SNRPA1(T180);SRSF9(S189);TPI1(S249);UPF3B(T169)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>PIK3CA</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>230</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>ABCF1(S109);ACLY(S455);ADAM9(S758);AFF1(T372);AFF4(S836);AHNAK(S5110);AKAP11(S18);AKAP13(S2563);AKT1S1(T246);ANKIB1(S737);ARAF(S257);ARHGAP25(S533);ARHGAP39(S407);ARHGEF11(S1295);ARHGEF5(S606);ASAP2(S822);ASIC3(S37);ASIC3(S39);ATP5F1C(S146);BASP1(S164);BAZ2A(S1397);BCL7C(S122);BCL7C(S126);BRCA1(S1189);BRCA1(S1191);C2CD5(S295);C5orf30(S167);CAD(S1859);CARHSP1(S30);CARHSP1(S32);CARHSP1(S52);CD2AP(S234);CD2AP(S458);CD2AP(T236);CDC42BPG(S1482);CECR2(T546);CHAF1A(S775);CHD4(T1553);CHD8(S1995);CPD(T1368);CPD(T1370);CTTN(T411);DDX17(S571);DOCK5(S1834);DYNC1H1(S4368);EDC3(S131);EEF2K(S72);EEF2K(S74);EHBP1L1(S310);EHMT2(S232);EIF3A(S1188);EIF4EBP1(T70);EIF4EBP1(T82);EIF4EBP1(Y34);EIF4EBP2(S65);EIF4EBP2(T37);EIF4EBP2(T41);EIF4EBP2(T46);EIF4EBP2(T70);EIF4EBP2(Y34);EIF4EBP3(T31);EIF4EBP3(T32);EIF4EBP3(Y20);EIF4G1(T205);EMB(S309);ENAH(S508);ERCC6L(S984);FAM117A(S178);FAM189A1(S18);FAM53B(S118);FBXL15(S262);FOXK2(S373);FRMD4B(Y674);FUBP3(S569);GAB2(S210);GJA1(S365);GLYR1(S130);GOLGA4(S41);GPBP1(S381);GSK3A(S21);GSK3B(S9);HBS1L(S67);HCLS1(T308);HDAC1(S410);HDGFL2(S454);HELB(S967);HIPK1(Y352);HIPK2(Y361);HMOX1(S229);ID2(S14);INCENP(T195);INCENP(T219);IRS1(S329);IRS1(T351);IRS2(S594);IWS1(S720);KIAA0319L(S978);KIAA1217(S1044);KIF23(S867);KIF23(S902);KIF4A(S801);L3MBTL2(S683);L3MBTL2(S689);LARP1(S766);LARP1(T376);LARP1(Y777);LINC00322(S226);LINC00322(S228);LLGL2(S1000);LRRC47(S518);LYL1(S260);LYSMD2(S33);MAP4(S280);MAP4K4(S631);MAP7D1(S552);MAPRE1(S155);MASTL(S453);MDC1(S376);MDC1(S495);MDC1(S498);MEF2D(S121);METTL1(S27);MPHOSPH8(S136);MPHOSPH8(S138);MTMR4(S610);MTMR6(S561);MVD(S96);MYC(S293);MYC(S62);MYCN(S62);NDRG3(S334);NOL8(S432);NUCKS1(S19);NUP188(S1708);NUP188(S1717);NUSAP1(S255);PAK2(S141);PALM3(S143);PATL1(T194);PCBP1(S264);PCBP2(S272);PCDH1(S973);PCDH1(S984);PDCD4(S457);PDHA1(S293);PDHA2(S291);PGAM1(S14);PGM2L1(S175);PGRMC1(S57);PGRMC2(S90);PI4K2A(S462);POM121C(S372);PPP1R12A(S422);PPP1R12C(S427);PRKAA2(S377);PROSER2(S312);PUM2(S82);RAB3IP(S157);RAI1(S1374);RANBP2(S1128);RAP1GAP2(S564);RBL2(S639);RBM14(S618);RET(S696);RICTOR(S1591);RPRD2(S485);RPS27(S78);RPS27L(S78);RPS6(S236);RPS6(S240);RPS6KB1(S427);RPTOR(S863);RRAS2(S186);RREB1(S1167);RTKN(S520);SALL4(S126);SART1(S448);SDCCAG3(S247);SENP1(S132);SF3B1(T257);SF3B1(T261);SKIV2L(S131);SKIV2L(S133);SLTM(S551);SON(S94);SPP1(S303);SRGAP1(S932);SRRM2(S2121);SRRM2(S2407);SRSF7(S165);SRSF7(S167);SUPT6H(T1523);TACC2(T2073);TBC1D4(S588);TMPO(S66);TNKS1BP1(S893);TNS3(S776);TOP2A(S1247);TOR1AIP1(S156);TOR1AIP1(S157);TOX4(S182);TRIM33(S1119);TRIM37(S771);TRIM37(S773);TRIP10(S296);TSC1(S1102);U2AF2(S79);UCK1(S253);ULK1(S450);ULK1(S477);ULK1(T717);UTF1(S18);VIRMA(S173);WASHC2A(S284);WASHC2C(S284);WNK3(S1585);WRNIP1(S75);XPR1(S666);XPR1(S668);YBX1(S209);ZEB1(S646);ZNF219(S698);ZNF219(T695);ZNF326(S270);ZNF609(S467);ZNF687(S1118);ZNRF2(S21);ZSCAN10(S6);ZSCAN29(S153);ZSWIM8(S53)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>PIK3CB</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>159</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>ABCF1(S109);ABL2(S620);AFF1(T372);AFF1(T376);AFF4(S179);AHCTF1(S1232);AHNAK(S115);AHNAK(S5110);AKAP13(S2563);ARAF(S257);ARFGAP2(S146);ASMTL(S228);ATG2B(S1582);ATG2B(S1583);ATG2B(Y1577);BRF2(S353);C19orf47(S151);C2CD3(S2132);CAD(S1859);CANX(S564);CCDC88B(S1348);CENPC(S316);CEP170(S1165);CHAMP1(S603);CHD4(T1553);CNOT2(S165);CPD(T1368);CPD(T1370);CSTF3(S691);CTDSPL2(S104);CTTN(T411);DAB2IP(S747);DBN1(S312);DDX17(S571);DEAF1(S176);DENND1A(S523);DNAJB6(S277);DNTTIP2(S151);EHMT2(S232);EIF4B(S445);EIF4G1(S1194);FAM117A(S145);FAM53B(S118);FNDC3A(S203);FUBP1(T153);GPATCH4(S130);GSK3A(S21);HCLS1(T308);HDGFL2(S454);HEATR6(S337);HIPK3(Y359);IARS(S1047);IRS2(S594);JPH1(S216);KIAA0319L(S978);KIAA0754(T122);KIDINS220(S918);KIF23(S867);KIF4A(S801);LARP1(S766);LARP1(T376);LARP1(Y777);MACF1(S4496);MAP1B(T1788);MAP4(S280);MAP7D1(S552);MARK2(S486);MSANTD3(S98);MTCL1(S549);NFATC1(S245);NUFIP2(S112);NUP210(T1844);NUP214(S678);NUP214(T670);PACS2(S390);PAK2(S141);PDHA1(S293);PDHA2(S291);PHLDB2(S204);PI4K2A(S462);PLPP3(S19);POM121(S395);POM121(S396);PPP1R12C(S427);PRRC2B(S1395);PUM1(S209);RAB11FIP1(S202);RAD54B(S14);RAI1(S1374);RAP1GAP2(S608);RAP1GAP2(S609);RBM10(S89);RBM14(S618);RBMX(S352);RETREG3(S258);RETREG3(S260);RETREG3(S360);RIF1(S2172);RIF1(S2176);RPS27(S78);RPS27L(S78);RPS6KA4(S682);RPS6KB1(S441);RRAS2(S186);SALL3(S1268);SALL4(S126);SART1(S448);SCAF4(S154);SEC16A(S1191);SEMA4B(S788);SF3B1(T257);SLC4A7(S242);SLC6A15(S687);SLC9A1(S703);SNTB2(S95);SON(S2129);SPAM1(S78);SPTBN1(T7);SRGAP1(S932);SRRM2(S2121);SRRM2(S2407);STIM2(S680);STIP1(S481);STRN(S376);TBC1D9B(S435);TCOF1(S583);TEX2(S732);TIMELESS(S1087);TNKS1BP1(S893);TNS3(S776);TOP2A(S1247);TOP2B(S1524);TOR1AIP1(T220);TTYH3(S496);TWISTNB(S304);TWISTNB(S316);UBE2E3(S8);UBR5(S2484);UBR5(S2486);UTF1(S18);VIRMA(S173);WDR59(S822);WIZ(S1012);YBX1(S209);YBX3(S293);YBX3(S38);YEATS2(S447);ZBTB17(S120);ZBTB7A(S337);ZC3H14(S620);ZC3H4(Y162);ZDHHC18(S19);ZDHHC5(S296);ZIC3(Y425);ZKSCAN8(S12);ZNF219(S698);ZNF219(T695);ZNF326(S270);ZSWIM8(S53)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>PKN1</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>2</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>AHNAK(S5830);ZNF185(S64)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>PKN2</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>16</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>ABI2(S368);BAIAP2(S261);CAD(S1859);CDC25B(S323);CDC42EP1(S192);EIF3A(S584);GPSM2(S565);JPH1(S216);LARP1(T649);MTBP(S755);NFATC2(S326);PIK3CD(T226);PPHLN1(S172);TBC1D10B(T697);ZFP36L1(S334);ZFP36L2(S490)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>PLK1</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>832</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>ABCF1(T108);ABI2(S242);ABL1(S569);ACD(S425);ACIN1(S838);ADD1(S436);ADD1(S465);ADGRL2(S1275);AFF1(T372);AFF1(T376);AFF4(S180);AHCTF1(S1232);AHCTF1(S528);AHNAK(S115);AHNAK(S93);AKAP11(S422);AKAP13(S1906);AKIRIN1(S22);ALDOA(S46);ALPK3(S1424);AMFR(S542);AMPD2(S76);ANAPC1(S355);ANKLE2(S662);ANKRD17(S1940);ANKRD17(S2401);ANKS1A(S628);ANLN(S54);ANLN(S927);ARFGEF2(S1528);ARFGEF2(S227);ARHGAP12(S240);ARHGAP12(T231);ARHGAP17(T682);ARHGAP21(S1526);ARHGAP39(S366);ARHGAP5(S1218);ARHGEF11(S1295);ARHGEF18(S1103);ARHGEF5(S1126);ARHGEF7(S257);ARID1A(S1755);ARID1A(T1206);ARID4B(S675);ARID5A(S463);ARMCX3(S110);ASMTL(S228);ASMTL(S239);ASXL2(S139);ATAD2(S342);ATAD2(T1152);ATAD2B(S16);ATF7IP(S113);ATG2B(S1582);ATG2B(S1583);ATG2B(Y1577);ATP13A3(S817);ATP5F1C(S146);ATRX(S889);ATXN2(S758);ATXN2(S857);ATXN2(S861);ATXN2L(S424);BAG3(T285);BAG6(S1117);BAP18(S110);BAZ1A(S1413);BAZ1A(T1547);BAZ2A(S135);BBX(S844);BCL11A(S332);BCL11A(S630);BCL7C(S126);BCL9(S687);BCLAF1(S268);BCLAF1(S287);BCLAF1(Y284);BCR(S463);BIN1(S303);BPTF(S2370);BRF2(S353);BRIP1(S1032);BUB1(S661);C12orf45(S15);C19orf47(S151);C2CD2(S441);C2CD2(S649);C2CD3(S2132);C2CD5(S295);C6orf106(S215);CABIN1(S1844);CAMSAP1(S563);CAMSAP1(S629);CAMSAP2(S464);CANX(S564);CARHSP1(S30);CASP8AP2(S875);CBARP(S200);CBY1(S20);CCAR2(S678);CCDC14(S798);CCDC6(S52);CCDC85C(S179);CCDC86(S18);CCDC88C(S1547);CCNK(S340);CCNL1(S335);CCNL1(S338);CCNL2(S348);CCNY(S83);CCP110(S551);CD2AP(S458);CD2AP(S510);CD3EAP(S490);CDAN1(S160);CDC20(S160);CDC20(T157);CDC42EP4(S118);CDC6(S106);CDK12(S1083);CDK12(S274);CDK12(S276);CDK12(S383);CDK12(S385);CDK12(T514);CDK13(S1048);CDK13(S525);CDK16(S153);CDK17(S137);CDS2(S33);CEBPB(S231);CENPC(S316);CENPF(S3119);CEP152(S1461);CEP170(S1165);CEP170(S1529);CEP170(S466);CEP170B(S829);CEP170B(S969);CEP170P1(S238);CEP350(S2460);CGN(S252);CHAF1A(S775);CHAF1A(S873);CHD4(S303);CHD7(S2559);CHD8(S1995);CHD8(T1338);CLASP1(S559);CLASP1(T798);CLASP2(S585);CLASP2(S596);CLDN3(T204);CLIP1(S204);CLIP1(S348);CLIP2(S352);CLIP2(S54);CLMN(S923);CNK3/IPCEF1(S892);CNNM3(S700);CNOT2(S165);CNOT2(S170);CNP(S170);CRKL(Y207);CRTC2(S136);CSPP1(S966);CSRP1(S192);CTTN(T411);DAB2IP(S747);DBN1(T343);DBNL(S269);DCLK1(S313);DCP1B(S147);DDX39A(T171);DDX54(S75);DENND1A(S523);DENND1C(S582);DHX29(S200);DHX57(S77);DIDO1(S1260);DLG5(S1232);DNAJB6(S277);DNMT1(S714);DNTTIP2(S117);DOCK7(S1438);DOT1L(S834);DTL(S656);DTNA(S662);DUSP28(S13);DYNC1H1(S4368);EAF1(S165);ECT2(S861);EEF2K(S74);EFCAB12(S172);EFR3A(S694);EHBP1(S436);EHD1(S456);EHMT2(S232);EIF3A(S1188);EIF4B(S283);EIF4EBP3(T31);EIF4EBP3(T32);EIF4EBP3(Y20);EIF4ENIF1(S564);EIF4G1(T205);ELF1(S187);EMD(S141);EMD(S142);EMD(S143);EPB41(S521);EPB41L1(S650);EPB41L1(S784);EPB41L3(S460);EPB41L3(T469);ERBB2(S1151);ESS2(S395);ESS2(T386);ESYT2(S693);ETV6(Y17);EXO1(S623);F11R(S284);FAF1(S582);FAM109A(S213);FAM117A(S145);FAM117A(S67);FAM122A(S189);FAM126B(S430);FAM208B(S2037);FAM214B(S319);FAM53B(S268);FAM53C(S122);FAM53C(S162);FAM53C(S299);FAM83B(S766);FAM83H(S7);FLI1(S241);FLNA(S1459);FNBP1(S299);FNDC3A(S203);FNDC3A(S213);FOXK1(S223);FOXK1(S441);FOXK2(S373);FTH1(S183);FTSJ3(S584);FTSJ3(S644);FUBP1(T153);FUS(S462);FXR1(S409);FXR2(S566);FXR2(T411);FYB1(S46);FZD6(S629);GATA3(S115);GATAD2A(S114);GBF1(S1318);GBF1(S1320);GJA1(S325);GNL1(T50);GOLGB1(S17);GON4L(S206);GPATCH2(S195);GPATCH2(S54);GPATCH2L(S447);GPATCH4(S130);GPATCH8(S1033);GPBP1(S381);GREB1(S1160);GTF3C2(S167);GTSE1(S580);GYS1(S641);GYS1(S645);HAUS6(T584);HBS1L(S67);HCN4(T1071);HDAC4(S467);HECTD4(S88);HIRIP3(S104);HIST1H1B(S18);HJURP(S557);HMGA1(S99);HMGCR(S872);HNRNPA2B1(S212);HNRNPA2B1(S344);HNRNPC(S253);HNRNPUL2(S655);HPS5(S534);HSP90AA1(T109);HSP90AA2P(T109);HSP90AB1(S226);HSP90AB1(S255);HSP90AB1(T104);HSP90AB2P(S177);HSP90AB2P(T104);HSP90AB3P(S205);HSPA4(S647);HSPH1(S809);IARS(S1047);IFI16(S153);IGF2R(S2484);INCENP(S143);INCENP(S311);INCENP(S312);INVS(S617);IPCEF1(S430);IQSEC2(S1143);IRF2BPL(S519);IRF2BPL(S659);IRS2(S1203);IRS2(S306);IRS2(S577);IRS2(S608);JMJD1C(S2053);JMJD1C(T1187);JPH1(S216);JUP(S182);KCTD15(S35);KCTD15(S38);KDM2A(S731);KIAA0754(T122);KIAA1522(S971);KIDINS220(S1555);KIDINS220(S1633);KIDINS220(S918);KIF13B(S1644);KIF18B(S685);KIF21A(S1239);KIF23(S867);KMT2A(S1837);KMT2A(S518);KMT2D(S2296);KMT2D(S3130);KMT2E(S531);KNOP1(S42);KNOP1(S48);KNOP1(T308);KPNA3(S60);KPNA4(S60);KRT76(T427);KRT8(S13);LARP6(S409);LEMD3(S144);LIMA1(S362);LIMA1(S609);LIMD1(S384);LMF1(S522);LRCH4(S313);LSM14B(S165);LUC7L(S327);LUZP1(S659);LYSMD2(S33);MADD(T1061);MAP1B(S1252);MAP1B(T1788);MAP2(T1616);MAP2K7(S61);MAP3K11(S524);MAP4(S1073);MAP4(S358);MAP4(S928);MAP4K4(S900);MAP7D1(S254);MAP7D1(S446);MAP7D1(S468);MAP7D1(S469);MAP7D1(S496);MAP7D3(S524);MAPK3(T207);MAPT(T498);MARK2(S456);MARK3(S469);MARK3(S583);MAST2(S1032);MASTL(S453);MATR3(S598);MAVS(S222);MAZ(S302);MCM3AP(S557);MEF2D(S121);MEX3B(S442);MEX3C(S545);MFF(S157);MGA(S2924);MIEF1(S59);MINDY2(S62);MINK1(S993);MIS18BP1(T702);MKI67(S1131);MKI67(S1329);MKI67(S2105);MKI67(S2344);MKI67(S2638);MKI67(S584);MPHOSPH8(S403);MPRIP(S993);MRPS18B(S38);MSANTD3(S98);MSL1(S126);MSX2(S91);MTCL1(S232);MTCL1(S549);MTMR1(S43);MTMR3(Y614);MTMR4(S115);MTX3(S284);MVD(S96);MXRA7(S144);MYBBP1A(S1241);MYC(S281);MYCBP2(S3467);MYH10(S1965);MYO9B(S1290);NADK(S48);NAF1(S315);NAV1(S1382);NAV1(S312);NAV2(S1245);NAV2(S1280);NCAPD2(S1333);NCOA1(S372);NCOA3(S1330);NDRG2(S350);NDRG2(S352);NDRG2(T334);NDRG2(T348);NDRG3(S334);NECAP2(S181);NELFA(S233);NFATC1(S245);NFATC2(S148);NIPBL(S306);NKTR(S463);NOMO2(S1205);NOMO3(S1205);NOP56(S520);NOVA1(S157);NPM1(S260);NSD1(S752);NSD2(T115);NTHL1(S22);NUF2(S247);NUFIP2(S112);NUMB(S425);NUP153(S333);NUP210(T1844);NUP210(Y1855);NUP98(S623);OGFR(S484);OIP5(S225);ORC2(T116);PABPN1(S150);PAK2(S152);PAK2(T169);PAPD5(S52);PARD3(S144);PARVA(S14);PARVA(S19);PATL1(S278);PBRM1(S13);PCDH7(S1011);PCM1(S93);PCNP(T139);PDS5B(S1182);PDS5B(S1358);PDXDC1(S718);PEAK1(S1036);PER1(S815);PEX19(S54);PFAS(S569);PHAX(S368);PHF3(S1133);PHLDB2(S204);PI4KB(S266);PIH1D1(S173);PIK3C2B(S155);PIKFYVE(S307);PININ_HUMAN_Phospho (ST);PIP5K1A(S460);PIPSL(S407);PJA1(T277);PKP4(S314);PLCL2(S17);PLEC(S4613);PLEKHA1(S332);PLEKHA5(S885);PLEKHA7(S556);PLXDC2(S506);POLR2A(S1875);POLR2A(S1878);POLR2A(S1906);POLR2A(S1910);POLR2A(S1913);POLR2A(T1885);POLR2A(Y1881);POLR2A(Y1916);POM121(S395);POM121(S396);POM121(S435);POM121B(S19);POM121C(S372);POM121C(S412);PPFIA1(S666);PPFIA1(S763);PPFIBP2(S363);PPHLN1(S201);PPHLN1(Y162);PPP1R13L(S102);PPP1R2(T89);PPP4R2(S224);PPP6R1(S531);PRAG1(S889);PRC1(S4);PRDM2(S796);PREX1(S1200);PREX1(S319);PRR12(S487);PRR12(S560);PRR12(S561);PRR36(S251);PRR5(S11);PRRC2B(S1395);PRRC2C(S1544);PRUNE2(S1842);PSMF1(S153);PSPC1(S477);PSRC1(S140);PTK2B(S375);PTPN14(S314);PTPRZ1(S293);R3HCC1(S236);RAB11FIP1(S156);RAB11FIP1(S202);RAB11FIP2(S150);RAB31(S35);RABL6(S492);RACGAP1(S203);RAF1(S259);RALBP1(S92);RALBP1(S93);RALGPS2(S329);RANBP2(S1128);RANBP2(S2454);RAP1GAP(S499);RAP1GAP2(S608);RAP1GAP2(S609);RAPGEF2(S1080);RAPGEF3(S918);RAPGEF6(S1094);RASAL3(S72);RB1(S807);RBBP6(S873);RBL2(S662);RBM12B(S278);RBM12B(S280);RBM12B(S839);RBM15(S292);RBM15B(S265);RBM39(S97);RBM39(Y95);RBM5(S624);RBMX(S332);RBMX(S91);RBMX2(S273);REPS1(S540);REPS1(Y126);RET(S696);RETREG3(S258);RETREG3(S260);RETREG3(S320);RFC1(S71);RFC1(Y67);RFX7(S424);RGL2(T752);RGPD1(S1463);RGPD2(S1471);RGPD3(S1479);RGPD4(S1479);RGPD5(S1478);RGPD8(S1478);RICTOR(S1284);RIF1(S1554);RIF1(S1707);RING1(S38);RLF(S1633);RMDN3(S46);RNF2(S168);RPA1(T180);RPL5(S185);RPRD2(S1099);RPS14(S139);RPS6(S235);RPS6KA1(S380);RPS6KA3(S227);RPS6KA4(S682);RPS6KA6(S232);RPS6KB1(S427);RPS6KB1(S441);RPTOR(S863);RREB1(S1167);RRP1B(S245);RRP1B(S453);RRP1B(S458);RSBN1L(S105);RSL1D1(S361);RTKN(S520);SACM1L(S514);SACS(S4246);SAFB(S601);SAFB2(S195);SALL3(S102);SALL3(S1268);SALL3(S39);SALL3(S98);SAMHD1(S33);SAMHD1(T21);SATB1(S637);SBNO1(S214);SCAF1(T976);SCARF2(S742);SCML2(S590);SEC16A(S136);SEC22B(S137);SEC31A(S799);SEC62(S357);SENP3(S169);SENP3(S181);SENP6(S352);SF3A1(S451);SF3B2(S307);SF3B2(T780);SFN(S45);SH3KBP1(S230);SH3KBP1(S587);SHANK2(S67);SHC3(S474);SHROOM3(S1221);SKIV2L(S256);SLAIN2(S48);SLC12A4(S47);SLC12A4(T926);SLC12A6(T991);SLC12A7(T926);SLC38A1(S52);SLC6A15(S687);SLC7A6(S22);SLC9A1(S605);SLC9A1(S703);SLC9A3R1(S269);SLTM(S1002);SLX4(S1028);SLX4(S1070);SLX4(S1309);SLX4(S1333);SLX4(S1469);SLX4(S584);SLX4IP(S396);SMG1(S3570);SMG1(T3573);SMG7(S270);SMG9(S32);SNRPA1(T180);SNTB2(S95);SNW1(S232);SNX17(S421);SORBS1(S475);SOX11(S137);SOX11(S332);SPAG9(S733);SPAM1(S78);SPECC1(S55);SPP1(S303);SPRY2(S142);SPTBN1(T7);SPTBN2(S2171);SRCAP(S1859);SRCAP(S274);SRRM1(S694);SRRM2(S1103);SRRM2(S994);SRRM2(T1531);SRSF11(S323);SSH3(S87);SSR1(S268);STAU1(S278);STIM1(S608);STIM2(S680);STIP1(S481);STK10(S448);STK3(T174);STK4(T177);STMN1(S46);STMN2(S80);STRN3(S229);STX17(S289);STXBP5L(S544);SUCO(S1226);SUPT5H(S671);SUPT5H(T799);SVIL(S221);SYNJ1(S1392);TANC2(S1545);TBC1D1(S237);TBC1D10B(S132);TBC1D10B(T148);TBC1D13(S184);TBC1D4(S588);TBC1D5(S554);TBKBP1(S504);TBX2(S379);TBX2(S386);TET2(S1107);TEX10(S637);TEX2(S732);TGS1(S154);THRAP3(S379);TICRR(S1413);TICRR(S1430);TICRR(S1433);TINF2(S330);TJAP1(T422);TJP2(S1067);TJP2(S1159);TJP2(T455);TJP3(S164);TLK1(S744);TLK2(S111);TMEM9(S137);TMF1(S344);TMOD3(S25);TMPO(S184);TNIK(S688);TNK2(Y827);TNKS1BP1(S983);TNRC18(S1989);TNS3(S363);TOMM34(S186);TOP2A(S1106);TOP2A(S1393);TOP2B(S1466);TP53BP1(S1086);TP53BP1(S831);TRAF4(S426);TRAPPC12(S184);TRIP10(S296);TRIP11(S464);TRMT1(S625);TRO(S155);TSC1(S505);TSPYL2(S16);TSPYL2(S20);TTC7B(S160);TTYH3(S496);TTYH3(S522);UBA1(S21);UBA1(S820);UBAP2L(S470);UBE2E3(S8);UBE2O(S515);UBR4(S2885);UBR5(S1549);UBR5(S2484);UBR5(S2486);ULK1(S450);UNKL(S15);UPF3B(T169);USO1(S942);USP32(S1423);USP36(S682);UTP11(S241);VANGL1(T47);VAV3(S116);VDAC2(S115);WAC(S523);WAPL(S77);WDR44(S561);WDR48(S335);WDR59(S822);WDR62(S1144);WDR77(T5);WIPF2(S235);WIPI2(S413);WIZ(S996);WNK1(S2270);WNK3(S1471);WRAP53(S26);WWC1(S899);XRN1(S1645);YBX3(S38);YEATS2(S447);YWHAB(S47);YWHAE(S46);YWHAG(S46);YWHAH(S46);YWHAQ(S45);YWHAZ(S45);ZBTB17(S120);ZBTB7A(S337);ZBTB7A(S549);ZC3H13(S873);ZC3H15(S360);ZC3HAV1(S271);ZC3HAV1(S275);ZC3HAV1(S378);ZC3HAV1(T273);ZC3HC1(S359);ZDHHC18(S19);ZDHHC5(S296);ZEB1(S646);ZFAND5(S48);ZFC3H1(S352);ZFP91(S103);ZFP91(S82);ZFP91(S83);ZFPM1(S909);ZIC3(Y425);ZKSCAN2(S789);ZKSCAN8(S12);ZNF106(S641);ZNF142(S904);ZNF281(T888);ZNF362(S410);ZNF521(S605);ZNF579(S483);ZNF609(S491);ZNF639(S88);ZNF687(S1118);ZNRF2(S21);ZRSR2(S384);ZSCAN10(S167);ZSCAN29(S153);ZSWIM8(S53);ZSWIM9(S107)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>PRKAA1</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>6</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>CIC(S173);DCLK1(S332);EGLN1(S125);PPP1R12A(S445);PRAM1(S334);SH3PXD2B(S291)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>PRKACA</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>110</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>ABLIM1(S452);AFDN(S1799);ALDH1A3(S95);ALKBH5(S361);ANKRD2(S99);ARHGEF17(S420);ASIC3(S39);AUTS2(S941);BAIAP2(S366);BTF3(S30);CAD(S1859);CANX(S554);CDK12(T893);CFL1(S3);CLASP1(S636);COBLL1(S394);COL4A3BP(S373);DBNL(T291);DCUN1D5(S9);DDX17(S571);DENND4C(S989);DENND5B(S1076);DIP2B(S100);ECD(S205);EML3(S176);ERBIN(S1168);ERCC6L(S820);ESS2(T386);FAM102B(S228);FAM189A1(S18);FAM208B(S340);FAM83G(S634);FARP2(S389);FBXL15(S262);GPN1(S338);GSK3A(S21);GTF3C2(S167);HDAC1(S421);HDAC1(S423);HDGFL2(S454);HMGCR(S872);HSPB1(S82);ID2(S14);IRS2(S306);ITPR3(S1832);ITSN1(S978);JPT1(S28);KHDRBS1(S20);KIF21A(S855);KLC2(S610);LIMD2(S29);LINC00322(S228);LRRTM4(S195);LUZP1(S995);MAP3K2(S153);MAPRE1(S155);MARCKS(S167);MARCKS(S170);MEPCE(S152);MPRIP(S993);MRGBP(S195);MTFR1L(S103);MTMR12(S564);MYL12A(S19);MYL12B(S20);MYL9(S20);NASP(S705);NEK6(S206);PDCD5(S119);PGM5(S510);PHACTR4(S590);PHC3(S823);PHIP(S1315);PPHLN1(Y162);PPP1R12A(S445);PRMT9(S81);PRRC2A(S1386);PXN(Y88);RAB3IP(S157);RBMX(S352);RFX7(S1081);RPL15(S34);RPL34(S12);RPS6KB1(S441);RPTOR(S722);RRP9(S293);SAFB2(S787);SF3A1(S329);SH3BP1(S612);SH3BP1(S613);SH3BP2(S278);SH3PXD2B(S291);SKIV2L(S133);SLTM(S1014);SLTM(S551);SLTM(S553);SNRNP200(S225);SRSF7(S167);SSH3(S37);TMEM201(S441);TMX1(S270);TRA2B(T201);TRIM37(S773);TRPV3(S372);ULK1(S556);VRTN(S432);XPR1(S668);ZNF185(S64);ZNRF1(S123);ZSCAN10(S6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>PRKACB</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>18</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>ALDH1A3(S95);CFL1(S3);DDX17(S571);DENND5B(S1076);DIP2B(S100);EML3(S176);HDGFL2(S454);ITSN1(S978);LIMD2(S29);MARCKS(S170);MEPCE(S152);MTMR12(S564);PHACTR4(S590);PHC3(S823);PRMT9(S81);RPS6KB1(S441);RRP9(S293);ZNF185(S64)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>PRKCA.B</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>14</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>CAD(S1859);EIF4ENIF1(S120);GOLGA4(S1248);HCLS1(T308);HSPB1(S82);KHDRBS1(S20);MIA3(S1740);PCBP2(S272);PHACTR1(S505);RPS27(S78);RPS27L(S78);RPS6(S240);TMX1(S270);WT1(S273)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>PRKCI</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>1056</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>09/06/18 00:00:00(T418);AAAS(S495);AAK1(T653);ABI1(S183);ABI1(S222);ABI2(S183);ABI2(S227);ABRAXAS2(S372);ACIN1(S825);ACKR3(S347);ADAM17(S791);ADD1(T11);ADD3(S679);AFAP1(S278);AFAP1(S282);AFAP1(S668);AFDN(S1318);AFF1(T372);AFF1(T376);AGAP2(S929);AGAP3(S538);AGPS(S65);AHCTF1(S1142);AHDC1(S1064);AHNAK(S5737);AHNAK(S5739);AHNAK(T5729);AHSG(S138);AJUBA(S263);AKAP11(S1242);AKAP11(S1611);AKAP13(S1559);AKAP13(S1929);AKAP2(T399);ALKBH5(S361);AMPD2(S100);ANK3(S1459);ANKLE2(S914);ANKRD12(S149);ANKRD27(S962);ANKRD27(T1023);ANKS1A(T318);ANKZF1(S361);ANLN(S658);AP3D1(S829);ARAF(S214);ARFGAP2(S368);ARFIP1(S132);ARHGAP21(S476);ARHGAP25(S507);ARHGAP45(S23);ARHGAP45(S577);ARHGEF11(S1458);ARHGEF12(T736);ARHGEF16(S107);ARHGEF2(S122);ARHGEF2(T152);ARHGEF6(S684);ARID1A(S1138);ARID1A(S1140);ARID1A(T1146);ARPC2_HUMAN;ARPP19(S104);ASAP2(S822);ATAD2B(S83);ATG2A(S498);ATL1(S10);ATL2(S27);ATN1(S34);ATN1(T669);ATN1(T691);ATXN2(S850);ATXN2(T853);ATXN2L(T31);ATXN2L(T44);BAD(S99);BAG6(S1081);BAG6(S113);BAIAP2(S261);BAIAP2(S366);BAIAP2L1(S251);BAIAP2L1(S261);BAIAP2L1(T252);BAZ1A(S1281);BAZ1B(S1468);BAZ1B(S705);BAZ1B(S716);BAZ1B(T710);BCAM(S600);BCKDHA(S339);BCL7B(T109);BCL9(S917);BCL9(T315);BCL9L(S750);BCLAF1(S281);BCLAF1(S648);BICD1(S546);BIN2(S440);BIN2(S462);BRAF(S365);BTF3(S30);BUD13(T123);C1orf198(S175);C1orf226(S18);C1orf226(S258);C2CD2(S441);C2CD2L(S691);C2CD4C(S273);C2CD5(S260);C9orf40(S71);CAD(S1406);CAMK1(T181);CAMSAP1(S629);CAMSAP3(S431);CAP1(T307);CARD9(S425);CARHSP1(S52);CASC1(S504);CASK(S589);CASP3(S26);CBL(S486);CCDC120(S286);CCDC85A(S347);CCDC85C(S179);CCDC85C(S246);CCDC85C(S258);CCDC86(S110);CCNL2(S330);CCNT2(S480);CCSER1(S448);CD2BP2(S194);CD3EAP(S27);CD5L(S292);CDC25B(S230);CDC25B(S238);CDC25B(S323);CDC25B(S375);CDC42EP1(S192);CDC42EP4(S118);CDC42EP4(T23);CDC5L(T396);CDCA7L(T81);CDK11A(S271);CDK11A(T583);CDK11B(S283);CDK12(S383);CDK12(S385);CDK12(T893);CDK14(S24);CDK17(S137);CDK17(S180);CDK18(S132);CDK18(S14);CENPF(S2996);CENPF(S3150);CENPJ(S859);CGN(S149);CHAF1A(S772);CHAMP1(S184);CHAMP1(S389);CHD4(S1531);CHD4(T517);CHD8(S1995);CHEK1(S280);CHERP(S815);CHERP(S817);CHERP(S904);CHERP(T819);CIC(S173);CLASP2(S1013);CLN6(S23);CNN3(S285);CNN3(S293);CNN3(S296);CNN3(S298);COIL(T303);COL4A3BP(S373);COPB2(T861);CRIP2(S115);CRKL(Y198);CRTC1(S153);CRTC1(S158);CRTC1(S172);CRTC3(S329);CRTC3(S370);CSNK1D(S382);CSTF2(S513);CSTF2(S518);CTDSPL2(S104);CTNND1(S349);CTNND1(T906);CTTNBP2NL(S444);CTTNBP2NL(S484);CXXC1(S138);DAB2IP(S747);DAPK3(S312);DAXX(S671);DBN1(S341);DBNL(T271);DBP(S161);DCAF5(S655);DCLK1(S332);DCP1A(T531);DDA1(S33);DDX21(S89);DDX23(S109);DDX41(S68);DDX42(S751);DENND4C(S1184);DENR(S73);DHRS13(S330);DHX8(S460);DKC1(S455);DKC1(T458);DLG5(T1279);DLGAP4(S666);DLGAP4(T975);DMXL2(S1400);DNTTIP2(S82);DOK3(S330);DPPA4(S221);DPPA4(T215);DPYSL2(S518);DSN1(S109);DUS3L(S272);DVL3(S125);DYNC1LI1(T512);EGLN1(S125);EHBP1L1(S310);EIF3A(S1188);EIF3A(S1336);EIF3A(S882);EIF3D(S161);EIF4B(S283);EIF4EBP1(S65);EIF4ENIF1(S564);EIF4G1(S1187);EIF4G1(S1194);ELAC2(S199);ELMSAN1(S996);EML3(S176);EML4(S895);EP400(S943);EPB41(S709);EPB41L1(S510);EPB41L2(S39);EPB41L2(S58);EPB41L3(S11);EPB41L3(S420);EPB41L3(T3);EPN2(S173);EPRS(S885);ERC1(S17);ERC1(S7);ERF(S532);ESCO2(S75);ESS2(T386);ESYT1(S627);ESYT2(T753);EVL(S354);EZH2(S362);F5(S1574);FAM102A(S189);FAM102B(S228);FAM117A(S145);FAM117A(S29);FAM117B(S273);FAM122A(S62);FAM122B(T51);FAM129A(T590);FAM171A2(S810);FAM83B(S664);FBL(S124);FBRSL1(S790);FERMT3(S15);FNBP1(S299);FNBP1(S502);FNBP1(S517);FNBP1(S521);FNBP1(T507);FNBP1L(S505);FNBP4(S18);FNDC3B(S208);FOXK2(S369);FOXK2(S61);FOXO3(T32);FRMD3(S416);FRMD6(S522);FRMD6(S525);FRS2(S211);FXR2(T598);FYTTD1(S16);GAB1(S419);GAB2(S141);GAB2(S210);GAB2(T391);GAPVD1(S757);GAPVD1(S902);GATAD2B(S129);GATAD2B(S134);GATAD2B(S333);GCFC2(T428);GFI1(S96);GFI1(S98);GFPT1(T262);GIGYF2(S23);GIGYF2(T25);GJA1(S325);GLCCI1(S30);GLCCI1(T81);GMIP(S460);GOLGA4(S71);GON4L(S206);GPRIN1(S229);GPSM2(S565);GSK3A(S21);GTF2I(S412);GTF2I(T687);GTF3C1(S1543);GTF3C2(S167);GTPBP1(S580);GTPBP4(S558);GTSE1(S575);GZF1(S613);HDAC7(S358);HDAC7(S487);HECTD1(S1567);HELZ(T1163);HERC2(S1539);HIC2(S197);HIPK1(Y352);HIPK2(Y361);HIRA(S549);HJURP(S486);HMBOX1(S133);HMG20A(S105);HMGA1(S44);HMGA2(T100);HMGCR(S872);HNRNPA2B1(S341);HNRNPK(S216);HNRNPK(T107);HNRNPUL1(S718);HSF1(S303);HSH2D(S194);HTATSF1(S409);HUWE1(S726);HUWE1(S727);ICE1(S1712);ID2(S14);ID2(S5);ID2B(S5);IFRD1(S15);IGLL1(S62);INAVA(S246);INCENP(S831);INCENP(T832);INPP4A(S210);INPP5J(S278);INTS1(S13);IRF2BP2(S360);IRF2BP2(T404);IRF2BP2(T412);IRS1(T1103);IRS2(S577);IRS2(S620);ITGB3BP(S33);JMJD1C(T1187);JPH1(S216);JPH1(S452);JUP(S665);KAT5(S199);KBTBD11(S314);KDM2A(S721);KDM2B(S1031);KHDRBS1(S20);KIAA0754(S42);KIAA0930(S306);KIAA1671(S1499);KIDINS220(S1633);KIF13B(S1410);KIF1B(S1057);KIF21A(S855);KIF21B(S1149);KIFC1(S351);KLC2(S582);KLC2(S610);KLF16(S105);KLF16(S108);KNOP1(S42);KRI1(S136);KRI1(S622);KRT13(S427);KRT18(S398);KRT8(S253);KRT8(S43);L1RE1(S33);L1TD1(S173);L1TD1(S578);LARP1(S1056);LARP1(S546);LARP1(S824);LARP1(S847);LARP1(T622);LARP1(T770);LARP1B(S343);LARP4B(S498);LARP6(T450);LAT2(S44);LDB1(S265);LDB1(S309);LIG1(T108);LIMD2(S29);LIN9(S321);LINC00337(S30);LRCH4(S515);LRCH4(S517);LRMP(S131);LRMP(T133);LRRC41(T327);LRRFIP1(S115);LSM14A(S182);LSM14A(S216);LSM14A(T201);LSM14B(S165);LSP1(S177);LUC7L2(S18);LUC7L2(S347);LZTS1(S233);MACF1(S7279);MAF1(S68);MAK16(S197);MAK16(T202);MAP1B(S1254);MAP1B(S1256);MAP1B(S1312);MAP1B(S541);MAP1B(T1799);MAP1B(T1964);MAP1S(S741);MAP2(S1555);MAP3K1(S292);MAP3K2(S153);MAP3K20(S727);MAP3K4(S1274);MAP4(S1073);MAP4(S928);MAP4(T942);MAP4K4(S900);MAP7D1(S113);MAP7D1(S254);MAP7D1(S552);MAPRE2(S200);MARCKS(S159);MARCKSL1(S104);MARK3(S400);MARK3(S419);MAST2(S148);MAST3(S747);MATR3(S598);MAVS(S222);MBD1(S297);MCM3(S704);MCMBP(S298);MED13(S530);MED13(S537);MED13(T326);MEF2D(S121);MELK(S505);MELK(S529);MEPCE(S152);MEPCE(S254);METAP2(S45);MFAP1(T267);MFSD10(S271);MFSD2B(S494);MGA(S1457);MGA(S924);MICALL2(S143);MINK1(S733);MIS18BP1(S541);MKI67(T1557);MKL1(S335);MPRIP(S993);MSH6(S309);MTA1(S576);MTA1(T564);MTA2(S433);MTCL1(S263);MTDH(S568);MTFR1L(S103);MTFR1L(S238);MTM1(S590);MTMR12(S564);MTSS1L(S601);MVB12A(S170);MYBBP1A(S1310);MYBPC2(S105);MYCBP2(S2315);MYCBP2(S2749);MYCBP2(S2751);MYH10(S1937);MYH9(S1943);MYO7B(S1279);MYOF(S1915);NAB2(S193);NASP(S480);NAV1(S296);NAV1(S528);NAV1(S806);NCBP1(T21);NCOA3(Y574);NCOR1(S70);NDRG1(S333);NDRG2(S350);NDRG3(S338);NEK4(S639);NELFA(S225);NELFB(S557);NEO1(S1194);NES(S1016);NES(S455);NES(S475);NES(S476);NEURL4(S502);NFATC1(S245);NFATC2(S236);NFATC2(S243);NFATC2(S255);NFATC2(S326);NFATC2IP(S366);NFRKB(S1291);NFX1(Y48);NHSL1(S1233);NIFK(T220);NIPBL(S2658);NMT1(S47);NMT2(S38);NOL8(S1099);NONO(T440);NOP56(S570);NOP58(T508);NPY1R(S368);NSD2(S121);NSUN2(S469);NUMB(S247);NUP107(S86);NUP214(S1023);NUP214(S678);NUP214(T670);OBSL1(T1669);OGFR(S378);ORC1(S383);OSBP(S240);OSBP(S379);OSBPL11(S189);OSBPL5(S12);OSER1(S82);OSER1(S84);OTUD5(S452);P2RX7(S470);P2RX7(T467);PAK1(T212);PAK4(S104);PAK4(S163);PALLD(S893);PALM3(S303);PANK2(S168);PAPD5(S52);PAPD5(S55);PARD3(S717);PATL1(S184);PAXBP1(T563);PBRM1(S13);PBRM1(S14);PBRM1(T43);PCBP1(S246);PCDH1(S962);PCM1(S1765);PCYT1A(S331);PDAP1(S57);PDE3B(S318);PDE3B(S495);PDHA1(S300);PDHA2(S298);PDLIM4(S112);PDS5A(T1208);PDS5B(S1162);PDYN(S101);PER2(S977);PGK1(S203);PGM1(S117);PGRMC1(S181);PHACTR1(S505);PHACTR2(S235);PHACTR4(S628);PHAX(S368);PHF14(S147);PHF14(S774);PHF6(S154);PHKA2(S1015);PHLDB1(S334);PHLDB1(S430);PHRF1(S1229);PI4KB(S428);PI4KB(S511);PIGT(S235);PIK3AP1(S759);PIK3C2B(S155);PIK3CD(T226);PINX1(S163);PITPNC1(S299);PITPNM1(T665);PKD2(S832);PKP2(S329);PLCG1(S1263);PLEC(S4386);PML(S36);POC5(S78);POGZ(T439);POLA1(S186);POLA2(S150);POLH(S380);POLM(S12);POLR2A(S1868);POLR2A(S1878);POLR2A(S1910);POLR2A(Y1860);POLR2M(S10);PPAN(S359);PPFIBP1(S466);PPFIBP1(S599);PPFIBP1(S601);PPHLN1(S110);PPHLN1(S133);PPIG(S687);PPIP5K1(S1152);PPIP5K2(S1074);PPM1H(S119);PPP1R12A(S445);PPP1R12A(S910);PPP1R13L(S102);PPP1R18(S125);PPP1R2(S121);PPP1R2(S122);PPP1R2(S72);PPP1R2(T92);PPP1R2P3(S121);PPP1R2P3(S122);PPP1R35(S87);PPP1R35(T84);PPP1R9B(S100);PPP4R2(S226);PPP4R3A(S741);PPP6R3(S523);PRAG1(S745);PRAG1(S827);PRAM1(S473);PRAM1(S48);PRC1(S4);PRDM2(S739);PRKAR2A(S99);PRKD1(S205);PRKD1(S397);PRKD1(S742);PRKD3(S391);PRKD3(S735);PRKRA(T20);PRPF6(S279);PRPF6(T275);PRRC2A(S1110);PRRC2A(S1386);PRRC2A(S146);PRRC2B(S1395);PRRC2C(S1544);PRRC2C(T2673);PSIP1(S271);PSIP1(T272);PSMD1(T270);PTK2(S716);PTPN1(S378);PTPN12(S435);PTPN12(S449);PTPN13(S1029);PTPN14(S760);PTPN2(S293);PTPRK(T854);PUM1(S124);PUM1(S209);RAB12(S21);RABEP1(S377);RABEP2(S193);RAF1(S294);RAI14(S412);RAI14(T283);RALGAPA1(S797);RALY(S135);RALY(T286);RANBP1(S60);RANBP1(T18);RANBP2(S1835);RANBP2(S21);RAPGEF1(S217);RARG(S43);RASAL3(S51);RASAL3(S865);RASGRP2(S391);RASGRP2(S576);RASGRP2(S578);RB1(T353);RB1(T601);RBBP6(S873);RBL1(S640);RBL1(T369);RBM10(S736);RBM14(S618);RBM15(S700);RBM15B(S113);RBM15B(S265);RBM15B(S267);RBM15B(T532);RBM23(S140);RBM23(S142);RBM39(S117);RBMS1(S27);RBMS1(S49);RBMX(S208);RBMX(S326);RBMX(S332);RBMX(S352);RBMX(S88);RBMXL1(S208);RBSN(S211);REEP3(S242);REEP4(S152);RGPD5(T19);RGPD8(T19);RIC8A(S502);RICTOR(S1284);RIF1(S1542);RILPL2(S107);RLIM(S228);RLIM(S230);ROBO2(T1154);ROCK1(T1101);RPA1(T180);RPL24(S149);RPL28(S115);RPS14(S139);RPS27(S78);RPS27L(S78);RPTOR(T865);RREB1(S1219);RREB1(S1238);RRP1B(S245);RSF1(S1359);RSF1(T1278);RSL1D1(T358);RTKN(S520);RUBCN(S388);RYBP(S99);SAFB(S234);SAFB(S601);SAFB(S604);SAFB2(S233);SALL3(T935);SALL4(S748);SALL4(S753);SAMD1(T107);SASH1(S90);SBNO1(T819);SCAF1(S874);SCAF1(T976);SCAF11(S726);SCAF11(S796);SCAF11(T331);SCAF11(T799);SCAMP3(S32);SCRIB(T475);SEC22B(S137);SELENOK(S16);SEMA4C(T97);SEMA6A(T996);SETD5(S865);SF3A1(S329);SF3B1(T261);SF3B1(T273);SF3B1(T434);SF3B1(T436);SF3B2(S303);SF3B2(T780);SFPQ(S33);SFSWAP(S868);SFSWAP(S870);SGPP1(S101);SH2D5(S231);SH3BP1(S585);SH3BP1(S586);SH3BP4(S296);SH3GL1(S288);SH3KBP1(S183);SH3KBP1(S410);SH3KBP1(S587);SH3PXD2B(S291);SHANK1(T946);SHANK2(S1069);SHANK2(S452);SHC1(S139);SHROOM2(S413);SHROOM2(T647);SHROOM3(S913);SHROOM3(T243);SIK3(S551);SIK3(S866);SIN3A(T292);SIPA1(S839);SIPA1L1(S1568);SKAP2(S5);SLAIN2(S391);SLAIN2(S413);SLBP(S111);SLC12A4(T926);SLC12A6(T991);SLC12A7(T926);SLC13A4(T244);SLC30A1(S468);SLC4A10(S238);SLC4A7(S233);SLC4A7(S400);SLTM(S1014);SLTM(S553);SMAP(S24);SMAP(S25);SMAP2(S231);SMAP2(S240);SMARCA4(S610);SMARCA4(T609);SMARCC2(S283);SMARCD1(S206);SMARCD2(S229);SMARCD3(S181);SMC3(S1067);SMC3(S1085);SMCR8(S489);SNRPA1(S178);SNRPA1(T180);SNX1(S39);SON(T1555);SOX15(S37);SPAG9(S730);SPAG9(S733);SPECC1(S914);SPTAN1(S1031);SPTBN1(S2102);SPTBN1(S2164);SQSTM1(S287);SRRM1(S391);SRRM1(S393);SRRM1(S549);SRRM1(S551);SRRM1(S597);SRRM1(S740);SRRM1(S775);SRRM1(T385);SRRM1(T572);SRRM1(T574);SRRM1(T614);SRRM2(S1132);SRRM2(S1444);SRRM2(S1458);SRRM2(S1691);SRRM2(S1694);SRRM2(S1925);SRRM2(S311);SRRM2(S317);SRRM2(S387);SRRM2(S395);SRRM2(S449);SRRM2(S774);SRRM2(T1531);SRRM2(T1927);SRRM2(T2125);SRRM2(T2397);SRRM2(T289);SRRM2(T315);SRRM2(T316);SRRM2(T326);SRSF10(S133);SRSF11(S449);SRSF2(S189);SRSF2(S191);SRSF4(S113);SRSF4(S446);SRSF5(S117);SRSF6(S119);SRSF9(S204);SSH3(S37);SSSCA1(S78);ST13(S75);ST13(S76);ST13(T93);ST13P4(T103);STAT5A(S780);STIM2(S680);STIM2(S719);STK4(S414);STX17(S289);SUGP2(S315);SUGP2(T281);SURF2(S234);SURF6(T229);SYN1(S553);SYNRG(S1075);SYNRG(T931);TAF3(S183);TAF4(S543);TAOK1(S9);TBC1D1(S237);TBC1D15(S70);TBC1D4(S588);TBC1D4(S751);TBC1D5(S544);TBX2(T335);TCEA1(S97);TCOF1(S1378);TCOF1(S156);TFAP4(S123);THOC5(S307);THRAP3(S232);THRAP3(S682);TJP1(S968);TJP2(T1054);TJP2(T462);TJP3(S369);TJP3(S371);TJP3(S591);TK1(S231);TLE1(S284);TLE3(S263);TLE4(S208);TMCC1(S414);TMCC2(S438);TMCC3(S216);TMEM131(S1604);TMEM163(S12);TMEM201(S441);TMEM201(S454);TMF1(S925);TNKS1BP1(S429);TNKS1BP1(S983);TOP2B(S1471);TOP2B(S1526);TOP2B(S1581);TOPORS(S194);TOPORS(S585);TP53BP1(S1316);TP53BP1(S1317);TP53BP1(S379);TP53BP1(T1214);TP53BP1(T382);TP53BP2(S698);TPR(T2116);TPRN(S241);TRA2A(T202);TRA2B(S102);TRA2B(T201);TRA2B(T212);TRAF4(S426);TRAPPC10(S711);TRIM11(S85);TRIP10(S296);TRIP11(S1891);TRIP12(T941);TSC2(S1448);TSEN54(S229);TSEN54(S238);TUBB(S75);TUBB2A(S75);TUBB2B(S75);TUBB3(S75);TUBB8(S138);TWISTNB(S304);UBAP2L(S445);UBAP2L(S471);UBE2O(S515);UBE2O(T834);UBQLN4(S100);UBQLN4(S98);UBR5(T637);UIMC1(S653);ULK1(S556);ULK1(S719);ULK1(T717);UNG(S63);USP32(S1416);USP32(S1423);USP36(S611);USP42(S754);USP54(S1036);USP6(S1214);USP8(S716);UTP20(T1741);VASP(S329);VIPAS39(S121);VPS8(S1338);WAPL(S223);WASHC2A(S288);WASHC2A(S522);WASHC2A(S728);WASHC2C(S288);WASHC2C(S726);WDR20(S434);WDR20(S492);WDR33(S1219);WDR44(T163);WDR48(T343);WIZ(S1010);WWC3(S563);WWTR1(S90);XRCC1(S446);YAP1(S105);YAP1(T110);YAP1(T119);YBX3(S293);YRDC(S37);ZBED6(S14);ZBTB21(S343);ZBTB48(S179);ZC3H11A(S758);ZC3H13(T364);ZC3H14(S343);ZC3H3(S571);ZC3H4(S1110);ZC3H4(S1267);ZC3H4(S159);ZC3H4(Y162);ZC3HAV1(S257);ZC3HAV1(S335);ZC3HAV1(T273);ZC3HAV1(Y348);ZC3HC1(S354);ZFAND5(S54);ZFHX3(S3432);ZFPM1(S786);ZFYVE19(S354);ZMYM4(S122);ZMYND8(S425);ZNF136(S405);ZNF148(S306);ZNF185(S64);ZNF318(S709);ZNF408(T322);ZNF574(T154);ZNF609(S1055);ZNRF2(S21);ZP2(S454)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>PRKCQ</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>1</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>ZNF185(S64)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>PRKD2</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>5</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(T142);AMBRA1(S1205);APPL1(S401);CDK14(S134);CTU2(S419)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>PRKD3</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>4</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>EPB41L5(S436);IRS1(S374);KHDRBS1(S20);SLTM(S551)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>RIPK3</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>3</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>FXR1(S409);HAUS6(T584);TET2(S1107)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>ROCK1.2</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>105</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>AFF4(S1043);AHNAK(S5830);ALDH1A3(S95);ANKRD20A1(T762);ANKRD20A12P(T54);ANKRD20A2(T762);ANKRD20A3(T762);ANKRD20A4(T762);ANKRD20A8P(T762);APPL1(S401);ARHGEF18(S1124);ARID1A(S604);ASIC3(S39);BAIAP2(S261);BAIAP2(S366);BTF3(S30);CANX(S554);CDC25B(S323);CDC42EP1(S192);CLASP1(S636);DCAF15(S50);DEF6(S590);DEK(S32);DTX3L(S202);EIF2B1(S105);EIF2B1(S107);EPB41L1(S510);EPX(S670);EPX(S672);FAM111A(S62);FAM189A1(S18);FAM193B(S785);FARP2(S389);FBXL15(S262);GPN1(S338);GPSM2(S565);GTF3C2(S167);HSPB1(S199);HSPB1(S82);HSPH1(S809);JUN(S63);KAZN(S387);KDM2B(S1031);KIFC1(S349);KIFC1(S351);KMT2B(S821);LARP1(T649);LEMD2(S499);LINC00322(S228);LRRTM4(S195);LUZP1(S995);LZTS2(S570);MAP1B(S1427);MAP7D1(S460);MARCKS(S167);MARCKS(S170);MFSD10(S270);MRGBP(S195);MTBP(S755);NFATC2(S326);PATL1(T194);PDAP1(S176);PDCD5(S119);PGM5(S510);PGRMC1(S181);POLH(S379);PRAM1(S204);PRMT9(S81);PXN(S258);PXN(Y88);RAB11FIP1(S156);RAB11FIP2(S150);RAB3IP(S157);RHPN2(T655);RHPN2P1(T552);RPS6(S235);RRP9(S293);SCRIB(S1508);SERBP1(S203);SFRP2(S287);SFRP2(S289);SH3BP1(S612);SH3BP1(S613);SH3BP2(S278);SHROOM3(S439);SIRT1(S47);SKIV2L(S133);SLTM(S553);SNRNP200(S225);SP110(S380);SRSF7(S167);TMX1(S270);TNIK(S688);TNK2(Y827);TP53BP1(S580);TPX2(T369);TRIM37(S773);TRPV3(S372);XPR1(S668);ZC3H15(S381);ZC3H3(S569);ZC3H3(S571);ZFR(S1054);ZNF185(S64);ZSCAN10(S6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>RPS6KA2</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>814</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>09/05/18 00:00:00(S225);09/06/18 00:00:00(S416);09/09/18 00:00:00(S30);AAGAB(S311);AAK1(S14);AAK1(T653);ABI1(S222);ABI2(S227);ABLIM1(S640);ACIN1(S825);ACIN1(S838);ADAM10(S740);ADAM17(S791);AFAP1(S668);AFDN(S1318);AFF4(S703);AGAP1(S521);AGAP3(S538);AGO2(S387);AGPS(S65);AHNAK(S5031);AHNAK(S5739);AJUBA(S263);AKAP12(S598);AKAP12(S612);AKAP13(S1559);AKAP13(S1929);AKIRIN1(S22);AKT1S1(S88);AKT1S1(S92);ALDH5A1(S122);AMOTL2(S183);AMOTL2(S602);AMPD2(S100);ANKRD13D(S465);ANKRD13D(T469);ANKS1A(T318);APC(S1360);ARAF(S582);ARFGAP2(S368);ARFGAP2(S432);ARFIP1(S132);ARHGAP1(S50);ARHGAP17(T682);ARHGAP21(S476);ARHGAP25(S507);ARHGAP29(S930);ARHGAP45(S23);ARHGAP45(S67);ARHGEF16(S208);ARHGEF19(S336);ARHGEF2(S122);ARHGEF2(S886);ARHGEF2(S956);ARHGEF2(S960);ARHGEF2(T152);ARHGEF38(S553);ARHGEF6(S684);ARID4B(S778);ARL6IP4(S239);ARL6IP6(S80);ARPP19(S104);ASIC3(S37);ATAD2(S327);ATG2A(S498);ATL1(S10);ATRX(S1244);ATRX(S1245);BAG6(S1081);BAIAP2(S366);BAIAP2(T340);BCAR3(S290);BCKDK(T32);BCL11A(S608);BCL9(T315);BCL9L(S915);BCORL1(S1033);BCR(S215);BEST4(S173);BIN2(S259);BOD1L1(S1531);BRD4(S1083);BTF3(S30);C12orf43(S61);C1orf198(S175);C1orf226(S18);C1orf52(S158);C2CD2L(S411);C2CD5(S281);C5orf30(S167);C9orf78(T100);CALD1(T730);CAMKK1(S74);CAMKK2(S100);CAMSAP1(S629);CARMIL1(S933);CARS(S19);CASC1(S504);CASKIN2(S858);CASP3(S26);CASP8AP2(S875);CBL(S486);CCDC6(S323);CCDC6(S52);CCDC85C(S246);CCDC88A(S1417);CCDC97(S212);CCSER1(S448);CD97(S818);CDC25B(S230);CDC25B(S238);CDC25B(S375);CDC42EP1(S195);CDC42EP4(S118);CDC42EP4(S80);CDC42EP4(T23);CDCA3(S68);CDK11A(S271);CDK11B(S283);CDK12(S383);CDK12(S385);CDK12(T893);CDK14(S24);CDK14(S78);CDK5RAP2(S1887);CEP170(S1160);CEP170B(S1114);CEP170B(S772);CHAF1A(S206);CHAF1A(S873);CHD2(S1728);CHD4(S1531);CHD8(S1978);CHD8(S1995);CHD8(S2008);CHERP(S904);CIC(S173);CLASP1(S559);CLASP1(S688);CLASP2(S327);CLASP2(S360);CLASP2(S529);CLCC1(S532);CLDN10(S203);CLK1(S140);CLK3(S283);COBLL1(S394);COG2(T480);COL4A3BP(S132);COL4A3BP(S373);CPA6(S60);CPSF7(S48);CRAMP1(S70);CRTC1(S153);CRTC2(S70);CRTC3(S370);CTNND1(S349);CUX1(S1218);DAB2IP(S978);DBNL(S269);DCLK1(S332);DCP1A(S353);DDA1(S33);DDX10(S831);DDX3X(S594);DDX3X(S90);DDX3Y(S592);DENND4C(S1278);DENND4C(S989);DGKH_HUMAN_3 Phospho (ST);DLG5(S1115);DLGAP4(T975);DMXL2(S1400);DOCK11(S12);DOCK2(S587);DOCK7(S180);DOCK7(S888);DPH7(S353);DPPA4(T215);DSN1(S109);DSN1(S81);DUSP27(S966);DVL2(S480);DVL3(S125);DYRK1A(Y321);DYRK1B(Y273);EEF2(T435);EGLN1(S125);EHBP1(S432);EHBP1L1(S1257);EIF2B1(S107);EIF3A(S1188);EIF3A(S1336);EIF3A(S882);EIF4B(S283);EIF4B(S359);EIF4EBP2(T46);EIF4ENIF1(S577);EIF4ENIF1(S74);EIF4G1(S1194);EIF4H(S21);ELF1(S168);EMSY(S209);EMSY(T207);EPB41(S709);EPB41(S85);EPB41L3(S760);EPB41L4B(S390);EPB41L5(S348);EPN1(T460);EPN2(S173);EPRS(S882);EPX(S672);ERCC6L(S14);ERF(S532);ERLIN1(S324);ESCO1(S412);ESS2(T386);ESYT1(S627);EZH2(S363);EZH2(T367);FAM102A(S189);FAM102B(S228);FAM102B(S321);FAM109A(S213);FAM117A(S29);FAM122A(S143);FAM124A(T493);FAM208A(S1103);FAM47A(S259);FAM53B(S268);FAM53C(S232);FAM53C(S234);FAM53C(S247);FAM83H(S8);FAM83H(S892);FAM91A1(T353);FARP1(S340);FASN(T2204);FBXO21(S116);FERMT3(S15);FLNC(S2624);FNBP1(S296);FOXK1(S420);FOXK1(S428);FOXK1(T436);FRMD3(S334);FRMD6(S522);FRMD6(S525);FRMPD1(S342);FRS2(S211);FRY(S1936);FTSJ1(S271);FYTTD1(S16);GAB2(S141);GAB2(T391);GAPVD1(S902);GCFC2(S429);GCFC2(S430);GEMIN5(S770);GFI1(S94);GINS2(S182);GON4L(S206);GPBP1L1(S49);GRAMD1A(S263);GSE1(S909);GSK3A(S21);GSK3A(Y279);GSK3B(S9);GSK3B(Y216);GTF2F1(S385);GTF2F1(S433);GTF2I(S412);GTF2I(S823);GTPBP1(S44);GTPBP1(S47);GTSE1(S575);GYS1(S641);GYS1(S645);H1FX(S31);HDAC1(S393);HDAC4(S467);HDAC7(S358);HECTD1(S1387);HECW1(S1344);HECW2(S1310);HIPK1(Y352);HIPK2(Y361);HMGA1(S44);HMGCR(S872);HNRNPA3(S358);HPDL(S173);HSH2D(S194);HSPB1(S82);HUWE1(S3553);ICAM3(T526);ICE1(S1712);IGLL1(S62);INPP5D(S971);IQSEC2(S744);IRS1(S374);ITPR1(S1598);JMJD1C(S2053);JPH1(S216);JUP(S665);KANK1(S186);KANK2(S172);KANK2(S175);KHDRBS1(S20);KIAA1191(S183);KIAA1217(S361);KIAA1522(S404);KIF13B(S1410);KIF15(S1141);KIF1A(S1337);KIF21A(S855);KIFC1(S351);KLC2(S610);KMT2C(S2937);KNOP1(T310);KRT8(S475);L1TD1(S557);L3MBTL1(S676);L3MBTL2(S683);L3MBTL2(S689);LARP1(S774);LARP1(S824);LARP4B(S498);LARP7(S337);LARP7(T338);LAT2(S102);LAT2(S205);LINC00322(S226);LINC00337(S30);LMF1(S522);LMNB2(T34);LRCH4(S513);LRRFIP1(S120);LRRFIP2(S324);LRWD1(S259);LSM11(S21);LSM14B(S165);LSP1(S204);LSP1(S218);LUC7L(S327);LUC7L2(S18);LUC7L2(S347);LZTS1(S233);MACF1(S7279);MACO1(S332);MAP2(S1555);MAP3K1(S292);MAP3K2(S153);MAP3K20(S648);MAP3K20(S727);MAP3K4(S1274);MAP3K7(S439);MAP4(S928);MAP7D1(S113);MAP7D1(S93);MAP7D1(T97);MAPRE1(S155);MARCKSL1(S104);MARK2(S631);MARK3(S400);MAST2(S876);MAST3(S747);MATR3(S9);MCPH1(S333);MDC1(S1814);MDM4(S367);MELK(S505);MELK(S529);MEPCE(S152);METTL25(S193);MEX3C(S540);MEX3C(T541);MFF(S157);MFSD10(S271);MFSD2B(S494);MKI67(T1557);MLLT10(S519);MMACHC(S275);MMRN2(S562);MNAT1(S279);MPLKIP(S47);MPRIP(S993);MSL1(S362);MTA1(S639);MTCL1(S776);MTFR1L(S103);MTFR1L(S238);MTM1(S18);MTM1(S591);MTMR12(S716);MUC16(S10570);MVB12A(S170);MYCBP2(S2749);MYCBP2(S2751);MYH10(S1937);MYOF(S1915);NAA30(S199);NAB2(S193);NADK(S64);NAV1(S808);NAV2(S1808);NCBP1(S22);NCBP3(S415);NCBP3(T413);NCOA3(Y574);NCOA5(S381);NCOR1(S2120);NDRG1(S333);NDRG2(S332);NDRG2(S353);NDRG2(T330);NDRG2(T334);NDRG3(S331);NECTIN2(S433);NEK3(S355);NFIX(S265);NFX1(Y48);NHSL1(S1233);NIFK(T223);NOTCH2(S2093);NTHL1(S22);NUFIP2(S608);NUP210(S1877);OSBP(S193);OSBPL11(S189);OSBPL8(S807);OSBPL8(S808);OSER1(S82);OSER1(S84);OTUD4(S416);PAK4(S163);PALLD(S1116);PALLD(S1118);PALLD(S1121);PALM3(S303);PARD3(S717);PBRM1(S10);PBRM1(S13);PBRM1(S14);PBX2(S330);PCDH18(T442);PCDHGC3(S60);PCF11(S494);PCNP(S119);PCSK9(S47);PCYT1A(S343);PDE3B(S445);PDE7A(S113);PDE7B(S74);PDS5A(T1208);PDYN(S101);PFKL(S775);PGM2L1(S175);PHACTR1(S505);PHACTR4(S590);PHAX(S368);PHLDB1(S334);PHLDB1(S419);PHLDB1(S461);PHLDB1(S518);PHLDB1(T516);PI4KB(S428);PIGT(S235);PIK3C2A(S338);PJA1(S365);PJA1(S367);PKD2(S832);PLCG1(S1263);PLCH1(S970);PLEKHA2(S349);PLEKHA6(S808);PLEKHA6(S867);PLIN5(S203);PML(S518);POGZ(S746);POLA1(S186);POLH(S380);POLM(S12);POLR2A(S1868);POLR2A(S1878);POLR2A(S1910);POLR2A(Y1860);PPAN(S359);PPFIBP1(S466);PPFIBP1(S601);PPHLN1(S133);PPIG(S356);PPIP5K2(S1074);PPP1R12A(S445);PPP1R35(S87);PPP1R35(T84);PPP1R9A(S840);PPP1R9B(S100);PPP6R1(S529);PRAG1(S510);PRC1(S4);PRCC(S157);PRCC(S159);PRKAB1(S108);PRKAR2A(S78);PRKAR2A(S80);PRKRA(S18);PRPF6(S279);PRPF6(T275);PRRC2A(S1386);PRRC2C(S1544);PRRC2C(S1568);PTK2(S716);PTPN12(S435);PTPN12(S449);PTPN14(S760);PTPRZ1(S293);PUM1(S124);PUM2(S82);Phospho (ST);QSER1(S1211);RABEP1(S377);RABL6(S359);RAF1(S621);RALGAPA1(S797);RANBP1(S60);RANBP2(S1400);RANBP2(T2450);RANBP2(T799);RAPGEF6(S1094);RASAL3(S51);RASAL3(S72);RASGRP2(S576);RB1(T601);RBL1(S640);RBL1(T369);RBM14(S520);RBM15(S292);RBM15(S700);RBM15(S97);RBM15B(S113);RBM15B(S265);RBM15B(S267);RBM15B(T532);RBM17(S169);RBM23(S140);RBM23(S142);RBM39(S117);RBMX(S208);RBMX(S326);RBMX(S332);RBMX(S352);RBMX(S88);RBMXL1(S208);RBMXL1(S88);REPS1(S272);REPS1(T539);RFWD3(S425);RGPD1(T1459);RGPD1(T790);RGPD2(T1467);RGPD2(T798);RGPD3(T1475);RGPD3(T800);RGPD4(T1475);RGPD4(T800);RGPD5(T1474);RGPD8(T1474);RIPOR1(S349);RIPOR1(S351);RLIM(S228);RLIM(S230);ROBO1(S1055);RPGR(S961);RPL15(S34);RPL22L1(S118);RPL28(S115);RPRD2(S1099);RPRD2(T732);RPS14(S139);RPTOR(S859);RRAGC(S95);RRAGD(S96);RRN3(S170);RRN3(S172);RRP1B(S735);RRP1B(T728);RSF1(S629);SACS(S4246);SAFB(S601);SAFB(S604);SAFB2(S787);SAMD1(T107);SAMD4A(S420);SAMD4B(S172);SAP130(S465);SASH1(S90);SBNO1(S214);SCAF1(S874);SCAF11(S796);SCAF11(S802);SCAMP2(S320);SCAMP3(S32);SCRIB(S835);SCRIB(T475);SEC16A(S1194);SEC16A(S411);SEC16A(T19);SETD2(S2080);SETD2(S2082);SF1(S80);SF1(S82);SF3B1(T261);SF3B1(T267);SF3B1(T434);SF3B1(T436);SF3B2(S431);SF3B2(S435);SF3B2(S436);SFSWAP(S283);SGPP1(S101);SH3BP4(S296);SH3KBP1(S410);SH3PXD2B(S291);SHROOM2(T647);SHROOM3(S1497);SIK3(S866);SIPA1(S839);SKIV2L(S131);SLAIN2(S413);SLC12A4(T926);SLC12A6(T991);SLC12A7(T926);SLC38A1(S49);SLC4A10(S238);SLC4A7(S233);SLC9A1(S605);SLC9A1(S703);SLTM(S1014);SLTM(S551);SLTM(S553);SLU7(S215);SMAP2(S240);SMARCA4(S610);SMARCD1(S206);SMARCD2(S229);SMARCD3(S181);SMC4(S22);SMCR8(S489);SMG9(S32);SNAPC4(S599);SNRNP70(S320);SON(S2013);SON(S2129);SPAG9(S730);SPAG9(S733);SPEN(S725);SPN(S355);SPN(T341);SPTAN1(S1031);SPTBN1(S2169);SRP72(S621);SRP72(T624);SRRM1(S391);SRRM1(S431);SRRM1(S713);SRRM1(S738);SRRM1(T718);SRRM2(S1458);SRRM2(S1694);SRRM2(S1925);SRRM2(S2067);SRRM2(S2449);SRRM2(S2688);SRRM2(S2690);SRRM2(S508);SRRM2(S774);SRRM2(T1927);SRRM2(T2069);SRRM2(Y1049);SRSF10(S133);SRSF4(S113);SRSF4(S431);SRSF4(S446);SRSF5(S117);SRSF6(S119);SRSF7(S165);SRSF7(S194);SSH3(S37);SSSCA1(S78);STIM2(S680);STIM2(S719);STK10(S514);STK4(S414);STX17(S289);STXBP5L(S544);SUCO(S1081);SUDS3(S237);SUGP1(S485);SURF6(T229);SYNJ1(S1049);SYNRG(S752);TAF9(S155);TAF9(S158);TAOK2(S473);TAOK3(S442);TATDN2(S80);TBC1D1(S237);TBC1D10B(S687);TBC1D10B(T697);TBC1D10C(T439);TBC1D22A(S167);TBC1D5(S730);TCOF1(S1350);TCOF1(S156);TGFB1I1(S68);TGFBR2(S352);THAP4(S128);THRAP3(S232);THRAP3(S406);THRAP3(S408);THYN1(S14);TIAM2(S767);TJP1(S617);TJP1(S968);TJP2(T462);TJP3(S369);TJP3(S371);TJP3(S591);TLK2(S771);TMC6(S127);TMEM201(S441);TMX1(S270);TMX2(S288);TNKS1BP1(S429);TNKS1BP1(S601);TNKS1BP1(S983);TNS3(S363);TOP2B(S1413);TP53BP1(S1317);TPD52L2(S21);TRA2A(T202);TRAF4(S426);TRAFD1(S470);TRAPPC10(S711);TRIM11(S85);TRIM37(S771);TRIP10(S296);TSC22D4(S62);TSPYL2(S18);TSPYL2(S20);TWISTNB(S316);UBAP2L(S462);UHRF1BP1L(S414);UIMC1(S653);ULK1(S556);ULK1(S719);UPF1(S1107);USP1(S475);USP33(S439);USP54(S1036);UTP20(T1741);UVRAG(S689);VASP(S314);VCP(S770);VCPIP1(S997);VCPIP1(S998);VIM(S55);VIPAS39(S121);WASHC2A(S288);WASHC2C(S288);WDR20(S434);WDR44(S403);WIPF1(S214);WIPF1(S340);WNK1(S2011);WNK1(S2032);WNK3(S1471);XPR1(S666);XRN2(S471);YAP1(T110);YBX3(S293);YEATS2(S465);ZC3H13(S993);ZC3H13(T364);ZC3H14(S343);ZC3H3(S408);ZC3H3(S571);ZC3H4(S159);ZC3HAV1(S257);ZC3HAV1(S335);ZC3HAV1(T273);ZC3HAV1(Y348);ZDHHC5(S380);ZDHHC5(S425);ZFC3H1(S1303);ZFC3H1(S1304);ZFHX4(S2996);ZFR(S1054);ZHX3(S946);ZMYND8(S425);ZMYND8(S460);ZMYND8(S462);ZNF106(T640);ZNF136(S405);ZNF281(T888);ZNF408(T322);ZNF517(S218);ZNF75A(S287);ZNF75D(S491);ZNRF2(S135);ZP2(S454);ZRSR2(S349);ZSWIM8(S1156)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>RPS6KA3</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>37</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>ARFGAP2(S368);ATL1(S10);CDC42EP4(T23);CDK14(S78);COBLL1(S394);COL4A3BP(S373);EPB41L5(S436);FAM102A(S189);GON4L(S206);IRS1(S374);KHDRBS1(S20);KIF21A(S855);MAP3K2(S153);MAPRE1(S155);NCBP1(S22);NCOA5(S381);PAPOLG(S708);PHAX(S368);RBM15(S292);RBM15B(S265);RBMX(S326);RBMX(S352);RBMXL1(S88);RIPOR1(S351);SAFB2(S787);SF3B1(T261);SIK3(S866);SLTM(S551);SRSF4(S113);SRSF5(S117);SRSF6(S119);TMEM201(S441);TNS3(S363);WASHC2A(S288);WASHC2C(S288);ZMYND8(S425);ZNF185(S64)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>RPS6KA4</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>25</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>COL4A3BP(S373);EIF4ENIF1(S564);GON4L(S206);GSK3A(S21);GTF3C2(S167);KHDRBS1(S20);MEPCE(S152);MTMR12(S564);PHACTR1(S505);PHAX(S368);RALY(S135);RBM15B(S265);RBMX(S352);RPA1(T180);RPS27(S78);RPS27L(S78);SLTM(S551);SNRPA1(T180);TMEM201(S441);TRA2A(T202);TRA2B(T201);TRA2B(T212);USP32(S1416);USP6(S1214);ZNF185(S64)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>RPS6KA6</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>10</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>COBLL1(S394);EIF4B(S283);KHDRBS1(S20);NCOA5(S381);RBM15(S292);RBM15B(S265);RBMXL1(S88);SAFB2(S787);SLTM(S551);SRSF9(S189)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>RPS6KB1</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>15</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>AHNAK(S5731);CAD(S1859);DMXL2(S1400);FAM53B(S118);HNRNPA2B1(S212);KRT8(S477);LRRTM4(S195);MEPCE(S152);NUP50(S208);RPS6(S240);SH3BP1(S612);SH3BP1(S613);TNS3(S363);TRPV3(S372);YBX1(S209)</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>SIK2</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>191</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(S30);09/09/18 00:00:00(T142);AFDN(T1330);AFF4(S487);AMBRA1(S1205);ANK1(S15);ANKRD17(S2401);AP1M1(T154);ARFGAP2(S368);ARHGAP17(S162);ARHGEF11(S255);ARID1A(S772);ARPC1B(T315);ASCC3(S2195);ATF7(S434);ATF7IP(S474);ATF7IP(S477);ATXN2L(S32);BICRAL(S675);CAMKV(T435);CAMSAP1(S793);CAMSAP3(S814);CDC42SE1(S74);CDC6(S106);CDK14(S134);CDK18(S117);CENPF(S276);CHAF1A(S775);CHD1(S1677);COBL(S269);COL4A3BP(S373);CRAMP1(S1268);CRTC1(S172);CRTC1(T149);CRTC3(S62);CSNK1D(S331);CTU2(S419);DCDC2(S270);DCLRE1C(S518);DLG5(T1279);EEF2K(S72);EEF2K(S74);EEF2K(Y69);EIF3A(S1188);EIF3A(S882);EIF3F(S258);EIF4EBP1(T82);EIF4ENIF1(S752);EIF4G1(S1092);ELAVL1(S202);ENAH(S531);ETV6(S203);EVPL(S2025);FAM120A(Y452);FAM193B(S785);FOXK1(S223);FUBP3(S569);FZR1(S163);GLCCI1(S30);GRAMD1B(S274);GSE1(S826);GSE1(S828);GSK3B(S25);GSK3B(S9);GTF2F1(T389);HIPK1(T351);HIPK1(Y352);HIPK2(T360);HIPK2(Y361);HSPB1(S82);HUWE1(T2889);ICE1(S255);IKBKB(S672);IQSEC1(S180);IRF2BPL(S215);ISCU(S20);ITSN1(S315);JPH4(S157);KIAA1551(S1358);KIF21A(S1239);KIFC1(S26);LIMK1(S298);LIMK1(S310);LMNA(S628);MAP3K11(S524);MAP7D1(S399);MARCKS(S167);MARK2(S456);MARK3(S585);MCRIP2(S82);MED13(S890);MICALL1(S486);MICALL2(S249);MNAT1(S279);MON1B(S59);MON1B(S61);MPHOSPH8(S403);MTA1(S576);MTA1(S639);MTBP(S755);MTX3(S284);MYC(S62);MYCN(S62);NAA30(S39);NAV1(S1265);NCKIPSD(T181);NCOA3(S857);NECTIN1(T391);NSRP1(S33);NSUN2(S456);NSUN2(S473);NUP214(S1045);OSBPL11(S181);OTUD4(S416);PAK4(T207);PALD1(S406);PARD3(S174);PARVA(S14);PCDH1(S949);PDHA1(S232);PDS5B(S1358);PHACTR1(S505);PKN1(S562);PKP2(S329);PKP4(S337);PKP4(S406);PLEKHA2(S349);PLPPR3(S508);PPM1H(S221);PPP1R12A(S903);PPP1R13L(S102);PRAG1(S889);PREX1(S1182);PTPN12(S449);PTPN22(S692);PXN(S258);R3HDM1(S381);RABGEF1(S302);RALGAPA1(T754);RB1(S249);RB1(T821);RBL1(S640);RBL1(T369);RBM10(S797);RBMX(S332);RCSD1(S116);RCSD1(S120);RFX7(S225);RFX7(S424);RICTOR(S1284);RIOK1(S22);RIPK2(S363);RREB1(S42);SEC16A(S136);SHC3(S474);SHROOM3(S242);SHROOM3(S816);SIK3(S866);SIRT1(S27);SLC12A7(T980);SLC4A7(S556);SLC9A3R1(S280);SNIP1(S35);SNTB1(S87);SOX2(S250);SRRM2(S1404);SRRM2(S2272);SRRM2(S322);STK33(S470);TBKBP1(S365);TEX2(S266);TNS1(S1269);TNS1(T1173);TPD52L2(S166);TRA2A(T202);TRAFD1(S470);TRAPPC12(S184);TRIO(S1724);TTC28(S2224);TVP23C(S223);USP1(S67);USP32(S1423);VGLL4(S149);WDR20(S434);ZFPM1(S786);ZNF106(S641);ZNF516(T930);ZNF552(S86);ZNF609(S1055);ZNF777(S47);ZNF814(S87)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>SLK</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>4</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>DLGAP4(S666);EIF4B(S283);TBC1D10B(S687);VIPAS39(S121)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>SRPK1</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>887</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>09/07/18 00:00:00(T426);09/09/18 00:00:00(T142);AAK1(S14);AAK1(S21);ABCF1(S140);ABI1(S222);ABI1(S231);ABI2(S368);ABL1(S569);ABLIM1(S655);ABLIM1(S706);ACIN1(S478);ACTA1(S241);ACTA1(S54);ACTA2(S241);ACTA2(S54);ACTB(S239);ACTB(S52);ACTBL2(S240);ACTC1(S241);ACTC1(S54);ACTG1(S239);ACTG1(S52);ACTG2(S240);ACTG2(S53);ADAD2(S522);AEBP2(S390);AFF4(S487);AHCTF1(S528);AHDC1(S1403);AHDC1(S1507);AKAP1(S107);AKAP11(T1100);AKAP13(S1565);ALDH5A1(S122);ALG3(S13);AMOTL2(S183);AMOTL2(S540);AMOTL2(S602);AMPD3(S85);AMPH(S262);AMPH(T260);ANAPC1(S355);ANKRD34A(S291);ANKRD50(S1165);ANKS1A(S887);ANLN(S485);ANLN(S661);AP3B1(S276);APC(S2674);APPL1(S401);ARFGAP1(S361);ARFGAP2(S368);ARFGEF2(S240);ARFGEF2(T244);ARHGAP25(S379);ARHGAP25(S507);ARHGAP29(S499);ARHGAP29(S930);ARHGAP35(S970);ARHGAP39(S251);ARHGEF11(S1480);ARHGEF11(S255);ARHGEF11(S663);ARHGEF11(T668);ARHGEF18(S1111);ARHGEF19(S336);ARHGEF26(S98);ARHGEF38(S553);ARID1A(S1600);ARID1A(S363);ARID1A(S604);ARID3B(S311);ARL6IP6(S80);ARRB1(S412);ARVCF(T642);ASIC3(S37);ATAD2B(S318);ATF7IP(S113);ATG2B(S1582);ATG2B(S1583);ATG2B(Y1577);ATP11B(S1154);ATP2A2(S663);ATXN2(S667);ATXN2(S863);ATXN2L(S559);AXIN1(S77);BAG3(S289);BAG4(S179);BAIAP2L1(S261);BAIAP2L1(T257);BCL11A(S714);BCL11A(S718);BCL11A(S721);BCL11A(S735);BCL2L12(S113);BCL2L12(S121);BCL2L12(T117);BCL7C(T118);BCL9L(S813);BCL9L(S915);BCLAF1(S183);BCR(S463);BICRA(S1413);BICRA(T921);BMP2K(S14);BPTF(S216);BPTF(S2367);BRCA1(S1542);BRCA1(S1613);BRD4(S1064);BRSK2(S423);BRSK2(T459);BRSK2(T463);C11orf95(S408);C19orf47(S151);C1orf226(S18);C1orf52(S158);C2CD5(S281);C2orf49(S189);CAMK4(S356);CAMK4(S360);CAMKK2(S129);CAMKK2(S132);CAMKK2(S133);CAMKK2(Y128);CAMSAP2(S464);CAMSAP3(S431);CASP8AP2(S567);CBARP(S200);CBL(S619);CBY1(S20);CCDC130(S332);CCDC18(S1355);CCDC6(S240);CCDC6(T434);CCDC61(S373);CCDC61(S376);CCDC61(S447);CCDC61(S458);CCDC86(S58);CCDC86(S80);CCDC88A(S237);CCNK(S9);CCNY(T75);CCNYL1(T97);CCZ1(S368);CCZ1B(S368);CD244(S334);CD2AP(T87);CDC20(S160);CDC20(T157);CDC42EP4(S80);CDK1(T161);CDK11A(S271);CDK11A(T583);CDK11A(T739);CDK11B(S283);CDK11B(T751);CDK12(S383);CDK12(S385);CDK13(T1056);CDK14(S78);CDYL(S149);CECR2(S1312);CENPF(S2996);CEP170(S1160);CEP170(S881);CEP170B(S972);CEP57(T58);CFDP1(S250);CGNL1(S196);CGNL1(S198);CGNL1(S202);CHAMP1(S319);CHAMP1(S379);CHAMP1(S382);CHAMP1(S386);CHAMP1(S427);CHAMP1(S432);CHAMP1(S436);CHAMP1(S603);CHD2(S1728);CHD4(S1531);CHD8(S1978);CHD8(T1982);CHEK1(S280);CLASP1(S559);CLASP1(S646);CLASP2(S327);CLASP2(S360);CLASP2(S370);CLASP2(S459);CLASP2(S525);CLASP2(S529);CLCC1(S532);CLIC6(S293);CLINT1(S299);CLINT1(Y293);CLK3(S283);CLNS1A(S102);CMTR1(S31);CNK3/IPCEF1(S892);CNNM2(S129);CNTROB(S62);COBLL1(S294);CPA6(S60);CRAMP1(S1201);CRKL(Y207);CRTC1(S153);CRTC2(S178);CRTC3(S329);CSRP1(S192);CTAGE5(S594);CTNNAL1(S538);CTNND1(S230);CTNND1(T906);CTPS1(S573);CTPS1(S574);CTPS1(Y567);CTTN(T411);CTTNBP2NL(S481);CUX1(S1218);CXXC5(S80);CYBA(T147);DAP(S51);DBN1(S312);DCAF12(S15);DCP1A(S319);DCP1B(S275);DDX3X(S90);DENND4A(S1256);DENND4C(S968);DENND4C(S973);DGCR8(S271);DGCR8(S373);DGCR8(S377);DIDO1(S1242);DIDO1(Y1244);DIP2B(S1343);DIP2B(S53);DLG5(S1254);DLG5(S1795);DLGAP4(T915);DNAAF2(T703);DNAJB6(S277);DNM1(S619);DNM2(S619);DNTTIP2(S141);DNTTIP2(S145);DOCK11(S440);DPYSL2(T514);DTL(T196);DUSP27(S966);DYNC1LI1(T513);E2F7(S825);ECT2(S842);EDC3(S131);EEF1AKMT2(S21);EEF1D(S37);EEF2(T57);EHBP1(S432);EIF2B1(S107);EIF3A(S584);EIF4B(S406);EIF4EBP1(T41);EIF4EBP2(T46);EIF4ENIF1(S345);EIF4G1(S1092);EIF4G3(S230);EIF5B(S113);ENAH(S531);EPB41L3(S760);EPN1(T460);EPRS(S882);EPS15L1(S229);EPS15L1(S793);EPX(S672);ERCC6(S1346);ERRFI1(S326);ETV4(S140);EVL(S331);EVL(S369);EZH2(S363);EZH2(T367);FAM102B(S228);FAM117A(S193);FAM122A(S143);FAM122B(S115);FAM122B(S119);FAM122B(S137);FAM122B(S141);FAM129B(S696);FAM208B(S1220);FAM47A(S259);FAM53C(S234);FAM53C(S247);FARP2(S439);FBXW9(S59);FCHO2(S387);FLNB(S1505);FNBP1(S296);FNBP1L(S501);FNDC3A(S203);FNDC3A(S206);FNDC3A(S207);FNDC3B(S208);FOXO1(S298);FOXO1(S303);FRMD4A(S604);FRY(S1936);FTSJ3(S584);FXR2(S566);FZD6(S620);GAPVD1(S761);GAPVD1(S902);GAPVD1(T762);GATAD2A(S100);GATAD2A(S107);GATAD2A(S114);GATAD2A(S548);GATAD2B(S340);GIGYF1(S24);GIGYF2(S236);GIGYF2(S26);GIT1(S410);GIT1(S592);GLCCI1(S223);GORASP2(T415);GPATCH8(S1033);GPR183(S343);GRAMD1A(S263);GRAMD1A(S267);GSE1(S710);GSE1(S84);GSE1(S909);GSK3A(Y279);GSK3B(S25);GSK3B(S9);GSK3B(Y216);GTF2F1(S377);GTF2F1(S380);GTF2F1(S385);GYS1(S641);GYS1(S645);HCFC1(S666);HCN4(S935);HDAC1(S421);HDAC1(S423);HDAC2(S422);HDAC2(S424);HDAC6(S22);HDAC7(S487);HECTD1(S1387);HECTD1(S1567);HID1(S653);HNRNPK(S379);HNRNPU(S271);HSH2D(S251);HSPB1(S82);HUWE1(S2534);HUWE1(T2889);IGF2R(S2409);IGLL1(S76);ILF3(T592);INO80B(S351);INPP5D(S1057);INPP5D(T963);INTS3(S994);IPCEF1(S430);IQSEC1(S107);IRF2BP1(S453);IRF2BP1(T480);IRF2BPL(S519);IRS2(S915);ITSN1(S559);IWS1(S333);JMY(S713);JPH1(S216);JUN(S63);KANK1(S186);KANSL3(S535);KAT7(S57);KCTD12(S185);KDM3A(S445);KHSRP(T100);KIAA1217(S357);KIAA1522(S404);KIAA1551(S1358);KIAA1551(S715);KIAA1671(S1224);KIDINS220(S1411);KIDINS220(Y1416);KIF1A(S1528);KIF1A(S1532);KIF21B(T1237);KIF2C(S187);KIF4A(T1181);KIFC1(S351);KLC4(S609);KMT2B(S2348);KNOP1(S42);KPNA3(S60);KPNA4(S60);KRT8(S330);L1TD1(S173);L3MBTL3(S608);LAD1(S301);LAMTOR1(S27);LARP1(S517);LARP1(S850);LARP1(T526);LARP6(S447);LARP6(S56);LARP6(S58);LARP7(S337);LARP7(T338);LASP1(T104);LAT2(S102);LEMD2(S82);LIG3(S912);LIN54(S314);LINC00322(S226);LMO7(S706);LRCH1(S532);LRRFIP1(S116);LRRFIP1(S120);LSM14A(S178);LSM14A(S183);LSP1(S252);LTBP1(Y1422);LUZP1(S995);LUZP1(T441);LUZP1(T958);LYSMD2(S24);LYSMD2(S29);LZTS1(S209);MAF1(S68);MAGOH(S106);MAGOHB(S108);MAP1A(S1675);MAP2(S1790);MAP3K11(S748);MAP3K2(S239);MAP4(S1073);MAP4K5(S335);MAP7D1(S93);MAP7D1(T97);MAPKAP1(S510);MAPT(S713);MAPT(S717);MARCKSL1(T85);MARK2(S456);MARK2(S619);MARK3(S583);MARK3(S585);MARVELD2(S116);MARVELD2(S120);MAST2(S1032);MAST2(S74);MAVS(S258);MAZ(S361);MBP(T39);MCPH1(S333);MDH1(S241);MED1(S1223);MED19(S226);MEPCE(S217);MEPCE(T213);MEX3B(S442);MEX3B(S63);MEX3C(S540);MEX3C(T541);MEX3D(S176);MEX3D(S514);MFSD10(S270);MFSD10(S271);MFSD2B(S494);MGA(S924);MGMT(S201);MIA2(S1202);MICAL3(S1310);MICAL3(S649);MIER1(T448);MIIP(S303);MIS18BP1(S594);MISP(S394);MKI67(S579);MKI67(S827);MKI67(T1557);MMACHC(S275);MORC3(S765);MPPE1(S325);MRGBP(S194);MSANTD2(S27);MSH6(S256);MTA1(S639);MTOR(S2448);MTX3(S284);MYBBP1A(S11);MYC(T58);MYO1F(S992);MYO9B(S1405);MYO9B(S717);MYO9B(T1271);NAA10(S182);NAA10(S186);NAB1(S403);NAB2(S479);NACA(S166);NACA(S2029);NAV2(S1559);NAV2(S1808);NCBP1(S22);NCOR2(S1018);NCOR2(S1331);NCOR2(S1783);NCOR2(T1391);NDE1(S211);NDRG1(S333);NDRG2(S332);NDRG2(T330);NELFA(T212);NEXN(S160);NLN(S485);NMNAT1(S117);NOL8(S432);NOP16(S16);NOP58(S351);NPM1(S260);NPM1(S70);NSF(S437);NSFL1C(S114);NSRP1(S33);NSUN2(S473);NUMA1(S1840);NUP214(T436);OSBP(S190);OSBP(S193);P2RX7(S470);P2RX7(T467);PAK4(S148);PANK2(S189);PANX1(S73);PBDC1(S197);PBX2(S330);PCDHGC3(S60);PCM1(S1958);PCYT1A(S347);PDZD4(S564);PEAK1(S823);PGK1(S203);PHAX(S368);PHF3(S1614);PHIP(S677);PHKA2(S1043);PHKA2(S1044);PHLDA2(S144);PHLDB1(S518);PHLDB1(T516);PHRF1(S936);PHRF1(S973);PIK3C2A(S338);PIK3CD(T226);PIK3R4(T927);PJA1(S126);PKP2(S82);PKP3(S331);PLEKHA6(S251);PLEKHA6(S867);PLEKHG2(S1261);PLEKHG2(T1257);PLEKHG4B(S729);PLEKHG7(S162);PLIN5(S203);PLXNA1(S1004);PODXL(S519);POLH(S379);POLH(S380);POLN(S75);POM121(S269);POM121C(S246);POTEE(S939);POTEF(S939);POTEKP(S239);PPFIA1(S1172);PPFIBP1(S540);PPHLN1(S201);PPHLN1(T200);PPIG(S356);PPIP5K2(S1074);PPP4R2(S159);PRAG1(S782);PRKD1(S205);PRKD1(S208);PRKRA(S18);PRPF4B(S852);PRPF4B(Y849);PRRC2C(S1568);PTGES3(S44);PTPN1(S378);PTPN13(S1082);PTPN13(S1085);PTPN22(S414);PTPN22(T450);PTTG1(S165);PTTG2(S165);PUM1(S209);R3HDM2(S349);RAB11FIP1(S156);RAB11FIP2(S150);RAB3GAP1(S537);RABL6(S359);RAD51AP1(S19);RAF1(S642);RAF1(T239);RALB(S6);RALY(S239);RANBP1(S60);RANBP2(S2454);RANBP2(T1396);RANBP2(T2450);RANBP3(S108);RAPGEF2(S585);RASAL2(S634);RB1(S807);RBBP8NL(S141);RBBP8NL(T140);RBM14(S618);RBM15(Y266);RBM15B(S552);RBMX(S189);RBMXL1(S189);RBMXL1(S88);RCOR1(S460);RCSD1(S116);RCSD1(S120);RCSD1(S123);RCSD1(S126);REPS1(S162);REPS1(S166);REPS1(S170);REPS1(T173);REPS1(T539);REXO4(S15);RFX1(S204);RFX7(S1028);RGPD1(S1463);RGPD1(T1459);RGPD2(S1471);RGPD2(T1467);RGPD3(S1479);RGPD3(T1475);RGPD4(S1479);RGPD4(T1475);RGPD5(S1478);RGPD5(T1474);RGPD8(S1478);RGPD8(T1474);RIC1(T992);RICTOR(S1284);RIF1(T1047);RIPOR1(S349);RNH1(T82);ROR1(S776);RPGR(S518);RPL5(S286);RPRD2(S930);RPS10(S146);RPS10P5(S157);RPS27(S11);RPS27(S27);RPS27(S78);RPS27L(S27);RPS27L(S78);RPS28(S23);RPS6(S235);RPTOR(S859);RREB1(S1238);RRP1B(T728);RUNX1(T14);SAFB(T200);SARNP(S163);SCAF1(S992);SCAF11(S802);SCFD1(S303);SCRIB(S1348);SCYL3(S707);SDAD1(S585);SEC16A(S1194);SEC16A(S1905);SEC16A(S23);SEC16A(T19);SEMA6A(T761);SETD2(S1084);SF3B1(T207);SF3B1(T211);SF3B1(T261);SF3B2(S431);SF3B2(S435);SF3B2(S436);SFPQ(S33);SGTA(S77);SGTA(T81);SH3BP4(S246);SH3BP5L(S362);SHC3(S474);SHROOM3(S1497);SHROOM3(T576);SHTN1(S506);SIK3(S551);SIPA1(S839);SIPA1L3(S1364);SKIV2L(S131);SLAIN2(S377);SLC20A2(Y389);SLC43A1(S267);SLC4A7(S403);SLC9A1(S703);SLTM(S1014);SMAP2(S219);SMARCA2(S588);SMG7(S781);SMN1(S28);SND1(S426);SNRNP200(S225);SNX8(S456);SNX8(T452);SPAG9(S550);SPAG9(S557);SPECC1(S364);SPECC1(S914);SPEN(S1918);SPEN(T2421);SPN(T341);SPP1(S219);SRCAP(S2787);SRP72(S621);SRP72(T624);SRPK1(S309);SRRM1(S391);SRRM1(S597);SRRM1(T718);SRRM2(S144);SRRM2(S1925);SRRM2(S323);SRRM2(S377);SRRM2(S435);SRRM2(S440);SRRM2(S534);SRRM2(S536);SRRM2(S774);SRRM2(S876);SRRM2(T1413);SRRM2(T1927);SRRM2(T400);SRRT(S74);SRSF8(S156);SRSF8(S158);ST6GALNAC4(S298);STAT5A(S193);STK10(T952);STK3(S385);STK3(T174);STK4(T177);STX7(S131);SYN1(S551);SYN1(S553);SZRD1(S107);TACC1(S276);TAF6(S634);TAF6(S636);TAF6(S653);TAGLN2(S163);TANC1(S67);TANC2(S169);TATDN2(S420);TATDN2(S80);TBC1D10B(S658);TBC1D10B(S661);TBC1D10B(T152);TBC1D10B(T697);TBC1D22A(S167);TBC1D4(S588);TCOF1(S1378);TGFB1I1(S141);TGFBR2(S352);THAP4(S128);THRAP3(S698);THYN1(S14);TIPIN(T224);TMF1(S72);TMPO(S159);TMPO(S184);TMPO(S306);TMPO(S424);TMX2(S288);TNKS1BP1(S1533);TNKS1BP1(S1620);TNKS1BP1(S1621);TNRC18(S1644);TNS2(S1003);TNS3(S332);TOP2A(S1393);TP53BP2(S121);TPI1(S58);TRAFD1(S470);TRAK1(S919);TRAPPC10(S711);TRIM24(S687);TRIM32(S335);TRIM37(S771);TRIT1(S443);TSC2(S1448);TSC22D4(S24);U2SURP(S485);UBA1(S816);UBAP2L(S462);UBAP2L(S605);UBE2C(S23);UBE2O(S896);UBE4B(T64);UHRF1BP1L(S414);UNG(S23);UNG(T60);UPF1(S1107);USP10(S576);USP36(S682);VASP(S239);VCAM1(S346);VCL(S755);VCPIP1(S998);WARS(S467);WASHC2A(S1180);WASHC2A(S704);WASHC2C(S1157);WASHC2C(S702);WASHC2D(S147);WDFY4(S3123);WDR44(S561);WIPF1(S340);WIPI2(S413);WNK1(S167);WTIP(S88);WWC1(S899);WWC1(T895);WWC3(S563);XPO4(S521);XPR1(S666);XRCC1(S447);XRN2(S499);XRN2(S501);YAP1(S164);YEATS2(T478);YTHDC2(S1090);ZBTB21(S983);ZBTB3(S549);ZBTB48(S179);ZC3H15(S360);ZC3H3(S571);ZC3H4(S1108);ZC3H4(S1114);ZC3H4(S1269);ZC3HC1(S24);ZDHHC5(S425);ZEB1(S679);ZFP36L1(S334);ZFP36L2(S438);ZFP36L2(S490);ZFYVE26(S1764);ZKSCAN8(S12);ZMYM4(S242);ZNF106(S893);ZNF226(S765);ZNF318(S136);ZNF45(S314);ZNF592(S691);ZNF609(S578);ZNF639(S88);ZNF655(S285);ZNF697(S299);ZNF75A(S287);ZNF75D(S491);ZSCAN25(S300);ZSCAN5A(S296);ZSCAN5B(S295)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>SRPK3</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>353</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>ABI1(S222);ACIN1(S478);ACTA1(S241);ACTA2(S241);ACTB(S239);ACTBL2(S240);ACTC1(S241);ACTG1(S239);ACTG2(S240);AHCTF1(S1222);AKAP11(T1100);ALG3(S13);AMPD3(S85);AP3D1(S829);APPL1(S401);ARHGAP25(S379);ARHGAP25(S507);ARHGAP35(S970);ARID3B(S311);ASIC3(S39);ATP11B(S1154);ATXN2(S667);ATXN2(S863);ATXN2L(S559);AXIN1(S77);BAG4(S179);BAIAP2L1(S261);BAIAP2L1(T257);BCL11A(S714);BCL11A(S718);BCL11A(S721);BCL11A(S735);BCL7C(T118);BCR(S463);BMP2K(S14);BRCA1(S1542);BRIP1(S990);C1orf226(S18);C2CD5(S295);CAMKK2(S129);CAMKK2(S132);CAMKK2(S133);CAMKK2(Y128);CANX(S564);CASC3(T143);CCDC61(S373);CCDC61(S376);CCDC61(S447);CCDC61(S458);CCDC86(S58);CCDC86(S80);CD244(S334);CDK11A(S271);CDK11A(T739);CDK11B(S283);CDK11B(T751);CDK13(T1056);CDT1(S394);CDYL(S149);CEP170(S1160);CEP170(S881);CFDP1(S250);CHAMP1(S379);CHAMP1(S382);CHAMP1(S386);CHAMP1(S427);CHAMP1(S432);CHAMP1(S436);CHAMP1(S507);CHAMP1(S603);CHD4(S1531);CHD8(S1978);CHD8(T1982);CLASP2(S327);CLASP2(S370);CLASP2(S525);CLNS1A(S102);CNK3/IPCEF1(S892);CRAMP1(S1201);CSRP1(S192);CTAGE5(S594);CTDP1(S839);CTPS1(S573);CTPS1(S574);CYBA(T147);DBN1(S312);DDB2(S26);DDX21(S121);DDX54(S782);DGCR8(S373);DGCR8(S377);DIDO1(S1242);DIDO1(Y1244);DIS3L2(S875);DLGAP4(T915);DNTTIP2(S141);DNTTIP2(S145);DOCK11(S440);EHBP1(S432);EIF4EBP1(T37);EIF4EBP3(T31);EIF4EBP3(T32);EIF4EBP3(Y20);EPB41L2(S499);EPB41L3(S760);EPN1(T460);EPRS(S882);EPS15L1(S793);ERCC6(S1346);EZH2(T367);FAM122A(S143);FAM122B(S115);FAM122B(S119);FAM122B(S137);FAM122B(S141);FNDC3A(S203);FRY(S1936);GATAD2A(S100);GATAD2A(S107);GATAD2A(S114);GATAD2B(S340);GIGYF2(S26);GLCCI1(S223);GPR183(S343);GSE1(S710);GTF2F1(S377);GTF2F1(S380);GTF2F1(S385);GTF3C1(S1068);HAUS6(T584);HCN4(S935);HDAC1(S421);HDAC1(S423);HDAC2(S422);HDAC2(S424);HDGF(S132);HDGF(S133);HELZ(S1317);HMGCS1(S4);HNRNPK(S284);HSH2D(S251);HSPB1(S98);ID2(S14);IGF2BP1(S181);IGF2R(S2409);INPP5D(S1057);INTS3(S994);IPCEF1(S430);IRF2BP1(S453);IRF2BP1(T480);IWS1(S720);JMY(S713);KANK1(S186);KAT6A(S1000);KIAA1522(S404);KIF4A(T1181);KLC4(S609);KPNA4(S60);L3MBTL3(S608);LARP1(S850);LARP1(T526);LARP1(T649);LASP1(T104);LAT2(S102);LIG3(S912);LINC00322(S228);LMO7(S706);LRCH1(S532);LRRFIP1(S116);LSP1(S252);LUZP1(S995);LUZP1(T958);MAF1(S68);MAP1A(S1675);MAP4K5(S335);MAP7(S209);MAP7D1(S93);MAP7D1(T97);MARK3(S585);MAVS(S258);MAZ(S361);MBP(T39);MCPH1(S333);MDH1(S241);MED1(S1481);MED1(S1482);MEX3B(S63);MEX3C(S540);MEX3C(T541);MEX3D(S176);MFSD10(S270);MGA(S924);MGMT(S201);MIA2(S1202);MICAL3(S1310);MKI67(S579);MKI67(S827);MKI67(T1557);MMACHC(S275);MORC3(S765);MPLKIP(S115);MRGBP(S194);MSH6(S256);MTMR4(S629);NAA10(S182);NAA10(S186);NAB1(S403);NCBP1(S22);NCOR1(S1980);NCOR1(S1981);NDRG1(S333);NOL8(S432);NOP16(S16);NSUN2(S473);NUMA1(S2047);P2RX7(S470);P2RX7(T467);PCDHGC3(S60);PCYT1A(S347);PDCD5(S119);PHAX(S368);PHF3(S1614);PHRF1(S936);PHRF1(S973);PLIN5(S203);POLD3(S307);POLH(S379);POM121(S269);POM121C(S246);POM121C(S372);POTEE(S939);POTEF(S939);POTEKP(S239);PPHLN1(S201);PRRC2A(S342);PRRC2A(S350);PSMB10(S229);PTGES3(S113);PTGES3(S44);PTTG1(S165);PTTG2(S165);PXN(Y118);RALY(S239);RANBP1(S60);RANBP2(S2454);RB1(S807);RB1(Y790);RBM15B(S552);RBMX(S189);RBMX2(S273);RBMXL1(S189);RCOR1(S460);RCSD1(S116);RCSD1(S120);RCSD1(S123);RCSD1(S126);REPS1(S162);REPS1(S166);REPS1(S170);REPS1(T173);REPS1(T539);RGPD1(S1463);RGPD2(S1471);RGPD3(S1479);RGPD4(S1479);RGPD5(S1478);RGPD8(S1478);RIC1(T992);RNH1(T82);RPL34(S12);RPS10(S146);RPS10P5(S157);RPS27(S27);RPS27L(S27);RPS6(S235);RREB1(S1238);RTN4(S184);SAFB(T200);SCAF1(S992);SCAF11(S802);SCRIB(S1348);SEC16A(S1905);SEC16A(S23);SEC16A(T19);SFPQ(S33);SIPA1(S839);SKIV2L(S133);SLAIN2(S377);SLC43A1(S267);SMAP2(S219);SMN1(S28);SNX17(S333);SPP1(S219);SRCAP(S2787);SRRM1(S874);SRRM1(T718);SRRM2(S144);SRRM2(S1925);SRRM2(T1927);SRSF4(S448);SRSF7(S167);STK10(T952);STK3(S385);TAF6(S653);TAGLN2(S163);TATDN2(S420);TGFBR2(S352);THAP4(S128);TMPO(S159);TMPO(S184);TMPO(S424);TMX1(S247);TNKS1BP1(S1620);TNKS1BP1(S1621);TOP2A(S1393);TP53BP1(T1648);TPI1(S58);TRAK1(S919);TRIM24(S687);TRIM37(S773);TXLNG(T102);U2SURP(S485);UBAP2L(S462);UBE2O(S896);UBE4B(T64);ULK1(S623);UNG(T60);UPF1(S1107);UTP18(S121);UTP18(S124);WARS(S467);WDFY4(S3123);WIPF1(S340);XPR1(S668);XRCC1(S266);XRCC1(S447);YTHDF1(S291);ZBTB21(S983);ZBTB3(S549);ZBTB48(S179);ZC3H4(S1108);ZC3H4(S1269);ZDHHC5(S425);ZEB1(S646);ZEB1(S679);ZFYVE26(S1764);ZKSCAN1(S13);ZMYM4(S122);ZNF592(S691);ZNF639(S88);ZNF655(S285);ZNRF2(S145);ZRANB2(S153)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>STK10</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>41</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(S30);ADAM17(S791);AHNAK(S3426);AKIRIN1(S22);BRIP1(S956);C2CD2L(S411);CLASP1(S636);DDX54(S75);DNTTIP2(S434);FAM109A(S213);FAM53B(S268);FLNC(S2624);GIGYF2(S26);IRF2BP2(S406);IRF2BPL(S519);KNOP1(T310);LRCH4(S520);MAP2(S1540);MAPK3(T207);MTMR1(S43);MTMR3(S613);NSD1(S2471);PARD3(S221);PEA15(S116);PLEKHA1(S332);PLK1(T214);PPHLN1(Y162);RB1(S788);RBM17(S169);REPS1(S709);SAMHD1(S33);SAMHD1(T21);SF3B1(T434);SMARCA2(S588);SNURF(S32);SRRM1(T718);TBX2(S653);TWISTNB(S316);VANGL1(T47);XPO4(S521);ZNF24(S274)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>STK17A</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>58</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(T49);ADAM10(S740);ADAM10(Y741);ADAM17(S791);AHCTF1(S528);AKAP11(S422);AMFR(S542);ANAPC1(S355);ANLN(S182);ANLN(T194);ATXN2L(S424);CNK3/IPCEF1(S892);DBNL(T291);DGCR8(S271);DIP2B(S259);DOCK7(S898);FUS(S462);FXR2(T411);GTF3C2(S167);HIST1H1B(S18);HNRNPM(S528);HNRNPM(S618);HPS5(S534);INCENP(S311);IPCEF1(S430);LARP1(S90);LARP1(T649);LRCH4(S520);MLLT6(S378);MLLT6(S382);MYCBP2(S3467);NADK(S48);NUMA1(T2000);NUP107(S11);PBRM1(S13);PCNP(T139);PHF3(S1614);PKP4(S273);PKP4(S314);PPHLN1(S163);PRRC2C(S779);RALY(S135);RBM39(S97);RBM39(Y95);RPA1(T180);SATB1(S637);SHANK2(S67);SNRPA1(T180);SUPT6H(T1523);TCOF1(S1227);THRAP3(S253);TLN1(S425);TNIK(S766);TPD52L2(S166);UPF3B(T169);ZC3H13(S64);ZCCHC8(S598);ZFR(S1054)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>STK3</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>65</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>ABLIM1(S452);ABLIM1(S706);AGAP2(T809);ALKBH5(S361);ARHGAP35(S1150);C17orf53(S332);C1orf226(S18);CBL(S619);CD2AP(S458);COL4A3BP(S373);DENND4C(S1099);DOCK7(S888);EIF4B(S207);EIF4ENIF1(S564);EIF4G1(S1092);EPB41(T710);ERCC6L(S820);FAM53C(S232);GPRIN1(S389);GSK3A(S21);HECTD1(S1387);HID1(S593);ID2(S14);INSRR(S72);IQSEC1(S180);IRS1(S1145);IRS2(S306);ITSN1(S978);KIF21A(S855);LIMA1(S15);LRRC41(S308);LUC7L2(S18);MAP7D1(S254);MAPRE1(S155);MYC(S62);MYO18A(S102);MYO7B(S689);NBN(S432);NCBP1(S22);PAK2(T143);PAPOLG(S708);PLEKHA5(S471);PPP1R12A(S554);PRKAB1(S108);PRPF4B(S852);PRPF4B(Y849);PTPN14(S642);RALGAPA1(T754);RAP1GAP2(S564);RAPGEF6(S1237);RAPGEF6(S1241);RBM14(S618);SEPT9(S30);SPP2(S182);SVIL(S968);TBC1D4(S588);TNS2(S1003);TNS3(S363);TPD52(S176);VASN(S284);XPO4(S521);ZC3HAV1(S335);ZNF609(S1055);ZNRF1(S123);ZP2(S454)</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>STK4</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>85</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>ABLIM1(S706);ADAM17(S791);AHNAK(S5731);AHNAK(S819);AKIRIN2(S21);ALKBH5(S361);APC(S2125);ATXN2(T672);ATXN7L3(S281);BAIAP2L1(S261);CBL(S619);CCDC86(S102);CDK12(S274);CHAMP1(S432);CHAMP1(S436);CLSPN(S954);COBLL1(S294);CUX1(S1215);CYBRD1(S260);DDX3X(S90);EDN3(S34);EIF4B(S207);EIF4G1(S1092);ELMO1(S344);ERBIN(S1168);FAM53C(S232);FBRSL1(S1034);GAPDH(T153);GPR183(S343);GSK3A(S21);HECTD1(S1387);HNRNPA2B1(S212);IQSEC1(S180);IRS1(S329);IRS1(T351);ITSN1(S978);KIDINS220(S1361);KIF21A(S855);KRT17(S32);LRCH4(S520);LUC7L2(S18);MEPCE(S152);NAB1(S407);NAP1L4(S125);NCBP1(S22);NOP14(S96);NSD2(T115);NUMA1(S2047);PALLD(S893);PATJ(S645);PPP1R12A(S871);PRPF4B(S852);PRPF4B(Y849);PXN(Y88);RAB11FIP1(S202);RBM14(S618);RIF1(S1554);RRBP1(S1277);RSF1(S570);RSF1(S629);RSF1(T628);SAMD4B(S628);SCAF1(S992);SCAF11(S802);SCNM1(S183);SEC31A(S799);SEPT9(S30);SGTA(S77);SGTA(T81);SH3BP2(S278);SIN3A(S1112);SKA3(S110);SRRM1(T718);TATDN2(S420);TBC1D4(S588);TJP2(S979);TNRC18(S1038);TNS2(S1003);TNS3(S363);TPD52(S176);TRIM24(S687);TWISTNB(S316);VIPAS39(S121);XPO4(S521);ZC3HC1(S359)</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>TAOK1</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>18</v>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>AHCTF1(S528);AKAP11(S422);ANAPC1(S355);CNK3/IPCEF1(S892);FUS(S462);FXR2(T411);GTF3C2(S167);HPS5(S534);IPCEF1(S430);NADK(S48);PBRM1(S13);PCNP(T139);PEA15(S116);PKP4(S314);RBM39(S97);RBM39(Y95);SHANK2(S67);UPF3B(T169)</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>TAOK3</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>757</v>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(S30);AAK1(S14);ABI1(S216);ABI1(Y213);ABLIM1(S431);ABR(T74);ACIN1(T414);ACTA1(S241);ACTA2(S241);ACTB(S239);ACTBL2(S240);ACTC1(S241);ACTG1(S239);ACTG2(S240);ADAM10(S740);ADAM10(Y741);ADAM17(S791);ADD1(S12);ADD1(S431);ADD1(S726);ADD2(S713);ADD3(S693);AFDN(S1721);AFF4(S1043);AFF4(S1058);AFF4(S32);AGAP2(S808);AGFG1(T177);AHCTF1(S528);AHDC1(S1064);AHDC1(S1507);AHNAK(S115);AHNAK(S216);AHNAK(S3412);AHNAK(S3426);AHNAK(S5731);AKAP11(S1580);AKAP11(S422);AKAP11(S448);AKAP13(S2728);AMBRA1(S1205);AMBRA1(S639);ANAPC1(S355);ANKRD17(S2401);ANKS1A(S382);ANKZF1(S675);ANLN(S518);ANP32B(T244);APPL1(S401);ARFGAP1(T135);ARFGAP2(S368);ARFGAP2(S432);ARHGAP1(S44);ARHGAP1(S51);ARHGAP17(S625);ARHGAP21(S856);ARHGEF11(S150);ARHGEF11(S35);ARHGEF17(S735);ARHGEF18(S1111);ARHGEF26(S80);ARID1A(S1184);ARID1A(S1604);ARID1A(S730);ARID3B(S381);ARL6IP6(S80);ARVCF(S887);ASF1B(T179);ATAD2(S327);ATG2B(S1582);ATG2B(S1583);ATG2B(Y1577);ATN1(S661);ATN1(T653);ATXN2(S684);ATXN2(T666);BAG3(S289);BAG3(T285);BAP18(S110);BAZ1B(S349);BCAM(S600);BCL11A(S328);BCL2L12(S113);BCL2L12(S121);BCL2L12(T117);BCR(S459);BIN2(S259);BPTF(S1300);BRD4(S1126);BRIP1(S956);BRSK2(T459);BRSK2(T463);BUB1(S655);C16orf54(S194);C16orf72(S167);C2CD2L(S662);C2CD5(S281);C2CD5(S662);C6orf132(S449);C7orf50(S175);CABLES1(S291);CALU(S35);CALU(S44);CAMSAP1(S563);CARHSP1(S41);CARMIL2(S1315);CAT(S515);CBL(S799);CBX8(S311);CCDC6(S240);CCDC9(S376);CCDC93(S305);CCL13(S44);CD97(S818);CD97(S831);CDC25C(S216);CDCA7L(S261);CDK13(T1056);CDK9(S347);CDV3(T182);CENPF(S276);CENPF(S3119);CEP170(S1260);CEP170(S881);CEP55(S428);CEP97(S308);CHAF1A(S206);CHAMP1(S376);CHAMP1(S405);CHAMP1(S432);CHAMP1(S436);CHAMP1(S445);CHAMP1(S452);CHAMP1(S472);CHAMP1(S507);CHD4(S303);CHD8(S1978);CHD8(T1982);CIT(S1322);CLASP1(S636);CLASP2(S325);CLASP2(S360);CLASP2(S529);CLASRP(S547);CLINT1(T308);CLK2(S142);CMTR1(S31);CNK3/IPCEF1(S892);CNP(S170);COL4A3BP(S373);CPSF7(S48);CREB1(S111);CREB1(S271);CSPP1(S901);CTAGE1(S616);CTAGE5(S647);CTPS1(S573);CTU2(S419);CYBA(T147);DACH1(S727);DAXX(S671);DBF4(S381);DBNL(T291);DDX10(S7);DDX21(S89);DDX3Y(S592);DENND4A(T1019);DGCR8(S271);DGCR8(S275);DGCR8(Y267);DIP2B(S259);DLG5(S1000);DLG5(T984);DLGAP5(S725);DNTTIP2(S434);DNTTIP2(T172);DOCK7(S898);DOCK7(S946);DOCK8(S451);DPYSL2(T509);DTL(S425);DYNC1LI1(S398);DYNC1LI1(S421);EEPD1(S21);EIF3E(S399);EML4(S144);EML4(S146);ENAH(T538);EP400(S722);EP400(S736);EPB41L1(S784);EPS15L1(S793);ERCC5(S384);ERRFI1(S461);ESF1(S198);EZH2(S363);EZH2(T367);FADD(S194);FAM117B(S10);FAM117B(S106);FAM122A(S143);FAM122A(S189);FAM129B(S665);FAM129B(S681);FAM129B(S696);FAM207A(T34);FAM53B(S179);FAM76B(S193);FAM83B(S766);FAM83H(S914);FANCI(S1121);FARSA(S301);FBRSL1(T1010);FBXW9(S59);FGD6(S692);FIP1L1(S259);FLYWCH2(S21);FOXK1(S416);FOXK1(S420);FOXK1(S441);FOXO1(S329);FRMD3(S416);FTSJ3(S677);FTSJ3(T573);FUS(S462);FXR2(S601);FXR2(T411);GAB2(S141);GAGE13(S33);GAGE2A(S32);GAGE2B(S32);GAGE2D(S32);GAPVD1(S902);GATAD2A(T189);GATAD2B(S334);GATAD2B(S486);GBF1(S1061);GBF1(S1298);GFI1(S94);GIGYF2(S26);GJA1(S262);GLUD1(S391);GLUD2(S391);GNL3(S529);GPATCH2(S195);GRIP1(S847);GTF2F1(S385);GTF2F1(T389);GTF2F1(T446);GTF3C1(S1068);GTF3C2(S132);GTF3C2(S167);HCFC1(S598);HCFC1(S666);HDAC1(S406);HELB(S1050);HIC2(S348);HIST1H1E(T18);HJURP(S557);HMGA1(S36);HMGCS1(T490);HNRNPA1(S338);HNRNPA2B1(S344);HNRNPA3(S358);HNRNPC(S253);HNRNPLL(S61);HNRNPM(S528);HNRNPM(S618);HPS5(S534);HRNR(S903);HRNR(S905);HSPB1(S15);HSPB1(S82);HUWE1(S1084);IBTK(S1045);IGLL1(S58);INCENP(T292);INPP5D(S971);INPP5D(T963);INTS12(S128);IPCEF1(S430);IRF2BP1(S421);IRF2BP2(S175);IRF2BP2(S318);IRF2BP2(S406);IRF2BPL(S519);ITGAL(S37);ITSN2(S884);ITSN2(S889);JADE3(S566);JMJD1C(S1223);JMJD1C(S641);JPT2(T76);KANK2(S172);KANK2(S175);KCAB2_HUMAN_Phospho (ST);KCNK2(S366);KIAA0319L(S978);KIAA0930(S304);KIAA1217(S357);KIAA1217(S361);KIAA1468(T143);KIAA1522(S545);KIAA1522(S858);KIAA1522(S862);KIAA1522(S929);KIF1A(S1094);KIF1A(S1528);KIF1A(S1532);KNOP1(S119);KPNA4(S60);KRT13(S427);KRT8(S36);L1TD1(S557);LAD1(S301);LAMTOR1(S27);LARP1(S1056);LARP1(S90);LARP1(T526);LARP1(T649);LAT2(S135);LAT2(S86);LEMD3(S187);LIMA1(S617);LIN28B(S203);LIN54(S310);LMNA(S22);LMNA(S390);LMNB2(S37);LRCH1(S532);LRCH4(S520);LRRFIP1(S116);LRRFIP2(S324);LSM11(S21);LSR(S464);LSR(T453);LUZP1(S745);MACF1(S7330);MAML1(S360);MAP1A(S1675);MAP1A(S1776);MAP2(S1540);MAP2(S1653);MAP2(T1649);MAP7D1(S93);MARCKS(S163);MARK1(S588);MAST2(S876);MAZ(S361);MCM3(Y708);MCM3AP(S557);MCM4(S120);MDC1(T378);MEPCE(S217);MEPCE(T213);MEX3C(S540);MEX3C(T541);MFAP1(S116);MIA2(S1255);MIA3(S1741);MICAL3(S649);MICALL1(S391);MICALL1(S486);MICALL1(S640);MICALL2(S143);MICALL2(S153);MIS18BP1(S1042);MKI67(S1937);MKI67(S2223);MLC1(S179);MLLT6(S378);MLLT6(S382);MORC2(S696);MORC2(S725);MPLKIP(S47);MPLKIP(T51);MPLKIP(Y45);MTA1(S386);MTA1(S449);MTA1(S522);MTA2(S435);MTBP(S755);MTFMT(S23);MTMR3(S613);MTMR4(S961);MTOR(S2454);MTSS1L(S342);MYBBP1A(S11);MYC(T58);MYCBP2(S3467);MYCN(S156);MZT2A(S139);MZT2B(S139);N4BP3(S211);NAA10(S186);NAA30(S199);NAB1(S403);NAB2(S171);NADK(S48);NADK(S64);NASP(T390);NAV1(S808);NAV2(S1800);NCAPD2(Y1325);NCL(T121);NCL(T76);NCOR1(S1980);NCOR1(S1981);NCOR2(S1547);NCOR2(S2424);NCOR2(S54);NECAP2(S181);NES(S768);NFATC1(S282);NFATC2(S217);NFATC2(S814);NOLC1(S397);NOLC1(S508);NOLC1(S622);NOLC1(S643);NONO(T450);NOP16(S16);NOP2(S732);NOP53(S29);NOP58(S351);NSD1(S2471);NUCKS1(T179);NUFIP2(S230);NUMA1(S1862);NUMA1(S1887);NUMA1(T2000);NUMBL(S263);NUP153(S209);NUP210(S1877);NUP210(S1881);NUP210(T1844);NUP35(S66);OBSL1(S10);OSBPL8(S68);PABPN1(S150);PAGR1(S237);PARD3(S221);PARVA(S19);PATL1(S278);PBRM1(S12);PBRM1(S13);PBX2(S330);PCBP1(S190);PCBP1(S231);PCM1(T79);PCM1(T82);PCNP(T139);PCYT1A(S315);PCYT1A(S347);PCYT1B(S315);PDCD6IP(S730);PDLIM2(S129);PDLIM4(S112);PDLIM5(S111);PDS5B(T1301);PDZD8(S521);PEA15(S116);PEAK1(S823);PFKL(S775);PGRMC1(S181);PHACTR2(T25);PHF3(S1614);PHF8(S880);PHKA2(S1043);PI4K2A(S51);PIK3AP1(S759);PKP4(S273);PKP4(S314);PLCB3(S926);PLEC(S1435);PLEKHA5(S937);PLEKHA5(T857);PLEKHA7(S903);PLEKHG4B(T727);PLK1(T214);PLPPR3(S353);PML(S505);POLA2(T127);POLD2(S15);POLM(S372);POM121(S298);POM121C(S275);POMZP3(S33);POTEE(S939);POTEF(S939);POTEKP(S239);PPFIBP1(S636);PPHLN1(S163);PPHLN1(S172);PPHLN1(S201);PPHLN1(T200);PPHLN1(T204);PPME1(S15);PPP1CC(T311);PPP1R12A(T696);PPP1R13L(S358);PPP1R13L(S395);PPP1R9B(S100);PRAG1(S510);PRKDC(T1045);PRR11(S40);PRR12(S314);PRR36(T1082);PRRC2A(S1147);PRRC2A(S2113);PSMF1(S153);PTDSS2(S16);PXN(S85);R3HDM2(S349);RAB11FIP1(S529);RAD18(S103);RALGAPB(T379);RANBP2(S2454);RANBP2(S2900);RANBP2(T1396);RANBP3(S211);RANBP9(S477);RANBP9(S482);RASAL3(S18);RASGRP2(S391);RB1(S249);RB1(S788);RB1(S795);RB1(T356);RB1(T821);RB1(T826);RB1(Y790);RBL1(S749);RBM10(S845);RBM15(S294);RBM15(S622);RBM17(S169);RBM39(S97);RBM39(Y95);RBM6(S1025);RBMX(S208);RBMX(S249);RBMXL1(S208);RBMXL1(S249);RBMXL1(S88);RECQL5(S815);REPS1(S709);RFX7(S1028);RGPD1(S1463);RGPD2(S1471);RGPD3(S1479);RGPD4(S1479);RGPD5(S1478);RGPD8(S1478);RIF1(S1688);RIF1(S2205);RPL18(S161);RPL18(T158);RPRD2(S665);RPRD2(T732);RRM2(T33);RRP15(T104);RRP1B(S735);RSL1D1(S392);RSL1D1(S396);RSL1D1(T465);SACS(S1779);SALL2(S806);SALL3(S940);SALL4(T541);SAMD1(S161);SAMD4B(S172);SAP130(S442);SAPCD2(S157);SASH3(S21);SCML2(S267);SCRIB(S1348);SCRIB(S1448);SCRIB(S504);SCRIB(S853);SEC16A(S1905);SEC31A(S799);SEPT9(S22);SET(S7);SF3B1(S129);SF3B1(T257);SF3B1(T303);SF3B1(T313);SFPQ(S33);SFPQ(T687);SFRP2(S287);SFRP2(S289);SFSWAP(S909);SGO1(S468);SH3BP2(S427);SHANK2(S67);SHROOM3(T576);SIK3(T469);SIPA1L1(S1565);SLC25A20(S208);SLC4A1AP(S82);SLTM(S1002);SLTM(S553);SLX4(S1309);SLX4(S1333);SMARCA2(S588);SMARCAD1(S146);SMNDC1(S201);SNRK(S518);SNRNP200(S225);SNRNP70(S226);SNURF(S32);SNX17(S336);SNX17(S409);SNX17(S415);SPECC1(S55);SPEG(S2109);SRRM1(S695);SRRM2(S1499);SRRM2(S510);SRSF1(S199);SRSF1(S201);SRSF9(S216);SSB(S366);STAM(S156);STIM2(S523);STK10(S450);STK17A(S28);STMN1(S38);SUPT6H(T1523);SURF6(S138);SVIL(S968);SYNJ1(S1053);SYTL2(S344);TACC3(S25);TACC3(S250);TACC3(S317);TAF6(S634);TAF6(S636);TAF7(S201);TAOK1(S965);TBC1D1(S211);TBC1D9B(S435);TBX2(S653);TCF20(S574);TCF20(S966);TCOF1(S1227);TCOF1(S156);TCOF1(S503);TCOF1(T914);TELO2(S836);TEX2(S732);THAP4(S128);THOC5(S314);THRAP3(S248);THRAP3(S575);THRAP3(S928);TICRR(T1260);TJAP1(S320);TJAP1(T318);TJAP1(Y316);TJP1(S617);TJP2(S1159);TJP2(S266);TK1(S231);TLN1(S425);TMC8(S714);TMEM201(S441);TMPO(S306);TMPO(S354);TMX1(S270);TNIK(S764);TNIK(S766);TNKS1BP1(S1103);TNKS1BP1(S836);TNRC6C(S714);TOM1(S464);TOR1AIP1(S135);TP53BP2(S558);TPD52L2(S166);TPR(S379);TRA2B(T201);TRA2B(T212);TRIM24(S654);TRIM33(S862);TRIM71(S187);TRIP12(S312);TRPM7(S1477);TRPS1(S216);TRPS1(T751);TSHZ2(T646);TUBA1A(S48);TUBA1B(S48);TUBA1C(S48);TUBA3C(S48);TUBA3E(S48);TXLNG(S97);U2SURP(S37);UBAP2L(S605);UBE2O(T838);UBE4B(S65);UBE4B(T64);UCK1(S253);ULK1(S450);UNC13B(S367);UNC93B1(S547);UNC93B1(S550);UNG(T60);UPF3B(T169);USP10(S211);USP10(S547);USP15(S242);USP20(S134);USP36(S546);USP36(S742);USP36(T653);USP7(S18);VCL(S290);VGLL4(S149);VPS13D(S1042);WBP11(S237);WDFY4(S3123);WIPF1(S340);WIZ(S1012);WT1(S273);XPO4(S521);XRCC1(S226);XRCC1(S229);XRCC1(T198);XRCC1(Y211);XRCC6(S477);YAP1(S289);YBX2(S189);YBX3(T67);YTHDC2(S1223);ZC3H11A(S132);ZC3H4(S907);ZC3HAV1(S378);ZCCHC8(S598);ZCCHC8(T479);ZCCHC8(T485);ZDHHC5(S425);ZFHX4(S2996);ZFP64(S547);ZFP91(S101);ZFP91(S103);ZFYVE26(S1764);ZMYM2(S305);ZMYM4(T217);ZNF24(S274);ZNF318(S1896);ZNF318(S501);ZNF462(S1251);ZNF574(S164);ZNF639(S88);ZNF687(S374);ZYX(S308)</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>TNK2</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>656</v>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>09/07/18 00:00:00(T228);09/09/18 00:00:00(S30);ABCA2(S1238);ABCF1(S105);ABCF1(T108);ABL1(S718);ACIN1(S481);ACIN1(S490);ADAM17(S791);ADGRL2(S1430);AGAP2(T809);AHCTF1(S1142);AHNAK(S3426);AHNAK(S5110);AHNAK(S570);AHNAK(S5731);AHNAK(S819);AKAP2(S152);AKAP2(S748);AKIRIN1(S22);AKIRIN2(S21);ANKRD2(S99);ANKS1A(S677);APC(S2125);APRT(S30);ARFGEF1(S1569);ARFGEF2(S240);ARFGEF2(T244);ARHGAP5(S1218);ARHGEF17(S420);ARHGEF6(S488);ARID1A(S1755);ARVCF(S887);ATF1(S36);ATL2(S24);ATRX(S34);ATXN1(S88);ATXN2(S863);ATXN2(T672);ATXN2L(S594);ATXN7L3(S281);BAG3(S386);BAIAP2L1(S261);BAIAP2L1(S331);BAZ2A(S1785);BCL9L(S1004);BCL9L(S1010);BCL9L(S750);BCL9L(S813);BCL9L(S999);BCLAF1(S222);BCLAF1(S282);BCLAF1(S512);BCLAF1(S564);BRIP1(S956);BRWD1(S696);BYSL(S98);C17orf53(S332);C2CD2L(S411);C2CD5(S260);C9orf78(S101);CAMKK2(S129);CAMKK2(S133);CAMSAP3(S685);CARMIL1(S1094);CASKIN2(S403);CASKIN2(T807);CASP3(S26);CBL(S619);CBX5(S92);CC2D1A(S208);CC2D1A(T204);CCDC86(S102);CCDC86(S47);CCDC86(S80);CCDC86(T42);CCDC88A(S230);CD2AP(S458);CDC25A(S18);CDC42EP2(S141);CDC42EP2(T137);CDC42SE1(S74);CDCA3(S87);CDK1(T161);CDK11A(T739);CDK11B(T751);CDK12(S274);CDK12(S276);CDK12(T1244);CDK13(T1058);CDK2(T160);CDK3(T160);CENPF(S3119);CENPF(T144);CEP170(S1160);CHAMP1(S427);CHAMP1(S432);CHAMP1(S436);CHD4(S515);CHD4(S531);CLASP1(S636);CLK2(S142);CLSPN(S954);COBLL1(S294);COL4A3BP(S132);COL4A3BP(S373);CRTC1(S153);CSNK1D(S382);CTAGE5(S594);CTAGE5(S596);CTDP1(S416);CTNNB1(S191);CTNND1(Y865);CTTN(S418);CTTN(T401);CTTN(T411);CUX1(S1215);CUX1(T1071);CYBRD1(S260);DBF4(S359);DCP2(S284);DDX3X(S90);DDX41(S23);DDX54(S75);DDX59(S76);DENND1A(S523);DENND4C(S989);DGCR8(S373);DGCR8(S377);DLGAP4(S666);DLGAP5(S662);DNTTIP2(S141);DNTTIP2(S330);DNTTIP2(S434);DOCK5(S1834);DOCK7(S888);DOCK8(S904);DPF2(S200);DPYSL3(T509);DSP(S176);DTL(S512);DTNA(S662);DYNC1LI1(S398);DYNC1LI1(S465);DYNC1LI1(S468);EBAG9(S36);EDN3(S34);EHMT2(S173);EIF2AK4(S555);EIF4EBP1(S83);EIF4EBP1(T82);EIF4ENIF1(S74);EIF4G1(S1092);EIF4G1(S1231);EIF4G2(T508);EIF4G3(S230);EML4(T899);ENAH(S506);EP300(S1726);EPB41(S560);EPB41(T710);EPHA1(S906);EPHA1(S910);EPN1(S435);EPRS(S886);EPS15L1(S229);ERBIN(S1168);ERF(S161);ERF(T526);ERF_HUMAN_2 Phospho (ST);ERF_HUMAN_Phospho (ST);ERRFI1(S461);ETV1(S97);ETV3(S139);FAM109A(S213);FAM122B(S115);FAM193A(S1129);FAM53B(S268);FAM53C(S251);FAM53C(S254);FAM53C(S255);FAM76B(S193);FAM83H(S9);FARP2(S389);FBRSL1(S1034);FBXL19(S408);FEZ1(S298);FGD1(S50);FKBP15(S1164);FLNC(S2624);FNBP1(S497);FNDC3A(S213);FOXO3(S284);FRY(T1956);FTSJ3(S688);FTSJ3(T573);FUBP1(S630);G3BP2(S163);GAPDH(T153);GAPVD1(S569);GAPVD1(S950);GBF1(S1320);GBF1(S1773);GFPT1(S261);GIGYF2(S26);GIGYF2(S30);GIGYF2(S593);GJA1(S255);GLCCI1(S406);GMIP(S923);GOLGA4(S266);GOLGA5(S116);GON4L(S346);GPAT3(S68);GPR161(S356);GPR183(S343);GPRIN1(S389);GTF3C2(S132);GTF3C2(S765);GTPBP6(S43);HCFC1(S1507);HCFC1(S598);HDGFL2(S137);HEATR1(S1190);HEATR6(S643);HECTD1(S1387);HERC1(S1428);HID1(S653);HIRIP3(S196);HIRIP3(S199);HMGCS1(S4);HMGCS1(T476);HMGN1(S25);HNRNPA2B1(S212);HNRNPD(S190);HNRNPU(S59);HSH2D(S251);HSPB8(T87);HSPBP1(S354);ICAM3(S544);ICE1(S1331);ICE1(S1903);IFIH1(S301);IL17RA(S708);IMPDH2(S122);INCENP(S275);INPP5D(T963);INSRR(S72);INTS3(S502);IQSEC1(S180);IQSEC1(S512);IRF2BP2(S175);IRF2BP2(S406);IRF2BPL(S519);IRS1(S329);IRS1(T351);IRS2(S1203);ITPKB(S43);ITPR3(S1832);ITSN1(S904);ITSN1(S978);IVNS1ABP(S277);JPT1(T54);KANSL1(S991);KANSL1(S994);KAT6A(S1000);KDM1A(S166);KIAA0754(S666);KIAA0930(S324);KIAA1468(T143);KIAA1671(S1488);KIDINS220(S1361);KIF1A(S1370);KIF21B(S1149);KMT2D(S2274);KNOP1(T310);KPNA2(S62);KRT17(S32);KRT8(S13);L3MBTL2(S688);LARP1(T376);LEMD3(S144);LIG3(S912);LIMA1(S15);LIN28A(S200);LMNA(S301);LMO7(S706);LPIN1(S162);LRCH4(S520);LRMP(S131);LRRC40(S71);LRWD1(S251);LUC7L2(T17);MACF1(T7287);MAP1B(S1400);MAP1B(S1797);MAP2(S1540);MAP2K2(T394);MAP3K7(S367);MAP3K7(S389);MAP4(T571);MAP7D3(S165);MAPK1(T185);MAPK1(Y187);MAPK3(T202);MAPK3(T207);MAPK3(Y204);MAST2(S148);MAST2(S209);MBD1(S391);MBP(T39);MCM6(S689);MCRIP1(S21);MED13(S530);MED13(S537);MED24(S873);MEPCE(S152);METTL6(S274);MIA2(S1202);MIA2(S1204);MIS18BP1(S1104);MIS18BP1(T702);MKI67(S538);MORC3(S765);MSL1(S205);MTA1(S386);MTBP(S639);MTMR1(S43);MTMR1(S653);MTMR3(S613);MYC(S62);MYC(T58);MYCN(S156);MYCN(S62);MYO18A(S102);MYO7B(S689);N4BP3(S211);NAB1(S407);NAP1L4(S125);NAV1(S1014);NBN(S432);NCBP1(S22);NCKIPSD(S122);NCOR2(S215);NDRG1(S367);NEK6(S206);NES(S905);NFAT5(S145);NIN(S1550);NIPBL(S280);NKAP(S9);NOP14(S96);NSD1(S2471);NSD2(T115);NSUN2(S473);NUMA1(S1834);NUMA1(S2047);NUP107(T46);NUP153(S343);NUP160(S1157);OIP5(S225);ORC2(S280);OSBP(S240);PAICS(S27);PAK2(S141);PAK2(T143);PALLD(S893);PALM3(S143);PANK2(S189);PAPOLA(S558);PAPOLG(S708);PARD3(S144);PARD3(S152);PARD3(S221);PATJ(S645);PAWR(T163);PAXBP1(S557);PAXBP1(S558);PCDHGC3(S60);PCM1(S65);PCM1(S861);PDCD6IP(S718);PDE7A(S113);PDE7B(S74);PDLIM2(S197);PDLIM2(S266);PEA15(S116);PFDN4(S125);PGAM1(S118);PGAM4(S118);PGM5(S510);PHACTR4(S427);PHF3(S1133);PHKA2(S1015);PHLDB1(S583);PHRF1(S1229);PI4KB(S266);PIKFYVE(S307);PJA1(S265);PLCB2(S964);PLEKHA1(S332);PLEKHA5(S471);PLIN5(S203);PLK1(T214);PNN(S347);PPFIBP1(S601);PPHLN1(S201);PPHLN1(Y162);PPP1R12A(S871);PPP1R13L(S597);PPP1R1A(T78);PPP1R2(T89);PPP1R7(S27);PPP6R1(S759);PPP6R3(S617);PRAG1(T801);PRKAB1(S182);PRPF4B(S852);PRPF4B(Y849);PRR12(S487);PRR15(S49);PRR5(S11);PRRC2A(S2113);PRRC2B(S1691);PSD4(S134);PSMA5(S56);PSMD2(S16);PTBP1(S16);PTGFRN(S875);PTPN1(S352);PTPN12(S332);PTPN13(S1082);PTPN14(S620);PTPN14(S642);PTPRA(Y798);PXN(S119);PXN(S126);PXN(S258);PXN(Y88);PYGO2(S40);Phospho (ST);RAB11FIP1(S202);RAI14(S281);RAI14(S286);RALGAPA1(T754);RALGPS2(S329);RANBP2(S1869);RAP1GAP2(S45);RAP1GAP2(S564);RAPGEF1(S311);RASAL2(S665);RASAL3(S167);RB1(S608);RB1(S612);RB1(S788);RB1(S795);RB1(S807);RB1(S811);RB1(T601);RB1(Y606);RB1(Y805);RBL1(S749);RBM14(S520);RBM14(S618);RBM15B(S113);RBM17(S169);RC3H1(S535);REPS1(S709);REPS1(T539);RIF1(S1554);RIF1(S782);RIF1(T1047);RNF20(S525);RNF214(S511);ROBO4(S125);RPAP3(S481);RPP38(S235);RPS17(S113);RPS6KA1(S363);RPS6KA1(S380);RPS6KA3(S369);RPTOR(S863);RRBP1(S1277);RREB1(S1238);RRM2(T33);RRP1B(S679);RSF1(S570);RSF1(S622);RSF1(S629);RSF1(T628);RSL1D1(T465);RTF1(S697);RUNX1(S212);SAFB(T200);SAMD4B(S628);SAMHD1(S33);SAMHD1(T21);SAP30(S138);SASH1(S839);SCAF1(S992);SCAF11(S802);SCNM1(S183);SCRIB(S1445);SEC16A(S25);SEC31A(S527);SEC31A(S799);SENP1(S157);SENP7(S443);SENP7(S444);SEPT9(S30);SERBP1(S234);SF3B1(T434);SFPQ(S33);SFSWAP(S604);SGTA(S77);SGTA(T81);SH3BP2(S278);SHROOM2(S208);SHROOM3(S1221);SHROOM3(S890);SIN3A(S1112);SIPA1L1(S162);SIPA1L2(S162);SIRT1(T719);SLC9A1(S599);SLC9A3R1(S269);SLC9A3R2(S303);SMARCA2(S588);SMARCA4(S1382);SMARCA4(S613);SMG8(T743);SMTN(S357);SNURF(S32);SPIN1(S199);SPP2(S182);SRA1(S69);SRRM1(T718);SRRM2(S1124);SRRM2(S1404);SRRM2(S144);SRRM2(S2740);SRRM2(T1003);SRRM2(T1856);SRRM2(T2409);SRRM2(T2738);SSH1(S897);STAT5A(S193);STAT5A(S780);STMN1(S16);STMN1(S46);STMN2(S80);STRIP1(S335);STRN(Y135);SUDS3(S237);SUPT20H(T494);SYTL1(S253);TACC2(S2317);TACC2(S2321);TACC3(S177);TANC2(T434);TATDN2(S420);TBC1D10B(S687);TBC1D5(S522);TBX2(S653);TBX2(S657);TCF25(S602);TCOF1(S906);TEAD3(S148);TELO2(S836);TEPSIN(S333);TGFBR2(S352);THRAP3(S575);TIAM1(S311);TJAP1(T422);TJP1(S131);TJP1(S1579);TJP2(S979);TLE3(S286);TLK1(S159);TMCO1(S184);TMPO(S159);TMPO(S66);TNKS1BP1(S1024);TNKS1BP1(S893);TNRC18(S1033);TNRC18(S1038);TNS2(S1003);TNS3(S776);TOPORS(S194);TP53BP1(S366);TPR(T2116);TRAPPC12(S184);TRIM2(S456);TRIM24(S687);TRIM33(S1119);TRO(S155);TRPS1(S115);TSC22D4(S279);TUBA1A(S287);TUBA1B(S287);TUBA3C(S287);TUBA3E(S287);TUBA4A(S287);TWISTNB(S316);TXLNA(S515);UBA1(S21);UBAP1(S146);UBE4B(S65);UBE4B(T64);UHRF1BP1L(S414);UHRF1BP1L(S418);UTP3(S37);VANGL1(T47);VASN(S284);VCL(S346);VIPAS39(S121);VIRMA(T184);VRTN(S432);WAPL(S226);WAPL(S380);WASHC2A(S1075);WASHC2C(S1052);WASHC2D(S42);WASL(Y256);WDR44(S162);WWC3(T909);XPO1(S391);XPO4(S521);YAP1(S367);YY1(S187);ZC3H11A(S108);ZC3H11A(S758);ZC3H13(S242);ZC3H14(S620);ZC3HAV1(S387);ZC3HAV1(T393);ZC3HC1(S359);ZC3HC1(S395);ZCCHC17(S114);ZDHHC5(S299);ZDHHC5(S429);ZEB1(S679);ZFC3H1(S1046);ZFP36L1(S54);ZHX3(S946);ZMYND8(S462);ZNF106(S1302);ZNF106(S1304);ZNF24(S274);ZNF330(T293);ZNF592(S78);ZNF609(S1055);ZNF609(S427);ZNF609(S433);ZZEF1(S1518);ZZZ3(S113)</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>TTK</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>1154</v>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>09/02/18 00:00:00(S218);09/09/18 00:00:00(S30);AAK1(S14);ABCF1(S109);ABI1(S216);ABI1(Y213);ABLIM1(S431);ABR(T74);ACIN1(T414);ACTA1(S241);ACTA2(S241);ACTB(S239);ACTBL2(S240);ACTC1(S241);ACTG1(S239);ACTG2(S240);ADAM10(S740);ADAM10(Y741);ADAM17(S791);ADD1(S12);ADD1(S431);ADD1(S465);ADD1(S726);ADD2(S713);ADD3(S693);ADNP(S970);AFDN(S1721);AFF1(T372);AFF1(T376);AFF4(S1043);AFF4(S1058);AFF4(S32);AGAP1(S605);AGAP2(S808);AHCTF1(S1222);AHCTF1(S528);AHDC1(S1064);AHDC1(S1507);AHNAK(S115);AHNAK(S216);AHNAK(S3412);AHNAK(S3426);AKAP11(S1242);AKAP11(S1580);AKAP11(S422);AKAP11(S448);AKAP13(S2728);AKT1S1(S183);ALMS1(T3036);AMBRA1(S639);ANAPC1(S355);ANKIB1(S737);ANKRD17(S2401);ANKS1A(S382);ANKZF1(S675);ANP32B(T244);APPL1(S401);ARFGAP2(S201);ARFGAP2(S368);ARFGAP2(S432);ARHGAP1(S44);ARHGAP1(S51);ARHGAP10(S591);ARHGAP17(S625);ARHGAP21(S856);ARHGAP32(S1203);ARHGAP4(S930);ARHGEF11(S150);ARHGEF11(S35);ARHGEF11(T1292);ARHGEF17(S735);ARHGEF35(S184);ARID1A(S1184);ARID1A(S1604);ARID1A(S730);ARID3A(S77);ARID3B(S381);ARID4B(S1029);ARID4B(T1025);ARID4B(T1026);ARL6IP6(S80);ASAP2(S822);ASIC3(S37);ATAD1(S322);ATAD2(S327);ATAD2(T1152);ATF7IP(S477);ATG2B(S1582);ATG2B(S1583);ATG2B(Y1577);ATG9A(S828);ATN1(S661);ATN1(T653);ATP5F1C(S146);ATRX(S890);ATXN2(S667);BCAM(S600);BCL11A(S328);BCL2L12(S113);BCL2L12(S121);BCL2L12(T117);BCL7C(S126);BCL9L(S1010);BCR(S459);BIN2(S259);BORCS8(S109);BRAF(T401);BRCA1(S1189);BRCA1(S1191);BRD4(S1126);BRD9(S56);BRIP1(S956);BRIP1(S990);BRPF1(S460);BRPF1(S462);BRSK2(T459);BRSK2(T463);BRWD1(S2018);BUB1(S655);BUD13(S151);BUD13(T147);C16orf54(S194);C2CD2L(S662);C2CD5(S281);C2CD5(S295);C2CD5(S662);C6orf132(S449);C7orf50(S175);C9orf78(T100);CABLES1(S291);CAD(S1859);CALU(S35);CALU(S44);CAMK1D(T184);CAMKV(T430);CAMSAP1(S563);CANX(S564);CARD9(S460);CARHSP1(S52);CARMIL2(S1315);CASC3(S363);CASC3(T143);CAT(S515);CBFA2T3(S459);CBL(S799);CBX8(S311);CCDC6(S240);CCDC86(S66);CCDC9(S376);CCDC93(S305);CCL13(S44);CCNL1(S335);CCNL1(S338);CD2AP(T236);CD2BP2(S49);CD97(S818);CD97(S831);CDC25C(S216);CDCA7L(S261);CDK11A(S72);CDK11B(S72);CDK13(T1056);CDK13(T871);CDK9(S347);CDT1(S394);CDV3(T182);CENPF(S276);CEP170(S881);CEP55(S428);CEP97(S308);CHAF1A(S206);CHAF1A(S775);CHAMP1(S376);CHAMP1(S432);CHAMP1(S436);CHAMP1(S445);CHAMP1(S452);CHAMP1(S472);CHAMP1(S507);CHAMP1(S652);CHAMP1(S653);CHD3(S324);CHD4(S1535);CHD4(S303);CHD8(S1420);CHD8(S1424);CHD8(S1978);CHD8(T1982);CIT(S1322);CLASP1(S636);CLASP2(S325);CLASP2(S529);CLASRP(S547);CLINT1(T308);CLK1(S140);CLK1(T138);CLK2(S142);CLSPN(S775);CMTR1(S31);CNK3/IPCEF1(S892);CNP(S170);COL4A3BP(S373);CPSF7(S48);CREB1(S111);CREB1(S271);CRMP1(S522);CSNK1E(S363);CSPP1(S901);CTAGE1(S616);CTAGE5(S647);CTDP1(S839);CTDSPL2(S28);CTPS1(S573);CTTN(T411);CTU2(S419);CYBA(T147);CYBRD1(T285);DACH1(S727);DAXX(S671);DBF4(S381);DBNL(T291);DCTN2(S83);DCTN2(Y81);DDB2(S26);DDX17(S571);DDX21(S121);DDX21(S89);DDX3Y(S592);DDX42(S96);DDX54(S782);DEF6(S590);DENND4A(T1019);DENND4C(S1277);DENND4C(S1301);DGCR8(S271);DGCR8(S275);DGCR8(Y267);DIP2B(S259);DIS3L2(S875);DLG5(S1000);DLG5(S1795);DLG5(T984);DLGAP1(S406);DLGAP2(S570);DLGAP3(S502);DLGAP4(S512);DLGAP5(S725);DNAAF1(T269);DNTTIP2(S434);DNTTIP2(S88);DNTTIP2(T172);DNTTIP2(T87);DOCK11(S440);DOCK7(S898);DOCK7(S946);DOCK8(S451);DOT1L(S374);DSN1(S81);DTL(S425);DVL2(S211);DYNC1LI1(S398);E2F8(S71);EDC3(S131);EDN3(S34);EEF1D(T147);EEF2K(S72);EEF2K(S74);EEF2K(Y37);EEF2K(Y69);EEPD1(S21);EHBP1(T378);EIF2B1(S107);EIF3A(S1188);EIF3A(S584);EIF3C(S9);EIF3CL(S9);EIF3E(S399);EIF4EBP1(S44);EIF4EBP1(S65);EIF4EBP1(T37);EIF4EBP1(T41);EIF4EBP1(T46);EIF4EBP1(T70);EIF4EBP1(T82);EIF4EBP1(Y34);EIF4EBP2(S65);EIF4EBP2(T37);EIF4EBP2(T41);EIF4EBP2(T46);EIF4EBP2(Y34);EIF4EBP3(T31);EIF4EBP3(T32);EIF4EBP3(Y20);EMD(S141);EMD(S142);EMD(S143);EML4(S144);EML4(S146);ENAH(T538);EP400(S722);EP400(S736);EPB41L1(S784);EPB41L2(S499);EPS15L1(S793);EPX(S672);ERBIN(S1168);ERCC5(S384);ERCC6L(S820);ERRFI1(S461);ESRP1(S543);EZH2(S363);EZH2(T367);F11R(S284);F11R(S287);FADD(S194);FAM117B(S10);FAM122A(S143);FAM122A(S189);FAM129B(S665);FAM129B(S681);FAM129B(S696);FAM207A(T34);FAM53B(S179);FAM76B(S193);FAM83B(S766);FAM83H(S1003);FAM83H(S914);FAM84B(T289);FANCI(S1121);FARSA(S301);FBRSL1(T1010);FBXW9(S59);FERMT3(S8);FGD6(S692);FIP1L1(S259);FMN2(S295);FNBP1L(S501);FOXK1(S101);FOXK1(S257);FOXK1(S416);FOXK1(S420);FOXK1(S441);FOXK1(S445);FOXK2(S373);FOXK2(S61);FOXO1(S329);FOXO3(S55);FRMD3(S416);FUS(S462);FXR2(S453);FXR2(S601);FXR2(T411);FYTTD1(S16);GAB2(S141);GAGE13(S33);GAGE2A(S32);GAGE2B(S32);GAGE2D(S32);GAPVD1(S902);GATAD2A(T189);GATAD2B(S334);GATAD2B(S486);GBF1(S1061);GBF1(S1298);GCN1(S786);GFI1(S94);GIGYF2(S26);GJA1(S262);GNL3(S529);GON4L(S1268);GORASP1(S220);GPATCH2(S195);GPATCH4(S128);GPATCH4(S130);GPHN(S188);GPHN(S194);GPHN(T198);GRIP1(S847);GRWD1(S122);GTF2F1(S385);GTF2F1(T389);GTF2F1(T446);GTF3C1(S1068);GTF3C1(S1865);GTF3C1(S1868);GTF3C2(S132);GTF3C2(S167);GTPBP1(S44);GTPBP1(S47);HAUS6(T584);HBS1L(S67);HCFC1(S598);HCFC1(S666);HCLS1(T308);HDAC1(S406);HDAC1(S421);HDAC1(S423);HDAC2(S422);HDAC2(S424);HDGF(S132);HDGF(S133);HDGFL2(S652);HELB(S1050);HELZ(S1317);HIC2(S348);HID1(S653);HIRIP3(S102);HIRIP3(S87);HLA-A(S356);HMGCS1(S4);HMGCS1(T490);HNRNPA1(S199);HNRNPA1(S338);HNRNPA2B1(S344);HNRNPA3(S116);HNRNPA3(S358);HNRNPC(S253);HNRNPC(S260);HNRNPDL(S241);HNRNPK(S284);HNRNPLL(S61);HNRNPM(S528);HNRNPM(S618);HPS5(S534);HRNR(S903);HSPB1(S15);HSPB1(S82);HSPB1(S98);HUWE1(S1084);HUWE1(S2362);HUWE1(S2365);IBTK(S1045);ICE1(S1895);ICE1(S1903);ID2(S14);IGF2BP1(S181);IGLL1(S58);INCENP(T292);INPP5D(T963);INTS12(S128);IPCEF1(S430);IRF2BP1(S421);IRF2BP1(S66);IRF2BP2(S175);IRF2BP2(S318);IRF2BP2(S406);IRF2BPL(S519);IRS1(S1101);IRS1(S329);IRS1(T351);IRS2(S620);ITGAL(S37);ITSN2(S884);ITSN2(S889);IWS1(S720);JADE1(S89);JADE3(S566);JMJD1C(S1223);JMJD1C(S641);JPT2(T76);KANK2(S172);KANK2(S175);KAT5(S90);KAT6A(S1000);KAT6A(S450);KAT7(T128);KAT7(T88);KCAB2_HUMAN_Phospho (ST);KCNK2(S366);KDM2B(S1031);KIAA0319L(S978);KIAA1143(S50);KIAA1217(S357);KIAA1217(S361);KIAA1468(T143);KIAA1522(S404);KIAA1522(S858);KIAA1522(S862);KIAA1522(S929);KIF1A(S1094);KIF1A(S1528);KIF1A(S1532);KIF21A(S1271);KIF21A(S1274);KIF4A(S801);KIFC1(S351);KLC1(S524);KLC2(S445);KMT2B(S1035);KMT2B(S1092);KMT2B(S1095);KNOP1(S119);KPNA4(S60);KRT13(S427);KRT8(S36);KRT8(S410);L1TD1(S557);LAD1(S301);LAMTOR1(S27);LARP1(S1056);LARP1(S1067);LARP1(S631);LARP1(S766);LARP1(S90);LARP1(T526);LARP1(T649);LARP1(Y777);LARP1(Y862);LARP4(T389);LARP6(T70);LAT2(S135);LAT2(S86);LEMD3(S187);LIMA1(S230);LIMA1(S617);LIMA1(S686);LIN28B(S203);LIN54(S310);LINC00322(S226);LLGL2(S965);LMNA(S390);LMNB2(S37);LRCH1(S532);LRCH4(S520);LRRFIP1(S116);LRRFIP2(S324);LSM11(S21);LSR(S464);LSR(T453);LUZP1(S745);LYSMD2(S33);LZTS2(S570);MACF1(S5592);MACF1(S7330);MAF1(S60);MAF1(S68);MAML1(S360);MAP1A(S1288);MAP1A(S1675);MAP1A(S1776);MAP1B(S1265);MAP2(S1540);MAP2(S1653);MAP2(T1649);MAP3K7(S389);MAP4K4(S639);MAP7(S209);MAP7D1(S93);MARCKS(S163);MARK1(S588);MAST2(S876);MASTL(S453);MAZ(S361);MCM3(Y708);MCM3AP(S557);MCM9(S883);MDC1(S495);MDC1(S498);MDC1(T378);MED1(S1481);MED1(S1482);MEF2D(S121);MEPCE(S217);MEPCE(T213);MEX3C(S320);MFAP1(S116);MFAP1(S52);MFAP1(S53);MFSD10(S270);MFSD10(S271);MGEA5(S515);MIA2(S1255);MIA3(S1741);MICAL3(S649);MICALL1(S391);MICALL1(S486);MICALL1(S640);MICALL2(S143);MICALL2(S153);MIER1(S377);MIS18BP1(S1042);MKI67(S2223);MLC1(S179);MLLT6(S378);MLLT6(S382);MORC2(S696);MORC2(S725);MPDZ(S1287);MPHOSPH8(S403);MPLKIP(S115);MTA1(S386);MTA1(S449);MTA1(S522);MTA2(S435);MTFMT(S23);MTMR3(S613);MTMR4(S610);MTMR4(S629);MTMR4(S961);MTOR(S2454);MTSS1L(S342);MVD(S96);MYBBP1A(S11);MYBBP1A(S1186);MYC(S62);MYC(T58);MYCBP2(S3467);MYCN(S156);MYCN(S62);NAA30(S199);NAB1(S403);NAB2(S171);NADK(S48);NADK(S64);NAP1L4(S125);NASP(T390);NAV1(S808);NCAPD2(Y1325);NCL(S145);NCL(S153);NCL(S184);NCL(S206);NCOR1(S1472);NCOR1(S1980);NCOR1(S1981);NCOR2(S1547);NCOR2(S2057);NCOR2(S2065);NCOR2(S2424);NCOR2(S54);NDRG3(S334);NEO1(S1214);NES(S768);NEXN(S160);NFATC1(S282);NFATC1(S359);NFATC2(S217);NFATC2(S814);NGDN(S142);NGDN(S143);NGRN(S41);NHSL1(S930);NHSL1(S941);NOL8(S432);NOLC1(S397);NOLC1(S508);NOLC1(S622);NOLC1(S643);NONO(T450);NOP16(S16);NOP53(S29);NOP58(S351);NOP58(S514);NRIP1(S356);NSD1(S2471);NSMCE4A(S63);NUCKS1(T179);NUFIP2(S230);NUMA1(S1862);NUMA1(S1887);NUMA1(S2047);NUMBL(S263);NUP153(S209);NUP188(S1708);NUP188(S1717);NUP210(S1877);NUP210(S1881);NUP214(S1081);NUP35(S66);NUP50(S208);OBSL1(S10);OSBPL8(S68);PABPN1(S150);PAGR1(S237);PAK4(S163);PALM(S116);PALM(S124);PANK2(S189);PARD3(S221);PARVA(S19);PATL1(S184);PATL1(S278);PATL1(T194);PBRM1(S12);PBRM1(S13);PBX2(S330);PCBP1(S190);PCBP1(S231);PCBP1(S264);PCM1(T79);PCM1(T82);PCNP(S147);PCNP(T139);PCYT1A(S315);PCYT1A(S347);PCYT1B(S315);PDCD5(S119);PDCD6IP(S730);PDLIM2(S129);PDLIM2(S266);PDLIM4(S112);PDS5B(S1166);PDS5B(S1257);PDS5B(T1301);PDZD8(S521);PEAK1(S823);PFKL(S775);PGRMC1(S181);PGRMC2(T211);PHACTR2(T25);PHF14(S280);PHF3(S1614);PHF8(S880);PHKA2(S1043);PI4K2A(S462);PI4K2A(S51);PIK3AP1(S740);PIK3AP1(S759);PIKFYVE(T28);PKP4(S273);PKP4(S314);PLCB3(S926);PLEC(S1435);PLEC(S4386);PLEC(S4648);PLEC(Y4393);PLEKHA5(T857);PLEKHG3(S433);PLEKHG4B(T727);PLK1(T214);PLPPR3(S353);PLRG1(S255);PML(S505);PNISR(S311);PNISR(S313);PNISR(S321);POLA2(T127);POLD2(S15);POLD3(S307);POLH(S379);POLH(S380);POLM(S372);POM121(S298);POM121(S395);POM121(S396);POM121C(S275);POM121C(S372);POM121C(S373);POMZP3(S33);POTEE(S939);POTEF(S939);POTEKP(S239);PPFIBP1(S636);PPHLN1(S163);PPHLN1(T200);PPIG(S256);PPIG(S257);PPIG(S259);PPME1(S15);PPP1CC(T311);PPP1R12A(S862);PPP1R12A(S871);PPP1R12C(S427);PPP1R13L(S358);PPP1R2(S87);PPP1R9B(S100);PPP6R3(S523);PRAG1(S510);PRKAR2A(S99);PRKDC(T1045);PRMT3(S25);PRMT3(S27);PRPF3(S619);PRR12(S314);PRR36(T1082);PRRC2A(S1106);PRRC2A(S1147);PRRC2A(S2113);PRRC2A(S342);PRRC2A(S350);PRRC2B(S1691);PRRC2B(Y1693);PSMB10(S229);PSMF1(S153);PTDSS2(S16);PTGES3(S113);PTPN14(S642);PTPN22(S414);PXN(S106);PXN(S85);PXN(Y118);QSER1(S1348);QSER1(T1341);R3HDM2(S349);RAD51AP1(Y13);RALGAPB(T379);RANBP2(S2454);RANBP2(S2900);RANBP3(S125);RANBP3(S211);RANBP9(S477);RANBP9(S482);RASAL3(S18);RASGRP2(S391);RB1(S788);RB1(T356);RB1(Y790);RBL1(S749);RBL1(S762);RBL2(S639);RBM10(S845);RBM15(S294);RBM15B(S562);RBM17(S169);RBM39(S136);RBM39(S97);RBM39(Y95);RBM6(S1025);RBMX(S208);RBMX(S249);RBMX2(S273);RBMXL1(S208);RBMXL1(S249);RBMXL1(S88);RCOR1(S260);RECQL5(S815);REPS1(S709);REPS1(T173);RET(S696);RFC1(S71);RFC1(Y67);RFX7(S1028);RFX7(S1081);RGPD1(S1463);RGPD2(S1471);RGPD3(S1479);RGPD4(S1479);RGPD5(S1478);RGPD8(S1478);RIC8A(S436);RIC8A(T441);RIF1(S1688);RIF1(S2205);RIPK2(S357);RMDN3(S46);RNF25(T303);ROBO1(T1240);RPL18(S161);RPL18(T158);RPL34(S12);RPRD2(S665);RPRD2(T723);RPRD2(T732);RPS10(S146);RPS10P5(S157);RPS6(S235);RPS6(S236);RPS6(S240);RPS6KA3(S227);RPS6KA6(S232);RPS6KB1(S441);RPTOR(S863);RPTOR(S877);RPTOR(T889);RREB1(S1167);RRP1B(S453);RRP1B(S458);RRP1B(S735);RSF1(T628);RSL1D1(S392);RSL1D1(S396);RTN4(S184);RUNX3(S395);RUNX3(S397);SACS(S1779);SAFB(S344);SAFB2(S343);SALL2(S806);SAMD1(S161);SAMD4B(S172);SASH3(S21);SCAF11(S776);SCML2(S267);SCRIB(S1348);SCRIB(S1448);SCRIB(S504);SEC16A(S1905);SEC31A(S799);SEPT9(S22);SET(S7);SF3A1(S329);SF3B1(S129);SF3B1(T142);SF3B1(T303);SF3B1(T313);SF3B1(T434);SFSWAP(S909);SGO1(S468);SH3BP2(S427);SH3GL1(S288);SHANK2(S67);SHROOM3(T576);SIK3(T469);SKA3(S110);SKIV2L(S131);SLC4A1AP(S466);SLC4A7(T559);SLX4(S1309);SLX4(S1333);SMARCA2(S588);SMARCAD1(S146);SMCR8(S417);SMG7(S781);SMN1(S31);SMNDC1(S201);SMPD4(S792);SNRK(S518);SNRNP200(S225);SNRNP70(S226);SNURF(S32);SNX17(S333);SNX17(S336);SNX17(S409);SNX17(S421);SON(S1783);SPAM1(S78);SPECC1(S55);SPEG(S2109);SPP1(S303);SPP1(S62);SPP1(S63);SRCAP(S274);SRRM1(S695);SRRM1(S769);SRRM1(S775);SRRM1(S874);SRRM1(T872);SRRM2(S1463);SRRM2(S1499);SRRM2(S1501);SRRM2(S1502);SRRM2(S2100);SRRM2(S510);SRRM2(S952);SRRM2(S954);SRSF1(S199);SRSF1(S201);SRSF4(S448);SRSF7(S165);SRSF7(S167);SRSF9(S216);SSB(S366);SSRP1(S444);STAM(S156);STEAP3(S17);STIM2(S523);STIM2(S700);STK10(S450);STK17A(S28);STMN1(S38);STRN(Y135);STX10(S143);SUPT6H(T1523);SURF6(S138);SVIL(S968);SYNJ1(S1053);SYTL2(S344);TACC2(S2317);TACC3(S250);TACC3(S317);TAF7(S201);TAF7(S264);TAOK1(S965);TBC1D1(S211);TBC1D4(S588);TBC1D9B(S435);TBX2(S653);TCF20(S574);TCOF1(S1227);TCOF1(S503);TCOF1(T914);TEX2(S732);TEX264(S244);TFE3(S548);TFE3(S556);TFIP11(S210);THAP4(S128);THOC5(S314);THRAP3(S248);THRAP3(S575);THRAP3(S928);TICRR(T1260);TIMELESS(S1149);TJAP1(S320);TJAP1(T318);TJAP1(Y316);TJP1(S617);TJP2(S266);TK1(S231);TLE3(S267);TLN1(S425);TMC6(S63);TMPO(S306);TMPO(S354);TMX1(S247);TMX1(S270);TNIK(S764);TNIK(S766);TNKS1BP1(S1103);TNKS1BP1(S1473);TNRC6C(S714);TOM1(S464);TOR1AIP1(S135);TOX4(S174);TOX4(S182);TP53BP1(S1678);TP53BP1(T1648);TP53BP2(S558);TPD52L2(S166);TPR(S379);TRA2B(T201);TRA2B(T212);TRAPPC10(S711);TRIM24(S654);TRIM28(S440);TRIM37(S771);TRIM71(S187);TRIP10(S296);TRIP12(S312);TRPM7(S1477);TRPS1(S216);TRPS1(T751);TSC1(S1080);TSC1(S1102);TSC2(S1449);TTK(S436);TTYH3(S519);TTYH3(S522);TUBA1A(S48);TUBA1B(S48);TUBA1C(S48);TUBA3C(S48);TUBA3E(S48);TWISTNB(S328);TXLNA(S19);TXLNG(S97);TXLNG(T102);U2SURP(S37);UBE2O(T838);UBE4B(S65);UBE4B(T64);UBR5(T158);UCK1(S253);ULK1(S450);ULK1(S467);ULK1(S479);ULK1(S623);UNC13B(S367);UNC93B1(S547);UNC93B1(S550);UNG(T60);UPF3B(T169);USP10(S211);USP15(S242);USP20(S134);USP32(S1371);USP32(T1326);USP36(S464);USP36(S742);USP36(T653);USP7(S18);UTF1(S211);UTP14A(S407);UTP18(S121);UTP18(S124);UTP3(S37);UTP3(Y43);VCL(S290);VGLL4(S149);VIRMA(S173);VPS13D(S1042);WASHC2A(S158);WASHC2A(S160);WASHC2C(S158);WASHC2C(S160);WDFY4(S3123);WDHD1(S868);WDR59(S830);WDR7(S1154);WIPF1(S340);WT1(S273);XPO4(S521);XPR1(S666);XPR1(S668);XRCC1(S226);XRCC1(S266);XRCC1(T198);XRCC6(S477);XRN2(S448);XRN2(S499);XRN2(S501);YAP1(S289);YBX1(S209);YBX3(S346);YBX3(T67);YTHDC2(S1223);YTHDF1(S291);YY1(S247);ZBTB21(S435);ZBTB21(S983);ZC3H3(S571);ZC3H4(S1108);ZC3H4(S1110);ZC3HAV1(S275);ZC3HAV1(T273);ZC3HC1(S24);ZCCHC11(S841);ZCCHC8(S598);ZCCHC8(T479);ZCCHC8(T485);ZDHHC5(S425);ZEB1(S646);ZFHX4(S2996);ZFP64(S547);ZFP91(S101);ZFP91(S103);ZFPM1(S909);ZFYVE26(S1764);ZFYVE9(S306);ZKSCAN1(S13);ZMYM4(S122);ZMYND8(S444);ZNF106(S1370);ZNF180(S643);ZNF24(S274);ZNF281(S651);ZNF318(S1896);ZNF318(S501);ZNF335(S418);ZNF367(S123);ZNF462(S1251);ZNF574(S164);ZNF609(S467);ZNF639(S88);ZNF687(S374);ZNF800(S426);ZNRF2(S145);ZNRF2(S21);ZNRF2(S82);ZRANB2(S153);ZSCAN29(S153);ZSWIM8(S1092);ZSWIM8(S1156);ZYX(S308)</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>TYK2</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>33</v>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>AMFR(S542);ANKRD17(S2401);ATXN2L(S424);C2CD2(S649);CDK12(S383);CDK12(S385);CNOT2(S170);CRKL(Y207);DDX54(S75);DHX57(S77);DLG5(S1232);FAM53C(S122);GPATCH8(S1033);HIST1H1B(S18);INCENP(S311);IQSEC1(S180);IRF2BPL(S519);KMT2D(S3130);MAPK3(T207);MTMR1(S43);PLEKHA1(S332);PPHLN1(Y162);PRAG1(S889);RNF2(S168);RPA1(T180);SAMHD1(S33);SAMHD1(T21);SATB1(S637);SNRPA1(T180);TSC1(S505);UPF3B(T169);VANGL1(T47);ZC3H15(S360)</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>ULK1</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>41</v>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(S30);ANKRD17(S2401);ARHGEF2(S174);ASIC3(S37);BAG3(T285);CDC42SE1(S74);EIF4B(S283);EPB41L5(S436);GTF3C2(S167);HAUS6(T584);HTT(S1199);IRS1(S374);KIAA1522(S971);LARP6(S409);LINC00322(S226);MAP4(S928);MAP7D1(S399);MARK2(S456);MARK3(S469);MAST2(S1364);OTUD4(S416);PLCL2(S17);PLEKHA5(S885);PRAG1(S148);PRAG1(S889);PRAM1(S334);R3HDM1(S381);RANBP1(S60);RBM15(S292);RICTOR(S1284);SKIV2L(S131);SLTM(S553);SRRM1(S429);SRSF7(S165);SRSF9(S189);TET2(S1107);TPI1(S249);TRIM37(S771);UBE2O(S515);WIPF2(S235);XPR1(S666)</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>YES1</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>721</v>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>09/09/18 00:00:00(S30);AAK1(T653);ABI1(T215);ABI2(S368);ABLIM1(S655);ABLIM1(S706);ACIN1(S388);ADAM17(S791);ADGRL2(S1275);AFAP1(S668);AFDN(S1318);AFDN(T1330);AFF1(T372);AFF1(T376);AGAP1(S605);AGAP3(S538);AGO2(S387);AGPS(S65);AHNAK(S5448);AHNAK(S5739);AJUBA(S263);AKAP13(S1559);AKAP13(S1929);AKAP2(S720);AMPD2(S100);ANKRD17(S1696);ANKRD17(S2401);ANKS1A(S663);ANKS1A(S887);AP1M1(T154);ARFGAP2(S368);ARHGAP17(S162);ARHGAP17(T682);ARHGAP21(S1862);ARHGAP21(S476);ARHGAP21(S856);ARHGAP4(S906);ARHGAP45(S23);ARHGEF11(S255);ARHGEF11(S35);ARHGEF16(S107);ARHGEF16(S578);ARHGEF2(S122);ARHGEF2(T152);ARHGEF6(S684);ARHGEF9(S502);ARID1A(S604);ARID1A(S772);ARID3A(S119);ARL6IP4(S239);ASAP2(S822);ASCC3(S2195);ATAD5(S306);ATAT1(S315);ATF7(S434);ATF7IP(S474);ATF7IP(S477);ATG2A(S498);ATL1(S10);ATP1A1(S16);ATXN2L(S32);BAG6(S1081);BAIAP2(S366);BAIAP2(T340);BCL9(T315);BCOR(S488);BICRAL(S675);BRAF(S365);BRCA1(S1524);BTF3(S30);BUB1B(S543);C17orf47(S195);C17orf53(S332);C1orf198(S175);C2CD2(S649);C9orf40(S69);C9orf78(T100);CAAP1(S312);CAMKV(T435);CAMSAP1(S793);CAMSAP3(S814);CARD9(S425);CARHSP1(S30);CASC1(S504);CASKIN2(S711);CASP3(S26);CBL(S486);CCDC14(S798);CCDC85C(S246);CCDC86(S160);CCDC86(Y164);CCDC88A(S1820);CCNL2(S369);CCNY(S83);CCSER1(S448);CD2AP(S458);CD2AP(S510);CDC25B(S230);CDC25B(S238);CDC25B(S323);CDC25B(S375);CDC42BPG(S1482);CDC42EP1(S350);CDC42EP4(S118);CDC42EP4(T23);CDC42SE1(S74);CDC6(S106);CDCA8(S219);CDK11A(S577);CDK11B(S589);CDK12(S32);CDK12(S383);CDK12(S385);CDK12(T893);CDK14(S24);CDK16(S119);CDK17(S146);CDK17(S180);CDK18(S117);CDK18(S132);CDK18(S14);CENPA(T21);CEP170(T1533);CEP170P1(T242);CEP76(S83);CFL1(S3);CGN(S149);CHAF1A(S206);CHD4(S1531);CHD8(S1995);CHD8(S2008);CIC(S173);CNOT2(S101);CNOT2(S170);COL4A3BP(S373);CPSF4(S202);CRAMP1(S1268);CREB1(S143);CRKL(Y207);CRTC1(S153);CRTC2(S613);CRTC3(S329);CRTC3(S370);CRTC3(S62);CSNK1D(S331);CTAGE5(S635);CTNND1(S349);DAB2IP(S747);DCLK1(S332);DCLRE1C(S518);DDX17(S571);DDX41(S21);DHX57(S77);DHX8(S460);DIP2B(S100);DLG5(S1115);DLG5(S1232);DLG5(S1254);DLGAP4(T975);DNMT3B(S136);DOCK5(S1766);DOCK7(S888);DOPEY2(S681);DSP(S2209);DUSP16(S612);DVL3(S125);DYNC1H1(S4368);EDC4(S729);EEF1D(T147);EEF1G(T46);EEF2K(S72);EEF2K(S74);EEF2K(Y69);EGLN1(S125);EIF3A(S1188);EIF3A(S1336);EIF3A(S882);EIF4ENIF1(S752);EIF4G1(S1187);EIF4G1(S1194);EIF4G3(S232);EML3(S176);EML4(S146);ENAH(S531);EPB41(S560);EPB41(S709);EPN2(S173);EPS15(S563);EPS15(S796);EPS15L1(S593);ERF(S327);ESS2(T386);ESYT1(S627);ETV6(S203);EVPL(S2025);EXO1(S623);FAM102A(S189);FAM117A(S29);FAM120A(Y452);FAM193A(S393);FAM193B(S785);FAM234B(S62);FAM53C(S122);FAM83H(S1025);FAM83H(S647);FERMT3(S15);FLNA(S2158);FOXK1(S223);FOXK2(S373);FRMD6(S522);FRMD6(S525);FRS2(S211);FRYL(T1959);FUBP3(S569);FYB1(S46);FYTTD1(S16);GAB2(S141);GAB2(T391);GAPDH(S151);GAPVD1(S902);GATA3(S115);GLCCI1(S30);GON4L(S206);GPATCH8(S738);GPRIN1(S389);GRAMD1B(S274);GSK3B(S25);GSK3B(S9);GTF2F1(T389);GTF2I(S412);GTF3C1(S1865);GTF3C2(S765);GTSE1(S575);HIPK1(T351);HIPK1(Y352);HIPK2(T360);HIPK2(Y361);HMGA1(S44);HMGCR(S872);HMGCS1(S516);HOXC9(S159);HRNR(S903);HSH2D(S194);HSP90AA1(S263);HSP90AB1(S226);HSP90AB3P(S205);HTATSF1(S642);HUWE1(T2889);ICE1(S1712);IFI16(S153);IGLL1(S62);IKBKB(S672);INCENP(S481);INSRR(S72);IQSEC1(S180);IRF2BPL(S215);ITSN1(S315);ITSN1(S978);IWS1(S235);IWS1(S237);JAZF1(T109);JAZF1(T113);JMJD1C(S2053);JUN(S63);JUP(S665);KANSL1(S829);KANSL1(S839);KIAA1522(S971);KIDINS220(S1633);KIF13B(S1410);KIF1A(S1548);KIF21A(S855);KIF23(S902);KIFC1(S26);KIFC1(S351);KLC2(S610);KLC4(S590);KMT2D(S3130);KTN1(S75);LARP1(S824);LIG1(S76);LIG1(T195);LINC00337(S30);LSM14A(S178);LSM14A(S183);LSM14B(S165);LUC7L2(S18);LUC7L2(S347);LYST(S2627);LZTS1(S233);MACF1(S7279);MACF1(S7330);MAGED2(S265);MAP2(S1555);MAP3K1(S292);MAP3K11(S524);MAP3K2(S153);MAP3K20(S727);MAP3K21(S514);MAP3K4(S1274);MAP3K9(S519);MAP4(S928);MAP4K2(S328);MAP7D1(S113);MAP7D1(S460);MAP9(S79);MARCKS(S167);MARK1(S394);MARK3(S400);MAST3(S747);MATK(S501);MCM3AP(S527);MCRIP2(S82);MED13(S890);MELK(S505);MELK(S529);MEPCE(S152);MEX3B(S4);MFSD10(S271);MIA2(S1243);MINK1(S733);MKI67(T1557);MNAT1(S279);MON1B(S59);MON1B(S61);MPHOSPH8(S403);MPHOSPH8(T89);MPRIP(S289);MPRIP(S292);MPRIP(S993);MTA1(S576);MTFR1L(S103);MTFR1L(S238);MTMR3(S647);MVB12A(S170);MYB(S599);MYC(S62);MYCBP2(S2749);MYCBP2(S2751);MYCN(S62);MYH10(S1937);MYO18A(S102);MYO7B(S689);MYOF(S1915);N4BP3(S211);NAA30(S39);NAB2(S193);NAV1(S1265);NAV1(S528);NAV1(S672);NAV1(S695);NCBP1(S22);NCOA3(S857);NCOA3(Y574);NCOR1(S1472);NDRG2(S332);NDRG3(S331);NDRG3(S334);NECTIN1(T391);NEDD4L(S448);NEDD4L(S487);NFATC2IP(S204);NFX1(Y48);NHSL1(S1233);NINL(S585);NMNAT1(S117);NOC2L(S49);NOL8(S432);NOP58(S502);NSMCE3(S64);NSRP1(S33);NSUN2(S456);NSUN2(S473);OSER1(S82);OSER1(S84);PAK1(S137);PAK1(S144);PAK2(S141);PAK2(T143);PAK4(S163);PAK4(S181);PAK4(T207);PALD1(S406);PALM3(S303);PAPOLG(S708);PARD3(S174);PARD3(S717);PATL1(T194);PBRM1(S13);PBRM1(S14);PCBP1(S173);PCDH18(T442);PCDH7(S1011);PCIF1(S144);PCYT1A(S343);PDE3B(S495);PDHA1(S232);PDHA1(S293);PDHA1(S300);PDHA2(S291);PDHA2(S298);PDS5A(T1208);PDS5B(S1358);PFKP(S386);PHACTR1(S505);PHAX(S368);PHC3(T609);PHIP(S1315);PHKA2(S729);PHLDB1(S334);PHLDB2(T404);PI4KB(S428);PIGT(S235);PKD2(S832);PKN1(S562);PKP2(S289);PKP2(S293);PKP2(S329);PKP4(S337);PKP4(S406);PLCG1(S1263);PLEKHA5(S471);PLEKHA5(S885);PLEKHA6(S808);PML(S518);PML(S527);PNPO(S241);POLH(S380);POLM(S12);POLR2A(S1868);POLR2A(S1878);POLR2A(S1910);POLR2A(Y1860);PPFIA1(S666);PPFIBP1(S466);PPFIBP1(S601);PPFIBP2(S387);PPHLN1(S133);PPIP5K2(S1074);PPM1H(S124);PPP1R12A(S445);PPP1R12A(S903);PPP1R13L(S102);PPP1R35(S87);PPP1R35(T84);PPP1R9B(S100);PRAG1(S889);PRAG1(S907);PRC1(S4);PREX1(S1182);PRKD2(S214);PROSER1(S613);PROSER2(S179);PRPF38B(S268);PRPF38B(S5);PRPF40B(S764);PRPF6(S279);PRPF6(T275);PRRC2A(S1386);PRRC2C(S1544);PRRC2C(T2673);PTK2(S716);PTPN12(S435);PTPN12(S449);PTPN13(S214);PTPN13(S908);PTPN14(S642);PTPN14(S760);PTPN22(S692);PUM1(S124);PXN(S258);R3HDM1(S381);RABEP1(S377);RALGAPA1(S797);RALGAPA1(T754);RALGPS2(S296);RANBP1(S60);RANBP2(S2510);RANBP2(S955);RAP1GAP2(S45);RAP1GAP2(S564);RAPGEF6(S1094);RAPH1(S539);RASAL2(S16);RASAL3(S51);RB1(S249);RB1(T601);RBL1(S640);RBL1(T369);RBM10(S797);RBM14(S256);RBM15(S700);RBM15B(S113);RBM15B(S265);RBM15B(S267);RBM15B(T532);RBM20(S644);RBM23(S140);RBM23(S142);RBM27(S120);RBMX(S208);RBMX(S326);RBMX(S332);RBMX(S352);RBMX(S88);RBMXL1(S208);RCOR1(S260);RCSD1(S116);RCSD1(S120);RFX7(S225);RFX7(S424);RGPD1(S1519);RGPD2(S1527);RGPD3(S1535);RGPD4(S1535);RGPD5(S1534);RGPD8(S1534);RICTOR(S1284);RIF1(S1554);RIOK1(S22);RLIM(S228);RLIM(S230);RNF2(S168);RNF39(S244);ROR2(S449);RPL28(S115);RPRD2(S374);RPRD2(T723);RPS14(S139);RREB1(S42);RYBP(S127);SAFB(S601);SAFB(S604);SAMD1(T107);SASH1(S407);SASH1(S813);SASH1(S90);SBNO1(T819);SCAF1(S874);SCAF11(S796);SCRIB(S1508);SCRIB(T475);SCYL3(T153);SEC24B(T329);SEC62(T375);SERPING1(S198);SF3A1(S359);SF3B1(T261);SF3B1(T350);SF3B1(T434);SF3B1(T436);SGPP1(S101);SH2B3(S150);SH2D3A(S147);SH3BP4(S279);SH3BP4(S296);SH3GL1(S288);SH3KBP1(S230);SH3PXD2B(S291);SHC3(S474);SHCBP1(S42);SHROOM2(S193);SHROOM2(T647);SHROOM3(S664);SHROOM3(S816);SHTN1(S506);SIK3(S866);SIPA1(S839);SIRT1(S27);SLAIN2(S413);SLC20A2(S256);SLC20A2(S259);SLC43A1(T256);SLC4A10(S238);SLC4A7(S233);SLC4A7(S556);SLC4A7(T559);SLC9A1(S703);SLTM(S1014);SLTM(S553);SMAD1(S463);SMAD1(S465);SMAD9(S465);SMAD9(S467);SMAP(S93);SMAP2(S240);SMARCA4(S610);SMARCC2(S347);SMARCD1(S206);SMARCD2(S229);SMARCD3(S181);SMCR8(S489);SMG8(T743);SMG8(Y746);SNIP1(S35);SPAG9(S730);SPAG9(S733);SPP2(S182);SPTAN1(S1031);SPTAN1(S1217);SPTBN2(S2384);SRRM2(S1144);SRRM2(S1404);SRRM2(S1458);SRRM2(S2123);SRRM2(S322);SRRM2(T318);SRRM2(Y1145);SRSF1(S199);SRSF1(S201);SRSF10(S133);SRSF4(S113);SRSF4(S446);SRSF4(S450);SRSF5(S117);SRSF6(S119);SSBP3(S347);SSH3(S37);SSSCA1(S78);STAT5A(S193);STAU1(S390);STIM1(S618);STIM2(S680);STIM2(S719);STK33(S470);STX17(S289);SURF6(T229);SYMPK(S1243);SYNRG(S1075);SYT6(S187);SYT6(Y190);TBC1D1(S237);TBC1D22A(S167);TBKBP1(S365);TCF4(S372);TCOF1(S156);TERF2IP(S154);TEX2(S266);THRAP3(S232);TJP1(S168);TJP1(S968);TJP2(T462);TJP3(S164);TJP3(S369);TJP3(S371);TJP3(S591);TLE4(S208);TMEM201(S441);TNK2(T829);TNK2(Y827);TNKS1BP1(S429);TNKS1BP1(S872);TNKS1BP1(S893);TNKS1BP1(S983);TNRC6C(S714);TNS1(S1269);TOP2B(S1400);TP53BP1(S1317);TP53BP1(S580);TPD52(S176);TPD52L1(S149);TPD52L2(S166);TRA2A(T202);TRAF4(S426);TRAFD1(S470);TRAM1(S365);TRAPPC10(S711);TRAPPC12(S184);TRIM11(S85);TRIO(S1724);TRIP10(S296);TRMT2A(S602);TRUB1(T27);TSC1(S505);TSC22D4(S62);TTN(S1406);TVP23C(S223);UBA1(S13);UFD1(S299);ULK1(S556);ULK1(S719);UPF1(S1127);UPF3B(T169);USP1(S67);USP32(S1423);USP54(S1036);UTP20(T1741);UTP3(S365);UTP3(S368);VASN(S284);VCPIP1(S747);WDFY4(S3123);WDR20(S434);WDR44(S403);WEE1(T190);XRN2(S471);YBX1(Y162);YBX3(S293);ZBTB37(S164);ZC3H13(T364);ZC3H3(S571);ZC3HAV1(S257);ZC3HAV1(S335);ZC3HAV1(T273);ZC3HAV1(Y348);ZFC3H1(S949);ZKSCAN8(S12);ZMYND8(S425);ZNF106(S641);ZNF136(S405);ZNF185(S64);ZNF280D(S545);ZNF408(T322);ZNF513(S85);ZNF516(T930);ZNF518A(S655);ZNF552(S86);ZNF609(S1055);ZNF814(S87);ZNRF2(S21);ZRANB2(S153)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>